<commit_message>
📈 Pointage automatique du 01/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -812,6 +812,176 @@
         <v>7.91</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E12" t="n">
+        <v>41.121</v>
+      </c>
+      <c r="F12" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G12" t="n">
+        <v>164.48</v>
+      </c>
+      <c r="H12" t="n">
+        <v>25.46</v>
+      </c>
+      <c r="I12" t="n">
+        <v>18.31</v>
+      </c>
+      <c r="J12" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E13" t="n">
+        <v>21.907</v>
+      </c>
+      <c r="F13" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G13" t="n">
+        <v>65.72</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J13" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E14" t="n">
+        <v>105.22</v>
+      </c>
+      <c r="F14" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G14" t="n">
+        <v>105.22</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="J14" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E15" t="n">
+        <v>10.756</v>
+      </c>
+      <c r="F15" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G15" t="n">
+        <v>32.27</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>9</v>
+      </c>
+      <c r="D16" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E16" t="n">
+        <v>6.788</v>
+      </c>
+      <c r="F16" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G16" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4.94</v>
+      </c>
+      <c r="I16" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
📈 Pointage automatique du 02/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E7" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F7" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G7" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H7" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I7" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E8" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F8" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G8" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H8" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I8" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E9" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F9" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G9" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H9" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I9" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E10" t="n">
-        <v>11.262</v>
+        <v>40.247</v>
       </c>
       <c r="F10" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G10" t="n">
-        <v>33.79</v>
+        <v>160.99</v>
       </c>
       <c r="H10" t="n">
-        <v>2.63</v>
+        <v>21.97</v>
       </c>
       <c r="I10" t="n">
-        <v>8.44</v>
+        <v>15.8</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E11" t="n">
-        <v>6.781</v>
+        <v>22.34</v>
       </c>
       <c r="F11" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G11" t="n">
-        <v>61.03</v>
+        <v>67.02</v>
       </c>
       <c r="H11" t="n">
-        <v>4.88</v>
+        <v>1.35</v>
       </c>
       <c r="I11" t="n">
-        <v>8.69</v>
+        <v>2.06</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -979,6 +979,176 @@
         <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E17" t="n">
+        <v>10.662</v>
+      </c>
+      <c r="F17" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G17" t="n">
+        <v>31.99</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="J17" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E18" t="n">
+        <v>41.789</v>
+      </c>
+      <c r="F18" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G18" t="n">
+        <v>167.16</v>
+      </c>
+      <c r="H18" t="n">
+        <v>28.14</v>
+      </c>
+      <c r="I18" t="n">
+        <v>20.24</v>
+      </c>
+      <c r="J18" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E19" t="n">
+        <v>21.915</v>
+      </c>
+      <c r="F19" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G19" t="n">
+        <v>65.75</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="J19" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E20" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G20" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="I20" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="J20" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="F21" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G21" t="n">
+        <v>61.38</v>
+      </c>
+      <c r="H21" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="I21" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="J21" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 03/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E13" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F13" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G13" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>10.756</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>32.27</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>1.11</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>3.56</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1149,6 +1149,176 @@
         <v>9.31</v>
       </c>
       <c r="J21" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E22" t="n">
+        <v>41.336</v>
+      </c>
+      <c r="F22" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G22" t="n">
+        <v>165.34</v>
+      </c>
+      <c r="H22" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="I22" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="J22" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E23" t="n">
+        <v>21.669</v>
+      </c>
+      <c r="F23" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G23" t="n">
+        <v>65.01000000000001</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-1.01</v>
+      </c>
+      <c r="J23" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E24" t="n">
+        <v>105.78</v>
+      </c>
+      <c r="F24" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G24" t="n">
+        <v>105.78</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E25" t="n">
+        <v>10.536</v>
+      </c>
+      <c r="F25" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G25" t="n">
+        <v>31.61</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="J25" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>9</v>
+      </c>
+      <c r="D26" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E26" t="n">
+        <v>6.799</v>
+      </c>
+      <c r="F26" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G26" t="n">
+        <v>61.19</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="I26" t="n">
+        <v>8.98</v>
+      </c>
+      <c r="J26" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 04/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E14" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F14" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G14" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H14" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I14" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E22" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F22" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G22" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H22" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I22" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E23" t="n">
-        <v>21.669</v>
+        <v>10.536</v>
       </c>
       <c r="F23" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G23" t="n">
-        <v>65.01000000000001</v>
+        <v>31.61</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.66</v>
+        <v>0.45</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.01</v>
+        <v>1.44</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E24" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F24" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G24" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H24" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I24" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E25" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F25" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G25" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I25" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,31 +1294,201 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E26" t="n">
+        <v>105.78</v>
+      </c>
+      <c r="F26" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G26" t="n">
+        <v>105.78</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="I26" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="J26" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="F27" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G27" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="J27" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E28" t="n">
+        <v>40.532</v>
+      </c>
+      <c r="F28" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G28" t="n">
+        <v>162.13</v>
+      </c>
+      <c r="H28" t="n">
+        <v>23.11</v>
+      </c>
+      <c r="I28" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="J28" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E29" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="F29" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G29" t="n">
+        <v>65.94</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J29" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E30" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="F30" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G30" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="H30" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="I30" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="J30" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C31" t="n">
         <v>9</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D31" t="n">
         <v>6.239</v>
       </c>
-      <c r="E26" t="n">
-        <v>6.799</v>
-      </c>
-      <c r="F26" t="n">
+      <c r="E31" t="n">
+        <v>6.795</v>
+      </c>
+      <c r="F31" t="n">
         <v>56.15</v>
       </c>
-      <c r="G26" t="n">
-        <v>61.19</v>
-      </c>
-      <c r="H26" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="I26" t="n">
-        <v>8.98</v>
-      </c>
-      <c r="J26" t="n">
+      <c r="G31" t="n">
+        <v>61.16</v>
+      </c>
+      <c r="H31" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="I31" t="n">
+        <v>8.92</v>
+      </c>
+      <c r="J31" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 05/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E7" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F7" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G7" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H7" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I7" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E8" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F8" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G8" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H8" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I8" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E9" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F9" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G9" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H9" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I9" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E10" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F10" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G10" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H10" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I10" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E11" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F11" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G11" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H11" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I11" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D17" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E17" t="n">
-        <v>10.662</v>
+        <v>6.82</v>
       </c>
       <c r="F17" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G17" t="n">
-        <v>31.99</v>
+        <v>61.38</v>
       </c>
       <c r="H17" t="n">
-        <v>0.83</v>
+        <v>5.23</v>
       </c>
       <c r="I17" t="n">
-        <v>2.66</v>
+        <v>9.31</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E18" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F18" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G18" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H18" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I18" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E20" t="n">
-        <v>105.6</v>
+        <v>41.789</v>
       </c>
       <c r="F20" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G20" t="n">
-        <v>105.6</v>
+        <v>167.16</v>
       </c>
       <c r="H20" t="n">
-        <v>5.51</v>
+        <v>28.14</v>
       </c>
       <c r="I20" t="n">
-        <v>5.51</v>
+        <v>20.24</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E21" t="n">
-        <v>6.82</v>
+        <v>10.662</v>
       </c>
       <c r="F21" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G21" t="n">
-        <v>61.38</v>
+        <v>31.99</v>
       </c>
       <c r="H21" t="n">
-        <v>5.23</v>
+        <v>0.83</v>
       </c>
       <c r="I21" t="n">
-        <v>9.31</v>
+        <v>2.66</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D27" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E27" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F27" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G27" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H27" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I27" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E28" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F28" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G28" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H28" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I28" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>40.532</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>162.13</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>23.11</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>16.62</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,31 +1464,201 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E31" t="n">
+        <v>21.98</v>
+      </c>
+      <c r="F31" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G31" t="n">
+        <v>65.94</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="J31" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E32" t="n">
+        <v>10.714</v>
+      </c>
+      <c r="F32" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G32" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I32" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="J32" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4</v>
+      </c>
+      <c r="D33" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E33" t="n">
+        <v>38.849</v>
+      </c>
+      <c r="F33" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G33" t="n">
+        <v>155.4</v>
+      </c>
+      <c r="H33" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="I33" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="J33" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E34" t="n">
+        <v>22.053</v>
+      </c>
+      <c r="F34" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G34" t="n">
+        <v>66.16</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J34" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E35" t="n">
+        <v>103.08</v>
+      </c>
+      <c r="F35" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G35" t="n">
+        <v>103.08</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="I35" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="J35" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C36" t="n">
         <v>9</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D36" t="n">
         <v>6.239</v>
       </c>
-      <c r="E31" t="n">
-        <v>6.795</v>
-      </c>
-      <c r="F31" t="n">
+      <c r="E36" t="n">
+        <v>6.762</v>
+      </c>
+      <c r="F36" t="n">
         <v>56.15</v>
       </c>
-      <c r="G31" t="n">
-        <v>61.16</v>
-      </c>
-      <c r="H31" t="n">
-        <v>5.01</v>
-      </c>
-      <c r="I31" t="n">
-        <v>8.92</v>
-      </c>
-      <c r="J31" t="n">
+      <c r="G36" t="n">
+        <v>60.86</v>
+      </c>
+      <c r="H36" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="I36" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="J36" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 08/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E7" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F7" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G7" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H7" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I7" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E8" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F8" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G8" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H8" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I8" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E9" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F9" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G9" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H9" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I9" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E10" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F10" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G10" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H10" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I10" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E11" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F11" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G11" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H11" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I11" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E17" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F17" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G17" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H17" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I17" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E18" t="n">
-        <v>105.6</v>
+        <v>21.915</v>
       </c>
       <c r="F18" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G18" t="n">
-        <v>105.6</v>
+        <v>65.75</v>
       </c>
       <c r="H18" t="n">
-        <v>5.51</v>
+        <v>0.08</v>
       </c>
       <c r="I18" t="n">
-        <v>5.51</v>
+        <v>0.12</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E19" t="n">
-        <v>21.915</v>
+        <v>10.662</v>
       </c>
       <c r="F19" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G19" t="n">
-        <v>65.75</v>
+        <v>31.99</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08</v>
+        <v>0.83</v>
       </c>
       <c r="I19" t="n">
-        <v>0.12</v>
+        <v>2.66</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E20" t="n">
-        <v>41.789</v>
+        <v>6.82</v>
       </c>
       <c r="F20" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G20" t="n">
-        <v>167.16</v>
+        <v>61.38</v>
       </c>
       <c r="H20" t="n">
-        <v>28.14</v>
+        <v>5.23</v>
       </c>
       <c r="I20" t="n">
-        <v>20.24</v>
+        <v>9.31</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E21" t="n">
-        <v>10.662</v>
+        <v>105.6</v>
       </c>
       <c r="F21" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G21" t="n">
-        <v>31.99</v>
+        <v>105.6</v>
       </c>
       <c r="H21" t="n">
-        <v>0.83</v>
+        <v>5.51</v>
       </c>
       <c r="I21" t="n">
-        <v>2.66</v>
+        <v>5.51</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>6.795</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>61.16</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>5.01</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>8.92</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E28" t="n">
-        <v>104.9</v>
+        <v>40.532</v>
       </c>
       <c r="F28" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G28" t="n">
-        <v>104.9</v>
+        <v>162.13</v>
       </c>
       <c r="H28" t="n">
-        <v>4.81</v>
+        <v>23.11</v>
       </c>
       <c r="I28" t="n">
-        <v>4.81</v>
+        <v>16.62</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E29" t="n">
-        <v>40.532</v>
+        <v>10.66</v>
       </c>
       <c r="F29" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G29" t="n">
-        <v>162.13</v>
+        <v>31.98</v>
       </c>
       <c r="H29" t="n">
-        <v>23.11</v>
+        <v>0.82</v>
       </c>
       <c r="I29" t="n">
-        <v>16.62</v>
+        <v>2.63</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>104.9</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>104.9</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>4.81</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>4.81</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1659,6 +1659,176 @@
         <v>8.390000000000001</v>
       </c>
       <c r="J36" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E37" t="n">
+        <v>10.67</v>
+      </c>
+      <c r="F37" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G37" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="I37" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="J37" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>4</v>
+      </c>
+      <c r="D38" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E38" t="n">
+        <v>38.879</v>
+      </c>
+      <c r="F38" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G38" t="n">
+        <v>155.52</v>
+      </c>
+      <c r="H38" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I38" t="n">
+        <v>11.87</v>
+      </c>
+      <c r="J38" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E39" t="n">
+        <v>21.839</v>
+      </c>
+      <c r="F39" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G39" t="n">
+        <v>65.52</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="J39" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E40" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="F40" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G40" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="H40" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="I40" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="J40" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>9</v>
+      </c>
+      <c r="D41" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6.728</v>
+      </c>
+      <c r="F41" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G41" t="n">
+        <v>60.55</v>
+      </c>
+      <c r="H41" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="I41" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="J41" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 09/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>41.121</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>164.48</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>25.46</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>18.31</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E22" t="n">
-        <v>6.799</v>
+        <v>105.78</v>
       </c>
       <c r="F22" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G22" t="n">
-        <v>61.19</v>
+        <v>105.78</v>
       </c>
       <c r="H22" t="n">
-        <v>5.04</v>
+        <v>5.69</v>
       </c>
       <c r="I22" t="n">
-        <v>8.98</v>
+        <v>5.68</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E23" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F23" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G23" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H23" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I23" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E25" t="n">
-        <v>41.336</v>
+        <v>10.536</v>
       </c>
       <c r="F25" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G25" t="n">
-        <v>165.34</v>
+        <v>31.61</v>
       </c>
       <c r="H25" t="n">
-        <v>26.32</v>
+        <v>0.45</v>
       </c>
       <c r="I25" t="n">
-        <v>18.93</v>
+        <v>1.44</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E26" t="n">
-        <v>105.78</v>
+        <v>6.799</v>
       </c>
       <c r="F26" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G26" t="n">
-        <v>105.78</v>
+        <v>61.19</v>
       </c>
       <c r="H26" t="n">
-        <v>5.69</v>
+        <v>5.04</v>
       </c>
       <c r="I26" t="n">
-        <v>5.68</v>
+        <v>8.98</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E32" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F32" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G32" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H32" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I32" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E33" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F33" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G33" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H33" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I33" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E34" t="n">
-        <v>22.053</v>
+        <v>103.08</v>
       </c>
       <c r="F34" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G34" t="n">
-        <v>66.16</v>
+        <v>103.08</v>
       </c>
       <c r="H34" t="n">
-        <v>0.49</v>
+        <v>2.99</v>
       </c>
       <c r="I34" t="n">
-        <v>0.75</v>
+        <v>2.99</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E35" t="n">
-        <v>103.08</v>
+        <v>10.714</v>
       </c>
       <c r="F35" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G35" t="n">
-        <v>103.08</v>
+        <v>32.14</v>
       </c>
       <c r="H35" t="n">
-        <v>2.99</v>
+        <v>0.98</v>
       </c>
       <c r="I35" t="n">
-        <v>2.99</v>
+        <v>3.15</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E36" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F36" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G36" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H36" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I36" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1829,6 +1829,176 @@
         <v>7.84</v>
       </c>
       <c r="J41" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>3</v>
+      </c>
+      <c r="D42" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E42" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="F42" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G42" t="n">
+        <v>31.83</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="J42" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E43" t="n">
+        <v>38.497</v>
+      </c>
+      <c r="F43" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G43" t="n">
+        <v>153.99</v>
+      </c>
+      <c r="H43" t="n">
+        <v>14.97</v>
+      </c>
+      <c r="I43" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="J43" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>3</v>
+      </c>
+      <c r="D44" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E44" t="n">
+        <v>22</v>
+      </c>
+      <c r="F44" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G44" t="n">
+        <v>66</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J44" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E45" t="n">
+        <v>100.06</v>
+      </c>
+      <c r="F45" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G45" t="n">
+        <v>100.06</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="J45" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>9</v>
+      </c>
+      <c r="D46" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E46" t="n">
+        <v>6.629</v>
+      </c>
+      <c r="F46" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G46" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="H46" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="I46" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="J46" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 10/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
+  <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E22" t="n">
-        <v>105.78</v>
+        <v>10.536</v>
       </c>
       <c r="F22" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G22" t="n">
-        <v>105.78</v>
+        <v>31.61</v>
       </c>
       <c r="H22" t="n">
-        <v>5.69</v>
+        <v>0.45</v>
       </c>
       <c r="I22" t="n">
-        <v>5.68</v>
+        <v>1.44</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E23" t="n">
-        <v>41.336</v>
+        <v>21.669</v>
       </c>
       <c r="F23" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G23" t="n">
-        <v>165.34</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>26.32</v>
+        <v>-0.66</v>
       </c>
       <c r="I23" t="n">
-        <v>18.93</v>
+        <v>-1.01</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E24" t="n">
-        <v>21.669</v>
+        <v>6.799</v>
       </c>
       <c r="F24" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G24" t="n">
-        <v>65.01000000000001</v>
+        <v>61.19</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.66</v>
+        <v>5.04</v>
       </c>
       <c r="I24" t="n">
-        <v>-1.01</v>
+        <v>8.98</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E25" t="n">
-        <v>10.536</v>
+        <v>105.78</v>
       </c>
       <c r="F25" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G25" t="n">
-        <v>31.61</v>
+        <v>105.78</v>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>5.69</v>
       </c>
       <c r="I25" t="n">
-        <v>1.44</v>
+        <v>5.68</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E26" t="n">
-        <v>6.799</v>
+        <v>41.336</v>
       </c>
       <c r="F26" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G26" t="n">
-        <v>61.19</v>
+        <v>165.34</v>
       </c>
       <c r="H26" t="n">
-        <v>5.04</v>
+        <v>26.32</v>
       </c>
       <c r="I26" t="n">
-        <v>8.98</v>
+        <v>18.93</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D37" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E37" t="n">
-        <v>10.67</v>
+        <v>6.728</v>
       </c>
       <c r="F37" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G37" t="n">
-        <v>32.01</v>
+        <v>60.55</v>
       </c>
       <c r="H37" t="n">
-        <v>0.85</v>
+        <v>4.4</v>
       </c>
       <c r="I37" t="n">
-        <v>2.73</v>
+        <v>7.84</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E38" t="n">
-        <v>38.879</v>
+        <v>102.8</v>
       </c>
       <c r="F38" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G38" t="n">
-        <v>155.52</v>
+        <v>102.8</v>
       </c>
       <c r="H38" t="n">
-        <v>16.5</v>
+        <v>2.71</v>
       </c>
       <c r="I38" t="n">
-        <v>11.87</v>
+        <v>2.71</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E39" t="n">
-        <v>21.839</v>
+        <v>38.879</v>
       </c>
       <c r="F39" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G39" t="n">
-        <v>65.52</v>
+        <v>155.52</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.15</v>
+        <v>16.5</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.23</v>
+        <v>11.87</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E40" t="n">
-        <v>102.8</v>
+        <v>10.67</v>
       </c>
       <c r="F40" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G40" t="n">
-        <v>102.8</v>
+        <v>32.01</v>
       </c>
       <c r="H40" t="n">
-        <v>2.71</v>
+        <v>0.85</v>
       </c>
       <c r="I40" t="n">
-        <v>2.71</v>
+        <v>2.73</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E41" t="n">
-        <v>6.728</v>
+        <v>21.839</v>
       </c>
       <c r="F41" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G41" t="n">
-        <v>60.55</v>
+        <v>65.52</v>
       </c>
       <c r="H41" t="n">
-        <v>4.4</v>
+        <v>-0.15</v>
       </c>
       <c r="I41" t="n">
-        <v>7.84</v>
+        <v>-0.23</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -1999,6 +1999,176 @@
         <v>6.25</v>
       </c>
       <c r="J46" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E47" t="n">
+        <v>10.562</v>
+      </c>
+      <c r="F47" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G47" t="n">
+        <v>31.69</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J47" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E48" t="n">
+        <v>38.312</v>
+      </c>
+      <c r="F48" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G48" t="n">
+        <v>153.25</v>
+      </c>
+      <c r="H48" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="I48" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="J48" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E49" t="n">
+        <v>21.778</v>
+      </c>
+      <c r="F49" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G49" t="n">
+        <v>65.33</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="J49" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E50" t="n">
+        <v>99.83</v>
+      </c>
+      <c r="F50" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G50" t="n">
+        <v>99.83</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="J50" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>9</v>
+      </c>
+      <c r="D51" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E51" t="n">
+        <v>6.622</v>
+      </c>
+      <c r="F51" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G51" t="n">
+        <v>59.6</v>
+      </c>
+      <c r="H51" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="I51" t="n">
+        <v>6.14</v>
+      </c>
+      <c r="J51" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 11/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>105.22</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>105.22</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>5.13</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>5.13</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>104.9</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>104.9</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>4.81</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>4.81</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E28" t="n">
-        <v>40.532</v>
+        <v>6.795</v>
       </c>
       <c r="F28" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G28" t="n">
-        <v>162.13</v>
+        <v>61.16</v>
       </c>
       <c r="H28" t="n">
-        <v>23.11</v>
+        <v>5.01</v>
       </c>
       <c r="I28" t="n">
-        <v>16.62</v>
+        <v>8.92</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E30" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F30" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G30" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H30" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I30" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E31" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F31" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G31" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H31" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I31" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>6.629</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>59.66</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>3.51</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>6.25</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>38.497</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>153.99</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>14.97</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>10.77</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E46" t="n">
-        <v>6.629</v>
+        <v>22</v>
       </c>
       <c r="F46" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G46" t="n">
-        <v>59.66</v>
+        <v>66</v>
       </c>
       <c r="H46" t="n">
-        <v>3.51</v>
+        <v>0.33</v>
       </c>
       <c r="I46" t="n">
-        <v>6.25</v>
+        <v>0.5</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2169,6 +2169,176 @@
         <v>6.14</v>
       </c>
       <c r="J51" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>3</v>
+      </c>
+      <c r="D52" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E52" t="n">
+        <v>10.702</v>
+      </c>
+      <c r="F52" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G52" t="n">
+        <v>32.11</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="I52" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="J52" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>4</v>
+      </c>
+      <c r="D53" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E53" t="n">
+        <v>38.544</v>
+      </c>
+      <c r="F53" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G53" t="n">
+        <v>154.18</v>
+      </c>
+      <c r="H53" t="n">
+        <v>15.16</v>
+      </c>
+      <c r="I53" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="J53" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>3</v>
+      </c>
+      <c r="D54" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E54" t="n">
+        <v>21.703</v>
+      </c>
+      <c r="F54" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G54" t="n">
+        <v>65.11</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="J54" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E55" t="n">
+        <v>100.34</v>
+      </c>
+      <c r="F55" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G55" t="n">
+        <v>100.34</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J55" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>9</v>
+      </c>
+      <c r="D56" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E56" t="n">
+        <v>6.629</v>
+      </c>
+      <c r="F56" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G56" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="H56" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="I56" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="J56" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 12/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>105.22</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>105.22</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>5.13</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>5.13</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>41.121</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>164.48</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>25.46</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>18.31</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E27" t="n">
-        <v>104.9</v>
+        <v>40.532</v>
       </c>
       <c r="F27" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G27" t="n">
-        <v>104.9</v>
+        <v>162.13</v>
       </c>
       <c r="H27" t="n">
-        <v>4.81</v>
+        <v>23.11</v>
       </c>
       <c r="I27" t="n">
-        <v>4.81</v>
+        <v>16.62</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E28" t="n">
-        <v>6.795</v>
+        <v>10.66</v>
       </c>
       <c r="F28" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G28" t="n">
-        <v>61.16</v>
+        <v>31.98</v>
       </c>
       <c r="H28" t="n">
-        <v>5.01</v>
+        <v>0.82</v>
       </c>
       <c r="I28" t="n">
-        <v>8.92</v>
+        <v>2.63</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E29" t="n">
-        <v>10.66</v>
+        <v>21.98</v>
       </c>
       <c r="F29" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G29" t="n">
-        <v>31.98</v>
+        <v>65.94</v>
       </c>
       <c r="H29" t="n">
-        <v>0.82</v>
+        <v>0.27</v>
       </c>
       <c r="I29" t="n">
-        <v>2.63</v>
+        <v>0.41</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E30" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F30" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G30" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H30" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I30" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E42" t="n">
-        <v>6.629</v>
+        <v>22</v>
       </c>
       <c r="F42" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G42" t="n">
-        <v>59.66</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>3.51</v>
+        <v>0.33</v>
       </c>
       <c r="I42" t="n">
-        <v>6.25</v>
+        <v>0.5</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>100.06</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>100.06</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.03</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.03</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E44" t="n">
-        <v>38.497</v>
+        <v>10.61</v>
       </c>
       <c r="F44" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G44" t="n">
-        <v>153.99</v>
+        <v>31.83</v>
       </c>
       <c r="H44" t="n">
-        <v>14.97</v>
+        <v>0.67</v>
       </c>
       <c r="I44" t="n">
-        <v>10.77</v>
+        <v>2.15</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D45" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E45" t="n">
-        <v>10.61</v>
+        <v>6.629</v>
       </c>
       <c r="F45" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G45" t="n">
-        <v>31.83</v>
+        <v>59.66</v>
       </c>
       <c r="H45" t="n">
-        <v>0.67</v>
+        <v>3.51</v>
       </c>
       <c r="I45" t="n">
-        <v>2.15</v>
+        <v>6.25</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E46" t="n">
-        <v>22</v>
+        <v>100.06</v>
       </c>
       <c r="F46" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G46" t="n">
-        <v>66</v>
+        <v>100.06</v>
       </c>
       <c r="H46" t="n">
-        <v>0.33</v>
+        <v>-0.03</v>
       </c>
       <c r="I46" t="n">
-        <v>0.5</v>
+        <v>-0.03</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D52" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E52" t="n">
-        <v>10.702</v>
+        <v>6.629</v>
       </c>
       <c r="F52" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G52" t="n">
-        <v>32.11</v>
+        <v>59.66</v>
       </c>
       <c r="H52" t="n">
-        <v>0.95</v>
+        <v>3.51</v>
       </c>
       <c r="I52" t="n">
-        <v>3.05</v>
+        <v>6.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E53" t="n">
-        <v>38.544</v>
+        <v>100.34</v>
       </c>
       <c r="F53" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G53" t="n">
-        <v>154.18</v>
+        <v>100.34</v>
       </c>
       <c r="H53" t="n">
-        <v>15.16</v>
+        <v>0.25</v>
       </c>
       <c r="I53" t="n">
-        <v>10.9</v>
+        <v>0.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E54" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F54" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G54" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H54" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E55" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F55" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G55" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H55" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I55" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,31 +2314,201 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>3</v>
+      </c>
+      <c r="D56" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E56" t="n">
+        <v>21.703</v>
+      </c>
+      <c r="F56" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G56" t="n">
+        <v>65.11</v>
+      </c>
+      <c r="H56" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-0.85</v>
+      </c>
+      <c r="J56" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>3</v>
+      </c>
+      <c r="D57" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E57" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F57" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G57" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="H57" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="I57" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J57" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E58" t="n">
+        <v>39.845</v>
+      </c>
+      <c r="F58" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G58" t="n">
+        <v>159.38</v>
+      </c>
+      <c r="H58" t="n">
+        <v>20.36</v>
+      </c>
+      <c r="I58" t="n">
+        <v>14.65</v>
+      </c>
+      <c r="J58" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>3</v>
+      </c>
+      <c r="D59" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E59" t="n">
+        <v>22.289</v>
+      </c>
+      <c r="F59" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G59" t="n">
+        <v>66.87</v>
+      </c>
+      <c r="H59" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I59" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="J59" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E60" t="n">
+        <v>102.86</v>
+      </c>
+      <c r="F60" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G60" t="n">
+        <v>102.86</v>
+      </c>
+      <c r="H60" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I60" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="J60" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C56" t="n">
+      <c r="C61" t="n">
         <v>9</v>
       </c>
-      <c r="D56" t="n">
+      <c r="D61" t="n">
         <v>6.239</v>
       </c>
-      <c r="E56" t="n">
-        <v>6.629</v>
-      </c>
-      <c r="F56" t="n">
+      <c r="E61" t="n">
+        <v>6.736</v>
+      </c>
+      <c r="F61" t="n">
         <v>56.15</v>
       </c>
-      <c r="G56" t="n">
-        <v>59.66</v>
-      </c>
-      <c r="H56" t="n">
-        <v>3.51</v>
-      </c>
-      <c r="I56" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="J56" t="n">
+      <c r="G61" t="n">
+        <v>60.62</v>
+      </c>
+      <c r="H61" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="I61" t="n">
+        <v>7.96</v>
+      </c>
+      <c r="J61" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 15/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E7" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F7" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G7" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H7" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I7" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E8" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F8" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G8" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H8" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I8" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E9" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F9" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G9" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H9" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I9" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E10" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F10" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G10" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H10" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I10" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E11" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F11" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G11" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H11" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I11" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E17" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F17" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G17" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H17" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I17" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E18" t="n">
-        <v>21.915</v>
+        <v>6.82</v>
       </c>
       <c r="F18" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G18" t="n">
-        <v>65.75</v>
+        <v>61.38</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08</v>
+        <v>5.23</v>
       </c>
       <c r="I18" t="n">
-        <v>0.12</v>
+        <v>9.31</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E19" t="n">
-        <v>10.662</v>
+        <v>41.789</v>
       </c>
       <c r="F19" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G19" t="n">
-        <v>31.99</v>
+        <v>167.16</v>
       </c>
       <c r="H19" t="n">
-        <v>0.83</v>
+        <v>28.14</v>
       </c>
       <c r="I19" t="n">
-        <v>2.66</v>
+        <v>20.24</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E20" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F20" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G20" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H20" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I20" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E21" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F21" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G21" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H21" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I21" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E32" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F32" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G32" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H32" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I32" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E33" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F33" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G33" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H33" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I33" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E35" t="n">
-        <v>10.714</v>
+        <v>22.053</v>
       </c>
       <c r="F35" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G35" t="n">
-        <v>32.14</v>
+        <v>66.16</v>
       </c>
       <c r="H35" t="n">
-        <v>0.98</v>
+        <v>0.49</v>
       </c>
       <c r="I35" t="n">
-        <v>3.15</v>
+        <v>0.75</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D36" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E36" t="n">
-        <v>38.849</v>
+        <v>6.762</v>
       </c>
       <c r="F36" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G36" t="n">
-        <v>155.4</v>
+        <v>60.86</v>
       </c>
       <c r="H36" t="n">
-        <v>16.38</v>
+        <v>4.71</v>
       </c>
       <c r="I36" t="n">
-        <v>11.78</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E47" t="n">
-        <v>10.562</v>
+        <v>6.622</v>
       </c>
       <c r="F47" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G47" t="n">
-        <v>31.69</v>
+        <v>59.6</v>
       </c>
       <c r="H47" t="n">
-        <v>0.53</v>
+        <v>3.45</v>
       </c>
       <c r="I47" t="n">
-        <v>1.7</v>
+        <v>6.14</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E48" t="n">
-        <v>38.312</v>
+        <v>21.778</v>
       </c>
       <c r="F48" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G48" t="n">
-        <v>153.25</v>
+        <v>65.33</v>
       </c>
       <c r="H48" t="n">
-        <v>14.23</v>
+        <v>-0.34</v>
       </c>
       <c r="I48" t="n">
-        <v>10.24</v>
+        <v>-0.52</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E49" t="n">
-        <v>21.778</v>
+        <v>99.83</v>
       </c>
       <c r="F49" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G49" t="n">
-        <v>65.33</v>
+        <v>99.83</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.34</v>
+        <v>-0.26</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.52</v>
+        <v>-0.26</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E50" t="n">
-        <v>99.83</v>
+        <v>10.562</v>
       </c>
       <c r="F50" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G50" t="n">
-        <v>99.83</v>
+        <v>31.69</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.26</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.26</v>
+        <v>1.7</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D51" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E51" t="n">
-        <v>6.622</v>
+        <v>38.312</v>
       </c>
       <c r="F51" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G51" t="n">
-        <v>59.6</v>
+        <v>153.25</v>
       </c>
       <c r="H51" t="n">
-        <v>3.45</v>
+        <v>14.23</v>
       </c>
       <c r="I51" t="n">
-        <v>6.14</v>
+        <v>10.24</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D57" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E57" t="n">
-        <v>10.75</v>
+        <v>39.845</v>
       </c>
       <c r="F57" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G57" t="n">
-        <v>32.25</v>
+        <v>159.38</v>
       </c>
       <c r="H57" t="n">
-        <v>1.09</v>
+        <v>20.36</v>
       </c>
       <c r="I57" t="n">
-        <v>3.5</v>
+        <v>14.65</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>10.75</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>32.25</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>1.09</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>3.5</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2509,6 +2509,176 @@
         <v>7.96</v>
       </c>
       <c r="J61" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E62" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="F62" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G62" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="H62" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="I62" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="J62" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>3</v>
+      </c>
+      <c r="D63" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E63" t="n">
+        <v>10.712</v>
+      </c>
+      <c r="F63" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G63" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I63" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="J63" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D64" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E64" t="n">
+        <v>41.064</v>
+      </c>
+      <c r="F64" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G64" t="n">
+        <v>164.26</v>
+      </c>
+      <c r="H64" t="n">
+        <v>25.24</v>
+      </c>
+      <c r="I64" t="n">
+        <v>18.16</v>
+      </c>
+      <c r="J64" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>3</v>
+      </c>
+      <c r="D65" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E65" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="F65" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G65" t="n">
+        <v>68.09999999999999</v>
+      </c>
+      <c r="H65" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="I65" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J65" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>9</v>
+      </c>
+      <c r="D66" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E66" t="n">
+        <v>6.817</v>
+      </c>
+      <c r="F66" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G66" t="n">
+        <v>61.35</v>
+      </c>
+      <c r="H66" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I66" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="J66" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 16/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E7" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F7" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G7" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H7" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I7" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E8" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F8" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G8" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H8" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I8" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E9" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F9" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G9" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H9" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I9" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E10" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F10" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G10" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H10" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I10" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E11" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F11" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G11" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H11" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I11" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E17" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F17" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G17" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H17" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I17" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E18" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F18" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G18" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H18" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I18" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E19" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F19" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G19" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H19" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I19" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E20" t="n">
-        <v>21.915</v>
+        <v>6.82</v>
       </c>
       <c r="F20" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G20" t="n">
-        <v>65.75</v>
+        <v>61.38</v>
       </c>
       <c r="H20" t="n">
-        <v>0.08</v>
+        <v>5.23</v>
       </c>
       <c r="I20" t="n">
-        <v>0.12</v>
+        <v>9.31</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E21" t="n">
-        <v>10.662</v>
+        <v>41.789</v>
       </c>
       <c r="F21" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G21" t="n">
-        <v>31.99</v>
+        <v>167.16</v>
       </c>
       <c r="H21" t="n">
-        <v>0.83</v>
+        <v>28.14</v>
       </c>
       <c r="I21" t="n">
-        <v>2.66</v>
+        <v>20.24</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E32" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F32" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G32" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H32" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I32" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E33" t="n">
-        <v>10.714</v>
+        <v>103.08</v>
       </c>
       <c r="F33" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G33" t="n">
-        <v>32.14</v>
+        <v>103.08</v>
       </c>
       <c r="H33" t="n">
-        <v>0.98</v>
+        <v>2.99</v>
       </c>
       <c r="I33" t="n">
-        <v>3.15</v>
+        <v>2.99</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E34" t="n">
-        <v>103.08</v>
+        <v>6.762</v>
       </c>
       <c r="F34" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G34" t="n">
-        <v>103.08</v>
+        <v>60.86</v>
       </c>
       <c r="H34" t="n">
-        <v>2.99</v>
+        <v>4.71</v>
       </c>
       <c r="I34" t="n">
-        <v>2.99</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E35" t="n">
-        <v>22.053</v>
+        <v>38.849</v>
       </c>
       <c r="F35" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G35" t="n">
-        <v>66.16</v>
+        <v>155.4</v>
       </c>
       <c r="H35" t="n">
-        <v>0.49</v>
+        <v>16.38</v>
       </c>
       <c r="I35" t="n">
-        <v>0.75</v>
+        <v>11.78</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E36" t="n">
-        <v>6.762</v>
+        <v>10.714</v>
       </c>
       <c r="F36" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G36" t="n">
-        <v>60.86</v>
+        <v>32.14</v>
       </c>
       <c r="H36" t="n">
-        <v>4.71</v>
+        <v>0.98</v>
       </c>
       <c r="I36" t="n">
-        <v>8.390000000000001</v>
+        <v>3.15</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E42" t="n">
-        <v>22</v>
+        <v>100.06</v>
       </c>
       <c r="F42" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>100.06</v>
       </c>
       <c r="H42" t="n">
-        <v>0.33</v>
+        <v>-0.03</v>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>-0.03</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E45" t="n">
-        <v>6.629</v>
+        <v>38.497</v>
       </c>
       <c r="F45" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G45" t="n">
-        <v>59.66</v>
+        <v>153.99</v>
       </c>
       <c r="H45" t="n">
-        <v>3.51</v>
+        <v>14.97</v>
       </c>
       <c r="I45" t="n">
-        <v>6.25</v>
+        <v>10.77</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E46" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F46" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G46" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E52" t="n">
-        <v>6.629</v>
+        <v>10.702</v>
       </c>
       <c r="F52" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G52" t="n">
-        <v>59.66</v>
+        <v>32.11</v>
       </c>
       <c r="H52" t="n">
-        <v>3.51</v>
+        <v>0.95</v>
       </c>
       <c r="I52" t="n">
-        <v>6.25</v>
+        <v>3.05</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E53" t="n">
-        <v>100.34</v>
+        <v>21.703</v>
       </c>
       <c r="F53" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G53" t="n">
-        <v>100.34</v>
+        <v>65.11</v>
       </c>
       <c r="H53" t="n">
-        <v>0.25</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>0.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E54" t="n">
-        <v>38.544</v>
+        <v>100.34</v>
       </c>
       <c r="F54" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G54" t="n">
-        <v>154.18</v>
+        <v>100.34</v>
       </c>
       <c r="H54" t="n">
-        <v>15.16</v>
+        <v>0.25</v>
       </c>
       <c r="I54" t="n">
-        <v>10.9</v>
+        <v>0.25</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E55" t="n">
-        <v>10.702</v>
+        <v>6.629</v>
       </c>
       <c r="F55" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G55" t="n">
-        <v>32.11</v>
+        <v>59.66</v>
       </c>
       <c r="H55" t="n">
-        <v>0.95</v>
+        <v>3.51</v>
       </c>
       <c r="I55" t="n">
-        <v>3.05</v>
+        <v>6.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D56" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E56" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F56" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G56" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D62" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E62" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F62" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G62" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H62" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E64" t="n">
-        <v>41.064</v>
+        <v>10.712</v>
       </c>
       <c r="F64" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G64" t="n">
-        <v>164.26</v>
+        <v>32.14</v>
       </c>
       <c r="H64" t="n">
-        <v>25.24</v>
+        <v>0.98</v>
       </c>
       <c r="I64" t="n">
-        <v>18.16</v>
+        <v>3.15</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>105.5</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>105.5</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>5.41</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>5.41</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,31 +2654,201 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>4</v>
+      </c>
+      <c r="D66" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E66" t="n">
+        <v>41.064</v>
+      </c>
+      <c r="F66" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G66" t="n">
+        <v>164.26</v>
+      </c>
+      <c r="H66" t="n">
+        <v>25.24</v>
+      </c>
+      <c r="I66" t="n">
+        <v>18.16</v>
+      </c>
+      <c r="J66" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>3</v>
+      </c>
+      <c r="D67" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E67" t="n">
+        <v>10.796</v>
+      </c>
+      <c r="F67" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G67" t="n">
+        <v>32.39</v>
+      </c>
+      <c r="H67" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="I67" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="J67" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>4</v>
+      </c>
+      <c r="D68" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E68" t="n">
+        <v>40.567</v>
+      </c>
+      <c r="F68" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G68" t="n">
+        <v>162.27</v>
+      </c>
+      <c r="H68" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="I68" t="n">
+        <v>16.72</v>
+      </c>
+      <c r="J68" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>3</v>
+      </c>
+      <c r="D69" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E69" t="n">
+        <v>22.797</v>
+      </c>
+      <c r="F69" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G69" t="n">
+        <v>68.39</v>
+      </c>
+      <c r="H69" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="I69" t="n">
+        <v>4.14</v>
+      </c>
+      <c r="J69" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E70" t="n">
+        <v>104.58</v>
+      </c>
+      <c r="F70" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G70" t="n">
+        <v>104.58</v>
+      </c>
+      <c r="H70" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="I70" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="J70" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C66" t="n">
+      <c r="C71" t="n">
         <v>9</v>
       </c>
-      <c r="D66" t="n">
+      <c r="D71" t="n">
         <v>6.239</v>
       </c>
-      <c r="E66" t="n">
-        <v>6.817</v>
-      </c>
-      <c r="F66" t="n">
+      <c r="E71" t="n">
+        <v>6.807</v>
+      </c>
+      <c r="F71" t="n">
         <v>56.15</v>
       </c>
-      <c r="G66" t="n">
-        <v>61.35</v>
-      </c>
-      <c r="H66" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="I66" t="n">
-        <v>9.26</v>
-      </c>
-      <c r="J66" t="n">
+      <c r="G71" t="n">
+        <v>61.26</v>
+      </c>
+      <c r="H71" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="I71" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="J71" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 17/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E7" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F7" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G7" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H7" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I7" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E8" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F8" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G8" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H8" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I8" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E9" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F9" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G9" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H9" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I9" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E10" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F10" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G10" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H10" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I10" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E11" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F11" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G11" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H11" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I11" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E17" t="n">
-        <v>10.662</v>
+        <v>41.789</v>
       </c>
       <c r="F17" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G17" t="n">
-        <v>31.99</v>
+        <v>167.16</v>
       </c>
       <c r="H17" t="n">
-        <v>0.83</v>
+        <v>28.14</v>
       </c>
       <c r="I17" t="n">
-        <v>2.66</v>
+        <v>20.24</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E18" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F18" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G18" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I18" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E19" t="n">
-        <v>105.6</v>
+        <v>6.82</v>
       </c>
       <c r="F19" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G19" t="n">
-        <v>105.6</v>
+        <v>61.38</v>
       </c>
       <c r="H19" t="n">
-        <v>5.51</v>
+        <v>5.23</v>
       </c>
       <c r="I19" t="n">
-        <v>5.51</v>
+        <v>9.31</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E20" t="n">
-        <v>6.82</v>
+        <v>10.662</v>
       </c>
       <c r="F20" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G20" t="n">
-        <v>61.38</v>
+        <v>31.99</v>
       </c>
       <c r="H20" t="n">
-        <v>5.23</v>
+        <v>0.83</v>
       </c>
       <c r="I20" t="n">
-        <v>9.31</v>
+        <v>2.66</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E21" t="n">
-        <v>41.789</v>
+        <v>21.915</v>
       </c>
       <c r="F21" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G21" t="n">
-        <v>167.16</v>
+        <v>65.75</v>
       </c>
       <c r="H21" t="n">
-        <v>28.14</v>
+        <v>0.08</v>
       </c>
       <c r="I21" t="n">
-        <v>20.24</v>
+        <v>0.12</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E28" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F28" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G28" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H28" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I28" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>104.9</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>104.9</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>4.81</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>4.81</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E31" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F31" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G31" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H31" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I31" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E37" t="n">
-        <v>6.728</v>
+        <v>21.839</v>
       </c>
       <c r="F37" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G37" t="n">
-        <v>60.55</v>
+        <v>65.52</v>
       </c>
       <c r="H37" t="n">
-        <v>4.4</v>
+        <v>-0.15</v>
       </c>
       <c r="I37" t="n">
-        <v>7.84</v>
+        <v>-0.23</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E38" t="n">
-        <v>102.8</v>
+        <v>10.67</v>
       </c>
       <c r="F38" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G38" t="n">
-        <v>102.8</v>
+        <v>32.01</v>
       </c>
       <c r="H38" t="n">
-        <v>2.71</v>
+        <v>0.85</v>
       </c>
       <c r="I38" t="n">
-        <v>2.71</v>
+        <v>2.73</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E40" t="n">
-        <v>10.67</v>
+        <v>102.8</v>
       </c>
       <c r="F40" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G40" t="n">
-        <v>32.01</v>
+        <v>102.8</v>
       </c>
       <c r="H40" t="n">
-        <v>0.85</v>
+        <v>2.71</v>
       </c>
       <c r="I40" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D41" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E41" t="n">
-        <v>21.839</v>
+        <v>6.728</v>
       </c>
       <c r="F41" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G41" t="n">
-        <v>65.52</v>
+        <v>60.55</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.15</v>
+        <v>4.4</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.23</v>
+        <v>7.84</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E47" t="n">
-        <v>6.622</v>
+        <v>38.312</v>
       </c>
       <c r="F47" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G47" t="n">
-        <v>59.6</v>
+        <v>153.25</v>
       </c>
       <c r="H47" t="n">
-        <v>3.45</v>
+        <v>14.23</v>
       </c>
       <c r="I47" t="n">
-        <v>6.14</v>
+        <v>10.24</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E48" t="n">
-        <v>21.778</v>
+        <v>10.562</v>
       </c>
       <c r="F48" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G48" t="n">
-        <v>65.33</v>
+        <v>31.69</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.34</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.52</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E50" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F50" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G50" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I50" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D51" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E51" t="n">
-        <v>38.312</v>
+        <v>6.622</v>
       </c>
       <c r="F51" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G51" t="n">
-        <v>153.25</v>
+        <v>59.6</v>
       </c>
       <c r="H51" t="n">
-        <v>14.23</v>
+        <v>3.45</v>
       </c>
       <c r="I51" t="n">
-        <v>10.24</v>
+        <v>6.14</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D57" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E57" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F57" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G57" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H57" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I57" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E58" t="n">
-        <v>10.75</v>
+        <v>102.86</v>
       </c>
       <c r="F58" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G58" t="n">
-        <v>32.25</v>
+        <v>102.86</v>
       </c>
       <c r="H58" t="n">
-        <v>1.09</v>
+        <v>2.77</v>
       </c>
       <c r="I58" t="n">
-        <v>3.5</v>
+        <v>2.77</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>3</v>
       </c>
       <c r="D59" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E59" t="n">
-        <v>22.289</v>
+        <v>10.75</v>
       </c>
       <c r="F59" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G59" t="n">
-        <v>66.87</v>
+        <v>32.25</v>
       </c>
       <c r="H59" t="n">
-        <v>1.2</v>
+        <v>1.09</v>
       </c>
       <c r="I59" t="n">
-        <v>1.83</v>
+        <v>3.5</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E60" t="n">
-        <v>102.86</v>
+        <v>39.845</v>
       </c>
       <c r="F60" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G60" t="n">
-        <v>102.86</v>
+        <v>159.38</v>
       </c>
       <c r="H60" t="n">
-        <v>2.77</v>
+        <v>20.36</v>
       </c>
       <c r="I60" t="n">
-        <v>2.77</v>
+        <v>14.65</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>6.736</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>60.62</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>4.47</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>7.96</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E67" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F67" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G67" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H67" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I67" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E68" t="n">
-        <v>40.567</v>
+        <v>10.796</v>
       </c>
       <c r="F68" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G68" t="n">
-        <v>162.27</v>
+        <v>32.39</v>
       </c>
       <c r="H68" t="n">
-        <v>23.25</v>
+        <v>1.23</v>
       </c>
       <c r="I68" t="n">
-        <v>16.72</v>
+        <v>3.95</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2849,6 +2849,176 @@
         <v>9.1</v>
       </c>
       <c r="J71" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>1</v>
+      </c>
+      <c r="D72" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E72" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="F72" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G72" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="H72" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="I72" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="J72" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>3</v>
+      </c>
+      <c r="D73" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E73" t="n">
+        <v>10.892</v>
+      </c>
+      <c r="F73" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G73" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="H73" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I73" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="J73" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>4</v>
+      </c>
+      <c r="D74" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E74" t="n">
+        <v>41.15</v>
+      </c>
+      <c r="F74" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G74" t="n">
+        <v>164.6</v>
+      </c>
+      <c r="H74" t="n">
+        <v>25.58</v>
+      </c>
+      <c r="I74" t="n">
+        <v>18.4</v>
+      </c>
+      <c r="J74" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>3</v>
+      </c>
+      <c r="D75" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E75" t="n">
+        <v>23</v>
+      </c>
+      <c r="F75" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G75" t="n">
+        <v>69</v>
+      </c>
+      <c r="H75" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="I75" t="n">
+        <v>5.07</v>
+      </c>
+      <c r="J75" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>9</v>
+      </c>
+      <c r="D76" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E76" t="n">
+        <v>6.811</v>
+      </c>
+      <c r="F76" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G76" t="n">
+        <v>61.3</v>
+      </c>
+      <c r="H76" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="I76" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="J76" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 18/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E7" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F7" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G7" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H7" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I7" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E8" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F8" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G8" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H8" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I8" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E9" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F9" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G9" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H9" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I9" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E10" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F10" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G10" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H10" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I10" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E11" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F11" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G11" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H11" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I11" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E17" t="n">
-        <v>41.789</v>
+        <v>21.915</v>
       </c>
       <c r="F17" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G17" t="n">
-        <v>167.16</v>
+        <v>65.75</v>
       </c>
       <c r="H17" t="n">
-        <v>28.14</v>
+        <v>0.08</v>
       </c>
       <c r="I17" t="n">
-        <v>20.24</v>
+        <v>0.12</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E18" t="n">
-        <v>105.6</v>
+        <v>6.82</v>
       </c>
       <c r="F18" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G18" t="n">
-        <v>105.6</v>
+        <v>61.38</v>
       </c>
       <c r="H18" t="n">
-        <v>5.51</v>
+        <v>5.23</v>
       </c>
       <c r="I18" t="n">
-        <v>5.51</v>
+        <v>9.31</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E19" t="n">
-        <v>6.82</v>
+        <v>10.662</v>
       </c>
       <c r="F19" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G19" t="n">
-        <v>61.38</v>
+        <v>31.99</v>
       </c>
       <c r="H19" t="n">
-        <v>5.23</v>
+        <v>0.83</v>
       </c>
       <c r="I19" t="n">
-        <v>9.31</v>
+        <v>2.66</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E20" t="n">
-        <v>10.662</v>
+        <v>41.789</v>
       </c>
       <c r="F20" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G20" t="n">
-        <v>31.99</v>
+        <v>167.16</v>
       </c>
       <c r="H20" t="n">
-        <v>0.83</v>
+        <v>28.14</v>
       </c>
       <c r="I20" t="n">
-        <v>2.66</v>
+        <v>20.24</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E21" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F21" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G21" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H21" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I21" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>104.9</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>104.9</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>4.81</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>4.81</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E28" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F28" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G28" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H28" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I28" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E29" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F29" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G29" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H29" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I29" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E31" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F31" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G31" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H31" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I31" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E37" t="n">
-        <v>21.839</v>
+        <v>102.8</v>
       </c>
       <c r="F37" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G37" t="n">
-        <v>65.52</v>
+        <v>102.8</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.15</v>
+        <v>2.71</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.23</v>
+        <v>2.71</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D38" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E38" t="n">
-        <v>10.67</v>
+        <v>38.879</v>
       </c>
       <c r="F38" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G38" t="n">
-        <v>32.01</v>
+        <v>155.52</v>
       </c>
       <c r="H38" t="n">
-        <v>0.85</v>
+        <v>16.5</v>
       </c>
       <c r="I38" t="n">
-        <v>2.73</v>
+        <v>11.87</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E39" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F39" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G39" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H39" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I39" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E40" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F40" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G40" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H40" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I40" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E41" t="n">
-        <v>6.728</v>
+        <v>10.67</v>
       </c>
       <c r="F41" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G41" t="n">
-        <v>60.55</v>
+        <v>32.01</v>
       </c>
       <c r="H41" t="n">
-        <v>4.4</v>
+        <v>0.85</v>
       </c>
       <c r="I41" t="n">
-        <v>7.84</v>
+        <v>2.73</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E47" t="n">
-        <v>38.312</v>
+        <v>6.622</v>
       </c>
       <c r="F47" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G47" t="n">
-        <v>153.25</v>
+        <v>59.6</v>
       </c>
       <c r="H47" t="n">
-        <v>14.23</v>
+        <v>3.45</v>
       </c>
       <c r="I47" t="n">
-        <v>10.24</v>
+        <v>6.14</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E48" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F48" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G48" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E50" t="n">
-        <v>21.778</v>
+        <v>38.312</v>
       </c>
       <c r="F50" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G50" t="n">
-        <v>65.33</v>
+        <v>153.25</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.34</v>
+        <v>14.23</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.52</v>
+        <v>10.24</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E51" t="n">
-        <v>6.622</v>
+        <v>10.562</v>
       </c>
       <c r="F51" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G51" t="n">
-        <v>59.6</v>
+        <v>31.69</v>
       </c>
       <c r="H51" t="n">
-        <v>3.45</v>
+        <v>0.53</v>
       </c>
       <c r="I51" t="n">
-        <v>6.14</v>
+        <v>1.7</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>6.736</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>60.62</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>4.47</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>7.96</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E58" t="n">
-        <v>102.86</v>
+        <v>10.75</v>
       </c>
       <c r="F58" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G58" t="n">
-        <v>102.86</v>
+        <v>32.25</v>
       </c>
       <c r="H58" t="n">
-        <v>2.77</v>
+        <v>1.09</v>
       </c>
       <c r="I58" t="n">
-        <v>2.77</v>
+        <v>3.5</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E59" t="n">
-        <v>10.75</v>
+        <v>39.845</v>
       </c>
       <c r="F59" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G59" t="n">
-        <v>32.25</v>
+        <v>159.38</v>
       </c>
       <c r="H59" t="n">
-        <v>1.09</v>
+        <v>20.36</v>
       </c>
       <c r="I59" t="n">
-        <v>3.5</v>
+        <v>14.65</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E60" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F60" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G60" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H60" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I60" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E61" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F61" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G61" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I61" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E67" t="n">
-        <v>40.567</v>
+        <v>6.807</v>
       </c>
       <c r="F67" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G67" t="n">
-        <v>162.27</v>
+        <v>61.26</v>
       </c>
       <c r="H67" t="n">
-        <v>23.25</v>
+        <v>5.11</v>
       </c>
       <c r="I67" t="n">
-        <v>16.72</v>
+        <v>9.1</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C68" t="n">
         <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E68" t="n">
-        <v>10.796</v>
+        <v>22.797</v>
       </c>
       <c r="F68" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G68" t="n">
-        <v>32.39</v>
+        <v>68.39</v>
       </c>
       <c r="H68" t="n">
-        <v>1.23</v>
+        <v>2.72</v>
       </c>
       <c r="I68" t="n">
-        <v>3.95</v>
+        <v>4.14</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E69" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F69" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G69" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H69" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I69" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E70" t="n">
-        <v>104.58</v>
+        <v>40.567</v>
       </c>
       <c r="F70" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G70" t="n">
-        <v>104.58</v>
+        <v>162.27</v>
       </c>
       <c r="H70" t="n">
-        <v>4.49</v>
+        <v>23.25</v>
       </c>
       <c r="I70" t="n">
-        <v>4.49</v>
+        <v>16.72</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E71" t="n">
-        <v>6.807</v>
+        <v>10.796</v>
       </c>
       <c r="F71" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G71" t="n">
-        <v>61.26</v>
+        <v>32.39</v>
       </c>
       <c r="H71" t="n">
-        <v>5.11</v>
+        <v>1.23</v>
       </c>
       <c r="I71" t="n">
-        <v>9.1</v>
+        <v>3.95</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3019,6 +3019,176 @@
         <v>9.17</v>
       </c>
       <c r="J76" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>3</v>
+      </c>
+      <c r="D77" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E77" t="n">
+        <v>10.958</v>
+      </c>
+      <c r="F77" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G77" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="H77" t="n">
+        <v>1.71</v>
+      </c>
+      <c r="I77" t="n">
+        <v>5.49</v>
+      </c>
+      <c r="J77" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>4</v>
+      </c>
+      <c r="D78" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E78" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="F78" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G78" t="n">
+        <v>169</v>
+      </c>
+      <c r="H78" t="n">
+        <v>29.98</v>
+      </c>
+      <c r="I78" t="n">
+        <v>21.57</v>
+      </c>
+      <c r="J78" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>3</v>
+      </c>
+      <c r="D79" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E79" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="F79" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G79" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="H79" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="I79" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J79" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>1</v>
+      </c>
+      <c r="D80" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E80" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="F80" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G80" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="H80" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I80" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="J80" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>9</v>
+      </c>
+      <c r="D81" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E81" t="n">
+        <v>6.836</v>
+      </c>
+      <c r="F81" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G81" t="n">
+        <v>61.52</v>
+      </c>
+      <c r="H81" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="I81" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="J81" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 19/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E13" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F13" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G13" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H13" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I13" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E14" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F14" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G14" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H14" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I14" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E22" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F22" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G22" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H22" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I22" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E23" t="n">
-        <v>21.669</v>
+        <v>105.78</v>
       </c>
       <c r="F23" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G23" t="n">
-        <v>65.01000000000001</v>
+        <v>105.78</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.66</v>
+        <v>5.69</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.01</v>
+        <v>5.68</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E24" t="n">
-        <v>6.799</v>
+        <v>10.536</v>
       </c>
       <c r="F24" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G24" t="n">
-        <v>61.19</v>
+        <v>31.61</v>
       </c>
       <c r="H24" t="n">
-        <v>5.04</v>
+        <v>0.45</v>
       </c>
       <c r="I24" t="n">
-        <v>8.98</v>
+        <v>1.44</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E25" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F25" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G25" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I25" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E26" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F26" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G26" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H26" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I26" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E32" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F32" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G32" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I32" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E33" t="n">
-        <v>103.08</v>
+        <v>38.849</v>
       </c>
       <c r="F33" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G33" t="n">
-        <v>103.08</v>
+        <v>155.4</v>
       </c>
       <c r="H33" t="n">
-        <v>2.99</v>
+        <v>16.38</v>
       </c>
       <c r="I33" t="n">
-        <v>2.99</v>
+        <v>11.78</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E35" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F35" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G35" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H35" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I35" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E36" t="n">
-        <v>10.714</v>
+        <v>103.08</v>
       </c>
       <c r="F36" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G36" t="n">
-        <v>32.14</v>
+        <v>103.08</v>
       </c>
       <c r="H36" t="n">
-        <v>0.98</v>
+        <v>2.99</v>
       </c>
       <c r="I36" t="n">
-        <v>3.15</v>
+        <v>2.99</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E42" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F42" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G42" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>6.629</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>59.66</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>3.51</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>6.25</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D45" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E45" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F45" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G45" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H45" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I45" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E46" t="n">
-        <v>10.61</v>
+        <v>100.06</v>
       </c>
       <c r="F46" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G46" t="n">
-        <v>31.83</v>
+        <v>100.06</v>
       </c>
       <c r="H46" t="n">
-        <v>0.67</v>
+        <v>-0.03</v>
       </c>
       <c r="I46" t="n">
-        <v>2.15</v>
+        <v>-0.03</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E52" t="n">
-        <v>10.702</v>
+        <v>38.544</v>
       </c>
       <c r="F52" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G52" t="n">
-        <v>32.11</v>
+        <v>154.18</v>
       </c>
       <c r="H52" t="n">
-        <v>0.95</v>
+        <v>15.16</v>
       </c>
       <c r="I52" t="n">
-        <v>3.05</v>
+        <v>10.9</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E53" t="n">
-        <v>21.703</v>
+        <v>6.629</v>
       </c>
       <c r="F53" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G53" t="n">
-        <v>65.11</v>
+        <v>59.66</v>
       </c>
       <c r="H53" t="n">
-        <v>-0.5600000000000001</v>
+        <v>3.51</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.85</v>
+        <v>6.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E55" t="n">
-        <v>6.629</v>
+        <v>21.703</v>
       </c>
       <c r="F55" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G55" t="n">
-        <v>59.66</v>
+        <v>65.11</v>
       </c>
       <c r="H55" t="n">
-        <v>3.51</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I55" t="n">
-        <v>6.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E56" t="n">
-        <v>38.544</v>
+        <v>10.702</v>
       </c>
       <c r="F56" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G56" t="n">
-        <v>154.18</v>
+        <v>32.11</v>
       </c>
       <c r="H56" t="n">
-        <v>15.16</v>
+        <v>0.95</v>
       </c>
       <c r="I56" t="n">
-        <v>10.9</v>
+        <v>3.05</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E62" t="n">
-        <v>6.817</v>
+        <v>41.064</v>
       </c>
       <c r="F62" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G62" t="n">
-        <v>61.35</v>
+        <v>164.26</v>
       </c>
       <c r="H62" t="n">
-        <v>5.2</v>
+        <v>25.24</v>
       </c>
       <c r="I62" t="n">
-        <v>9.26</v>
+        <v>18.16</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E64" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F64" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G64" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H64" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I64" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D65" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E65" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F65" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G65" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H65" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I65" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E66" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F66" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G66" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H66" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I66" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E74" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F74" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G74" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H74" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I74" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E75" t="n">
-        <v>23</v>
+        <v>104.22</v>
       </c>
       <c r="F75" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G75" t="n">
-        <v>69</v>
+        <v>104.22</v>
       </c>
       <c r="H75" t="n">
-        <v>3.33</v>
+        <v>4.13</v>
       </c>
       <c r="I75" t="n">
-        <v>5.07</v>
+        <v>4.13</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D76" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E76" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F76" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G76" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H76" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I76" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D77" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E77" t="n">
-        <v>10.958</v>
+        <v>6.836</v>
       </c>
       <c r="F77" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G77" t="n">
-        <v>32.87</v>
+        <v>61.52</v>
       </c>
       <c r="H77" t="n">
-        <v>1.71</v>
+        <v>5.37</v>
       </c>
       <c r="I77" t="n">
-        <v>5.49</v>
+        <v>9.56</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E78" t="n">
-        <v>42.25</v>
+        <v>10.958</v>
       </c>
       <c r="F78" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G78" t="n">
-        <v>169</v>
+        <v>32.87</v>
       </c>
       <c r="H78" t="n">
-        <v>29.98</v>
+        <v>1.71</v>
       </c>
       <c r="I78" t="n">
-        <v>21.57</v>
+        <v>5.49</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D79" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E79" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F79" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G79" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H79" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I79" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,31 +3164,201 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E81" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="F81" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G81" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="H81" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I81" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="J81" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E82" t="n">
+        <v>106.26</v>
+      </c>
+      <c r="F82" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G82" t="n">
+        <v>106.26</v>
+      </c>
+      <c r="H82" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="I82" t="n">
+        <v>6.16</v>
+      </c>
+      <c r="J82" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D83" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E83" t="n">
+        <v>10.988</v>
+      </c>
+      <c r="F83" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G83" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="H83" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="I83" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="J83" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>4</v>
+      </c>
+      <c r="D84" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E84" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="F84" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G84" t="n">
+        <v>168.4</v>
+      </c>
+      <c r="H84" t="n">
+        <v>29.38</v>
+      </c>
+      <c r="I84" t="n">
+        <v>21.13</v>
+      </c>
+      <c r="J84" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>3</v>
+      </c>
+      <c r="D85" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E85" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="F85" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G85" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="H85" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="I85" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="J85" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="1" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C86" t="n">
         <v>9</v>
       </c>
-      <c r="D81" t="n">
+      <c r="D86" t="n">
         <v>6.239</v>
       </c>
-      <c r="E81" t="n">
-        <v>6.836</v>
-      </c>
-      <c r="F81" t="n">
+      <c r="E86" t="n">
+        <v>6.846</v>
+      </c>
+      <c r="F86" t="n">
         <v>56.15</v>
       </c>
-      <c r="G81" t="n">
-        <v>61.52</v>
-      </c>
-      <c r="H81" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="I81" t="n">
-        <v>9.56</v>
-      </c>
-      <c r="J81" t="n">
+      <c r="G86" t="n">
+        <v>61.61</v>
+      </c>
+      <c r="H86" t="n">
+        <v>5.46</v>
+      </c>
+      <c r="I86" t="n">
+        <v>9.720000000000001</v>
+      </c>
+      <c r="J86" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 22/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>21.907</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>65.72</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>0.08</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E22" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F22" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G22" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H22" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I22" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E23" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F23" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G23" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I23" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E24" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F24" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G24" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H24" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I24" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E25" t="n">
-        <v>21.669</v>
+        <v>105.78</v>
       </c>
       <c r="F25" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G25" t="n">
-        <v>65.01000000000001</v>
+        <v>105.78</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.66</v>
+        <v>5.69</v>
       </c>
       <c r="I25" t="n">
-        <v>-1.01</v>
+        <v>5.68</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E26" t="n">
-        <v>6.799</v>
+        <v>10.536</v>
       </c>
       <c r="F26" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G26" t="n">
-        <v>61.19</v>
+        <v>31.61</v>
       </c>
       <c r="H26" t="n">
-        <v>5.04</v>
+        <v>0.45</v>
       </c>
       <c r="I26" t="n">
-        <v>8.98</v>
+        <v>1.44</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E32" t="n">
-        <v>10.714</v>
+        <v>103.08</v>
       </c>
       <c r="F32" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G32" t="n">
-        <v>32.14</v>
+        <v>103.08</v>
       </c>
       <c r="H32" t="n">
-        <v>0.98</v>
+        <v>2.99</v>
       </c>
       <c r="I32" t="n">
-        <v>3.15</v>
+        <v>2.99</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E33" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F33" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G33" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H33" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I33" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E35" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F35" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G35" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H35" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I35" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E36" t="n">
-        <v>103.08</v>
+        <v>38.849</v>
       </c>
       <c r="F36" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G36" t="n">
-        <v>103.08</v>
+        <v>155.4</v>
       </c>
       <c r="H36" t="n">
-        <v>2.99</v>
+        <v>16.38</v>
       </c>
       <c r="I36" t="n">
-        <v>2.99</v>
+        <v>11.78</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>6.629</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>59.66</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>3.51</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>6.25</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>22</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>66</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>0.33</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>0.5</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>100.06</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>100.06</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>-0.03</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>-0.03</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>6.629</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>59.66</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>3.51</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>6.25</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D46" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E46" t="n">
-        <v>100.06</v>
+        <v>38.497</v>
       </c>
       <c r="F46" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G46" t="n">
-        <v>100.06</v>
+        <v>153.99</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.03</v>
+        <v>14.97</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03</v>
+        <v>10.77</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E52" t="n">
-        <v>38.544</v>
+        <v>21.703</v>
       </c>
       <c r="F52" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G52" t="n">
-        <v>154.18</v>
+        <v>65.11</v>
       </c>
       <c r="H52" t="n">
-        <v>15.16</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I52" t="n">
-        <v>10.9</v>
+        <v>-0.85</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E53" t="n">
-        <v>6.629</v>
+        <v>100.34</v>
       </c>
       <c r="F53" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G53" t="n">
-        <v>59.66</v>
+        <v>100.34</v>
       </c>
       <c r="H53" t="n">
-        <v>3.51</v>
+        <v>0.25</v>
       </c>
       <c r="I53" t="n">
-        <v>6.25</v>
+        <v>0.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E54" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F54" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G54" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H54" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I54" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D55" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E55" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F55" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G55" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H55" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I55" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D56" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E56" t="n">
-        <v>10.702</v>
+        <v>6.629</v>
       </c>
       <c r="F56" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G56" t="n">
-        <v>32.11</v>
+        <v>59.66</v>
       </c>
       <c r="H56" t="n">
-        <v>0.95</v>
+        <v>3.51</v>
       </c>
       <c r="I56" t="n">
-        <v>3.05</v>
+        <v>6.25</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>10.75</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>32.25</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>1.09</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>3.5</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>10.75</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>32.25</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>1.09</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>3.5</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D59" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E59" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F59" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G59" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H59" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I59" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E60" t="n">
-        <v>6.736</v>
+        <v>102.86</v>
       </c>
       <c r="F60" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G60" t="n">
-        <v>60.62</v>
+        <v>102.86</v>
       </c>
       <c r="H60" t="n">
-        <v>4.47</v>
+        <v>2.77</v>
       </c>
       <c r="I60" t="n">
-        <v>7.96</v>
+        <v>2.77</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E67" t="n">
-        <v>6.807</v>
+        <v>40.567</v>
       </c>
       <c r="F67" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G67" t="n">
-        <v>61.26</v>
+        <v>162.27</v>
       </c>
       <c r="H67" t="n">
-        <v>5.11</v>
+        <v>23.25</v>
       </c>
       <c r="I67" t="n">
-        <v>9.1</v>
+        <v>16.72</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C68" t="n">
         <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E68" t="n">
-        <v>22.797</v>
+        <v>10.796</v>
       </c>
       <c r="F68" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G68" t="n">
-        <v>68.39</v>
+        <v>32.39</v>
       </c>
       <c r="H68" t="n">
-        <v>2.72</v>
+        <v>1.23</v>
       </c>
       <c r="I68" t="n">
-        <v>4.14</v>
+        <v>3.95</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E69" t="n">
-        <v>104.58</v>
+        <v>22.797</v>
       </c>
       <c r="F69" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G69" t="n">
-        <v>104.58</v>
+        <v>68.39</v>
       </c>
       <c r="H69" t="n">
-        <v>4.49</v>
+        <v>2.72</v>
       </c>
       <c r="I69" t="n">
-        <v>4.49</v>
+        <v>4.14</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E70" t="n">
-        <v>40.567</v>
+        <v>6.807</v>
       </c>
       <c r="F70" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G70" t="n">
-        <v>162.27</v>
+        <v>61.26</v>
       </c>
       <c r="H70" t="n">
-        <v>23.25</v>
+        <v>5.11</v>
       </c>
       <c r="I70" t="n">
-        <v>16.72</v>
+        <v>9.1</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E71" t="n">
-        <v>10.796</v>
+        <v>104.58</v>
       </c>
       <c r="F71" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G71" t="n">
-        <v>32.39</v>
+        <v>104.58</v>
       </c>
       <c r="H71" t="n">
-        <v>1.23</v>
+        <v>4.49</v>
       </c>
       <c r="I71" t="n">
-        <v>3.95</v>
+        <v>4.49</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E77" t="n">
-        <v>6.836</v>
+        <v>105.8</v>
       </c>
       <c r="F77" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G77" t="n">
-        <v>61.52</v>
+        <v>105.8</v>
       </c>
       <c r="H77" t="n">
-        <v>5.37</v>
+        <v>5.71</v>
       </c>
       <c r="I77" t="n">
-        <v>9.56</v>
+        <v>5.7</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D78" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E78" t="n">
-        <v>10.958</v>
+        <v>42.25</v>
       </c>
       <c r="F78" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G78" t="n">
-        <v>32.87</v>
+        <v>169</v>
       </c>
       <c r="H78" t="n">
-        <v>1.71</v>
+        <v>29.98</v>
       </c>
       <c r="I78" t="n">
-        <v>5.49</v>
+        <v>21.57</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E79" t="n">
-        <v>42.25</v>
+        <v>23.4</v>
       </c>
       <c r="F79" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G79" t="n">
-        <v>169</v>
+        <v>70.2</v>
       </c>
       <c r="H79" t="n">
-        <v>29.98</v>
+        <v>4.53</v>
       </c>
       <c r="I79" t="n">
-        <v>21.57</v>
+        <v>6.9</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D80" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E80" t="n">
-        <v>23.4</v>
+        <v>6.836</v>
       </c>
       <c r="F80" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G80" t="n">
-        <v>70.2</v>
+        <v>61.52</v>
       </c>
       <c r="H80" t="n">
-        <v>4.53</v>
+        <v>5.37</v>
       </c>
       <c r="I80" t="n">
-        <v>6.9</v>
+        <v>9.56</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E81" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F81" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G81" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H81" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I81" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3359,6 +3359,176 @@
         <v>9.720000000000001</v>
       </c>
       <c r="J86" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>3</v>
+      </c>
+      <c r="D87" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E87" t="n">
+        <v>10.852</v>
+      </c>
+      <c r="F87" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G87" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="H87" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="I87" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="J87" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D88" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E88" t="n">
+        <v>43.005</v>
+      </c>
+      <c r="F88" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G88" t="n">
+        <v>172.02</v>
+      </c>
+      <c r="H88" t="n">
+        <v>33</v>
+      </c>
+      <c r="I88" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="J88" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>3</v>
+      </c>
+      <c r="D89" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E89" t="n">
+        <v>23.32</v>
+      </c>
+      <c r="F89" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G89" t="n">
+        <v>69.95999999999999</v>
+      </c>
+      <c r="H89" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="I89" t="n">
+        <v>6.53</v>
+      </c>
+      <c r="J89" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E90" t="n">
+        <v>106.28</v>
+      </c>
+      <c r="F90" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G90" t="n">
+        <v>106.28</v>
+      </c>
+      <c r="H90" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="I90" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="J90" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>9</v>
+      </c>
+      <c r="D91" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E91" t="n">
+        <v>6.856</v>
+      </c>
+      <c r="F91" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G91" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="H91" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="I91" t="n">
+        <v>9.880000000000001</v>
+      </c>
+      <c r="J91" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 23/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E13" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F13" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G13" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H13" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I13" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E22" t="n">
-        <v>6.799</v>
+        <v>10.536</v>
       </c>
       <c r="F22" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G22" t="n">
-        <v>61.19</v>
+        <v>31.61</v>
       </c>
       <c r="H22" t="n">
-        <v>5.04</v>
+        <v>0.45</v>
       </c>
       <c r="I22" t="n">
-        <v>8.98</v>
+        <v>1.44</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E23" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F23" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G23" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E24" t="n">
-        <v>41.336</v>
+        <v>105.78</v>
       </c>
       <c r="F24" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G24" t="n">
-        <v>165.34</v>
+        <v>105.78</v>
       </c>
       <c r="H24" t="n">
-        <v>26.32</v>
+        <v>5.69</v>
       </c>
       <c r="I24" t="n">
-        <v>18.93</v>
+        <v>5.68</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D25" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E25" t="n">
-        <v>105.78</v>
+        <v>6.799</v>
       </c>
       <c r="F25" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G25" t="n">
-        <v>105.78</v>
+        <v>61.19</v>
       </c>
       <c r="H25" t="n">
-        <v>5.69</v>
+        <v>5.04</v>
       </c>
       <c r="I25" t="n">
-        <v>5.68</v>
+        <v>8.98</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E26" t="n">
-        <v>10.536</v>
+        <v>21.669</v>
       </c>
       <c r="F26" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G26" t="n">
-        <v>31.61</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>0.45</v>
+        <v>-0.66</v>
       </c>
       <c r="I26" t="n">
-        <v>1.44</v>
+        <v>-1.01</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E32" t="n">
-        <v>103.08</v>
+        <v>38.849</v>
       </c>
       <c r="F32" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G32" t="n">
-        <v>103.08</v>
+        <v>155.4</v>
       </c>
       <c r="H32" t="n">
-        <v>2.99</v>
+        <v>16.38</v>
       </c>
       <c r="I32" t="n">
-        <v>2.99</v>
+        <v>11.78</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D33" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E33" t="n">
-        <v>22.053</v>
+        <v>6.762</v>
       </c>
       <c r="F33" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G33" t="n">
-        <v>66.16</v>
+        <v>60.86</v>
       </c>
       <c r="H33" t="n">
-        <v>0.49</v>
+        <v>4.71</v>
       </c>
       <c r="I33" t="n">
-        <v>0.75</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E34" t="n">
-        <v>6.762</v>
+        <v>10.714</v>
       </c>
       <c r="F34" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G34" t="n">
-        <v>60.86</v>
+        <v>32.14</v>
       </c>
       <c r="H34" t="n">
-        <v>4.71</v>
+        <v>0.98</v>
       </c>
       <c r="I34" t="n">
-        <v>8.390000000000001</v>
+        <v>3.15</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E35" t="n">
-        <v>10.714</v>
+        <v>103.08</v>
       </c>
       <c r="F35" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G35" t="n">
-        <v>32.14</v>
+        <v>103.08</v>
       </c>
       <c r="H35" t="n">
-        <v>0.98</v>
+        <v>2.99</v>
       </c>
       <c r="I35" t="n">
-        <v>3.15</v>
+        <v>2.99</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E36" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F36" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G36" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H36" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I36" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E42" t="n">
-        <v>6.629</v>
+        <v>10.61</v>
       </c>
       <c r="F42" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G42" t="n">
-        <v>59.66</v>
+        <v>31.83</v>
       </c>
       <c r="H42" t="n">
-        <v>3.51</v>
+        <v>0.67</v>
       </c>
       <c r="I42" t="n">
-        <v>6.25</v>
+        <v>2.15</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D43" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E43" t="n">
-        <v>22</v>
+        <v>6.629</v>
       </c>
       <c r="F43" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G43" t="n">
-        <v>66</v>
+        <v>59.66</v>
       </c>
       <c r="H43" t="n">
-        <v>0.33</v>
+        <v>3.51</v>
       </c>
       <c r="I43" t="n">
-        <v>0.5</v>
+        <v>6.25</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E45" t="n">
-        <v>10.61</v>
+        <v>100.06</v>
       </c>
       <c r="F45" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G45" t="n">
-        <v>31.83</v>
+        <v>100.06</v>
       </c>
       <c r="H45" t="n">
-        <v>0.67</v>
+        <v>-0.03</v>
       </c>
       <c r="I45" t="n">
-        <v>2.15</v>
+        <v>-0.03</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E47" t="n">
-        <v>6.622</v>
+        <v>10.562</v>
       </c>
       <c r="F47" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G47" t="n">
-        <v>59.6</v>
+        <v>31.69</v>
       </c>
       <c r="H47" t="n">
-        <v>3.45</v>
+        <v>0.53</v>
       </c>
       <c r="I47" t="n">
-        <v>6.14</v>
+        <v>1.7</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E48" t="n">
-        <v>21.778</v>
+        <v>38.312</v>
       </c>
       <c r="F48" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G48" t="n">
-        <v>65.33</v>
+        <v>153.25</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.34</v>
+        <v>14.23</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.52</v>
+        <v>10.24</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E50" t="n">
-        <v>38.312</v>
+        <v>21.778</v>
       </c>
       <c r="F50" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G50" t="n">
-        <v>153.25</v>
+        <v>65.33</v>
       </c>
       <c r="H50" t="n">
-        <v>14.23</v>
+        <v>-0.34</v>
       </c>
       <c r="I50" t="n">
-        <v>10.24</v>
+        <v>-0.52</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D51" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E51" t="n">
-        <v>10.562</v>
+        <v>6.622</v>
       </c>
       <c r="F51" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G51" t="n">
-        <v>31.69</v>
+        <v>59.6</v>
       </c>
       <c r="H51" t="n">
-        <v>0.53</v>
+        <v>3.45</v>
       </c>
       <c r="I51" t="n">
-        <v>1.7</v>
+        <v>6.14</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E57" t="n">
-        <v>10.75</v>
+        <v>102.86</v>
       </c>
       <c r="F57" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G57" t="n">
-        <v>32.25</v>
+        <v>102.86</v>
       </c>
       <c r="H57" t="n">
-        <v>1.09</v>
+        <v>2.77</v>
       </c>
       <c r="I57" t="n">
-        <v>3.5</v>
+        <v>2.77</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D59" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E59" t="n">
-        <v>6.736</v>
+        <v>22.289</v>
       </c>
       <c r="F59" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G59" t="n">
-        <v>60.62</v>
+        <v>66.87</v>
       </c>
       <c r="H59" t="n">
-        <v>4.47</v>
+        <v>1.2</v>
       </c>
       <c r="I59" t="n">
-        <v>7.96</v>
+        <v>1.83</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D60" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E60" t="n">
-        <v>102.86</v>
+        <v>10.75</v>
       </c>
       <c r="F60" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G60" t="n">
-        <v>102.86</v>
+        <v>32.25</v>
       </c>
       <c r="H60" t="n">
-        <v>2.77</v>
+        <v>1.09</v>
       </c>
       <c r="I60" t="n">
-        <v>2.77</v>
+        <v>3.5</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D61" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E61" t="n">
-        <v>22.289</v>
+        <v>39.845</v>
       </c>
       <c r="F61" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G61" t="n">
-        <v>66.87</v>
+        <v>159.38</v>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>20.36</v>
       </c>
       <c r="I61" t="n">
-        <v>1.83</v>
+        <v>14.65</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E72" t="n">
-        <v>23</v>
+        <v>41.15</v>
       </c>
       <c r="F72" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G72" t="n">
-        <v>69</v>
+        <v>164.6</v>
       </c>
       <c r="H72" t="n">
-        <v>3.33</v>
+        <v>25.58</v>
       </c>
       <c r="I72" t="n">
-        <v>5.07</v>
+        <v>18.4</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>104.22</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>104.22</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>4.13</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>4.13</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D74" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E74" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F74" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G74" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H74" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I74" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E75" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F75" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G75" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H75" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I75" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E76" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F76" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G76" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H76" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I76" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E82" t="n">
-        <v>106.26</v>
+        <v>23.3</v>
       </c>
       <c r="F82" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G82" t="n">
-        <v>106.26</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H82" t="n">
-        <v>6.17</v>
+        <v>4.23</v>
       </c>
       <c r="I82" t="n">
-        <v>6.16</v>
+        <v>6.44</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D83" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E83" t="n">
-        <v>10.988</v>
+        <v>6.846</v>
       </c>
       <c r="F83" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G83" t="n">
-        <v>32.96</v>
+        <v>61.61</v>
       </c>
       <c r="H83" t="n">
-        <v>1.8</v>
+        <v>5.46</v>
       </c>
       <c r="I83" t="n">
-        <v>5.78</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E84" t="n">
-        <v>42.1</v>
+        <v>10.988</v>
       </c>
       <c r="F84" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G84" t="n">
-        <v>168.4</v>
+        <v>32.96</v>
       </c>
       <c r="H84" t="n">
-        <v>29.38</v>
+        <v>1.8</v>
       </c>
       <c r="I84" t="n">
-        <v>21.13</v>
+        <v>5.78</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E85" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F85" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G85" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H85" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I85" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D86" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E86" t="n">
-        <v>6.846</v>
+        <v>42.1</v>
       </c>
       <c r="F86" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G86" t="n">
-        <v>61.61</v>
+        <v>168.4</v>
       </c>
       <c r="H86" t="n">
-        <v>5.46</v>
+        <v>29.38</v>
       </c>
       <c r="I86" t="n">
-        <v>9.720000000000001</v>
+        <v>21.13</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D87" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E87" t="n">
-        <v>10.852</v>
+        <v>6.856</v>
       </c>
       <c r="F87" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G87" t="n">
-        <v>32.56</v>
+        <v>61.7</v>
       </c>
       <c r="H87" t="n">
-        <v>1.4</v>
+        <v>5.55</v>
       </c>
       <c r="I87" t="n">
-        <v>4.49</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E88" t="n">
-        <v>43.005</v>
+        <v>10.852</v>
       </c>
       <c r="F88" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G88" t="n">
-        <v>172.02</v>
+        <v>32.56</v>
       </c>
       <c r="H88" t="n">
-        <v>33</v>
+        <v>1.4</v>
       </c>
       <c r="I88" t="n">
-        <v>23.74</v>
+        <v>4.49</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D89" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E89" t="n">
-        <v>23.32</v>
+        <v>43.005</v>
       </c>
       <c r="F89" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G89" t="n">
-        <v>69.95999999999999</v>
+        <v>172.02</v>
       </c>
       <c r="H89" t="n">
-        <v>4.29</v>
+        <v>33</v>
       </c>
       <c r="I89" t="n">
-        <v>6.53</v>
+        <v>23.74</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E90" t="n">
-        <v>106.28</v>
+        <v>23.32</v>
       </c>
       <c r="F90" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G90" t="n">
-        <v>106.28</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H90" t="n">
-        <v>6.19</v>
+        <v>4.29</v>
       </c>
       <c r="I90" t="n">
-        <v>6.18</v>
+        <v>6.53</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,31 +3504,201 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E91" t="n">
+        <v>106.28</v>
+      </c>
+      <c r="F91" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G91" t="n">
+        <v>106.28</v>
+      </c>
+      <c r="H91" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="I91" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="J91" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E92" t="n">
+        <v>103.88</v>
+      </c>
+      <c r="F92" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G92" t="n">
+        <v>103.88</v>
+      </c>
+      <c r="H92" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="I92" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="J92" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>3</v>
+      </c>
+      <c r="D93" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E93" t="n">
+        <v>10.876</v>
+      </c>
+      <c r="F93" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G93" t="n">
+        <v>32.63</v>
+      </c>
+      <c r="H93" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="I93" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="J93" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>4</v>
+      </c>
+      <c r="D94" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E94" t="n">
+        <v>40.575</v>
+      </c>
+      <c r="F94" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G94" t="n">
+        <v>162.3</v>
+      </c>
+      <c r="H94" t="n">
+        <v>23.28</v>
+      </c>
+      <c r="I94" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="J94" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>3</v>
+      </c>
+      <c r="D95" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E95" t="n">
+        <v>23.025</v>
+      </c>
+      <c r="F95" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G95" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="H95" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I95" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="J95" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>46196</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C91" t="n">
+      <c r="C96" t="n">
         <v>9</v>
       </c>
-      <c r="D91" t="n">
+      <c r="D96" t="n">
         <v>6.239</v>
       </c>
-      <c r="E91" t="n">
-        <v>6.856</v>
-      </c>
-      <c r="F91" t="n">
+      <c r="E96" t="n">
+        <v>6.797</v>
+      </c>
+      <c r="F96" t="n">
         <v>56.15</v>
       </c>
-      <c r="G91" t="n">
-        <v>61.7</v>
-      </c>
-      <c r="H91" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="I91" t="n">
-        <v>9.880000000000001</v>
-      </c>
-      <c r="J91" t="n">
+      <c r="G96" t="n">
+        <v>61.17</v>
+      </c>
+      <c r="H96" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="I96" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="J96" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 24/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>105.22</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>105.22</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>5.13</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>5.13</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>21.907</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>65.72</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>0.08</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E14" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F14" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G14" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H14" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I14" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E22" t="n">
-        <v>10.536</v>
+        <v>21.669</v>
       </c>
       <c r="F22" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G22" t="n">
-        <v>31.61</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>0.45</v>
+        <v>-0.66</v>
       </c>
       <c r="I22" t="n">
-        <v>1.44</v>
+        <v>-1.01</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E23" t="n">
-        <v>41.336</v>
+        <v>105.78</v>
       </c>
       <c r="F23" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G23" t="n">
-        <v>165.34</v>
+        <v>105.78</v>
       </c>
       <c r="H23" t="n">
-        <v>26.32</v>
+        <v>5.69</v>
       </c>
       <c r="I23" t="n">
-        <v>18.93</v>
+        <v>5.68</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E24" t="n">
-        <v>105.78</v>
+        <v>6.799</v>
       </c>
       <c r="F24" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G24" t="n">
-        <v>105.78</v>
+        <v>61.19</v>
       </c>
       <c r="H24" t="n">
-        <v>5.69</v>
+        <v>5.04</v>
       </c>
       <c r="I24" t="n">
-        <v>5.68</v>
+        <v>8.98</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E25" t="n">
-        <v>6.799</v>
+        <v>10.536</v>
       </c>
       <c r="F25" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G25" t="n">
-        <v>61.19</v>
+        <v>31.61</v>
       </c>
       <c r="H25" t="n">
-        <v>5.04</v>
+        <v>0.45</v>
       </c>
       <c r="I25" t="n">
-        <v>8.98</v>
+        <v>1.44</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E26" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F26" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G26" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I26" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E32" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F32" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G32" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H32" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I32" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E33" t="n">
-        <v>6.762</v>
+        <v>10.714</v>
       </c>
       <c r="F33" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G33" t="n">
-        <v>60.86</v>
+        <v>32.14</v>
       </c>
       <c r="H33" t="n">
-        <v>4.71</v>
+        <v>0.98</v>
       </c>
       <c r="I33" t="n">
-        <v>8.390000000000001</v>
+        <v>3.15</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E34" t="n">
-        <v>10.714</v>
+        <v>103.08</v>
       </c>
       <c r="F34" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G34" t="n">
-        <v>32.14</v>
+        <v>103.08</v>
       </c>
       <c r="H34" t="n">
-        <v>0.98</v>
+        <v>2.99</v>
       </c>
       <c r="I34" t="n">
-        <v>3.15</v>
+        <v>2.99</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E35" t="n">
-        <v>103.08</v>
+        <v>38.849</v>
       </c>
       <c r="F35" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G35" t="n">
-        <v>103.08</v>
+        <v>155.4</v>
       </c>
       <c r="H35" t="n">
-        <v>2.99</v>
+        <v>16.38</v>
       </c>
       <c r="I35" t="n">
-        <v>2.99</v>
+        <v>11.78</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D36" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E36" t="n">
-        <v>22.053</v>
+        <v>6.762</v>
       </c>
       <c r="F36" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G36" t="n">
-        <v>66.16</v>
+        <v>60.86</v>
       </c>
       <c r="H36" t="n">
-        <v>0.49</v>
+        <v>4.71</v>
       </c>
       <c r="I36" t="n">
-        <v>0.75</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>100.06</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>100.06</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>-0.03</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>-0.03</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E43" t="n">
-        <v>6.629</v>
+        <v>10.61</v>
       </c>
       <c r="F43" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G43" t="n">
-        <v>59.66</v>
+        <v>31.83</v>
       </c>
       <c r="H43" t="n">
-        <v>3.51</v>
+        <v>0.67</v>
       </c>
       <c r="I43" t="n">
-        <v>6.25</v>
+        <v>2.15</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>6.629</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>59.66</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>3.51</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>6.25</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E45" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F45" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G45" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C47" t="n">
         <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E47" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F47" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G47" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H47" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I47" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E48" t="n">
-        <v>38.312</v>
+        <v>99.83</v>
       </c>
       <c r="F48" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G48" t="n">
-        <v>153.25</v>
+        <v>99.83</v>
       </c>
       <c r="H48" t="n">
-        <v>14.23</v>
+        <v>-0.26</v>
       </c>
       <c r="I48" t="n">
-        <v>10.24</v>
+        <v>-0.26</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E49" t="n">
-        <v>99.83</v>
+        <v>6.622</v>
       </c>
       <c r="F49" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G49" t="n">
-        <v>99.83</v>
+        <v>59.6</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.26</v>
+        <v>3.45</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.26</v>
+        <v>6.14</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E50" t="n">
-        <v>21.778</v>
+        <v>10.562</v>
       </c>
       <c r="F50" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G50" t="n">
-        <v>65.33</v>
+        <v>31.69</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.34</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.52</v>
+        <v>1.7</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D51" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E51" t="n">
-        <v>6.622</v>
+        <v>38.312</v>
       </c>
       <c r="F51" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G51" t="n">
-        <v>59.6</v>
+        <v>153.25</v>
       </c>
       <c r="H51" t="n">
-        <v>3.45</v>
+        <v>14.23</v>
       </c>
       <c r="I51" t="n">
-        <v>6.14</v>
+        <v>10.24</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E57" t="n">
-        <v>102.86</v>
+        <v>10.75</v>
       </c>
       <c r="F57" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G57" t="n">
-        <v>102.86</v>
+        <v>32.25</v>
       </c>
       <c r="H57" t="n">
-        <v>2.77</v>
+        <v>1.09</v>
       </c>
       <c r="I57" t="n">
-        <v>2.77</v>
+        <v>3.5</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E58" t="n">
-        <v>6.736</v>
+        <v>22.289</v>
       </c>
       <c r="F58" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G58" t="n">
-        <v>60.62</v>
+        <v>66.87</v>
       </c>
       <c r="H58" t="n">
-        <v>4.47</v>
+        <v>1.2</v>
       </c>
       <c r="I58" t="n">
-        <v>7.96</v>
+        <v>1.83</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E59" t="n">
-        <v>22.289</v>
+        <v>39.845</v>
       </c>
       <c r="F59" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G59" t="n">
-        <v>66.87</v>
+        <v>159.38</v>
       </c>
       <c r="H59" t="n">
-        <v>1.2</v>
+        <v>20.36</v>
       </c>
       <c r="I59" t="n">
-        <v>1.83</v>
+        <v>14.65</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E60" t="n">
-        <v>10.75</v>
+        <v>102.86</v>
       </c>
       <c r="F60" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G60" t="n">
-        <v>32.25</v>
+        <v>102.86</v>
       </c>
       <c r="H60" t="n">
-        <v>1.09</v>
+        <v>2.77</v>
       </c>
       <c r="I60" t="n">
-        <v>3.5</v>
+        <v>2.77</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D61" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E61" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F61" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G61" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H61" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I61" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E72" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F72" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G72" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H72" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I72" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>104.22</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>104.22</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>4.13</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>4.13</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E74" t="n">
-        <v>6.811</v>
+        <v>23</v>
       </c>
       <c r="F74" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G74" t="n">
-        <v>61.3</v>
+        <v>69</v>
       </c>
       <c r="H74" t="n">
-        <v>5.15</v>
+        <v>3.33</v>
       </c>
       <c r="I74" t="n">
-        <v>9.17</v>
+        <v>5.07</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E75" t="n">
-        <v>23</v>
+        <v>41.15</v>
       </c>
       <c r="F75" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G75" t="n">
-        <v>69</v>
+        <v>164.6</v>
       </c>
       <c r="H75" t="n">
-        <v>3.33</v>
+        <v>25.58</v>
       </c>
       <c r="I75" t="n">
-        <v>5.07</v>
+        <v>18.4</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E76" t="n">
-        <v>10.892</v>
+        <v>104.22</v>
       </c>
       <c r="F76" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G76" t="n">
-        <v>32.68</v>
+        <v>104.22</v>
       </c>
       <c r="H76" t="n">
-        <v>1.52</v>
+        <v>4.13</v>
       </c>
       <c r="I76" t="n">
-        <v>4.88</v>
+        <v>4.13</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E87" t="n">
-        <v>6.856</v>
+        <v>106.28</v>
       </c>
       <c r="F87" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G87" t="n">
-        <v>61.7</v>
+        <v>106.28</v>
       </c>
       <c r="H87" t="n">
-        <v>5.55</v>
+        <v>6.19</v>
       </c>
       <c r="I87" t="n">
-        <v>9.880000000000001</v>
+        <v>6.18</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E88" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F88" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G88" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I88" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E89" t="n">
-        <v>43.005</v>
+        <v>10.852</v>
       </c>
       <c r="F89" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G89" t="n">
-        <v>172.02</v>
+        <v>32.56</v>
       </c>
       <c r="H89" t="n">
-        <v>33</v>
+        <v>1.4</v>
       </c>
       <c r="I89" t="n">
-        <v>23.74</v>
+        <v>4.49</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E90" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F90" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G90" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H90" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I90" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E91" t="n">
-        <v>106.28</v>
+        <v>43.005</v>
       </c>
       <c r="F91" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G91" t="n">
-        <v>106.28</v>
+        <v>172.02</v>
       </c>
       <c r="H91" t="n">
-        <v>6.19</v>
+        <v>33</v>
       </c>
       <c r="I91" t="n">
-        <v>6.18</v>
+        <v>23.74</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3699,6 +3699,176 @@
         <v>8.94</v>
       </c>
       <c r="J96" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>3</v>
+      </c>
+      <c r="D97" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E97" t="n">
+        <v>10.642</v>
+      </c>
+      <c r="F97" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G97" t="n">
+        <v>31.93</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I97" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="J97" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>4</v>
+      </c>
+      <c r="D98" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E98" t="n">
+        <v>40.65</v>
+      </c>
+      <c r="F98" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G98" t="n">
+        <v>162.6</v>
+      </c>
+      <c r="H98" t="n">
+        <v>23.58</v>
+      </c>
+      <c r="I98" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="J98" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>3</v>
+      </c>
+      <c r="D99" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E99" t="n">
+        <v>23.35</v>
+      </c>
+      <c r="F99" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G99" t="n">
+        <v>70.05</v>
+      </c>
+      <c r="H99" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I99" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="J99" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E100" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="F100" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G100" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="H100" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="I100" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="J100" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>9</v>
+      </c>
+      <c r="D101" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E101" t="n">
+        <v>6.839</v>
+      </c>
+      <c r="F101" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G101" t="n">
+        <v>61.55</v>
+      </c>
+      <c r="H101" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="I101" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="J101" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 25/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>105.22</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>105.22</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>5.13</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>5.13</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C15" t="n">
         <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>6.788</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>61.09</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>4.94</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E28" t="n">
-        <v>40.532</v>
+        <v>6.795</v>
       </c>
       <c r="F28" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G28" t="n">
-        <v>162.13</v>
+        <v>61.16</v>
       </c>
       <c r="H28" t="n">
-        <v>23.11</v>
+        <v>5.01</v>
       </c>
       <c r="I28" t="n">
-        <v>16.62</v>
+        <v>8.92</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E29" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F29" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G29" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H29" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I29" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E30" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F30" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G30" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H30" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I30" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D37" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E37" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F37" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G37" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H37" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I37" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D38" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E38" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F38" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G38" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H38" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I38" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E39" t="n">
-        <v>6.728</v>
+        <v>10.67</v>
       </c>
       <c r="F39" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G39" t="n">
-        <v>60.55</v>
+        <v>32.01</v>
       </c>
       <c r="H39" t="n">
-        <v>4.4</v>
+        <v>0.85</v>
       </c>
       <c r="I39" t="n">
-        <v>7.84</v>
+        <v>2.73</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E40" t="n">
-        <v>21.839</v>
+        <v>102.8</v>
       </c>
       <c r="F40" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G40" t="n">
-        <v>65.52</v>
+        <v>102.8</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.15</v>
+        <v>2.71</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.23</v>
+        <v>2.71</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E41" t="n">
-        <v>10.67</v>
+        <v>38.879</v>
       </c>
       <c r="F41" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G41" t="n">
-        <v>32.01</v>
+        <v>155.52</v>
       </c>
       <c r="H41" t="n">
-        <v>0.85</v>
+        <v>16.5</v>
       </c>
       <c r="I41" t="n">
-        <v>2.73</v>
+        <v>11.87</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D52" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E52" t="n">
-        <v>21.703</v>
+        <v>6.629</v>
       </c>
       <c r="F52" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G52" t="n">
-        <v>65.11</v>
+        <v>59.66</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.5600000000000001</v>
+        <v>3.51</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.85</v>
+        <v>6.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E53" t="n">
-        <v>100.34</v>
+        <v>38.544</v>
       </c>
       <c r="F53" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G53" t="n">
-        <v>100.34</v>
+        <v>154.18</v>
       </c>
       <c r="H53" t="n">
-        <v>0.25</v>
+        <v>15.16</v>
       </c>
       <c r="I53" t="n">
-        <v>0.25</v>
+        <v>10.9</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E55" t="n">
-        <v>38.544</v>
+        <v>100.34</v>
       </c>
       <c r="F55" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G55" t="n">
-        <v>154.18</v>
+        <v>100.34</v>
       </c>
       <c r="H55" t="n">
-        <v>15.16</v>
+        <v>0.25</v>
       </c>
       <c r="I55" t="n">
-        <v>10.9</v>
+        <v>0.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E56" t="n">
-        <v>6.629</v>
+        <v>21.703</v>
       </c>
       <c r="F56" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G56" t="n">
-        <v>59.66</v>
+        <v>65.11</v>
       </c>
       <c r="H56" t="n">
-        <v>3.51</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I56" t="n">
-        <v>6.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D62" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E62" t="n">
-        <v>41.064</v>
+        <v>6.817</v>
       </c>
       <c r="F62" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G62" t="n">
-        <v>164.26</v>
+        <v>61.35</v>
       </c>
       <c r="H62" t="n">
-        <v>25.24</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>18.16</v>
+        <v>9.26</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E64" t="n">
-        <v>105.5</v>
+        <v>22.7</v>
       </c>
       <c r="F64" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G64" t="n">
-        <v>105.5</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H64" t="n">
-        <v>5.41</v>
+        <v>2.43</v>
       </c>
       <c r="I64" t="n">
-        <v>5.41</v>
+        <v>3.7</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E65" t="n">
-        <v>6.817</v>
+        <v>41.064</v>
       </c>
       <c r="F65" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G65" t="n">
-        <v>61.35</v>
+        <v>164.26</v>
       </c>
       <c r="H65" t="n">
-        <v>5.2</v>
+        <v>25.24</v>
       </c>
       <c r="I65" t="n">
-        <v>9.26</v>
+        <v>18.16</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E66" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F66" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G66" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H66" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I66" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D77" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E77" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F77" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G77" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H77" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I77" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E78" t="n">
-        <v>42.25</v>
+        <v>23.4</v>
       </c>
       <c r="F78" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G78" t="n">
-        <v>169</v>
+        <v>70.2</v>
       </c>
       <c r="H78" t="n">
-        <v>29.98</v>
+        <v>4.53</v>
       </c>
       <c r="I78" t="n">
-        <v>21.57</v>
+        <v>6.9</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D79" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E79" t="n">
-        <v>23.4</v>
+        <v>6.836</v>
       </c>
       <c r="F79" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G79" t="n">
-        <v>70.2</v>
+        <v>61.52</v>
       </c>
       <c r="H79" t="n">
-        <v>4.53</v>
+        <v>5.37</v>
       </c>
       <c r="I79" t="n">
-        <v>6.9</v>
+        <v>9.56</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E80" t="n">
-        <v>6.836</v>
+        <v>105.8</v>
       </c>
       <c r="F80" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G80" t="n">
-        <v>61.52</v>
+        <v>105.8</v>
       </c>
       <c r="H80" t="n">
-        <v>5.37</v>
+        <v>5.71</v>
       </c>
       <c r="I80" t="n">
-        <v>9.56</v>
+        <v>5.7</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D81" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E81" t="n">
-        <v>10.958</v>
+        <v>42.25</v>
       </c>
       <c r="F81" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G81" t="n">
-        <v>32.87</v>
+        <v>169</v>
       </c>
       <c r="H81" t="n">
-        <v>1.71</v>
+        <v>29.98</v>
       </c>
       <c r="I81" t="n">
-        <v>5.49</v>
+        <v>21.57</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E87" t="n">
-        <v>106.28</v>
+        <v>43.005</v>
       </c>
       <c r="F87" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G87" t="n">
-        <v>106.28</v>
+        <v>172.02</v>
       </c>
       <c r="H87" t="n">
-        <v>6.19</v>
+        <v>33</v>
       </c>
       <c r="I87" t="n">
-        <v>6.18</v>
+        <v>23.74</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E88" t="n">
-        <v>23.32</v>
+        <v>106.28</v>
       </c>
       <c r="F88" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G88" t="n">
-        <v>69.95999999999999</v>
+        <v>106.28</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>6.19</v>
       </c>
       <c r="I88" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C89" t="n">
         <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E89" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F89" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G89" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H89" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I89" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E90" t="n">
-        <v>6.856</v>
+        <v>10.852</v>
       </c>
       <c r="F90" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G90" t="n">
-        <v>61.7</v>
+        <v>32.56</v>
       </c>
       <c r="H90" t="n">
-        <v>5.55</v>
+        <v>1.4</v>
       </c>
       <c r="I90" t="n">
-        <v>9.880000000000001</v>
+        <v>4.49</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D91" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E91" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F91" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G91" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H91" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I91" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D92" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E92" t="n">
-        <v>103.88</v>
+        <v>6.797</v>
       </c>
       <c r="F92" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G92" t="n">
-        <v>103.88</v>
+        <v>61.17</v>
       </c>
       <c r="H92" t="n">
-        <v>3.79</v>
+        <v>5.02</v>
       </c>
       <c r="I92" t="n">
-        <v>3.79</v>
+        <v>8.94</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C93" t="n">
         <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E93" t="n">
-        <v>10.876</v>
+        <v>23.025</v>
       </c>
       <c r="F93" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G93" t="n">
-        <v>32.63</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H93" t="n">
-        <v>1.47</v>
+        <v>3.4</v>
       </c>
       <c r="I93" t="n">
-        <v>4.72</v>
+        <v>5.18</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E94" t="n">
-        <v>40.575</v>
+        <v>10.876</v>
       </c>
       <c r="F94" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G94" t="n">
-        <v>162.3</v>
+        <v>32.63</v>
       </c>
       <c r="H94" t="n">
-        <v>23.28</v>
+        <v>1.47</v>
       </c>
       <c r="I94" t="n">
-        <v>16.75</v>
+        <v>4.72</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E95" t="n">
-        <v>23.025</v>
+        <v>103.88</v>
       </c>
       <c r="F95" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G95" t="n">
-        <v>69.06999999999999</v>
+        <v>103.88</v>
       </c>
       <c r="H95" t="n">
-        <v>3.4</v>
+        <v>3.79</v>
       </c>
       <c r="I95" t="n">
-        <v>5.18</v>
+        <v>3.79</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D96" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E96" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F96" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G96" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H96" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I96" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D97" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E97" t="n">
-        <v>10.642</v>
+        <v>6.839</v>
       </c>
       <c r="F97" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G97" t="n">
-        <v>31.93</v>
+        <v>61.55</v>
       </c>
       <c r="H97" t="n">
-        <v>0.77</v>
+        <v>5.4</v>
       </c>
       <c r="I97" t="n">
-        <v>2.47</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E98" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F98" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G98" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H98" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I98" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D99" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E99" t="n">
-        <v>23.35</v>
+        <v>40.65</v>
       </c>
       <c r="F99" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G99" t="n">
-        <v>70.05</v>
+        <v>162.6</v>
       </c>
       <c r="H99" t="n">
-        <v>4.38</v>
+        <v>23.58</v>
       </c>
       <c r="I99" t="n">
-        <v>6.67</v>
+        <v>16.96</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E100" t="n">
-        <v>104.22</v>
+        <v>23.35</v>
       </c>
       <c r="F100" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G100" t="n">
-        <v>104.22</v>
+        <v>70.05</v>
       </c>
       <c r="H100" t="n">
-        <v>4.13</v>
+        <v>4.38</v>
       </c>
       <c r="I100" t="n">
-        <v>4.13</v>
+        <v>6.67</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,31 +3844,201 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E101" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="F101" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G101" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="H101" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="I101" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="J101" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E102" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="F102" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G102" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="H102" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I102" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J102" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>3</v>
+      </c>
+      <c r="D103" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E103" t="n">
+        <v>10.556</v>
+      </c>
+      <c r="F103" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G103" t="n">
+        <v>31.67</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="I103" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="J103" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>4</v>
+      </c>
+      <c r="D104" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E104" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="F104" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G104" t="n">
+        <v>163.88</v>
+      </c>
+      <c r="H104" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="I104" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="J104" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>3</v>
+      </c>
+      <c r="D105" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E105" t="n">
+        <v>23.29</v>
+      </c>
+      <c r="F105" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G105" t="n">
+        <v>69.87</v>
+      </c>
+      <c r="H105" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="I105" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="J105" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C101" t="n">
+      <c r="C106" t="n">
         <v>9</v>
       </c>
-      <c r="D101" t="n">
+      <c r="D106" t="n">
         <v>6.239</v>
       </c>
-      <c r="E101" t="n">
-        <v>6.839</v>
-      </c>
-      <c r="F101" t="n">
+      <c r="E106" t="n">
+        <v>6.804</v>
+      </c>
+      <c r="F106" t="n">
         <v>56.15</v>
       </c>
-      <c r="G101" t="n">
-        <v>61.55</v>
-      </c>
-      <c r="H101" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="I101" t="n">
-        <v>9.619999999999999</v>
-      </c>
-      <c r="J101" t="n">
+      <c r="G106" t="n">
+        <v>61.24</v>
+      </c>
+      <c r="H106" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="I106" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="J106" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 26/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>21.907</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>65.72</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>0.05</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>0.08</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E28" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F28" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G28" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H28" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I28" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E29" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F29" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G29" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H29" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I29" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E30" t="n">
-        <v>40.532</v>
+        <v>6.795</v>
       </c>
       <c r="F30" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G30" t="n">
-        <v>162.13</v>
+        <v>61.16</v>
       </c>
       <c r="H30" t="n">
-        <v>23.11</v>
+        <v>5.01</v>
       </c>
       <c r="I30" t="n">
-        <v>16.62</v>
+        <v>8.92</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E31" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F31" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G31" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H31" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I31" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E37" t="n">
-        <v>21.839</v>
+        <v>102.8</v>
       </c>
       <c r="F37" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G37" t="n">
-        <v>65.52</v>
+        <v>102.8</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.15</v>
+        <v>2.71</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.23</v>
+        <v>2.71</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E38" t="n">
-        <v>6.728</v>
+        <v>10.67</v>
       </c>
       <c r="F38" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G38" t="n">
-        <v>60.55</v>
+        <v>32.01</v>
       </c>
       <c r="H38" t="n">
-        <v>4.4</v>
+        <v>0.85</v>
       </c>
       <c r="I38" t="n">
-        <v>7.84</v>
+        <v>2.73</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E39" t="n">
-        <v>10.67</v>
+        <v>38.879</v>
       </c>
       <c r="F39" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G39" t="n">
-        <v>32.01</v>
+        <v>155.52</v>
       </c>
       <c r="H39" t="n">
-        <v>0.85</v>
+        <v>16.5</v>
       </c>
       <c r="I39" t="n">
-        <v>2.73</v>
+        <v>11.87</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E40" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F40" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G40" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H40" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I40" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D41" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E41" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F41" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G41" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H41" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I41" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E52" t="n">
-        <v>6.629</v>
+        <v>100.34</v>
       </c>
       <c r="F52" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G52" t="n">
-        <v>59.66</v>
+        <v>100.34</v>
       </c>
       <c r="H52" t="n">
-        <v>3.51</v>
+        <v>0.25</v>
       </c>
       <c r="I52" t="n">
-        <v>6.25</v>
+        <v>0.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E53" t="n">
-        <v>38.544</v>
+        <v>10.702</v>
       </c>
       <c r="F53" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G53" t="n">
-        <v>154.18</v>
+        <v>32.11</v>
       </c>
       <c r="H53" t="n">
-        <v>15.16</v>
+        <v>0.95</v>
       </c>
       <c r="I53" t="n">
-        <v>10.9</v>
+        <v>3.05</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E54" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F54" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G54" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H54" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E55" t="n">
-        <v>100.34</v>
+        <v>6.629</v>
       </c>
       <c r="F55" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G55" t="n">
-        <v>100.34</v>
+        <v>59.66</v>
       </c>
       <c r="H55" t="n">
-        <v>0.25</v>
+        <v>3.51</v>
       </c>
       <c r="I55" t="n">
-        <v>0.25</v>
+        <v>6.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D56" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E56" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F56" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G56" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D67" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E67" t="n">
-        <v>40.567</v>
+        <v>104.58</v>
       </c>
       <c r="F67" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G67" t="n">
-        <v>162.27</v>
+        <v>104.58</v>
       </c>
       <c r="H67" t="n">
-        <v>23.25</v>
+        <v>4.49</v>
       </c>
       <c r="I67" t="n">
-        <v>16.72</v>
+        <v>4.49</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D68" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E68" t="n">
-        <v>10.796</v>
+        <v>6.807</v>
       </c>
       <c r="F68" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G68" t="n">
-        <v>32.39</v>
+        <v>61.26</v>
       </c>
       <c r="H68" t="n">
-        <v>1.23</v>
+        <v>5.11</v>
       </c>
       <c r="I68" t="n">
-        <v>3.95</v>
+        <v>9.1</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D69" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E69" t="n">
-        <v>22.797</v>
+        <v>40.567</v>
       </c>
       <c r="F69" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G69" t="n">
-        <v>68.39</v>
+        <v>162.27</v>
       </c>
       <c r="H69" t="n">
-        <v>2.72</v>
+        <v>23.25</v>
       </c>
       <c r="I69" t="n">
-        <v>4.14</v>
+        <v>16.72</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E70" t="n">
-        <v>6.807</v>
+        <v>10.796</v>
       </c>
       <c r="F70" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G70" t="n">
-        <v>61.26</v>
+        <v>32.39</v>
       </c>
       <c r="H70" t="n">
-        <v>5.11</v>
+        <v>1.23</v>
       </c>
       <c r="I70" t="n">
-        <v>9.1</v>
+        <v>3.95</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E71" t="n">
-        <v>104.58</v>
+        <v>22.797</v>
       </c>
       <c r="F71" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G71" t="n">
-        <v>104.58</v>
+        <v>68.39</v>
       </c>
       <c r="H71" t="n">
-        <v>4.49</v>
+        <v>2.72</v>
       </c>
       <c r="I71" t="n">
-        <v>4.49</v>
+        <v>4.14</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E82" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F82" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G82" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H82" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I82" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D83" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E83" t="n">
-        <v>6.846</v>
+        <v>42.1</v>
       </c>
       <c r="F83" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G83" t="n">
-        <v>61.61</v>
+        <v>168.4</v>
       </c>
       <c r="H83" t="n">
-        <v>5.46</v>
+        <v>29.38</v>
       </c>
       <c r="I83" t="n">
-        <v>9.720000000000001</v>
+        <v>21.13</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E84" t="n">
-        <v>10.988</v>
+        <v>6.846</v>
       </c>
       <c r="F84" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G84" t="n">
-        <v>32.96</v>
+        <v>61.61</v>
       </c>
       <c r="H84" t="n">
-        <v>1.8</v>
+        <v>5.46</v>
       </c>
       <c r="I84" t="n">
-        <v>5.78</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E85" t="n">
-        <v>106.26</v>
+        <v>23.3</v>
       </c>
       <c r="F85" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G85" t="n">
-        <v>106.26</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H85" t="n">
-        <v>6.17</v>
+        <v>4.23</v>
       </c>
       <c r="I85" t="n">
-        <v>6.16</v>
+        <v>6.44</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E86" t="n">
-        <v>42.1</v>
+        <v>10.988</v>
       </c>
       <c r="F86" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G86" t="n">
-        <v>168.4</v>
+        <v>32.96</v>
       </c>
       <c r="H86" t="n">
-        <v>29.38</v>
+        <v>1.8</v>
       </c>
       <c r="I86" t="n">
-        <v>21.13</v>
+        <v>5.78</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D97" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E97" t="n">
-        <v>6.839</v>
+        <v>104.22</v>
       </c>
       <c r="F97" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G97" t="n">
-        <v>61.55</v>
+        <v>104.22</v>
       </c>
       <c r="H97" t="n">
-        <v>5.4</v>
+        <v>4.13</v>
       </c>
       <c r="I97" t="n">
-        <v>9.619999999999999</v>
+        <v>4.13</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E98" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F98" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G98" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H98" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I98" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D99" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E99" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F99" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G99" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H99" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I99" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D100" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E100" t="n">
-        <v>23.35</v>
+        <v>6.839</v>
       </c>
       <c r="F100" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G100" t="n">
-        <v>70.05</v>
+        <v>61.55</v>
       </c>
       <c r="H100" t="n">
-        <v>4.38</v>
+        <v>5.4</v>
       </c>
       <c r="I100" t="n">
-        <v>6.67</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D101" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E101" t="n">
-        <v>104.22</v>
+        <v>40.65</v>
       </c>
       <c r="F101" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G101" t="n">
-        <v>104.22</v>
+        <v>162.6</v>
       </c>
       <c r="H101" t="n">
-        <v>4.13</v>
+        <v>23.58</v>
       </c>
       <c r="I101" t="n">
-        <v>4.13</v>
+        <v>16.96</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4039,6 +4039,176 @@
         <v>9.07</v>
       </c>
       <c r="J106" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>3</v>
+      </c>
+      <c r="D107" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E107" t="n">
+        <v>10.456</v>
+      </c>
+      <c r="F107" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G107" t="n">
+        <v>31.37</v>
+      </c>
+      <c r="H107" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I107" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="J107" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>4</v>
+      </c>
+      <c r="D108" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E108" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F108" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G108" t="n">
+        <v>162</v>
+      </c>
+      <c r="H108" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="I108" t="n">
+        <v>16.53</v>
+      </c>
+      <c r="J108" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>3</v>
+      </c>
+      <c r="D109" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E109" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="F109" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G109" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="H109" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="I109" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="J109" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E110" t="n">
+        <v>103.14</v>
+      </c>
+      <c r="F110" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G110" t="n">
+        <v>103.14</v>
+      </c>
+      <c r="H110" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="I110" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="J110" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>9</v>
+      </c>
+      <c r="D111" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E111" t="n">
+        <v>6.785</v>
+      </c>
+      <c r="F111" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G111" t="n">
+        <v>61.06</v>
+      </c>
+      <c r="H111" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="I111" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="J111" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 29/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J111"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E13" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F13" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G13" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>105.22</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>105.22</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>5.13</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>5.13</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E27" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F27" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G27" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H27" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I27" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E28" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F28" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G28" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H28" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I28" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>6.795</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>61.16</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>5.01</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>8.92</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E31" t="n">
-        <v>104.9</v>
+        <v>40.532</v>
       </c>
       <c r="F31" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G31" t="n">
-        <v>104.9</v>
+        <v>162.13</v>
       </c>
       <c r="H31" t="n">
-        <v>4.81</v>
+        <v>23.11</v>
       </c>
       <c r="I31" t="n">
-        <v>4.81</v>
+        <v>16.62</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E42" t="n">
-        <v>100.06</v>
+        <v>6.629</v>
       </c>
       <c r="F42" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G42" t="n">
-        <v>100.06</v>
+        <v>59.66</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.03</v>
+        <v>3.51</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.03</v>
+        <v>6.25</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>6.629</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>59.66</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>3.51</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>6.25</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E46" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F46" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G46" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H46" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I46" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D57" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E57" t="n">
-        <v>10.75</v>
+        <v>6.736</v>
       </c>
       <c r="F57" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G57" t="n">
-        <v>32.25</v>
+        <v>60.62</v>
       </c>
       <c r="H57" t="n">
-        <v>1.09</v>
+        <v>4.47</v>
       </c>
       <c r="I57" t="n">
-        <v>3.5</v>
+        <v>7.96</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E58" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F58" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G58" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H58" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I58" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D60" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E60" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F60" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G60" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H60" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I60" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E61" t="n">
-        <v>6.736</v>
+        <v>10.75</v>
       </c>
       <c r="F61" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G61" t="n">
-        <v>60.62</v>
+        <v>32.25</v>
       </c>
       <c r="H61" t="n">
-        <v>4.47</v>
+        <v>1.09</v>
       </c>
       <c r="I61" t="n">
-        <v>7.96</v>
+        <v>3.5</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E72" t="n">
-        <v>10.892</v>
+        <v>104.22</v>
       </c>
       <c r="F72" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G72" t="n">
-        <v>32.68</v>
+        <v>104.22</v>
       </c>
       <c r="H72" t="n">
-        <v>1.52</v>
+        <v>4.13</v>
       </c>
       <c r="I72" t="n">
-        <v>4.88</v>
+        <v>4.13</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E75" t="n">
-        <v>41.15</v>
+        <v>6.811</v>
       </c>
       <c r="F75" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G75" t="n">
-        <v>164.6</v>
+        <v>61.3</v>
       </c>
       <c r="H75" t="n">
-        <v>25.58</v>
+        <v>5.15</v>
       </c>
       <c r="I75" t="n">
-        <v>18.4</v>
+        <v>9.17</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E76" t="n">
-        <v>104.22</v>
+        <v>10.892</v>
       </c>
       <c r="F76" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G76" t="n">
-        <v>104.22</v>
+        <v>32.68</v>
       </c>
       <c r="H76" t="n">
-        <v>4.13</v>
+        <v>1.52</v>
       </c>
       <c r="I76" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D87" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E87" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F87" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G87" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H87" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I87" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E88" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F88" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G88" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H88" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I88" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D89" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E89" t="n">
-        <v>23.32</v>
+        <v>106.28</v>
       </c>
       <c r="F89" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G89" t="n">
-        <v>69.95999999999999</v>
+        <v>106.28</v>
       </c>
       <c r="H89" t="n">
-        <v>4.29</v>
+        <v>6.19</v>
       </c>
       <c r="I89" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D90" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E90" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F90" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G90" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H90" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I90" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E91" t="n">
-        <v>6.856</v>
+        <v>23.32</v>
       </c>
       <c r="F91" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G91" t="n">
-        <v>61.7</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H91" t="n">
-        <v>5.55</v>
+        <v>4.29</v>
       </c>
       <c r="I91" t="n">
-        <v>9.880000000000001</v>
+        <v>6.53</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D97" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E97" t="n">
-        <v>104.22</v>
+        <v>40.65</v>
       </c>
       <c r="F97" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G97" t="n">
-        <v>104.22</v>
+        <v>162.6</v>
       </c>
       <c r="H97" t="n">
-        <v>4.13</v>
+        <v>23.58</v>
       </c>
       <c r="I97" t="n">
-        <v>4.13</v>
+        <v>16.96</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E98" t="n">
-        <v>23.35</v>
+        <v>104.22</v>
       </c>
       <c r="F98" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G98" t="n">
-        <v>70.05</v>
+        <v>104.22</v>
       </c>
       <c r="H98" t="n">
-        <v>4.38</v>
+        <v>4.13</v>
       </c>
       <c r="I98" t="n">
-        <v>6.67</v>
+        <v>4.13</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C99" t="n">
         <v>3</v>
       </c>
       <c r="D99" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E99" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F99" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G99" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H99" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I99" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E100" t="n">
-        <v>6.839</v>
+        <v>10.642</v>
       </c>
       <c r="F100" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G100" t="n">
-        <v>61.55</v>
+        <v>31.93</v>
       </c>
       <c r="H100" t="n">
-        <v>5.4</v>
+        <v>0.77</v>
       </c>
       <c r="I100" t="n">
-        <v>9.619999999999999</v>
+        <v>2.47</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D101" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E101" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F101" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G101" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H101" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I101" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D102" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E102" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F102" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G102" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H102" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I102" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C103" t="n">
         <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E103" t="n">
-        <v>10.556</v>
+        <v>23.29</v>
       </c>
       <c r="F103" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G103" t="n">
-        <v>31.67</v>
+        <v>69.87</v>
       </c>
       <c r="H103" t="n">
-        <v>0.51</v>
+        <v>4.2</v>
       </c>
       <c r="I103" t="n">
-        <v>1.64</v>
+        <v>6.4</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D104" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E104" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F104" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G104" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H104" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I104" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D105" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E105" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F105" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G105" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H105" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I105" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D106" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E106" t="n">
-        <v>6.804</v>
+        <v>40.97</v>
       </c>
       <c r="F106" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G106" t="n">
-        <v>61.24</v>
+        <v>163.88</v>
       </c>
       <c r="H106" t="n">
-        <v>5.09</v>
+        <v>24.86</v>
       </c>
       <c r="I106" t="n">
-        <v>9.07</v>
+        <v>17.88</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D107" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E107" t="n">
-        <v>10.456</v>
+        <v>6.785</v>
       </c>
       <c r="F107" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G107" t="n">
-        <v>31.37</v>
+        <v>61.06</v>
       </c>
       <c r="H107" t="n">
-        <v>0.21</v>
+        <v>4.91</v>
       </c>
       <c r="I107" t="n">
-        <v>0.67</v>
+        <v>8.74</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E108" t="n">
-        <v>40.5</v>
+        <v>10.456</v>
       </c>
       <c r="F108" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G108" t="n">
-        <v>162</v>
+        <v>31.37</v>
       </c>
       <c r="H108" t="n">
-        <v>22.98</v>
+        <v>0.21</v>
       </c>
       <c r="I108" t="n">
-        <v>16.53</v>
+        <v>0.67</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D109" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E109" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F109" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G109" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H109" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I109" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E110" t="n">
-        <v>103.14</v>
+        <v>23.33</v>
       </c>
       <c r="F110" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G110" t="n">
-        <v>103.14</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H110" t="n">
-        <v>3.05</v>
+        <v>4.32</v>
       </c>
       <c r="I110" t="n">
-        <v>3.05</v>
+        <v>6.58</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,31 +4184,201 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E111" t="n">
+        <v>103.14</v>
+      </c>
+      <c r="F111" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G111" t="n">
+        <v>103.14</v>
+      </c>
+      <c r="H111" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="I111" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="J111" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E112" t="n">
+        <v>103.56</v>
+      </c>
+      <c r="F112" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G112" t="n">
+        <v>103.56</v>
+      </c>
+      <c r="H112" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="I112" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="J112" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>3</v>
+      </c>
+      <c r="D113" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E113" t="n">
+        <v>10.568</v>
+      </c>
+      <c r="F113" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G113" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="H113" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="I113" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="J113" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>4</v>
+      </c>
+      <c r="D114" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E114" t="n">
+        <v>40</v>
+      </c>
+      <c r="F114" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G114" t="n">
+        <v>160</v>
+      </c>
+      <c r="H114" t="n">
+        <v>20.98</v>
+      </c>
+      <c r="I114" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="J114" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>3</v>
+      </c>
+      <c r="D115" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E115" t="n">
+        <v>23.025</v>
+      </c>
+      <c r="F115" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G115" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="H115" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I115" t="n">
+        <v>5.18</v>
+      </c>
+      <c r="J115" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="1" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C111" t="n">
+      <c r="C116" t="n">
         <v>9</v>
       </c>
-      <c r="D111" t="n">
+      <c r="D116" t="n">
         <v>6.239</v>
       </c>
-      <c r="E111" t="n">
-        <v>6.785</v>
-      </c>
-      <c r="F111" t="n">
+      <c r="E116" t="n">
+        <v>6.797</v>
+      </c>
+      <c r="F116" t="n">
         <v>56.15</v>
       </c>
-      <c r="G111" t="n">
-        <v>61.06</v>
-      </c>
-      <c r="H111" t="n">
-        <v>4.91</v>
-      </c>
-      <c r="I111" t="n">
-        <v>8.74</v>
-      </c>
-      <c r="J111" t="n">
+      <c r="G116" t="n">
+        <v>61.17</v>
+      </c>
+      <c r="H116" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="I116" t="n">
+        <v>8.94</v>
+      </c>
+      <c r="J116" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 30/06/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>105.22</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>105.22</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>5.13</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>5.13</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>10.756</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>32.27</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>1.11</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>3.56</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>41.121</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>164.48</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>25.46</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>18.31</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E27" t="n">
-        <v>104.9</v>
+        <v>40.532</v>
       </c>
       <c r="F27" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G27" t="n">
-        <v>104.9</v>
+        <v>162.13</v>
       </c>
       <c r="H27" t="n">
-        <v>4.81</v>
+        <v>23.11</v>
       </c>
       <c r="I27" t="n">
-        <v>4.81</v>
+        <v>16.62</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E28" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F28" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G28" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H28" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I28" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E29" t="n">
-        <v>6.795</v>
+        <v>10.66</v>
       </c>
       <c r="F29" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G29" t="n">
-        <v>61.16</v>
+        <v>31.98</v>
       </c>
       <c r="H29" t="n">
-        <v>5.01</v>
+        <v>0.82</v>
       </c>
       <c r="I29" t="n">
-        <v>8.92</v>
+        <v>2.63</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E31" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F31" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G31" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H31" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I31" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E42" t="n">
-        <v>6.629</v>
+        <v>22</v>
       </c>
       <c r="F42" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G42" t="n">
-        <v>59.66</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>3.51</v>
+        <v>0.33</v>
       </c>
       <c r="I42" t="n">
-        <v>6.25</v>
+        <v>0.5</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E45" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F45" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G45" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H45" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I45" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E46" t="n">
-        <v>100.06</v>
+        <v>6.629</v>
       </c>
       <c r="F46" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G46" t="n">
-        <v>100.06</v>
+        <v>59.66</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.03</v>
+        <v>3.51</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03</v>
+        <v>6.25</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>6.736</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>60.62</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>4.47</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>7.96</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>102.86</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>102.86</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>2.77</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>2.77</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D59" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E59" t="n">
-        <v>39.845</v>
+        <v>10.75</v>
       </c>
       <c r="F59" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G59" t="n">
-        <v>159.38</v>
+        <v>32.25</v>
       </c>
       <c r="H59" t="n">
-        <v>20.36</v>
+        <v>1.09</v>
       </c>
       <c r="I59" t="n">
-        <v>14.65</v>
+        <v>3.5</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E60" t="n">
-        <v>22.289</v>
+        <v>6.736</v>
       </c>
       <c r="F60" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G60" t="n">
-        <v>66.87</v>
+        <v>60.62</v>
       </c>
       <c r="H60" t="n">
-        <v>1.2</v>
+        <v>4.47</v>
       </c>
       <c r="I60" t="n">
-        <v>1.83</v>
+        <v>7.96</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E61" t="n">
-        <v>10.75</v>
+        <v>102.86</v>
       </c>
       <c r="F61" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G61" t="n">
-        <v>32.25</v>
+        <v>102.86</v>
       </c>
       <c r="H61" t="n">
-        <v>1.09</v>
+        <v>2.77</v>
       </c>
       <c r="I61" t="n">
-        <v>3.5</v>
+        <v>2.77</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>10.892</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>32.68</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>1.52</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>41.15</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>164.6</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>25.58</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>18.4</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E75" t="n">
-        <v>6.811</v>
+        <v>104.22</v>
       </c>
       <c r="F75" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G75" t="n">
-        <v>61.3</v>
+        <v>104.22</v>
       </c>
       <c r="H75" t="n">
-        <v>5.15</v>
+        <v>4.13</v>
       </c>
       <c r="I75" t="n">
-        <v>9.17</v>
+        <v>4.13</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D76" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E76" t="n">
-        <v>10.892</v>
+        <v>41.15</v>
       </c>
       <c r="F76" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G76" t="n">
-        <v>32.68</v>
+        <v>164.6</v>
       </c>
       <c r="H76" t="n">
-        <v>1.52</v>
+        <v>25.58</v>
       </c>
       <c r="I76" t="n">
-        <v>4.88</v>
+        <v>18.4</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D87" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E87" t="n">
-        <v>6.856</v>
+        <v>23.32</v>
       </c>
       <c r="F87" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G87" t="n">
-        <v>61.7</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H87" t="n">
-        <v>5.55</v>
+        <v>4.29</v>
       </c>
       <c r="I87" t="n">
-        <v>9.880000000000001</v>
+        <v>6.53</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E88" t="n">
-        <v>10.852</v>
+        <v>106.28</v>
       </c>
       <c r="F88" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G88" t="n">
-        <v>32.56</v>
+        <v>106.28</v>
       </c>
       <c r="H88" t="n">
-        <v>1.4</v>
+        <v>6.19</v>
       </c>
       <c r="I88" t="n">
-        <v>4.49</v>
+        <v>6.18</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D89" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E89" t="n">
-        <v>106.28</v>
+        <v>43.005</v>
       </c>
       <c r="F89" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G89" t="n">
-        <v>106.28</v>
+        <v>172.02</v>
       </c>
       <c r="H89" t="n">
-        <v>6.19</v>
+        <v>33</v>
       </c>
       <c r="I89" t="n">
-        <v>6.18</v>
+        <v>23.74</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E90" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F90" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G90" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H90" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I90" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C91" t="n">
         <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E91" t="n">
-        <v>23.32</v>
+        <v>10.852</v>
       </c>
       <c r="F91" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G91" t="n">
-        <v>69.95999999999999</v>
+        <v>32.56</v>
       </c>
       <c r="H91" t="n">
-        <v>4.29</v>
+        <v>1.4</v>
       </c>
       <c r="I91" t="n">
-        <v>6.53</v>
+        <v>4.49</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D102" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E102" t="n">
-        <v>6.804</v>
+        <v>40.97</v>
       </c>
       <c r="F102" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G102" t="n">
-        <v>61.24</v>
+        <v>163.88</v>
       </c>
       <c r="H102" t="n">
-        <v>5.09</v>
+        <v>24.86</v>
       </c>
       <c r="I102" t="n">
-        <v>9.07</v>
+        <v>17.88</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C103" t="n">
         <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E103" t="n">
-        <v>23.29</v>
+        <v>10.556</v>
       </c>
       <c r="F103" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G103" t="n">
-        <v>69.87</v>
+        <v>31.67</v>
       </c>
       <c r="H103" t="n">
-        <v>4.2</v>
+        <v>0.51</v>
       </c>
       <c r="I103" t="n">
-        <v>6.4</v>
+        <v>1.64</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E104" t="n">
-        <v>10.556</v>
+        <v>103.46</v>
       </c>
       <c r="F104" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G104" t="n">
-        <v>31.67</v>
+        <v>103.46</v>
       </c>
       <c r="H104" t="n">
-        <v>0.51</v>
+        <v>3.37</v>
       </c>
       <c r="I104" t="n">
-        <v>1.64</v>
+        <v>3.37</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D105" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E105" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F105" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G105" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H105" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I105" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D106" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E106" t="n">
-        <v>40.97</v>
+        <v>23.29</v>
       </c>
       <c r="F106" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G106" t="n">
-        <v>163.88</v>
+        <v>69.87</v>
       </c>
       <c r="H106" t="n">
-        <v>24.86</v>
+        <v>4.2</v>
       </c>
       <c r="I106" t="n">
-        <v>17.88</v>
+        <v>6.4</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D112" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E112" t="n">
-        <v>103.56</v>
+        <v>6.797</v>
       </c>
       <c r="F112" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G112" t="n">
-        <v>103.56</v>
+        <v>61.17</v>
       </c>
       <c r="H112" t="n">
-        <v>3.47</v>
+        <v>5.02</v>
       </c>
       <c r="I112" t="n">
-        <v>3.47</v>
+        <v>8.94</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C113" t="n">
         <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E113" t="n">
-        <v>10.568</v>
+        <v>23.025</v>
       </c>
       <c r="F113" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G113" t="n">
-        <v>31.7</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H113" t="n">
-        <v>0.54</v>
+        <v>3.4</v>
       </c>
       <c r="I113" t="n">
-        <v>1.73</v>
+        <v>5.18</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E114" t="n">
-        <v>40</v>
+        <v>10.568</v>
       </c>
       <c r="F114" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G114" t="n">
-        <v>160</v>
+        <v>31.7</v>
       </c>
       <c r="H114" t="n">
-        <v>20.98</v>
+        <v>0.54</v>
       </c>
       <c r="I114" t="n">
-        <v>15.09</v>
+        <v>1.73</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E115" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F115" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G115" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H115" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I115" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,31 +4354,201 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>4</v>
+      </c>
+      <c r="D116" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E116" t="n">
+        <v>40</v>
+      </c>
+      <c r="F116" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G116" t="n">
+        <v>160</v>
+      </c>
+      <c r="H116" t="n">
+        <v>20.98</v>
+      </c>
+      <c r="I116" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="J116" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>3</v>
+      </c>
+      <c r="D117" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E117" t="n">
+        <v>10.756</v>
+      </c>
+      <c r="F117" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G117" t="n">
+        <v>32.27</v>
+      </c>
+      <c r="H117" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="I117" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="J117" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>4</v>
+      </c>
+      <c r="D118" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E118" t="n">
+        <v>41</v>
+      </c>
+      <c r="F118" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G118" t="n">
+        <v>164</v>
+      </c>
+      <c r="H118" t="n">
+        <v>24.98</v>
+      </c>
+      <c r="I118" t="n">
+        <v>17.97</v>
+      </c>
+      <c r="J118" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>3</v>
+      </c>
+      <c r="D119" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E119" t="n">
+        <v>23.145</v>
+      </c>
+      <c r="F119" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G119" t="n">
+        <v>69.44</v>
+      </c>
+      <c r="H119" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="I119" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="J119" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E120" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="F120" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G120" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="H120" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="I120" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="J120" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C116" t="n">
+      <c r="C121" t="n">
         <v>9</v>
       </c>
-      <c r="D116" t="n">
+      <c r="D121" t="n">
         <v>6.239</v>
       </c>
-      <c r="E116" t="n">
-        <v>6.797</v>
-      </c>
-      <c r="F116" t="n">
+      <c r="E121" t="n">
+        <v>6.861</v>
+      </c>
+      <c r="F121" t="n">
         <v>56.15</v>
       </c>
-      <c r="G116" t="n">
-        <v>61.17</v>
-      </c>
-      <c r="H116" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="I116" t="n">
-        <v>8.94</v>
-      </c>
-      <c r="J116" t="n">
+      <c r="G121" t="n">
+        <v>61.75</v>
+      </c>
+      <c r="H121" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="I121" t="n">
+        <v>9.970000000000001</v>
+      </c>
+      <c r="J121" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 01/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E7" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F7" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G7" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H7" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I7" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E8" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F8" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G8" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H8" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I8" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E9" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F9" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G9" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H9" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I9" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E10" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F10" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G10" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H10" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I10" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E11" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F11" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G11" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H11" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I11" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E17" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F17" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G17" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H17" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I17" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E18" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F18" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G18" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H18" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I18" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E19" t="n">
-        <v>10.662</v>
+        <v>21.915</v>
       </c>
       <c r="F19" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G19" t="n">
-        <v>31.99</v>
+        <v>65.75</v>
       </c>
       <c r="H19" t="n">
-        <v>0.83</v>
+        <v>0.08</v>
       </c>
       <c r="I19" t="n">
-        <v>2.66</v>
+        <v>0.12</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E20" t="n">
-        <v>41.789</v>
+        <v>6.82</v>
       </c>
       <c r="F20" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G20" t="n">
-        <v>167.16</v>
+        <v>61.38</v>
       </c>
       <c r="H20" t="n">
-        <v>28.14</v>
+        <v>5.23</v>
       </c>
       <c r="I20" t="n">
-        <v>20.24</v>
+        <v>9.31</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E21" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F21" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G21" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H21" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I21" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E32" t="n">
-        <v>22.053</v>
+        <v>6.762</v>
       </c>
       <c r="F32" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G32" t="n">
-        <v>66.16</v>
+        <v>60.86</v>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>4.71</v>
       </c>
       <c r="I32" t="n">
-        <v>0.75</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E33" t="n">
-        <v>10.714</v>
+        <v>38.849</v>
       </c>
       <c r="F33" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G33" t="n">
-        <v>32.14</v>
+        <v>155.4</v>
       </c>
       <c r="H33" t="n">
-        <v>0.98</v>
+        <v>16.38</v>
       </c>
       <c r="I33" t="n">
-        <v>3.15</v>
+        <v>11.78</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E34" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F34" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G34" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H34" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I34" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E35" t="n">
-        <v>38.849</v>
+        <v>10.714</v>
       </c>
       <c r="F35" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G35" t="n">
-        <v>155.4</v>
+        <v>32.14</v>
       </c>
       <c r="H35" t="n">
-        <v>16.38</v>
+        <v>0.98</v>
       </c>
       <c r="I35" t="n">
-        <v>11.78</v>
+        <v>3.15</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E36" t="n">
-        <v>6.762</v>
+        <v>103.08</v>
       </c>
       <c r="F36" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G36" t="n">
-        <v>60.86</v>
+        <v>103.08</v>
       </c>
       <c r="H36" t="n">
-        <v>4.71</v>
+        <v>2.99</v>
       </c>
       <c r="I36" t="n">
-        <v>8.390000000000001</v>
+        <v>2.99</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D47" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E47" t="n">
-        <v>21.778</v>
+        <v>38.312</v>
       </c>
       <c r="F47" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G47" t="n">
-        <v>65.33</v>
+        <v>153.25</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.34</v>
+        <v>14.23</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.52</v>
+        <v>10.24</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E48" t="n">
-        <v>99.83</v>
+        <v>10.562</v>
       </c>
       <c r="F48" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G48" t="n">
-        <v>99.83</v>
+        <v>31.69</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.26</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.26</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E50" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F50" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G50" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I50" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E51" t="n">
-        <v>38.312</v>
+        <v>99.83</v>
       </c>
       <c r="F51" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G51" t="n">
-        <v>153.25</v>
+        <v>99.83</v>
       </c>
       <c r="H51" t="n">
-        <v>14.23</v>
+        <v>-0.26</v>
       </c>
       <c r="I51" t="n">
-        <v>10.24</v>
+        <v>-0.26</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E62" t="n">
-        <v>6.817</v>
+        <v>10.712</v>
       </c>
       <c r="F62" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G62" t="n">
-        <v>61.35</v>
+        <v>32.14</v>
       </c>
       <c r="H62" t="n">
-        <v>5.2</v>
+        <v>0.98</v>
       </c>
       <c r="I62" t="n">
-        <v>9.26</v>
+        <v>3.15</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E63" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F63" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G63" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H63" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I63" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E65" t="n">
-        <v>41.064</v>
+        <v>105.5</v>
       </c>
       <c r="F65" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G65" t="n">
-        <v>164.26</v>
+        <v>105.5</v>
       </c>
       <c r="H65" t="n">
-        <v>25.24</v>
+        <v>5.41</v>
       </c>
       <c r="I65" t="n">
-        <v>18.16</v>
+        <v>5.41</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D66" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E66" t="n">
-        <v>10.712</v>
+        <v>6.817</v>
       </c>
       <c r="F66" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G66" t="n">
-        <v>32.14</v>
+        <v>61.35</v>
       </c>
       <c r="H66" t="n">
-        <v>0.98</v>
+        <v>5.2</v>
       </c>
       <c r="I66" t="n">
-        <v>3.15</v>
+        <v>9.26</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E77" t="n">
-        <v>10.958</v>
+        <v>42.25</v>
       </c>
       <c r="F77" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G77" t="n">
-        <v>32.87</v>
+        <v>169</v>
       </c>
       <c r="H77" t="n">
-        <v>1.71</v>
+        <v>29.98</v>
       </c>
       <c r="I77" t="n">
-        <v>5.49</v>
+        <v>21.57</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E78" t="n">
-        <v>23.4</v>
+        <v>105.8</v>
       </c>
       <c r="F78" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G78" t="n">
-        <v>70.2</v>
+        <v>105.8</v>
       </c>
       <c r="H78" t="n">
-        <v>4.53</v>
+        <v>5.71</v>
       </c>
       <c r="I78" t="n">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E81" t="n">
-        <v>42.25</v>
+        <v>10.958</v>
       </c>
       <c r="F81" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G81" t="n">
-        <v>169</v>
+        <v>32.87</v>
       </c>
       <c r="H81" t="n">
-        <v>29.98</v>
+        <v>1.71</v>
       </c>
       <c r="I81" t="n">
-        <v>21.57</v>
+        <v>5.49</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D92" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E92" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F92" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G92" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H92" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I92" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C93" t="n">
         <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E93" t="n">
-        <v>23.025</v>
+        <v>10.876</v>
       </c>
       <c r="F93" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G93" t="n">
-        <v>69.06999999999999</v>
+        <v>32.63</v>
       </c>
       <c r="H93" t="n">
-        <v>3.4</v>
+        <v>1.47</v>
       </c>
       <c r="I93" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D94" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E94" t="n">
-        <v>10.876</v>
+        <v>103.88</v>
       </c>
       <c r="F94" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G94" t="n">
-        <v>32.63</v>
+        <v>103.88</v>
       </c>
       <c r="H94" t="n">
-        <v>1.47</v>
+        <v>3.79</v>
       </c>
       <c r="I94" t="n">
-        <v>4.72</v>
+        <v>3.79</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D95" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E95" t="n">
-        <v>103.88</v>
+        <v>6.797</v>
       </c>
       <c r="F95" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G95" t="n">
-        <v>103.88</v>
+        <v>61.17</v>
       </c>
       <c r="H95" t="n">
-        <v>3.79</v>
+        <v>5.02</v>
       </c>
       <c r="I95" t="n">
-        <v>3.79</v>
+        <v>8.94</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D96" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E96" t="n">
-        <v>40.575</v>
+        <v>23.025</v>
       </c>
       <c r="F96" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G96" t="n">
-        <v>162.3</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H96" t="n">
-        <v>23.28</v>
+        <v>3.4</v>
       </c>
       <c r="I96" t="n">
-        <v>16.75</v>
+        <v>5.18</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E107" t="n">
-        <v>6.785</v>
+        <v>23.33</v>
       </c>
       <c r="F107" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G107" t="n">
-        <v>61.06</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H107" t="n">
-        <v>4.91</v>
+        <v>4.32</v>
       </c>
       <c r="I107" t="n">
-        <v>8.74</v>
+        <v>6.58</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E108" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F108" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G108" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H108" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I108" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D109" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E109" t="n">
-        <v>40.5</v>
+        <v>10.456</v>
       </c>
       <c r="F109" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G109" t="n">
-        <v>162</v>
+        <v>31.37</v>
       </c>
       <c r="H109" t="n">
-        <v>22.98</v>
+        <v>0.21</v>
       </c>
       <c r="I109" t="n">
-        <v>16.53</v>
+        <v>0.67</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D110" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E110" t="n">
-        <v>23.33</v>
+        <v>6.785</v>
       </c>
       <c r="F110" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G110" t="n">
-        <v>69.98999999999999</v>
+        <v>61.06</v>
       </c>
       <c r="H110" t="n">
-        <v>4.32</v>
+        <v>4.91</v>
       </c>
       <c r="I110" t="n">
-        <v>6.58</v>
+        <v>8.74</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D111" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E111" t="n">
-        <v>103.14</v>
+        <v>40.5</v>
       </c>
       <c r="F111" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G111" t="n">
-        <v>103.14</v>
+        <v>162</v>
       </c>
       <c r="H111" t="n">
-        <v>3.05</v>
+        <v>22.98</v>
       </c>
       <c r="I111" t="n">
-        <v>3.05</v>
+        <v>16.53</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D117" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E117" t="n">
-        <v>10.756</v>
+        <v>6.861</v>
       </c>
       <c r="F117" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G117" t="n">
-        <v>32.27</v>
+        <v>61.75</v>
       </c>
       <c r="H117" t="n">
-        <v>1.11</v>
+        <v>5.6</v>
       </c>
       <c r="I117" t="n">
-        <v>3.56</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E118" t="n">
-        <v>41</v>
+        <v>10.756</v>
       </c>
       <c r="F118" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G118" t="n">
-        <v>164</v>
+        <v>32.27</v>
       </c>
       <c r="H118" t="n">
-        <v>24.98</v>
+        <v>1.11</v>
       </c>
       <c r="I118" t="n">
-        <v>17.97</v>
+        <v>3.56</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D119" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E119" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F119" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G119" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H119" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I119" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>23.145</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>69.44</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>3.77</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>5.74</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,31 +4524,201 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E121" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="F121" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G121" t="n">
+        <v>105.96</v>
+      </c>
+      <c r="H121" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="I121" t="n">
+        <v>5.86</v>
+      </c>
+      <c r="J121" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E122" t="n">
+        <v>106</v>
+      </c>
+      <c r="F122" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G122" t="n">
+        <v>106</v>
+      </c>
+      <c r="H122" t="n">
+        <v>5.91</v>
+      </c>
+      <c r="I122" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="J122" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>3</v>
+      </c>
+      <c r="D123" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E123" t="n">
+        <v>11.038</v>
+      </c>
+      <c r="F123" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G123" t="n">
+        <v>33.11</v>
+      </c>
+      <c r="H123" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="I123" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="J123" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>4</v>
+      </c>
+      <c r="D124" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E124" t="n">
+        <v>40.395</v>
+      </c>
+      <c r="F124" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G124" t="n">
+        <v>161.58</v>
+      </c>
+      <c r="H124" t="n">
+        <v>22.56</v>
+      </c>
+      <c r="I124" t="n">
+        <v>16.23</v>
+      </c>
+      <c r="J124" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>3</v>
+      </c>
+      <c r="D125" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E125" t="n">
+        <v>23.165</v>
+      </c>
+      <c r="F125" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G125" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="H125" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="I125" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="J125" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C121" t="n">
+      <c r="C126" t="n">
         <v>9</v>
       </c>
-      <c r="D121" t="n">
+      <c r="D126" t="n">
         <v>6.239</v>
       </c>
-      <c r="E121" t="n">
-        <v>6.861</v>
-      </c>
-      <c r="F121" t="n">
+      <c r="E126" t="n">
+        <v>6.901</v>
+      </c>
+      <c r="F126" t="n">
         <v>56.15</v>
       </c>
-      <c r="G121" t="n">
-        <v>61.75</v>
-      </c>
-      <c r="H121" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="I121" t="n">
-        <v>9.970000000000001</v>
-      </c>
-      <c r="J121" t="n">
+      <c r="G126" t="n">
+        <v>62.11</v>
+      </c>
+      <c r="H126" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="I126" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="J126" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 02/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J126"/>
+  <dimension ref="A1:J131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E7" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F7" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G7" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H7" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I7" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E8" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F8" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G8" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H8" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I8" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E9" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F9" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G9" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H9" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I9" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E10" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F10" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G10" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H10" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I10" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E11" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F11" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G11" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H11" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I11" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E17" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F17" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G17" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H17" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I17" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E18" t="n">
-        <v>41.789</v>
+        <v>6.82</v>
       </c>
       <c r="F18" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G18" t="n">
-        <v>167.16</v>
+        <v>61.38</v>
       </c>
       <c r="H18" t="n">
-        <v>28.14</v>
+        <v>5.23</v>
       </c>
       <c r="I18" t="n">
-        <v>20.24</v>
+        <v>9.31</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E19" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F19" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G19" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I19" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E20" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F20" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G20" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H20" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I20" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C21" t="n">
         <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E21" t="n">
-        <v>10.662</v>
+        <v>21.915</v>
       </c>
       <c r="F21" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G21" t="n">
-        <v>31.99</v>
+        <v>65.75</v>
       </c>
       <c r="H21" t="n">
-        <v>0.83</v>
+        <v>0.08</v>
       </c>
       <c r="I21" t="n">
-        <v>2.66</v>
+        <v>0.12</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E32" t="n">
-        <v>6.762</v>
+        <v>103.08</v>
       </c>
       <c r="F32" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G32" t="n">
-        <v>60.86</v>
+        <v>103.08</v>
       </c>
       <c r="H32" t="n">
-        <v>4.71</v>
+        <v>2.99</v>
       </c>
       <c r="I32" t="n">
-        <v>8.390000000000001</v>
+        <v>2.99</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E33" t="n">
-        <v>38.849</v>
+        <v>10.714</v>
       </c>
       <c r="F33" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G33" t="n">
-        <v>155.4</v>
+        <v>32.14</v>
       </c>
       <c r="H33" t="n">
-        <v>16.38</v>
+        <v>0.98</v>
       </c>
       <c r="I33" t="n">
-        <v>11.78</v>
+        <v>3.15</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E34" t="n">
-        <v>22.053</v>
+        <v>6.762</v>
       </c>
       <c r="F34" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G34" t="n">
-        <v>66.16</v>
+        <v>60.86</v>
       </c>
       <c r="H34" t="n">
-        <v>0.49</v>
+        <v>4.71</v>
       </c>
       <c r="I34" t="n">
-        <v>0.75</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E35" t="n">
-        <v>10.714</v>
+        <v>38.849</v>
       </c>
       <c r="F35" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G35" t="n">
-        <v>32.14</v>
+        <v>155.4</v>
       </c>
       <c r="H35" t="n">
-        <v>0.98</v>
+        <v>16.38</v>
       </c>
       <c r="I35" t="n">
-        <v>3.15</v>
+        <v>11.78</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E36" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F36" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G36" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H36" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I36" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E47" t="n">
-        <v>38.312</v>
+        <v>99.83</v>
       </c>
       <c r="F47" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G47" t="n">
-        <v>153.25</v>
+        <v>99.83</v>
       </c>
       <c r="H47" t="n">
-        <v>14.23</v>
+        <v>-0.26</v>
       </c>
       <c r="I47" t="n">
-        <v>10.24</v>
+        <v>-0.26</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C48" t="n">
         <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E48" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F48" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G48" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E50" t="n">
-        <v>21.778</v>
+        <v>38.312</v>
       </c>
       <c r="F50" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G50" t="n">
-        <v>65.33</v>
+        <v>153.25</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.34</v>
+        <v>14.23</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.52</v>
+        <v>10.24</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E51" t="n">
-        <v>99.83</v>
+        <v>10.562</v>
       </c>
       <c r="F51" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G51" t="n">
-        <v>99.83</v>
+        <v>31.69</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.26</v>
+        <v>0.53</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.26</v>
+        <v>1.7</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E62" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F62" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G62" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H62" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I62" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E63" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F63" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G63" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I63" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E64" t="n">
-        <v>22.7</v>
+        <v>6.817</v>
       </c>
       <c r="F64" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G64" t="n">
-        <v>68.09999999999999</v>
+        <v>61.35</v>
       </c>
       <c r="H64" t="n">
-        <v>2.43</v>
+        <v>5.2</v>
       </c>
       <c r="I64" t="n">
-        <v>3.7</v>
+        <v>9.26</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>105.5</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>105.5</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>5.41</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>5.41</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D66" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E66" t="n">
-        <v>6.817</v>
+        <v>41.064</v>
       </c>
       <c r="F66" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G66" t="n">
-        <v>61.35</v>
+        <v>164.26</v>
       </c>
       <c r="H66" t="n">
-        <v>5.2</v>
+        <v>25.24</v>
       </c>
       <c r="I66" t="n">
-        <v>9.26</v>
+        <v>18.16</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D77" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E77" t="n">
-        <v>42.25</v>
+        <v>23.4</v>
       </c>
       <c r="F77" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G77" t="n">
-        <v>169</v>
+        <v>70.2</v>
       </c>
       <c r="H77" t="n">
-        <v>29.98</v>
+        <v>4.53</v>
       </c>
       <c r="I77" t="n">
-        <v>21.57</v>
+        <v>6.9</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D78" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E78" t="n">
-        <v>105.8</v>
+        <v>6.836</v>
       </c>
       <c r="F78" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G78" t="n">
-        <v>105.8</v>
+        <v>61.52</v>
       </c>
       <c r="H78" t="n">
-        <v>5.71</v>
+        <v>5.37</v>
       </c>
       <c r="I78" t="n">
-        <v>5.7</v>
+        <v>9.56</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E79" t="n">
-        <v>6.836</v>
+        <v>10.958</v>
       </c>
       <c r="F79" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G79" t="n">
-        <v>61.52</v>
+        <v>32.87</v>
       </c>
       <c r="H79" t="n">
-        <v>5.37</v>
+        <v>1.71</v>
       </c>
       <c r="I79" t="n">
-        <v>9.56</v>
+        <v>5.49</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D80" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E80" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F80" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G80" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H80" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I80" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E81" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F81" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G81" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H81" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I81" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E82" t="n">
-        <v>106.26</v>
+        <v>10.988</v>
       </c>
       <c r="F82" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G82" t="n">
-        <v>106.26</v>
+        <v>32.96</v>
       </c>
       <c r="H82" t="n">
-        <v>6.17</v>
+        <v>1.8</v>
       </c>
       <c r="I82" t="n">
-        <v>6.16</v>
+        <v>5.78</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E83" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F83" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G83" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H83" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I83" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D84" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E84" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F84" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G84" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H84" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I84" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D85" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E85" t="n">
-        <v>23.3</v>
+        <v>42.1</v>
       </c>
       <c r="F85" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G85" t="n">
-        <v>69.90000000000001</v>
+        <v>168.4</v>
       </c>
       <c r="H85" t="n">
-        <v>4.23</v>
+        <v>29.38</v>
       </c>
       <c r="I85" t="n">
-        <v>6.44</v>
+        <v>21.13</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D86" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E86" t="n">
-        <v>10.988</v>
+        <v>6.846</v>
       </c>
       <c r="F86" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G86" t="n">
-        <v>32.96</v>
+        <v>61.61</v>
       </c>
       <c r="H86" t="n">
-        <v>1.8</v>
+        <v>5.46</v>
       </c>
       <c r="I86" t="n">
-        <v>5.78</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D89" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E89" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F89" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G89" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H89" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I89" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E90" t="n">
-        <v>6.856</v>
+        <v>10.852</v>
       </c>
       <c r="F90" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G90" t="n">
-        <v>61.7</v>
+        <v>32.56</v>
       </c>
       <c r="H90" t="n">
-        <v>5.55</v>
+        <v>1.4</v>
       </c>
       <c r="I90" t="n">
-        <v>9.880000000000001</v>
+        <v>4.49</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E91" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F91" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G91" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H91" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I91" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D97" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E97" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F97" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G97" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H97" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I97" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E98" t="n">
-        <v>104.22</v>
+        <v>10.642</v>
       </c>
       <c r="F98" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G98" t="n">
-        <v>104.22</v>
+        <v>31.93</v>
       </c>
       <c r="H98" t="n">
-        <v>4.13</v>
+        <v>0.77</v>
       </c>
       <c r="I98" t="n">
-        <v>4.13</v>
+        <v>2.47</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D99" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E99" t="n">
-        <v>23.35</v>
+        <v>104.22</v>
       </c>
       <c r="F99" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G99" t="n">
-        <v>70.05</v>
+        <v>104.22</v>
       </c>
       <c r="H99" t="n">
-        <v>4.38</v>
+        <v>4.13</v>
       </c>
       <c r="I99" t="n">
-        <v>6.67</v>
+        <v>4.13</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E100" t="n">
-        <v>10.642</v>
+        <v>40.65</v>
       </c>
       <c r="F100" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G100" t="n">
-        <v>31.93</v>
+        <v>162.6</v>
       </c>
       <c r="H100" t="n">
-        <v>0.77</v>
+        <v>23.58</v>
       </c>
       <c r="I100" t="n">
-        <v>2.47</v>
+        <v>16.96</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E101" t="n">
-        <v>6.839</v>
+        <v>23.35</v>
       </c>
       <c r="F101" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G101" t="n">
-        <v>61.55</v>
+        <v>70.05</v>
       </c>
       <c r="H101" t="n">
-        <v>5.4</v>
+        <v>4.38</v>
       </c>
       <c r="I101" t="n">
-        <v>9.619999999999999</v>
+        <v>6.67</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E112" t="n">
-        <v>6.797</v>
+        <v>40</v>
       </c>
       <c r="F112" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G112" t="n">
-        <v>61.17</v>
+        <v>160</v>
       </c>
       <c r="H112" t="n">
-        <v>5.02</v>
+        <v>20.98</v>
       </c>
       <c r="I112" t="n">
-        <v>8.94</v>
+        <v>15.09</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C113" t="n">
         <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E113" t="n">
-        <v>23.025</v>
+        <v>10.568</v>
       </c>
       <c r="F113" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G113" t="n">
-        <v>69.06999999999999</v>
+        <v>31.7</v>
       </c>
       <c r="H113" t="n">
-        <v>3.4</v>
+        <v>0.54</v>
       </c>
       <c r="I113" t="n">
-        <v>5.18</v>
+        <v>1.73</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E114" t="n">
-        <v>10.568</v>
+        <v>103.56</v>
       </c>
       <c r="F114" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G114" t="n">
-        <v>31.7</v>
+        <v>103.56</v>
       </c>
       <c r="H114" t="n">
-        <v>0.54</v>
+        <v>3.47</v>
       </c>
       <c r="I114" t="n">
-        <v>1.73</v>
+        <v>3.47</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D115" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E115" t="n">
-        <v>103.56</v>
+        <v>6.797</v>
       </c>
       <c r="F115" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G115" t="n">
-        <v>103.56</v>
+        <v>61.17</v>
       </c>
       <c r="H115" t="n">
-        <v>3.47</v>
+        <v>5.02</v>
       </c>
       <c r="I115" t="n">
-        <v>3.47</v>
+        <v>8.94</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E116" t="n">
-        <v>40</v>
+        <v>23.025</v>
       </c>
       <c r="F116" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G116" t="n">
-        <v>160</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H116" t="n">
-        <v>20.98</v>
+        <v>3.4</v>
       </c>
       <c r="I116" t="n">
-        <v>15.09</v>
+        <v>5.18</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D122" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E122" t="n">
-        <v>106</v>
+        <v>6.901</v>
       </c>
       <c r="F122" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G122" t="n">
-        <v>106</v>
+        <v>62.11</v>
       </c>
       <c r="H122" t="n">
-        <v>5.91</v>
+        <v>5.96</v>
       </c>
       <c r="I122" t="n">
-        <v>5.9</v>
+        <v>10.61</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C123" t="n">
         <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E123" t="n">
-        <v>11.038</v>
+        <v>23.165</v>
       </c>
       <c r="F123" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G123" t="n">
-        <v>33.11</v>
+        <v>69.5</v>
       </c>
       <c r="H123" t="n">
-        <v>1.95</v>
+        <v>3.83</v>
       </c>
       <c r="I123" t="n">
-        <v>6.26</v>
+        <v>5.83</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E124" t="n">
-        <v>40.395</v>
+        <v>11.038</v>
       </c>
       <c r="F124" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G124" t="n">
-        <v>161.58</v>
+        <v>33.11</v>
       </c>
       <c r="H124" t="n">
-        <v>22.56</v>
+        <v>1.95</v>
       </c>
       <c r="I124" t="n">
-        <v>16.23</v>
+        <v>6.26</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D125" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E125" t="n">
-        <v>23.165</v>
+        <v>106</v>
       </c>
       <c r="F125" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G125" t="n">
-        <v>69.5</v>
+        <v>106</v>
       </c>
       <c r="H125" t="n">
-        <v>3.83</v>
+        <v>5.91</v>
       </c>
       <c r="I125" t="n">
-        <v>5.83</v>
+        <v>5.9</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,31 +4694,201 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>4</v>
+      </c>
+      <c r="D126" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E126" t="n">
+        <v>40.395</v>
+      </c>
+      <c r="F126" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G126" t="n">
+        <v>161.58</v>
+      </c>
+      <c r="H126" t="n">
+        <v>22.56</v>
+      </c>
+      <c r="I126" t="n">
+        <v>16.23</v>
+      </c>
+      <c r="J126" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>3</v>
+      </c>
+      <c r="D127" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E127" t="n">
+        <v>11.458</v>
+      </c>
+      <c r="F127" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G127" t="n">
+        <v>34.37</v>
+      </c>
+      <c r="H127" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="I127" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="J127" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>4</v>
+      </c>
+      <c r="D128" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E128" t="n">
+        <v>39.36</v>
+      </c>
+      <c r="F128" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G128" t="n">
+        <v>157.44</v>
+      </c>
+      <c r="H128" t="n">
+        <v>18.42</v>
+      </c>
+      <c r="I128" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="J128" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>3</v>
+      </c>
+      <c r="D129" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E129" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="F129" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G129" t="n">
+        <v>69.51000000000001</v>
+      </c>
+      <c r="H129" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="I129" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="J129" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E130" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="F130" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G130" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="H130" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I130" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J130" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C126" t="n">
+      <c r="C131" t="n">
         <v>9</v>
       </c>
-      <c r="D126" t="n">
+      <c r="D131" t="n">
         <v>6.239</v>
       </c>
-      <c r="E126" t="n">
-        <v>6.901</v>
-      </c>
-      <c r="F126" t="n">
+      <c r="E131" t="n">
+        <v>6.868</v>
+      </c>
+      <c r="F131" t="n">
         <v>56.15</v>
       </c>
-      <c r="G126" t="n">
-        <v>62.11</v>
-      </c>
-      <c r="H126" t="n">
-        <v>5.96</v>
-      </c>
-      <c r="I126" t="n">
-        <v>10.61</v>
-      </c>
-      <c r="J126" t="n">
+      <c r="G131" t="n">
+        <v>61.81</v>
+      </c>
+      <c r="H131" t="n">
+        <v>5.66</v>
+      </c>
+      <c r="I131" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="J131" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 03/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J131"/>
+  <dimension ref="A1:J136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E7" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F7" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G7" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H7" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I7" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E8" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F8" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G8" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H8" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I8" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E9" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F9" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G9" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H9" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I9" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E10" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F10" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G10" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H10" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I10" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E11" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F11" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G11" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H11" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I11" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E17" t="n">
-        <v>10.662</v>
+        <v>21.915</v>
       </c>
       <c r="F17" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G17" t="n">
-        <v>31.99</v>
+        <v>65.75</v>
       </c>
       <c r="H17" t="n">
-        <v>0.83</v>
+        <v>0.08</v>
       </c>
       <c r="I17" t="n">
-        <v>2.66</v>
+        <v>0.12</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E18" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F18" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G18" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H18" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I18" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E19" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F19" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G19" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H19" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I19" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E20" t="n">
-        <v>41.789</v>
+        <v>6.82</v>
       </c>
       <c r="F20" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G20" t="n">
-        <v>167.16</v>
+        <v>61.38</v>
       </c>
       <c r="H20" t="n">
-        <v>28.14</v>
+        <v>5.23</v>
       </c>
       <c r="I20" t="n">
-        <v>20.24</v>
+        <v>9.31</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E21" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F21" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G21" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H21" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I21" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E32" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F32" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G32" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H32" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I32" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D33" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E33" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F33" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G33" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H33" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I33" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E34" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F34" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G34" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H34" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I34" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E35" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F35" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G35" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H35" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I35" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E36" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F36" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G36" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H36" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E47" t="n">
-        <v>99.83</v>
+        <v>10.562</v>
       </c>
       <c r="F47" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G47" t="n">
-        <v>99.83</v>
+        <v>31.69</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.26</v>
+        <v>0.53</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.26</v>
+        <v>1.7</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E48" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F48" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G48" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I48" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E49" t="n">
-        <v>6.622</v>
+        <v>38.312</v>
       </c>
       <c r="F49" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G49" t="n">
-        <v>59.6</v>
+        <v>153.25</v>
       </c>
       <c r="H49" t="n">
-        <v>3.45</v>
+        <v>14.23</v>
       </c>
       <c r="I49" t="n">
-        <v>6.14</v>
+        <v>10.24</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E50" t="n">
-        <v>38.312</v>
+        <v>99.83</v>
       </c>
       <c r="F50" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G50" t="n">
-        <v>153.25</v>
+        <v>99.83</v>
       </c>
       <c r="H50" t="n">
-        <v>14.23</v>
+        <v>-0.26</v>
       </c>
       <c r="I50" t="n">
-        <v>10.24</v>
+        <v>-0.26</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E51" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F51" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G51" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H51" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I51" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>39.845</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>159.38</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>20.36</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>14.65</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>22.289</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>66.87</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>1.2</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>1.83</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D62" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E62" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F62" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G62" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H62" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E64" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F64" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G64" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H64" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I64" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E65" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F65" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G65" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H65" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I65" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E67" t="n">
-        <v>104.58</v>
+        <v>22.797</v>
       </c>
       <c r="F67" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G67" t="n">
-        <v>104.58</v>
+        <v>68.39</v>
       </c>
       <c r="H67" t="n">
-        <v>4.49</v>
+        <v>2.72</v>
       </c>
       <c r="I67" t="n">
-        <v>4.49</v>
+        <v>4.14</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E68" t="n">
-        <v>6.807</v>
+        <v>10.796</v>
       </c>
       <c r="F68" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G68" t="n">
-        <v>61.26</v>
+        <v>32.39</v>
       </c>
       <c r="H68" t="n">
-        <v>5.11</v>
+        <v>1.23</v>
       </c>
       <c r="I68" t="n">
-        <v>9.1</v>
+        <v>3.95</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E70" t="n">
-        <v>10.796</v>
+        <v>6.807</v>
       </c>
       <c r="F70" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G70" t="n">
-        <v>32.39</v>
+        <v>61.26</v>
       </c>
       <c r="H70" t="n">
-        <v>1.23</v>
+        <v>5.11</v>
       </c>
       <c r="I70" t="n">
-        <v>3.95</v>
+        <v>9.1</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E71" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F71" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G71" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H71" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I71" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D82" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E82" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F82" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G82" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H82" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I82" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D83" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E83" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F83" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G83" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H83" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I83" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E84" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F84" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G84" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H84" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I84" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E85" t="n">
-        <v>42.1</v>
+        <v>10.988</v>
       </c>
       <c r="F85" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G85" t="n">
-        <v>168.4</v>
+        <v>32.96</v>
       </c>
       <c r="H85" t="n">
-        <v>29.38</v>
+        <v>1.8</v>
       </c>
       <c r="I85" t="n">
-        <v>21.13</v>
+        <v>5.78</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E86" t="n">
-        <v>6.846</v>
+        <v>23.3</v>
       </c>
       <c r="F86" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G86" t="n">
-        <v>61.61</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H86" t="n">
-        <v>5.46</v>
+        <v>4.23</v>
       </c>
       <c r="I86" t="n">
-        <v>9.720000000000001</v>
+        <v>6.44</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E92" t="n">
-        <v>40.575</v>
+        <v>23.025</v>
       </c>
       <c r="F92" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G92" t="n">
-        <v>162.3</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H92" t="n">
-        <v>23.28</v>
+        <v>3.4</v>
       </c>
       <c r="I92" t="n">
-        <v>16.75</v>
+        <v>5.18</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D93" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E93" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F93" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G93" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H93" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I93" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D95" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E95" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F95" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G95" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H95" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I95" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C96" t="n">
         <v>3</v>
       </c>
       <c r="D96" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E96" t="n">
-        <v>23.025</v>
+        <v>10.876</v>
       </c>
       <c r="F96" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G96" t="n">
-        <v>69.06999999999999</v>
+        <v>32.63</v>
       </c>
       <c r="H96" t="n">
-        <v>3.4</v>
+        <v>1.47</v>
       </c>
       <c r="I96" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E102" t="n">
-        <v>40.97</v>
+        <v>23.29</v>
       </c>
       <c r="F102" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G102" t="n">
-        <v>163.88</v>
+        <v>69.87</v>
       </c>
       <c r="H102" t="n">
-        <v>24.86</v>
+        <v>4.2</v>
       </c>
       <c r="I102" t="n">
-        <v>17.88</v>
+        <v>6.4</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D103" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E103" t="n">
-        <v>10.556</v>
+        <v>6.804</v>
       </c>
       <c r="F103" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G103" t="n">
-        <v>31.67</v>
+        <v>61.24</v>
       </c>
       <c r="H103" t="n">
-        <v>0.51</v>
+        <v>5.09</v>
       </c>
       <c r="I103" t="n">
-        <v>1.64</v>
+        <v>9.07</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D104" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E104" t="n">
-        <v>103.46</v>
+        <v>10.556</v>
       </c>
       <c r="F104" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G104" t="n">
-        <v>103.46</v>
+        <v>31.67</v>
       </c>
       <c r="H104" t="n">
-        <v>3.37</v>
+        <v>0.51</v>
       </c>
       <c r="I104" t="n">
-        <v>3.37</v>
+        <v>1.64</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D105" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E105" t="n">
-        <v>6.804</v>
+        <v>40.97</v>
       </c>
       <c r="F105" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G105" t="n">
-        <v>61.24</v>
+        <v>163.88</v>
       </c>
       <c r="H105" t="n">
-        <v>5.09</v>
+        <v>24.86</v>
       </c>
       <c r="I105" t="n">
-        <v>9.07</v>
+        <v>17.88</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D106" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E106" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F106" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G106" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H106" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I106" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E117" t="n">
-        <v>6.861</v>
+        <v>23.145</v>
       </c>
       <c r="F117" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G117" t="n">
-        <v>61.75</v>
+        <v>69.44</v>
       </c>
       <c r="H117" t="n">
-        <v>5.6</v>
+        <v>3.77</v>
       </c>
       <c r="I117" t="n">
-        <v>9.970000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E118" t="n">
-        <v>10.756</v>
+        <v>105.96</v>
       </c>
       <c r="F118" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G118" t="n">
-        <v>32.27</v>
+        <v>105.96</v>
       </c>
       <c r="H118" t="n">
-        <v>1.11</v>
+        <v>5.87</v>
       </c>
       <c r="I118" t="n">
-        <v>3.56</v>
+        <v>5.86</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E119" t="n">
-        <v>41</v>
+        <v>10.756</v>
       </c>
       <c r="F119" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G119" t="n">
-        <v>164</v>
+        <v>32.27</v>
       </c>
       <c r="H119" t="n">
-        <v>24.98</v>
+        <v>1.11</v>
       </c>
       <c r="I119" t="n">
-        <v>17.97</v>
+        <v>3.56</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D120" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E120" t="n">
-        <v>23.145</v>
+        <v>6.861</v>
       </c>
       <c r="F120" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G120" t="n">
-        <v>69.44</v>
+        <v>61.75</v>
       </c>
       <c r="H120" t="n">
-        <v>3.77</v>
+        <v>5.6</v>
       </c>
       <c r="I120" t="n">
-        <v>5.74</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D121" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E121" t="n">
-        <v>105.96</v>
+        <v>41</v>
       </c>
       <c r="F121" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G121" t="n">
-        <v>105.96</v>
+        <v>164</v>
       </c>
       <c r="H121" t="n">
-        <v>5.87</v>
+        <v>24.98</v>
       </c>
       <c r="I121" t="n">
-        <v>5.86</v>
+        <v>17.97</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D127" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E127" t="n">
-        <v>11.458</v>
+        <v>6.868</v>
       </c>
       <c r="F127" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G127" t="n">
-        <v>34.37</v>
+        <v>61.81</v>
       </c>
       <c r="H127" t="n">
-        <v>3.21</v>
+        <v>5.66</v>
       </c>
       <c r="I127" t="n">
-        <v>10.3</v>
+        <v>10.08</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E128" t="n">
-        <v>39.36</v>
+        <v>11.458</v>
       </c>
       <c r="F128" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G128" t="n">
-        <v>157.44</v>
+        <v>34.37</v>
       </c>
       <c r="H128" t="n">
-        <v>18.42</v>
+        <v>3.21</v>
       </c>
       <c r="I128" t="n">
-        <v>13.25</v>
+        <v>10.3</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4796,29 +4796,29 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D129" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E129" t="n">
-        <v>23.17</v>
+        <v>39.36</v>
       </c>
       <c r="F129" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G129" t="n">
-        <v>69.51000000000001</v>
+        <v>157.44</v>
       </c>
       <c r="H129" t="n">
-        <v>3.84</v>
+        <v>18.42</v>
       </c>
       <c r="I129" t="n">
-        <v>5.85</v>
+        <v>13.25</v>
       </c>
       <c r="J129" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E130" t="n">
-        <v>103.46</v>
+        <v>23.17</v>
       </c>
       <c r="F130" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G130" t="n">
-        <v>103.46</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H130" t="n">
-        <v>3.37</v>
+        <v>3.84</v>
       </c>
       <c r="I130" t="n">
-        <v>3.37</v>
+        <v>5.85</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,31 +4864,201 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E131" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="F131" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G131" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="H131" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I131" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J131" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E132" t="n">
+        <v>104.02</v>
+      </c>
+      <c r="F132" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G132" t="n">
+        <v>104.02</v>
+      </c>
+      <c r="H132" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="I132" t="n">
+        <v>3.93</v>
+      </c>
+      <c r="J132" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>3</v>
+      </c>
+      <c r="D133" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E133" t="n">
+        <v>11.516</v>
+      </c>
+      <c r="F133" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G133" t="n">
+        <v>34.55</v>
+      </c>
+      <c r="H133" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="I133" t="n">
+        <v>10.88</v>
+      </c>
+      <c r="J133" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>4</v>
+      </c>
+      <c r="D134" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E134" t="n">
+        <v>40.54</v>
+      </c>
+      <c r="F134" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G134" t="n">
+        <v>162.16</v>
+      </c>
+      <c r="H134" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="I134" t="n">
+        <v>16.65</v>
+      </c>
+      <c r="J134" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>3</v>
+      </c>
+      <c r="D135" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E135" t="n">
+        <v>23.18</v>
+      </c>
+      <c r="F135" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G135" t="n">
+        <v>69.54000000000001</v>
+      </c>
+      <c r="H135" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="I135" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="J135" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C131" t="n">
+      <c r="C136" t="n">
         <v>9</v>
       </c>
-      <c r="D131" t="n">
+      <c r="D136" t="n">
         <v>6.239</v>
       </c>
-      <c r="E131" t="n">
-        <v>6.868</v>
-      </c>
-      <c r="F131" t="n">
+      <c r="E136" t="n">
+        <v>6.895</v>
+      </c>
+      <c r="F136" t="n">
         <v>56.15</v>
       </c>
-      <c r="G131" t="n">
-        <v>61.81</v>
-      </c>
-      <c r="H131" t="n">
-        <v>5.66</v>
-      </c>
-      <c r="I131" t="n">
-        <v>10.08</v>
-      </c>
-      <c r="J131" t="n">
+      <c r="G136" t="n">
+        <v>62.05</v>
+      </c>
+      <c r="H136" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I136" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="J136" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 06/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J136"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E7" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F7" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G7" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H7" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I7" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E8" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F8" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G8" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H8" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I8" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E9" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F9" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G9" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H9" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I9" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E10" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F10" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G10" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H10" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I10" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E11" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F11" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G11" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H11" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I11" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E17" t="n">
-        <v>21.915</v>
+        <v>105.6</v>
       </c>
       <c r="F17" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G17" t="n">
-        <v>65.75</v>
+        <v>105.6</v>
       </c>
       <c r="H17" t="n">
-        <v>0.08</v>
+        <v>5.51</v>
       </c>
       <c r="I17" t="n">
-        <v>0.12</v>
+        <v>5.51</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D18" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E18" t="n">
-        <v>41.789</v>
+        <v>6.82</v>
       </c>
       <c r="F18" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G18" t="n">
-        <v>167.16</v>
+        <v>61.38</v>
       </c>
       <c r="H18" t="n">
-        <v>28.14</v>
+        <v>5.23</v>
       </c>
       <c r="I18" t="n">
-        <v>20.24</v>
+        <v>9.31</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C19" t="n">
         <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E19" t="n">
-        <v>10.662</v>
+        <v>21.915</v>
       </c>
       <c r="F19" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G19" t="n">
-        <v>31.99</v>
+        <v>65.75</v>
       </c>
       <c r="H19" t="n">
-        <v>0.83</v>
+        <v>0.08</v>
       </c>
       <c r="I19" t="n">
-        <v>2.66</v>
+        <v>0.12</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D20" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E20" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F20" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G20" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H20" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I20" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E21" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F21" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G21" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H21" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I21" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E32" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F32" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G32" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I32" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E33" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F33" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G33" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H33" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I33" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E34" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F34" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G34" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H34" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I34" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E35" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F35" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G35" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H35" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I35" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D36" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E36" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F36" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G36" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H36" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I36" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C47" t="n">
         <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E47" t="n">
-        <v>10.562</v>
+        <v>21.778</v>
       </c>
       <c r="F47" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G47" t="n">
-        <v>31.69</v>
+        <v>65.33</v>
       </c>
       <c r="H47" t="n">
-        <v>0.53</v>
+        <v>-0.34</v>
       </c>
       <c r="I47" t="n">
-        <v>1.7</v>
+        <v>-0.52</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E48" t="n">
-        <v>6.622</v>
+        <v>38.312</v>
       </c>
       <c r="F48" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G48" t="n">
-        <v>59.6</v>
+        <v>153.25</v>
       </c>
       <c r="H48" t="n">
-        <v>3.45</v>
+        <v>14.23</v>
       </c>
       <c r="I48" t="n">
-        <v>6.14</v>
+        <v>10.24</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D49" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E49" t="n">
-        <v>38.312</v>
+        <v>99.83</v>
       </c>
       <c r="F49" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G49" t="n">
-        <v>153.25</v>
+        <v>99.83</v>
       </c>
       <c r="H49" t="n">
-        <v>14.23</v>
+        <v>-0.26</v>
       </c>
       <c r="I49" t="n">
-        <v>10.24</v>
+        <v>-0.26</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E50" t="n">
-        <v>99.83</v>
+        <v>10.562</v>
       </c>
       <c r="F50" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G50" t="n">
-        <v>99.83</v>
+        <v>31.69</v>
       </c>
       <c r="H50" t="n">
-        <v>-0.26</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="n">
-        <v>-0.26</v>
+        <v>1.7</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D51" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E51" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F51" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G51" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>39.845</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>159.38</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>20.36</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>14.65</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>22.289</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>66.87</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>1.2</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>1.83</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E62" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F62" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G62" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H62" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I62" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E64" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F64" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G64" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H64" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I64" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E67" t="n">
-        <v>22.797</v>
+        <v>6.807</v>
       </c>
       <c r="F67" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G67" t="n">
-        <v>68.39</v>
+        <v>61.26</v>
       </c>
       <c r="H67" t="n">
-        <v>2.72</v>
+        <v>5.11</v>
       </c>
       <c r="I67" t="n">
-        <v>4.14</v>
+        <v>9.1</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E68" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F68" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G68" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H68" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I68" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E69" t="n">
-        <v>40.567</v>
+        <v>104.58</v>
       </c>
       <c r="F69" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G69" t="n">
-        <v>162.27</v>
+        <v>104.58</v>
       </c>
       <c r="H69" t="n">
-        <v>23.25</v>
+        <v>4.49</v>
       </c>
       <c r="I69" t="n">
-        <v>16.72</v>
+        <v>4.49</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E70" t="n">
-        <v>6.807</v>
+        <v>22.797</v>
       </c>
       <c r="F70" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G70" t="n">
-        <v>61.26</v>
+        <v>68.39</v>
       </c>
       <c r="H70" t="n">
-        <v>5.11</v>
+        <v>2.72</v>
       </c>
       <c r="I70" t="n">
-        <v>9.1</v>
+        <v>4.14</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E71" t="n">
-        <v>104.58</v>
+        <v>10.796</v>
       </c>
       <c r="F71" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G71" t="n">
-        <v>104.58</v>
+        <v>32.39</v>
       </c>
       <c r="H71" t="n">
-        <v>4.49</v>
+        <v>1.23</v>
       </c>
       <c r="I71" t="n">
-        <v>4.49</v>
+        <v>3.95</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E82" t="n">
-        <v>42.1</v>
+        <v>10.988</v>
       </c>
       <c r="F82" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G82" t="n">
-        <v>168.4</v>
+        <v>32.96</v>
       </c>
       <c r="H82" t="n">
-        <v>29.38</v>
+        <v>1.8</v>
       </c>
       <c r="I82" t="n">
-        <v>21.13</v>
+        <v>5.78</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D83" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E83" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F83" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G83" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H83" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I83" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E84" t="n">
-        <v>6.846</v>
+        <v>23.3</v>
       </c>
       <c r="F84" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G84" t="n">
-        <v>61.61</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H84" t="n">
-        <v>5.46</v>
+        <v>4.23</v>
       </c>
       <c r="I84" t="n">
-        <v>9.720000000000001</v>
+        <v>6.44</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D85" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E85" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F85" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G85" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H85" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I85" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D86" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E86" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F86" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G86" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H86" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I86" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C92" t="n">
         <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E92" t="n">
-        <v>23.025</v>
+        <v>10.876</v>
       </c>
       <c r="F92" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G92" t="n">
-        <v>69.06999999999999</v>
+        <v>32.63</v>
       </c>
       <c r="H92" t="n">
-        <v>3.4</v>
+        <v>1.47</v>
       </c>
       <c r="I92" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D93" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E93" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F93" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G93" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H93" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I93" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E95" t="n">
-        <v>40.575</v>
+        <v>23.025</v>
       </c>
       <c r="F95" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G95" t="n">
-        <v>162.3</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H95" t="n">
-        <v>23.28</v>
+        <v>3.4</v>
       </c>
       <c r="I95" t="n">
-        <v>16.75</v>
+        <v>5.18</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D96" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E96" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F96" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G96" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H96" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I96" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D102" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E102" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F102" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G102" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H102" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I102" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E103" t="n">
-        <v>6.804</v>
+        <v>10.556</v>
       </c>
       <c r="F103" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G103" t="n">
-        <v>61.24</v>
+        <v>31.67</v>
       </c>
       <c r="H103" t="n">
-        <v>5.09</v>
+        <v>0.51</v>
       </c>
       <c r="I103" t="n">
-        <v>9.07</v>
+        <v>1.64</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D104" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E104" t="n">
-        <v>10.556</v>
+        <v>40.97</v>
       </c>
       <c r="F104" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G104" t="n">
-        <v>31.67</v>
+        <v>163.88</v>
       </c>
       <c r="H104" t="n">
-        <v>0.51</v>
+        <v>24.86</v>
       </c>
       <c r="I104" t="n">
-        <v>1.64</v>
+        <v>17.88</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E105" t="n">
-        <v>40.97</v>
+        <v>23.29</v>
       </c>
       <c r="F105" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G105" t="n">
-        <v>163.88</v>
+        <v>69.87</v>
       </c>
       <c r="H105" t="n">
-        <v>24.86</v>
+        <v>4.2</v>
       </c>
       <c r="I105" t="n">
-        <v>17.88</v>
+        <v>6.4</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D106" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E106" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F106" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G106" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H106" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I106" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E112" t="n">
-        <v>40</v>
+        <v>23.025</v>
       </c>
       <c r="F112" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G112" t="n">
-        <v>160</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H112" t="n">
-        <v>20.98</v>
+        <v>3.4</v>
       </c>
       <c r="I112" t="n">
-        <v>15.09</v>
+        <v>5.18</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D113" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E113" t="n">
-        <v>10.568</v>
+        <v>6.797</v>
       </c>
       <c r="F113" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G113" t="n">
-        <v>31.7</v>
+        <v>61.17</v>
       </c>
       <c r="H113" t="n">
-        <v>0.54</v>
+        <v>5.02</v>
       </c>
       <c r="I113" t="n">
-        <v>1.73</v>
+        <v>8.94</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D114" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E114" t="n">
-        <v>103.56</v>
+        <v>40</v>
       </c>
       <c r="F114" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G114" t="n">
-        <v>103.56</v>
+        <v>160</v>
       </c>
       <c r="H114" t="n">
-        <v>3.47</v>
+        <v>20.98</v>
       </c>
       <c r="I114" t="n">
-        <v>3.47</v>
+        <v>15.09</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E115" t="n">
-        <v>6.797</v>
+        <v>10.568</v>
       </c>
       <c r="F115" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G115" t="n">
-        <v>61.17</v>
+        <v>31.7</v>
       </c>
       <c r="H115" t="n">
-        <v>5.02</v>
+        <v>0.54</v>
       </c>
       <c r="I115" t="n">
-        <v>8.94</v>
+        <v>1.73</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D116" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E116" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F116" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G116" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H116" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I116" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E122" t="n">
-        <v>6.901</v>
+        <v>106</v>
       </c>
       <c r="F122" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G122" t="n">
-        <v>62.11</v>
+        <v>106</v>
       </c>
       <c r="H122" t="n">
-        <v>5.96</v>
+        <v>5.91</v>
       </c>
       <c r="I122" t="n">
-        <v>10.61</v>
+        <v>5.9</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D123" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E123" t="n">
-        <v>23.165</v>
+        <v>40.395</v>
       </c>
       <c r="F123" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G123" t="n">
-        <v>69.5</v>
+        <v>161.58</v>
       </c>
       <c r="H123" t="n">
-        <v>3.83</v>
+        <v>22.56</v>
       </c>
       <c r="I123" t="n">
-        <v>5.83</v>
+        <v>16.23</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C124" t="n">
         <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E124" t="n">
-        <v>11.038</v>
+        <v>23.165</v>
       </c>
       <c r="F124" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G124" t="n">
-        <v>33.11</v>
+        <v>69.5</v>
       </c>
       <c r="H124" t="n">
-        <v>1.95</v>
+        <v>3.83</v>
       </c>
       <c r="I124" t="n">
-        <v>6.26</v>
+        <v>5.83</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D125" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E125" t="n">
-        <v>106</v>
+        <v>6.901</v>
       </c>
       <c r="F125" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G125" t="n">
-        <v>106</v>
+        <v>62.11</v>
       </c>
       <c r="H125" t="n">
-        <v>5.91</v>
+        <v>5.96</v>
       </c>
       <c r="I125" t="n">
-        <v>5.9</v>
+        <v>10.61</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D126" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E126" t="n">
-        <v>40.395</v>
+        <v>11.038</v>
       </c>
       <c r="F126" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G126" t="n">
-        <v>161.58</v>
+        <v>33.11</v>
       </c>
       <c r="H126" t="n">
-        <v>22.56</v>
+        <v>1.95</v>
       </c>
       <c r="I126" t="n">
-        <v>16.23</v>
+        <v>6.26</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D132" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E132" t="n">
-        <v>104.02</v>
+        <v>6.895</v>
       </c>
       <c r="F132" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G132" t="n">
-        <v>104.02</v>
+        <v>62.05</v>
       </c>
       <c r="H132" t="n">
-        <v>3.93</v>
+        <v>5.9</v>
       </c>
       <c r="I132" t="n">
-        <v>3.93</v>
+        <v>10.51</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C133" t="n">
         <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E133" t="n">
-        <v>11.516</v>
+        <v>23.18</v>
       </c>
       <c r="F133" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G133" t="n">
-        <v>34.55</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H133" t="n">
-        <v>3.39</v>
+        <v>3.87</v>
       </c>
       <c r="I133" t="n">
-        <v>10.88</v>
+        <v>5.89</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E134" t="n">
-        <v>40.54</v>
+        <v>11.516</v>
       </c>
       <c r="F134" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G134" t="n">
-        <v>162.16</v>
+        <v>34.55</v>
       </c>
       <c r="H134" t="n">
-        <v>23.14</v>
+        <v>3.39</v>
       </c>
       <c r="I134" t="n">
-        <v>16.65</v>
+        <v>10.88</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D135" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E135" t="n">
-        <v>23.18</v>
+        <v>104.02</v>
       </c>
       <c r="F135" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G135" t="n">
-        <v>69.54000000000001</v>
+        <v>104.02</v>
       </c>
       <c r="H135" t="n">
-        <v>3.87</v>
+        <v>3.93</v>
       </c>
       <c r="I135" t="n">
-        <v>5.89</v>
+        <v>3.93</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,31 +5034,201 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>4</v>
+      </c>
+      <c r="D136" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E136" t="n">
+        <v>40.54</v>
+      </c>
+      <c r="F136" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G136" t="n">
+        <v>162.16</v>
+      </c>
+      <c r="H136" t="n">
+        <v>23.14</v>
+      </c>
+      <c r="I136" t="n">
+        <v>16.65</v>
+      </c>
+      <c r="J136" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>3</v>
+      </c>
+      <c r="D137" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E137" t="n">
+        <v>11.728</v>
+      </c>
+      <c r="F137" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G137" t="n">
+        <v>35.18</v>
+      </c>
+      <c r="H137" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="I137" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="J137" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>4</v>
+      </c>
+      <c r="D138" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E138" t="n">
+        <v>40.61</v>
+      </c>
+      <c r="F138" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G138" t="n">
+        <v>162.44</v>
+      </c>
+      <c r="H138" t="n">
+        <v>23.42</v>
+      </c>
+      <c r="I138" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="J138" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>3</v>
+      </c>
+      <c r="D139" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E139" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="F139" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G139" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="H139" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="I139" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="J139" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E140" t="n">
+        <v>104.76</v>
+      </c>
+      <c r="F140" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G140" t="n">
+        <v>104.76</v>
+      </c>
+      <c r="H140" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I140" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="J140" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C136" t="n">
+      <c r="C141" t="n">
         <v>9</v>
       </c>
-      <c r="D136" t="n">
+      <c r="D141" t="n">
         <v>6.239</v>
       </c>
-      <c r="E136" t="n">
-        <v>6.895</v>
-      </c>
-      <c r="F136" t="n">
+      <c r="E141" t="n">
+        <v>6.927</v>
+      </c>
+      <c r="F141" t="n">
         <v>56.15</v>
       </c>
-      <c r="G136" t="n">
-        <v>62.05</v>
-      </c>
-      <c r="H136" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="I136" t="n">
-        <v>10.51</v>
-      </c>
-      <c r="J136" t="n">
+      <c r="G141" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="H141" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="I141" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="J141" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 07/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E7" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F7" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G7" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H7" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I7" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E8" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F8" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G8" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H8" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I8" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E9" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F9" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G9" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H9" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I9" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E10" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F10" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G10" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H10" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I10" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E11" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F11" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G11" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H11" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I11" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E17" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F17" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G17" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H17" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I17" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E18" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F18" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G18" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H18" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I18" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E19" t="n">
-        <v>21.915</v>
+        <v>41.789</v>
       </c>
       <c r="F19" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G19" t="n">
-        <v>65.75</v>
+        <v>167.16</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08</v>
+        <v>28.14</v>
       </c>
       <c r="I19" t="n">
-        <v>0.12</v>
+        <v>20.24</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E20" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F20" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G20" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H20" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I20" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E21" t="n">
-        <v>10.662</v>
+        <v>6.82</v>
       </c>
       <c r="F21" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G21" t="n">
-        <v>31.99</v>
+        <v>61.38</v>
       </c>
       <c r="H21" t="n">
-        <v>0.83</v>
+        <v>5.23</v>
       </c>
       <c r="I21" t="n">
-        <v>2.66</v>
+        <v>9.31</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E27" t="n">
-        <v>40.532</v>
+        <v>10.66</v>
       </c>
       <c r="F27" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G27" t="n">
-        <v>162.13</v>
+        <v>31.98</v>
       </c>
       <c r="H27" t="n">
-        <v>23.11</v>
+        <v>0.82</v>
       </c>
       <c r="I27" t="n">
-        <v>16.62</v>
+        <v>2.63</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E28" t="n">
-        <v>6.795</v>
+        <v>21.98</v>
       </c>
       <c r="F28" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G28" t="n">
-        <v>61.16</v>
+        <v>65.94</v>
       </c>
       <c r="H28" t="n">
-        <v>5.01</v>
+        <v>0.27</v>
       </c>
       <c r="I28" t="n">
-        <v>8.92</v>
+        <v>0.41</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E29" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F29" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G29" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H29" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I29" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>6.795</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>61.16</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>5.01</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>8.92</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>40.532</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>162.13</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>23.11</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>16.62</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D37" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E37" t="n">
-        <v>102.8</v>
+        <v>6.728</v>
       </c>
       <c r="F37" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G37" t="n">
-        <v>102.8</v>
+        <v>60.55</v>
       </c>
       <c r="H37" t="n">
-        <v>2.71</v>
+        <v>4.4</v>
       </c>
       <c r="I37" t="n">
-        <v>2.71</v>
+        <v>7.84</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E38" t="n">
-        <v>10.67</v>
+        <v>21.839</v>
       </c>
       <c r="F38" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G38" t="n">
-        <v>32.01</v>
+        <v>65.52</v>
       </c>
       <c r="H38" t="n">
-        <v>0.85</v>
+        <v>-0.15</v>
       </c>
       <c r="I38" t="n">
-        <v>2.73</v>
+        <v>-0.23</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E39" t="n">
-        <v>38.879</v>
+        <v>102.8</v>
       </c>
       <c r="F39" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G39" t="n">
-        <v>155.52</v>
+        <v>102.8</v>
       </c>
       <c r="H39" t="n">
-        <v>16.5</v>
+        <v>2.71</v>
       </c>
       <c r="I39" t="n">
-        <v>11.87</v>
+        <v>2.71</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E40" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F40" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G40" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E41" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F41" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G41" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H41" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I41" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D52" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E52" t="n">
-        <v>100.34</v>
+        <v>6.629</v>
       </c>
       <c r="F52" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G52" t="n">
-        <v>100.34</v>
+        <v>59.66</v>
       </c>
       <c r="H52" t="n">
-        <v>0.25</v>
+        <v>3.51</v>
       </c>
       <c r="I52" t="n">
-        <v>0.25</v>
+        <v>6.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E53" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F53" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G53" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H53" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E54" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F54" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G54" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H54" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E55" t="n">
-        <v>6.629</v>
+        <v>100.34</v>
       </c>
       <c r="F55" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G55" t="n">
-        <v>59.66</v>
+        <v>100.34</v>
       </c>
       <c r="H55" t="n">
-        <v>3.51</v>
+        <v>0.25</v>
       </c>
       <c r="I55" t="n">
-        <v>6.25</v>
+        <v>0.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E56" t="n">
-        <v>38.544</v>
+        <v>10.702</v>
       </c>
       <c r="F56" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G56" t="n">
-        <v>154.18</v>
+        <v>32.11</v>
       </c>
       <c r="H56" t="n">
-        <v>15.16</v>
+        <v>0.95</v>
       </c>
       <c r="I56" t="n">
-        <v>10.9</v>
+        <v>3.05</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E62" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F62" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G62" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H62" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I62" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
         <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E65" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F65" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G65" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H65" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I65" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E66" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F66" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G66" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H66" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I66" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E72" t="n">
-        <v>10.892</v>
+        <v>41.15</v>
       </c>
       <c r="F72" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G72" t="n">
-        <v>32.68</v>
+        <v>164.6</v>
       </c>
       <c r="H72" t="n">
-        <v>1.52</v>
+        <v>25.58</v>
       </c>
       <c r="I72" t="n">
-        <v>4.88</v>
+        <v>18.4</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>104.22</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>104.22</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>4.13</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>4.13</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E75" t="n">
-        <v>104.22</v>
+        <v>6.811</v>
       </c>
       <c r="F75" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G75" t="n">
-        <v>104.22</v>
+        <v>61.3</v>
       </c>
       <c r="H75" t="n">
-        <v>4.13</v>
+        <v>5.15</v>
       </c>
       <c r="I75" t="n">
-        <v>4.13</v>
+        <v>9.17</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E76" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F76" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G76" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H76" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I76" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C87" t="n">
         <v>3</v>
       </c>
       <c r="D87" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E87" t="n">
-        <v>23.32</v>
+        <v>10.852</v>
       </c>
       <c r="F87" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G87" t="n">
-        <v>69.95999999999999</v>
+        <v>32.56</v>
       </c>
       <c r="H87" t="n">
-        <v>4.29</v>
+        <v>1.4</v>
       </c>
       <c r="I87" t="n">
-        <v>6.53</v>
+        <v>4.49</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D88" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E88" t="n">
-        <v>106.28</v>
+        <v>6.856</v>
       </c>
       <c r="F88" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G88" t="n">
-        <v>106.28</v>
+        <v>61.7</v>
       </c>
       <c r="H88" t="n">
-        <v>6.19</v>
+        <v>5.55</v>
       </c>
       <c r="I88" t="n">
-        <v>6.18</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D89" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E89" t="n">
-        <v>6.856</v>
+        <v>43.005</v>
       </c>
       <c r="F89" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G89" t="n">
-        <v>61.7</v>
+        <v>172.02</v>
       </c>
       <c r="H89" t="n">
-        <v>5.55</v>
+        <v>33</v>
       </c>
       <c r="I89" t="n">
-        <v>9.880000000000001</v>
+        <v>23.74</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C90" t="n">
         <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E90" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F90" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G90" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H90" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I90" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E91" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F91" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G91" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H91" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I91" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E97" t="n">
-        <v>6.839</v>
+        <v>23.35</v>
       </c>
       <c r="F97" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G97" t="n">
-        <v>61.55</v>
+        <v>70.05</v>
       </c>
       <c r="H97" t="n">
-        <v>5.4</v>
+        <v>4.38</v>
       </c>
       <c r="I97" t="n">
-        <v>9.619999999999999</v>
+        <v>6.67</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D98" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E98" t="n">
-        <v>10.642</v>
+        <v>40.65</v>
       </c>
       <c r="F98" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G98" t="n">
-        <v>31.93</v>
+        <v>162.6</v>
       </c>
       <c r="H98" t="n">
-        <v>0.77</v>
+        <v>23.58</v>
       </c>
       <c r="I98" t="n">
-        <v>2.47</v>
+        <v>16.96</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D100" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E100" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F100" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G100" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H100" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I100" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C101" t="n">
         <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E101" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F101" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G101" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H101" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I101" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D107" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E107" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F107" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G107" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H107" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I107" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E108" t="n">
-        <v>103.14</v>
+        <v>10.456</v>
       </c>
       <c r="F108" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G108" t="n">
-        <v>103.14</v>
+        <v>31.37</v>
       </c>
       <c r="H108" t="n">
-        <v>3.05</v>
+        <v>0.21</v>
       </c>
       <c r="I108" t="n">
-        <v>3.05</v>
+        <v>0.67</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D109" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E109" t="n">
-        <v>10.456</v>
+        <v>6.785</v>
       </c>
       <c r="F109" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G109" t="n">
-        <v>31.37</v>
+        <v>61.06</v>
       </c>
       <c r="H109" t="n">
-        <v>0.21</v>
+        <v>4.91</v>
       </c>
       <c r="I109" t="n">
-        <v>0.67</v>
+        <v>8.74</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D110" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E110" t="n">
-        <v>6.785</v>
+        <v>103.14</v>
       </c>
       <c r="F110" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G110" t="n">
-        <v>61.06</v>
+        <v>103.14</v>
       </c>
       <c r="H110" t="n">
-        <v>4.91</v>
+        <v>3.05</v>
       </c>
       <c r="I110" t="n">
-        <v>8.74</v>
+        <v>3.05</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E111" t="n">
-        <v>40.5</v>
+        <v>23.33</v>
       </c>
       <c r="F111" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G111" t="n">
-        <v>162</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H111" t="n">
-        <v>22.98</v>
+        <v>4.32</v>
       </c>
       <c r="I111" t="n">
-        <v>16.53</v>
+        <v>6.58</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E117" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F117" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G117" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H117" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I117" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D118" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E118" t="n">
-        <v>105.96</v>
+        <v>6.861</v>
       </c>
       <c r="F118" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G118" t="n">
-        <v>105.96</v>
+        <v>61.75</v>
       </c>
       <c r="H118" t="n">
-        <v>5.87</v>
+        <v>5.6</v>
       </c>
       <c r="I118" t="n">
-        <v>5.86</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E120" t="n">
-        <v>6.861</v>
+        <v>105.96</v>
       </c>
       <c r="F120" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G120" t="n">
-        <v>61.75</v>
+        <v>105.96</v>
       </c>
       <c r="H120" t="n">
-        <v>5.6</v>
+        <v>5.87</v>
       </c>
       <c r="I120" t="n">
-        <v>9.970000000000001</v>
+        <v>5.86</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E121" t="n">
-        <v>41</v>
+        <v>23.145</v>
       </c>
       <c r="F121" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G121" t="n">
-        <v>164</v>
+        <v>69.44</v>
       </c>
       <c r="H121" t="n">
-        <v>24.98</v>
+        <v>3.77</v>
       </c>
       <c r="I121" t="n">
-        <v>17.97</v>
+        <v>5.74</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D127" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E127" t="n">
-        <v>6.868</v>
+        <v>103.46</v>
       </c>
       <c r="F127" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G127" t="n">
-        <v>61.81</v>
+        <v>103.46</v>
       </c>
       <c r="H127" t="n">
-        <v>5.66</v>
+        <v>3.37</v>
       </c>
       <c r="I127" t="n">
-        <v>10.08</v>
+        <v>3.37</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C128" t="n">
         <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E128" t="n">
-        <v>11.458</v>
+        <v>23.17</v>
       </c>
       <c r="F128" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G128" t="n">
-        <v>34.37</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H128" t="n">
-        <v>3.21</v>
+        <v>3.84</v>
       </c>
       <c r="I128" t="n">
-        <v>10.3</v>
+        <v>5.85</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4796,29 +4796,29 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E129" t="n">
-        <v>39.36</v>
+        <v>11.458</v>
       </c>
       <c r="F129" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G129" t="n">
-        <v>157.44</v>
+        <v>34.37</v>
       </c>
       <c r="H129" t="n">
-        <v>18.42</v>
+        <v>3.21</v>
       </c>
       <c r="I129" t="n">
-        <v>13.25</v>
+        <v>10.3</v>
       </c>
       <c r="J129" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D130" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E130" t="n">
-        <v>23.17</v>
+        <v>6.868</v>
       </c>
       <c r="F130" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G130" t="n">
-        <v>69.51000000000001</v>
+        <v>61.81</v>
       </c>
       <c r="H130" t="n">
-        <v>3.84</v>
+        <v>5.66</v>
       </c>
       <c r="I130" t="n">
-        <v>5.85</v>
+        <v>10.08</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E131" t="n">
-        <v>103.46</v>
+        <v>39.36</v>
       </c>
       <c r="F131" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G131" t="n">
-        <v>103.46</v>
+        <v>157.44</v>
       </c>
       <c r="H131" t="n">
-        <v>3.37</v>
+        <v>18.42</v>
       </c>
       <c r="I131" t="n">
-        <v>3.37</v>
+        <v>13.25</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D137" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E137" t="n">
-        <v>11.728</v>
+        <v>6.927</v>
       </c>
       <c r="F137" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G137" t="n">
-        <v>35.18</v>
+        <v>62.34</v>
       </c>
       <c r="H137" t="n">
-        <v>4.02</v>
+        <v>6.19</v>
       </c>
       <c r="I137" t="n">
-        <v>12.9</v>
+        <v>11.02</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E138" t="n">
-        <v>40.61</v>
+        <v>11.728</v>
       </c>
       <c r="F138" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G138" t="n">
-        <v>162.44</v>
+        <v>35.18</v>
       </c>
       <c r="H138" t="n">
-        <v>23.42</v>
+        <v>4.02</v>
       </c>
       <c r="I138" t="n">
-        <v>16.85</v>
+        <v>12.9</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D139" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E139" t="n">
-        <v>23.3</v>
+        <v>40.61</v>
       </c>
       <c r="F139" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G139" t="n">
-        <v>69.90000000000001</v>
+        <v>162.44</v>
       </c>
       <c r="H139" t="n">
-        <v>4.23</v>
+        <v>23.42</v>
       </c>
       <c r="I139" t="n">
-        <v>6.44</v>
+        <v>16.85</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E140" t="n">
-        <v>104.76</v>
+        <v>23.3</v>
       </c>
       <c r="F140" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G140" t="n">
-        <v>104.76</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H140" t="n">
-        <v>4.67</v>
+        <v>4.23</v>
       </c>
       <c r="I140" t="n">
-        <v>4.67</v>
+        <v>6.44</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,31 +5204,201 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E141" t="n">
+        <v>104.76</v>
+      </c>
+      <c r="F141" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G141" t="n">
+        <v>104.76</v>
+      </c>
+      <c r="H141" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="I141" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="J141" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E142" t="n">
+        <v>102.06</v>
+      </c>
+      <c r="F142" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G142" t="n">
+        <v>102.06</v>
+      </c>
+      <c r="H142" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="I142" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="J142" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>3</v>
+      </c>
+      <c r="D143" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E143" t="n">
+        <v>11.498</v>
+      </c>
+      <c r="F143" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G143" t="n">
+        <v>34.49</v>
+      </c>
+      <c r="H143" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="I143" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="J143" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>4</v>
+      </c>
+      <c r="D144" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E144" t="n">
+        <v>38.89</v>
+      </c>
+      <c r="F144" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G144" t="n">
+        <v>155.56</v>
+      </c>
+      <c r="H144" t="n">
+        <v>16.54</v>
+      </c>
+      <c r="I144" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="J144" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>3</v>
+      </c>
+      <c r="D145" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E145" t="n">
+        <v>23.135</v>
+      </c>
+      <c r="F145" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G145" t="n">
+        <v>69.41</v>
+      </c>
+      <c r="H145" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="I145" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="J145" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C141" t="n">
+      <c r="C146" t="n">
         <v>9</v>
       </c>
-      <c r="D141" t="n">
+      <c r="D146" t="n">
         <v>6.239</v>
       </c>
-      <c r="E141" t="n">
-        <v>6.927</v>
-      </c>
-      <c r="F141" t="n">
+      <c r="E146" t="n">
+        <v>6.878</v>
+      </c>
+      <c r="F146" t="n">
         <v>56.15</v>
       </c>
-      <c r="G141" t="n">
-        <v>62.34</v>
-      </c>
-      <c r="H141" t="n">
-        <v>6.19</v>
-      </c>
-      <c r="I141" t="n">
-        <v>11.02</v>
-      </c>
-      <c r="J141" t="n">
+      <c r="G146" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="H146" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="I146" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="J146" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 08/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E7" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F7" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G7" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H7" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I7" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D8" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E8" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F8" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G8" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H8" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I8" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E9" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F9" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G9" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H9" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I9" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E10" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F10" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G10" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H10" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I10" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E11" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F11" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G11" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H11" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I11" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D17" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E17" t="n">
-        <v>10.662</v>
+        <v>6.82</v>
       </c>
       <c r="F17" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G17" t="n">
-        <v>31.99</v>
+        <v>61.38</v>
       </c>
       <c r="H17" t="n">
-        <v>0.83</v>
+        <v>5.23</v>
       </c>
       <c r="I17" t="n">
-        <v>2.66</v>
+        <v>9.31</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E18" t="n">
-        <v>21.915</v>
+        <v>41.789</v>
       </c>
       <c r="F18" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G18" t="n">
-        <v>65.75</v>
+        <v>167.16</v>
       </c>
       <c r="H18" t="n">
-        <v>0.08</v>
+        <v>28.14</v>
       </c>
       <c r="I18" t="n">
-        <v>0.12</v>
+        <v>20.24</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E19" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F19" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G19" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H19" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I19" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E20" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F20" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G20" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H20" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I20" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E21" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F21" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G21" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H21" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I21" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E27" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F27" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G27" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H27" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I27" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E28" t="n">
-        <v>21.98</v>
+        <v>40.532</v>
       </c>
       <c r="F28" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G28" t="n">
-        <v>65.94</v>
+        <v>162.13</v>
       </c>
       <c r="H28" t="n">
-        <v>0.27</v>
+        <v>23.11</v>
       </c>
       <c r="I28" t="n">
-        <v>0.41</v>
+        <v>16.62</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E29" t="n">
-        <v>104.9</v>
+        <v>6.795</v>
       </c>
       <c r="F29" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G29" t="n">
-        <v>104.9</v>
+        <v>61.16</v>
       </c>
       <c r="H29" t="n">
-        <v>4.81</v>
+        <v>5.01</v>
       </c>
       <c r="I29" t="n">
-        <v>4.81</v>
+        <v>8.92</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E30" t="n">
-        <v>6.795</v>
+        <v>21.98</v>
       </c>
       <c r="F30" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G30" t="n">
-        <v>61.16</v>
+        <v>65.94</v>
       </c>
       <c r="H30" t="n">
-        <v>5.01</v>
+        <v>0.27</v>
       </c>
       <c r="I30" t="n">
-        <v>8.92</v>
+        <v>0.41</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E31" t="n">
-        <v>40.532</v>
+        <v>10.66</v>
       </c>
       <c r="F31" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G31" t="n">
-        <v>162.13</v>
+        <v>31.98</v>
       </c>
       <c r="H31" t="n">
-        <v>23.11</v>
+        <v>0.82</v>
       </c>
       <c r="I31" t="n">
-        <v>16.62</v>
+        <v>2.63</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E37" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F37" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G37" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H37" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I37" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E38" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F38" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G38" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D39" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E39" t="n">
-        <v>102.8</v>
+        <v>6.728</v>
       </c>
       <c r="F39" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G39" t="n">
-        <v>102.8</v>
+        <v>60.55</v>
       </c>
       <c r="H39" t="n">
-        <v>2.71</v>
+        <v>4.4</v>
       </c>
       <c r="I39" t="n">
-        <v>2.71</v>
+        <v>7.84</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E40" t="n">
-        <v>10.67</v>
+        <v>21.839</v>
       </c>
       <c r="F40" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G40" t="n">
-        <v>32.01</v>
+        <v>65.52</v>
       </c>
       <c r="H40" t="n">
-        <v>0.85</v>
+        <v>-0.15</v>
       </c>
       <c r="I40" t="n">
-        <v>2.73</v>
+        <v>-0.23</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E41" t="n">
-        <v>38.879</v>
+        <v>102.8</v>
       </c>
       <c r="F41" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G41" t="n">
-        <v>155.52</v>
+        <v>102.8</v>
       </c>
       <c r="H41" t="n">
-        <v>16.5</v>
+        <v>2.71</v>
       </c>
       <c r="I41" t="n">
-        <v>11.87</v>
+        <v>2.71</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E52" t="n">
-        <v>6.629</v>
+        <v>100.34</v>
       </c>
       <c r="F52" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G52" t="n">
-        <v>59.66</v>
+        <v>100.34</v>
       </c>
       <c r="H52" t="n">
-        <v>3.51</v>
+        <v>0.25</v>
       </c>
       <c r="I52" t="n">
-        <v>6.25</v>
+        <v>0.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E53" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F53" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G53" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H53" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E54" t="n">
-        <v>38.544</v>
+        <v>10.702</v>
       </c>
       <c r="F54" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G54" t="n">
-        <v>154.18</v>
+        <v>32.11</v>
       </c>
       <c r="H54" t="n">
-        <v>15.16</v>
+        <v>0.95</v>
       </c>
       <c r="I54" t="n">
-        <v>10.9</v>
+        <v>3.05</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E55" t="n">
-        <v>100.34</v>
+        <v>6.629</v>
       </c>
       <c r="F55" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G55" t="n">
-        <v>100.34</v>
+        <v>59.66</v>
       </c>
       <c r="H55" t="n">
-        <v>0.25</v>
+        <v>3.51</v>
       </c>
       <c r="I55" t="n">
-        <v>0.25</v>
+        <v>6.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E56" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F56" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G56" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H56" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I56" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E62" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F62" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G62" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H62" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I62" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E65" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F65" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G65" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H65" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I65" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E66" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F66" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G66" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H66" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I66" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D72" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E72" t="n">
-        <v>41.15</v>
+        <v>6.811</v>
       </c>
       <c r="F72" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G72" t="n">
-        <v>164.6</v>
+        <v>61.3</v>
       </c>
       <c r="H72" t="n">
-        <v>25.58</v>
+        <v>5.15</v>
       </c>
       <c r="I72" t="n">
-        <v>18.4</v>
+        <v>9.17</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E73" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F73" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G73" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H73" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I73" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E74" t="n">
-        <v>23</v>
+        <v>10.892</v>
       </c>
       <c r="F74" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G74" t="n">
-        <v>69</v>
+        <v>32.68</v>
       </c>
       <c r="H74" t="n">
-        <v>3.33</v>
+        <v>1.52</v>
       </c>
       <c r="I74" t="n">
-        <v>5.07</v>
+        <v>4.88</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E75" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F75" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G75" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H75" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I75" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E76" t="n">
-        <v>10.892</v>
+        <v>104.22</v>
       </c>
       <c r="F76" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G76" t="n">
-        <v>32.68</v>
+        <v>104.22</v>
       </c>
       <c r="H76" t="n">
-        <v>1.52</v>
+        <v>4.13</v>
       </c>
       <c r="I76" t="n">
-        <v>4.88</v>
+        <v>4.13</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D92" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E92" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F92" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G92" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H92" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I92" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E93" t="n">
-        <v>40.575</v>
+        <v>23.025</v>
       </c>
       <c r="F93" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G93" t="n">
-        <v>162.3</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H93" t="n">
-        <v>23.28</v>
+        <v>3.4</v>
       </c>
       <c r="I93" t="n">
-        <v>16.75</v>
+        <v>5.18</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C95" t="n">
         <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E95" t="n">
-        <v>23.025</v>
+        <v>10.876</v>
       </c>
       <c r="F95" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G95" t="n">
-        <v>69.06999999999999</v>
+        <v>32.63</v>
       </c>
       <c r="H95" t="n">
-        <v>3.4</v>
+        <v>1.47</v>
       </c>
       <c r="I95" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D96" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E96" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F96" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G96" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H96" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I96" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D102" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E102" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F102" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G102" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H102" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I102" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C103" t="n">
         <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E103" t="n">
-        <v>10.556</v>
+        <v>23.29</v>
       </c>
       <c r="F103" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G103" t="n">
-        <v>31.67</v>
+        <v>69.87</v>
       </c>
       <c r="H103" t="n">
-        <v>0.51</v>
+        <v>4.2</v>
       </c>
       <c r="I103" t="n">
-        <v>1.64</v>
+        <v>6.4</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D104" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E104" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F104" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G104" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H104" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I104" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D105" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E105" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F105" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G105" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H105" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I105" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D106" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E106" t="n">
-        <v>6.804</v>
+        <v>40.97</v>
       </c>
       <c r="F106" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G106" t="n">
-        <v>61.24</v>
+        <v>163.88</v>
       </c>
       <c r="H106" t="n">
-        <v>5.09</v>
+        <v>24.86</v>
       </c>
       <c r="I106" t="n">
-        <v>9.07</v>
+        <v>17.88</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D112" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E112" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F112" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G112" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H112" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I112" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E113" t="n">
-        <v>6.797</v>
+        <v>10.568</v>
       </c>
       <c r="F113" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G113" t="n">
-        <v>61.17</v>
+        <v>31.7</v>
       </c>
       <c r="H113" t="n">
-        <v>5.02</v>
+        <v>0.54</v>
       </c>
       <c r="I113" t="n">
-        <v>8.94</v>
+        <v>1.73</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D114" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E114" t="n">
-        <v>40</v>
+        <v>6.797</v>
       </c>
       <c r="F114" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G114" t="n">
-        <v>160</v>
+        <v>61.17</v>
       </c>
       <c r="H114" t="n">
-        <v>20.98</v>
+        <v>5.02</v>
       </c>
       <c r="I114" t="n">
-        <v>15.09</v>
+        <v>8.94</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C115" t="n">
         <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E115" t="n">
-        <v>10.568</v>
+        <v>23.025</v>
       </c>
       <c r="F115" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G115" t="n">
-        <v>31.7</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H115" t="n">
-        <v>0.54</v>
+        <v>3.4</v>
       </c>
       <c r="I115" t="n">
-        <v>1.73</v>
+        <v>5.18</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D116" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E116" t="n">
-        <v>103.56</v>
+        <v>40</v>
       </c>
       <c r="F116" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G116" t="n">
-        <v>103.56</v>
+        <v>160</v>
       </c>
       <c r="H116" t="n">
-        <v>3.47</v>
+        <v>20.98</v>
       </c>
       <c r="I116" t="n">
-        <v>3.47</v>
+        <v>15.09</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E122" t="n">
-        <v>106</v>
+        <v>11.038</v>
       </c>
       <c r="F122" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G122" t="n">
-        <v>106</v>
+        <v>33.11</v>
       </c>
       <c r="H122" t="n">
-        <v>5.91</v>
+        <v>1.95</v>
       </c>
       <c r="I122" t="n">
-        <v>5.9</v>
+        <v>6.26</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D123" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E123" t="n">
-        <v>40.395</v>
+        <v>6.901</v>
       </c>
       <c r="F123" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G123" t="n">
-        <v>161.58</v>
+        <v>62.11</v>
       </c>
       <c r="H123" t="n">
-        <v>22.56</v>
+        <v>5.96</v>
       </c>
       <c r="I123" t="n">
-        <v>16.23</v>
+        <v>10.61</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D124" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E124" t="n">
-        <v>23.165</v>
+        <v>106</v>
       </c>
       <c r="F124" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G124" t="n">
-        <v>69.5</v>
+        <v>106</v>
       </c>
       <c r="H124" t="n">
-        <v>3.83</v>
+        <v>5.91</v>
       </c>
       <c r="I124" t="n">
-        <v>5.83</v>
+        <v>5.9</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D125" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E125" t="n">
-        <v>6.901</v>
+        <v>40.395</v>
       </c>
       <c r="F125" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G125" t="n">
-        <v>62.11</v>
+        <v>161.58</v>
       </c>
       <c r="H125" t="n">
-        <v>5.96</v>
+        <v>22.56</v>
       </c>
       <c r="I125" t="n">
-        <v>10.61</v>
+        <v>16.23</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C126" t="n">
         <v>3</v>
       </c>
       <c r="D126" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E126" t="n">
-        <v>11.038</v>
+        <v>23.165</v>
       </c>
       <c r="F126" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G126" t="n">
-        <v>33.11</v>
+        <v>69.5</v>
       </c>
       <c r="H126" t="n">
-        <v>1.95</v>
+        <v>3.83</v>
       </c>
       <c r="I126" t="n">
-        <v>6.26</v>
+        <v>5.83</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D132" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E132" t="n">
-        <v>6.895</v>
+        <v>104.02</v>
       </c>
       <c r="F132" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G132" t="n">
-        <v>62.05</v>
+        <v>104.02</v>
       </c>
       <c r="H132" t="n">
-        <v>5.9</v>
+        <v>3.93</v>
       </c>
       <c r="I132" t="n">
-        <v>10.51</v>
+        <v>3.93</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E133" t="n">
-        <v>23.18</v>
+        <v>40.54</v>
       </c>
       <c r="F133" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G133" t="n">
-        <v>69.54000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="H133" t="n">
-        <v>3.87</v>
+        <v>23.14</v>
       </c>
       <c r="I133" t="n">
-        <v>5.89</v>
+        <v>16.65</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C134" t="n">
         <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E134" t="n">
-        <v>11.516</v>
+        <v>23.18</v>
       </c>
       <c r="F134" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G134" t="n">
-        <v>34.55</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H134" t="n">
-        <v>3.39</v>
+        <v>3.87</v>
       </c>
       <c r="I134" t="n">
-        <v>10.88</v>
+        <v>5.89</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D135" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E135" t="n">
-        <v>104.02</v>
+        <v>6.895</v>
       </c>
       <c r="F135" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G135" t="n">
-        <v>104.02</v>
+        <v>62.05</v>
       </c>
       <c r="H135" t="n">
-        <v>3.93</v>
+        <v>5.9</v>
       </c>
       <c r="I135" t="n">
-        <v>3.93</v>
+        <v>10.51</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E136" t="n">
-        <v>40.54</v>
+        <v>11.516</v>
       </c>
       <c r="F136" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G136" t="n">
-        <v>162.16</v>
+        <v>34.55</v>
       </c>
       <c r="H136" t="n">
-        <v>23.14</v>
+        <v>3.39</v>
       </c>
       <c r="I136" t="n">
-        <v>16.65</v>
+        <v>10.88</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D142" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E142" t="n">
-        <v>102.06</v>
+        <v>6.878</v>
       </c>
       <c r="F142" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G142" t="n">
-        <v>102.06</v>
+        <v>61.9</v>
       </c>
       <c r="H142" t="n">
-        <v>1.97</v>
+        <v>5.75</v>
       </c>
       <c r="I142" t="n">
-        <v>1.97</v>
+        <v>10.24</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C143" t="n">
         <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E143" t="n">
-        <v>11.498</v>
+        <v>23.135</v>
       </c>
       <c r="F143" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G143" t="n">
-        <v>34.49</v>
+        <v>69.41</v>
       </c>
       <c r="H143" t="n">
-        <v>3.33</v>
+        <v>3.74</v>
       </c>
       <c r="I143" t="n">
-        <v>10.69</v>
+        <v>5.7</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5306,29 +5306,29 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D144" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E144" t="n">
-        <v>38.89</v>
+        <v>11.498</v>
       </c>
       <c r="F144" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G144" t="n">
-        <v>155.56</v>
+        <v>34.49</v>
       </c>
       <c r="H144" t="n">
-        <v>16.54</v>
+        <v>3.33</v>
       </c>
       <c r="I144" t="n">
-        <v>11.9</v>
+        <v>10.69</v>
       </c>
       <c r="J144" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E145" t="n">
-        <v>23.135</v>
+        <v>102.06</v>
       </c>
       <c r="F145" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G145" t="n">
-        <v>69.41</v>
+        <v>102.06</v>
       </c>
       <c r="H145" t="n">
-        <v>3.74</v>
+        <v>1.97</v>
       </c>
       <c r="I145" t="n">
-        <v>5.7</v>
+        <v>1.97</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,31 +5374,201 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>4</v>
+      </c>
+      <c r="D146" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E146" t="n">
+        <v>38.89</v>
+      </c>
+      <c r="F146" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G146" t="n">
+        <v>155.56</v>
+      </c>
+      <c r="H146" t="n">
+        <v>16.54</v>
+      </c>
+      <c r="I146" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="J146" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>3</v>
+      </c>
+      <c r="D147" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E147" t="n">
+        <v>11.162</v>
+      </c>
+      <c r="F147" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G147" t="n">
+        <v>33.49</v>
+      </c>
+      <c r="H147" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="I147" t="n">
+        <v>7.48</v>
+      </c>
+      <c r="J147" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>4</v>
+      </c>
+      <c r="D148" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E148" t="n">
+        <v>38.955</v>
+      </c>
+      <c r="F148" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G148" t="n">
+        <v>155.82</v>
+      </c>
+      <c r="H148" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="I148" t="n">
+        <v>12.08</v>
+      </c>
+      <c r="J148" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>3</v>
+      </c>
+      <c r="D149" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E149" t="n">
+        <v>22.755</v>
+      </c>
+      <c r="F149" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G149" t="n">
+        <v>68.27</v>
+      </c>
+      <c r="H149" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I149" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="J149" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E150" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="F150" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G150" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="H150" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="I150" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J150" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C146" t="n">
+      <c r="C151" t="n">
         <v>9</v>
       </c>
-      <c r="D146" t="n">
+      <c r="D151" t="n">
         <v>6.239</v>
       </c>
-      <c r="E146" t="n">
-        <v>6.878</v>
-      </c>
-      <c r="F146" t="n">
+      <c r="E151" t="n">
+        <v>6.826</v>
+      </c>
+      <c r="F151" t="n">
         <v>56.15</v>
       </c>
-      <c r="G146" t="n">
-        <v>61.9</v>
-      </c>
-      <c r="H146" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="I146" t="n">
-        <v>10.24</v>
-      </c>
-      <c r="J146" t="n">
+      <c r="G151" t="n">
+        <v>61.43</v>
+      </c>
+      <c r="H151" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="I151" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="J151" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 09/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E7" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F7" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G7" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H7" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I7" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E8" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F8" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G8" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H8" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I8" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E9" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F9" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G9" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H9" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I9" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E10" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F10" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G10" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H10" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I10" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D11" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E11" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F11" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G11" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H11" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I11" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E17" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F17" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G17" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H17" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I17" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E18" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F18" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G18" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H18" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I18" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E19" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F19" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G19" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H19" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I19" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D20" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E20" t="n">
-        <v>10.662</v>
+        <v>6.82</v>
       </c>
       <c r="F20" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G20" t="n">
-        <v>31.99</v>
+        <v>61.38</v>
       </c>
       <c r="H20" t="n">
-        <v>0.83</v>
+        <v>5.23</v>
       </c>
       <c r="I20" t="n">
-        <v>2.66</v>
+        <v>9.31</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E21" t="n">
-        <v>21.915</v>
+        <v>41.789</v>
       </c>
       <c r="F21" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G21" t="n">
-        <v>65.75</v>
+        <v>167.16</v>
       </c>
       <c r="H21" t="n">
-        <v>0.08</v>
+        <v>28.14</v>
       </c>
       <c r="I21" t="n">
-        <v>0.12</v>
+        <v>20.24</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D27" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E27" t="n">
-        <v>104.9</v>
+        <v>6.795</v>
       </c>
       <c r="F27" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G27" t="n">
-        <v>104.9</v>
+        <v>61.16</v>
       </c>
       <c r="H27" t="n">
-        <v>4.81</v>
+        <v>5.01</v>
       </c>
       <c r="I27" t="n">
-        <v>4.81</v>
+        <v>8.92</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E28" t="n">
-        <v>40.532</v>
+        <v>10.66</v>
       </c>
       <c r="F28" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G28" t="n">
-        <v>162.13</v>
+        <v>31.98</v>
       </c>
       <c r="H28" t="n">
-        <v>23.11</v>
+        <v>0.82</v>
       </c>
       <c r="I28" t="n">
-        <v>16.62</v>
+        <v>2.63</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E29" t="n">
-        <v>6.795</v>
+        <v>21.98</v>
       </c>
       <c r="F29" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G29" t="n">
-        <v>61.16</v>
+        <v>65.94</v>
       </c>
       <c r="H29" t="n">
-        <v>5.01</v>
+        <v>0.27</v>
       </c>
       <c r="I29" t="n">
-        <v>8.92</v>
+        <v>0.41</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E30" t="n">
-        <v>21.98</v>
+        <v>40.532</v>
       </c>
       <c r="F30" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G30" t="n">
-        <v>65.94</v>
+        <v>162.13</v>
       </c>
       <c r="H30" t="n">
-        <v>0.27</v>
+        <v>23.11</v>
       </c>
       <c r="I30" t="n">
-        <v>0.41</v>
+        <v>16.62</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E31" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F31" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G31" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H31" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I31" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E37" t="n">
-        <v>38.879</v>
+        <v>102.8</v>
       </c>
       <c r="F37" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G37" t="n">
-        <v>155.52</v>
+        <v>102.8</v>
       </c>
       <c r="H37" t="n">
-        <v>16.5</v>
+        <v>2.71</v>
       </c>
       <c r="I37" t="n">
-        <v>11.87</v>
+        <v>2.71</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D38" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E38" t="n">
-        <v>10.67</v>
+        <v>6.728</v>
       </c>
       <c r="F38" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G38" t="n">
-        <v>32.01</v>
+        <v>60.55</v>
       </c>
       <c r="H38" t="n">
-        <v>0.85</v>
+        <v>4.4</v>
       </c>
       <c r="I38" t="n">
-        <v>2.73</v>
+        <v>7.84</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E39" t="n">
-        <v>6.728</v>
+        <v>21.839</v>
       </c>
       <c r="F39" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G39" t="n">
-        <v>60.55</v>
+        <v>65.52</v>
       </c>
       <c r="H39" t="n">
-        <v>4.4</v>
+        <v>-0.15</v>
       </c>
       <c r="I39" t="n">
-        <v>7.84</v>
+        <v>-0.23</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E40" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F40" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G40" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I40" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D41" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E41" t="n">
-        <v>102.8</v>
+        <v>38.879</v>
       </c>
       <c r="F41" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G41" t="n">
-        <v>102.8</v>
+        <v>155.52</v>
       </c>
       <c r="H41" t="n">
-        <v>2.71</v>
+        <v>16.5</v>
       </c>
       <c r="I41" t="n">
-        <v>2.71</v>
+        <v>11.87</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E47" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F47" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G47" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E48" t="n">
-        <v>38.312</v>
+        <v>10.562</v>
       </c>
       <c r="F48" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G48" t="n">
-        <v>153.25</v>
+        <v>31.69</v>
       </c>
       <c r="H48" t="n">
-        <v>14.23</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="n">
-        <v>10.24</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E50" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F50" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G50" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I50" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E51" t="n">
-        <v>6.622</v>
+        <v>21.778</v>
       </c>
       <c r="F51" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G51" t="n">
-        <v>59.6</v>
+        <v>65.33</v>
       </c>
       <c r="H51" t="n">
-        <v>3.45</v>
+        <v>-0.34</v>
       </c>
       <c r="I51" t="n">
-        <v>6.14</v>
+        <v>-0.52</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E60" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F60" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G60" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H60" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I60" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E77" t="n">
-        <v>23.4</v>
+        <v>105.8</v>
       </c>
       <c r="F77" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G77" t="n">
-        <v>70.2</v>
+        <v>105.8</v>
       </c>
       <c r="H77" t="n">
-        <v>4.53</v>
+        <v>5.71</v>
       </c>
       <c r="I77" t="n">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D78" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E78" t="n">
-        <v>6.836</v>
+        <v>42.25</v>
       </c>
       <c r="F78" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G78" t="n">
-        <v>61.52</v>
+        <v>169</v>
       </c>
       <c r="H78" t="n">
-        <v>5.37</v>
+        <v>29.98</v>
       </c>
       <c r="I78" t="n">
-        <v>9.56</v>
+        <v>21.57</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D80" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E80" t="n">
-        <v>42.25</v>
+        <v>6.836</v>
       </c>
       <c r="F80" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G80" t="n">
-        <v>169</v>
+        <v>61.52</v>
       </c>
       <c r="H80" t="n">
-        <v>29.98</v>
+        <v>5.37</v>
       </c>
       <c r="I80" t="n">
-        <v>21.57</v>
+        <v>9.56</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E81" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F81" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G81" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H81" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I81" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E87" t="n">
-        <v>10.852</v>
+        <v>106.28</v>
       </c>
       <c r="F87" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G87" t="n">
-        <v>32.56</v>
+        <v>106.28</v>
       </c>
       <c r="H87" t="n">
-        <v>1.4</v>
+        <v>6.19</v>
       </c>
       <c r="I87" t="n">
-        <v>4.49</v>
+        <v>6.18</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E88" t="n">
-        <v>6.856</v>
+        <v>23.32</v>
       </c>
       <c r="F88" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G88" t="n">
-        <v>61.7</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>5.55</v>
+        <v>4.29</v>
       </c>
       <c r="I88" t="n">
-        <v>9.880000000000001</v>
+        <v>6.53</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E90" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F90" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G90" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H90" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I90" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E91" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F91" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G91" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H91" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I91" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C97" t="n">
         <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E97" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F97" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G97" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H97" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I97" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D98" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E98" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F98" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G98" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H98" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I98" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E100" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F100" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G100" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H100" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I100" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C101" t="n">
         <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E101" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F101" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G101" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H101" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I101" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E107" t="n">
-        <v>40.5</v>
+        <v>23.33</v>
       </c>
       <c r="F107" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G107" t="n">
-        <v>162</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H107" t="n">
-        <v>22.98</v>
+        <v>4.32</v>
       </c>
       <c r="I107" t="n">
-        <v>16.53</v>
+        <v>6.58</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E108" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F108" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G108" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H108" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I108" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E110" t="n">
-        <v>103.14</v>
+        <v>10.456</v>
       </c>
       <c r="F110" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G110" t="n">
-        <v>103.14</v>
+        <v>31.37</v>
       </c>
       <c r="H110" t="n">
-        <v>3.05</v>
+        <v>0.21</v>
       </c>
       <c r="I110" t="n">
-        <v>3.05</v>
+        <v>0.67</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D111" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E111" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F111" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G111" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H111" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I111" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E117" t="n">
-        <v>41</v>
+        <v>23.145</v>
       </c>
       <c r="F117" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G117" t="n">
-        <v>164</v>
+        <v>69.44</v>
       </c>
       <c r="H117" t="n">
-        <v>24.98</v>
+        <v>3.77</v>
       </c>
       <c r="I117" t="n">
-        <v>17.97</v>
+        <v>5.74</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E118" t="n">
-        <v>6.861</v>
+        <v>105.96</v>
       </c>
       <c r="F118" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G118" t="n">
-        <v>61.75</v>
+        <v>105.96</v>
       </c>
       <c r="H118" t="n">
-        <v>5.6</v>
+        <v>5.87</v>
       </c>
       <c r="I118" t="n">
-        <v>9.970000000000001</v>
+        <v>5.86</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D119" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E119" t="n">
-        <v>10.756</v>
+        <v>6.861</v>
       </c>
       <c r="F119" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G119" t="n">
-        <v>32.27</v>
+        <v>61.75</v>
       </c>
       <c r="H119" t="n">
-        <v>1.11</v>
+        <v>5.6</v>
       </c>
       <c r="I119" t="n">
-        <v>3.56</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>10.756</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>32.27</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>1.11</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>3.56</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D121" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E121" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F121" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G121" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H121" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I121" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D127" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E127" t="n">
-        <v>103.46</v>
+        <v>39.36</v>
       </c>
       <c r="F127" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G127" t="n">
-        <v>103.46</v>
+        <v>157.44</v>
       </c>
       <c r="H127" t="n">
-        <v>3.37</v>
+        <v>18.42</v>
       </c>
       <c r="I127" t="n">
-        <v>3.37</v>
+        <v>13.25</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D128" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E128" t="n">
-        <v>23.17</v>
+        <v>6.868</v>
       </c>
       <c r="F128" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G128" t="n">
-        <v>69.51000000000001</v>
+        <v>61.81</v>
       </c>
       <c r="H128" t="n">
-        <v>3.84</v>
+        <v>5.66</v>
       </c>
       <c r="I128" t="n">
-        <v>5.85</v>
+        <v>10.08</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E130" t="n">
-        <v>6.868</v>
+        <v>23.17</v>
       </c>
       <c r="F130" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G130" t="n">
-        <v>61.81</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H130" t="n">
-        <v>5.66</v>
+        <v>3.84</v>
       </c>
       <c r="I130" t="n">
-        <v>10.08</v>
+        <v>5.85</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D131" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E131" t="n">
-        <v>39.36</v>
+        <v>103.46</v>
       </c>
       <c r="F131" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G131" t="n">
-        <v>157.44</v>
+        <v>103.46</v>
       </c>
       <c r="H131" t="n">
-        <v>18.42</v>
+        <v>3.37</v>
       </c>
       <c r="I131" t="n">
-        <v>13.25</v>
+        <v>3.37</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D137" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E137" t="n">
-        <v>6.927</v>
+        <v>104.76</v>
       </c>
       <c r="F137" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G137" t="n">
-        <v>62.34</v>
+        <v>104.76</v>
       </c>
       <c r="H137" t="n">
-        <v>6.19</v>
+        <v>4.67</v>
       </c>
       <c r="I137" t="n">
-        <v>11.02</v>
+        <v>4.67</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C138" t="n">
         <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E138" t="n">
-        <v>11.728</v>
+        <v>23.3</v>
       </c>
       <c r="F138" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G138" t="n">
-        <v>35.18</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H138" t="n">
-        <v>4.02</v>
+        <v>4.23</v>
       </c>
       <c r="I138" t="n">
-        <v>12.9</v>
+        <v>6.44</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D139" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E139" t="n">
-        <v>40.61</v>
+        <v>11.728</v>
       </c>
       <c r="F139" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G139" t="n">
-        <v>162.44</v>
+        <v>35.18</v>
       </c>
       <c r="H139" t="n">
-        <v>23.42</v>
+        <v>4.02</v>
       </c>
       <c r="I139" t="n">
-        <v>16.85</v>
+        <v>12.9</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D140" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E140" t="n">
-        <v>23.3</v>
+        <v>6.927</v>
       </c>
       <c r="F140" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G140" t="n">
-        <v>69.90000000000001</v>
+        <v>62.34</v>
       </c>
       <c r="H140" t="n">
-        <v>4.23</v>
+        <v>6.19</v>
       </c>
       <c r="I140" t="n">
-        <v>6.44</v>
+        <v>11.02</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D141" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E141" t="n">
-        <v>104.76</v>
+        <v>40.61</v>
       </c>
       <c r="F141" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G141" t="n">
-        <v>104.76</v>
+        <v>162.44</v>
       </c>
       <c r="H141" t="n">
-        <v>4.67</v>
+        <v>23.42</v>
       </c>
       <c r="I141" t="n">
-        <v>4.67</v>
+        <v>16.85</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D147" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E147" t="n">
-        <v>11.162</v>
+        <v>6.826</v>
       </c>
       <c r="F147" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G147" t="n">
-        <v>33.49</v>
+        <v>61.43</v>
       </c>
       <c r="H147" t="n">
-        <v>2.33</v>
+        <v>5.28</v>
       </c>
       <c r="I147" t="n">
-        <v>7.48</v>
+        <v>9.4</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E148" t="n">
-        <v>38.955</v>
+        <v>11.162</v>
       </c>
       <c r="F148" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G148" t="n">
-        <v>155.82</v>
+        <v>33.49</v>
       </c>
       <c r="H148" t="n">
-        <v>16.8</v>
+        <v>2.33</v>
       </c>
       <c r="I148" t="n">
-        <v>12.08</v>
+        <v>7.48</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D149" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E149" t="n">
-        <v>22.755</v>
+        <v>38.955</v>
       </c>
       <c r="F149" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G149" t="n">
-        <v>68.27</v>
+        <v>155.82</v>
       </c>
       <c r="H149" t="n">
-        <v>2.6</v>
+        <v>16.8</v>
       </c>
       <c r="I149" t="n">
-        <v>3.96</v>
+        <v>12.08</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D150" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E150" t="n">
-        <v>101.7</v>
+        <v>22.755</v>
       </c>
       <c r="F150" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G150" t="n">
-        <v>101.7</v>
+        <v>68.27</v>
       </c>
       <c r="H150" t="n">
-        <v>1.61</v>
+        <v>2.6</v>
       </c>
       <c r="I150" t="n">
-        <v>1.61</v>
+        <v>3.96</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,31 +5544,201 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E151" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="F151" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G151" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="H151" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="I151" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="J151" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E152" t="n">
+        <v>104.12</v>
+      </c>
+      <c r="F152" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G152" t="n">
+        <v>104.12</v>
+      </c>
+      <c r="H152" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="I152" t="n">
+        <v>4.03</v>
+      </c>
+      <c r="J152" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>3</v>
+      </c>
+      <c r="D153" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E153" t="n">
+        <v>11.034</v>
+      </c>
+      <c r="F153" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G153" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="H153" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="I153" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="J153" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>4</v>
+      </c>
+      <c r="D154" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E154" t="n">
+        <v>39.915</v>
+      </c>
+      <c r="F154" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G154" t="n">
+        <v>159.66</v>
+      </c>
+      <c r="H154" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="I154" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="J154" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>3</v>
+      </c>
+      <c r="D155" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E155" t="n">
+        <v>23.045</v>
+      </c>
+      <c r="F155" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G155" t="n">
+        <v>69.14</v>
+      </c>
+      <c r="H155" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="I155" t="n">
+        <v>5.28</v>
+      </c>
+      <c r="J155" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C151" t="n">
+      <c r="C156" t="n">
         <v>9</v>
       </c>
-      <c r="D151" t="n">
+      <c r="D156" t="n">
         <v>6.239</v>
       </c>
-      <c r="E151" t="n">
-        <v>6.826</v>
-      </c>
-      <c r="F151" t="n">
+      <c r="E156" t="n">
+        <v>6.893</v>
+      </c>
+      <c r="F156" t="n">
         <v>56.15</v>
       </c>
-      <c r="G151" t="n">
-        <v>61.43</v>
-      </c>
-      <c r="H151" t="n">
-        <v>5.28</v>
-      </c>
-      <c r="I151" t="n">
-        <v>9.4</v>
-      </c>
-      <c r="J151" t="n">
+      <c r="G156" t="n">
+        <v>62.04</v>
+      </c>
+      <c r="H156" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="I156" t="n">
+        <v>10.49</v>
+      </c>
+      <c r="J156" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 10/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J156"/>
+  <dimension ref="A1:J161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E7" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F7" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G7" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H7" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I7" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E8" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F8" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G8" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H8" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I8" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E9" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F9" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G9" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H9" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I9" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E10" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F10" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G10" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H10" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I10" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E11" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F11" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G11" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H11" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I11" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E17" t="n">
-        <v>21.915</v>
+        <v>41.789</v>
       </c>
       <c r="F17" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G17" t="n">
-        <v>65.75</v>
+        <v>167.16</v>
       </c>
       <c r="H17" t="n">
-        <v>0.08</v>
+        <v>28.14</v>
       </c>
       <c r="I17" t="n">
-        <v>0.12</v>
+        <v>20.24</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E18" t="n">
-        <v>105.6</v>
+        <v>10.662</v>
       </c>
       <c r="F18" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G18" t="n">
-        <v>105.6</v>
+        <v>31.99</v>
       </c>
       <c r="H18" t="n">
-        <v>5.51</v>
+        <v>0.83</v>
       </c>
       <c r="I18" t="n">
-        <v>5.51</v>
+        <v>2.66</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D19" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E19" t="n">
-        <v>10.662</v>
+        <v>6.82</v>
       </c>
       <c r="F19" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G19" t="n">
-        <v>31.99</v>
+        <v>61.38</v>
       </c>
       <c r="H19" t="n">
-        <v>0.83</v>
+        <v>5.23</v>
       </c>
       <c r="I19" t="n">
-        <v>2.66</v>
+        <v>9.31</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E20" t="n">
-        <v>6.82</v>
+        <v>21.915</v>
       </c>
       <c r="F20" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G20" t="n">
-        <v>61.38</v>
+        <v>65.75</v>
       </c>
       <c r="H20" t="n">
-        <v>5.23</v>
+        <v>0.08</v>
       </c>
       <c r="I20" t="n">
-        <v>9.31</v>
+        <v>0.12</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E21" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F21" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G21" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H21" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I21" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>6.795</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>61.16</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>5.01</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>8.92</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E28" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F28" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G28" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H28" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I28" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>40.532</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>162.13</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>23.11</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>16.62</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>40.532</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>162.13</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>23.11</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>16.62</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E31" t="n">
-        <v>104.9</v>
+        <v>6.795</v>
       </c>
       <c r="F31" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G31" t="n">
-        <v>104.9</v>
+        <v>61.16</v>
       </c>
       <c r="H31" t="n">
-        <v>4.81</v>
+        <v>5.01</v>
       </c>
       <c r="I31" t="n">
-        <v>4.81</v>
+        <v>8.92</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E37" t="n">
-        <v>102.8</v>
+        <v>38.879</v>
       </c>
       <c r="F37" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G37" t="n">
-        <v>102.8</v>
+        <v>155.52</v>
       </c>
       <c r="H37" t="n">
-        <v>2.71</v>
+        <v>16.5</v>
       </c>
       <c r="I37" t="n">
-        <v>2.71</v>
+        <v>11.87</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E38" t="n">
-        <v>6.728</v>
+        <v>21.839</v>
       </c>
       <c r="F38" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G38" t="n">
-        <v>60.55</v>
+        <v>65.52</v>
       </c>
       <c r="H38" t="n">
-        <v>4.4</v>
+        <v>-0.15</v>
       </c>
       <c r="I38" t="n">
-        <v>7.84</v>
+        <v>-0.23</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E39" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F39" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G39" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E40" t="n">
-        <v>10.67</v>
+        <v>6.728</v>
       </c>
       <c r="F40" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G40" t="n">
-        <v>32.01</v>
+        <v>60.55</v>
       </c>
       <c r="H40" t="n">
-        <v>0.85</v>
+        <v>4.4</v>
       </c>
       <c r="I40" t="n">
-        <v>2.73</v>
+        <v>7.84</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E41" t="n">
-        <v>38.879</v>
+        <v>102.8</v>
       </c>
       <c r="F41" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G41" t="n">
-        <v>155.52</v>
+        <v>102.8</v>
       </c>
       <c r="H41" t="n">
-        <v>16.5</v>
+        <v>2.71</v>
       </c>
       <c r="I41" t="n">
-        <v>11.87</v>
+        <v>2.71</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E47" t="n">
-        <v>6.622</v>
+        <v>21.778</v>
       </c>
       <c r="F47" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G47" t="n">
-        <v>59.6</v>
+        <v>65.33</v>
       </c>
       <c r="H47" t="n">
-        <v>3.45</v>
+        <v>-0.34</v>
       </c>
       <c r="I47" t="n">
-        <v>6.14</v>
+        <v>-0.52</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E48" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F48" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G48" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E50" t="n">
-        <v>38.312</v>
+        <v>10.562</v>
       </c>
       <c r="F50" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G50" t="n">
-        <v>153.25</v>
+        <v>31.69</v>
       </c>
       <c r="H50" t="n">
-        <v>14.23</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="n">
-        <v>10.24</v>
+        <v>1.7</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D51" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E51" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F51" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G51" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E60" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F60" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G60" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H60" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I60" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E61" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F61" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G61" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I61" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D77" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E77" t="n">
-        <v>105.8</v>
+        <v>6.836</v>
       </c>
       <c r="F77" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G77" t="n">
-        <v>105.8</v>
+        <v>61.52</v>
       </c>
       <c r="H77" t="n">
-        <v>5.71</v>
+        <v>5.37</v>
       </c>
       <c r="I77" t="n">
-        <v>5.7</v>
+        <v>9.56</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E78" t="n">
-        <v>42.25</v>
+        <v>10.958</v>
       </c>
       <c r="F78" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G78" t="n">
-        <v>169</v>
+        <v>32.87</v>
       </c>
       <c r="H78" t="n">
-        <v>29.98</v>
+        <v>1.71</v>
       </c>
       <c r="I78" t="n">
-        <v>21.57</v>
+        <v>5.49</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C79" t="n">
         <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E79" t="n">
-        <v>10.958</v>
+        <v>23.4</v>
       </c>
       <c r="F79" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G79" t="n">
-        <v>32.87</v>
+        <v>70.2</v>
       </c>
       <c r="H79" t="n">
-        <v>1.71</v>
+        <v>4.53</v>
       </c>
       <c r="I79" t="n">
-        <v>5.49</v>
+        <v>6.9</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E80" t="n">
-        <v>6.836</v>
+        <v>105.8</v>
       </c>
       <c r="F80" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G80" t="n">
-        <v>61.52</v>
+        <v>105.8</v>
       </c>
       <c r="H80" t="n">
-        <v>5.37</v>
+        <v>5.71</v>
       </c>
       <c r="I80" t="n">
-        <v>9.56</v>
+        <v>5.7</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D81" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E81" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F81" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G81" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H81" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I81" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D87" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E87" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F87" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G87" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H87" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I87" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D88" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E88" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F88" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G88" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I88" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D89" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E89" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F89" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G89" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H89" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I89" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E90" t="n">
-        <v>6.856</v>
+        <v>23.32</v>
       </c>
       <c r="F90" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G90" t="n">
-        <v>61.7</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H90" t="n">
-        <v>5.55</v>
+        <v>4.29</v>
       </c>
       <c r="I90" t="n">
-        <v>9.880000000000001</v>
+        <v>6.53</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E91" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F91" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G91" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H91" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I91" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D97" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E97" t="n">
-        <v>10.642</v>
+        <v>40.65</v>
       </c>
       <c r="F97" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G97" t="n">
-        <v>31.93</v>
+        <v>162.6</v>
       </c>
       <c r="H97" t="n">
-        <v>0.77</v>
+        <v>23.58</v>
       </c>
       <c r="I97" t="n">
-        <v>2.47</v>
+        <v>16.96</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E98" t="n">
-        <v>6.839</v>
+        <v>23.35</v>
       </c>
       <c r="F98" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G98" t="n">
-        <v>61.55</v>
+        <v>70.05</v>
       </c>
       <c r="H98" t="n">
-        <v>5.4</v>
+        <v>4.38</v>
       </c>
       <c r="I98" t="n">
-        <v>9.619999999999999</v>
+        <v>6.67</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E100" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F100" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G100" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H100" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I100" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D101" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E101" t="n">
-        <v>23.35</v>
+        <v>6.839</v>
       </c>
       <c r="F101" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G101" t="n">
-        <v>70.05</v>
+        <v>61.55</v>
       </c>
       <c r="H101" t="n">
-        <v>4.38</v>
+        <v>5.4</v>
       </c>
       <c r="I101" t="n">
-        <v>6.67</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D107" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E107" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F107" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G107" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H107" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I107" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E108" t="n">
-        <v>103.14</v>
+        <v>10.456</v>
       </c>
       <c r="F108" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G108" t="n">
-        <v>103.14</v>
+        <v>31.37</v>
       </c>
       <c r="H108" t="n">
-        <v>3.05</v>
+        <v>0.21</v>
       </c>
       <c r="I108" t="n">
-        <v>3.05</v>
+        <v>0.67</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C110" t="n">
         <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E110" t="n">
-        <v>10.456</v>
+        <v>23.33</v>
       </c>
       <c r="F110" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G110" t="n">
-        <v>31.37</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H110" t="n">
-        <v>0.21</v>
+        <v>4.32</v>
       </c>
       <c r="I110" t="n">
-        <v>0.67</v>
+        <v>6.58</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D111" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E111" t="n">
-        <v>40.5</v>
+        <v>103.14</v>
       </c>
       <c r="F111" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G111" t="n">
-        <v>162</v>
+        <v>103.14</v>
       </c>
       <c r="H111" t="n">
-        <v>22.98</v>
+        <v>3.05</v>
       </c>
       <c r="I111" t="n">
-        <v>16.53</v>
+        <v>3.05</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E117" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F117" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G117" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H117" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I117" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D118" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E118" t="n">
-        <v>105.96</v>
+        <v>6.861</v>
       </c>
       <c r="F118" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G118" t="n">
-        <v>105.96</v>
+        <v>61.75</v>
       </c>
       <c r="H118" t="n">
-        <v>5.87</v>
+        <v>5.6</v>
       </c>
       <c r="I118" t="n">
-        <v>5.86</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E119" t="n">
-        <v>6.861</v>
+        <v>10.756</v>
       </c>
       <c r="F119" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G119" t="n">
-        <v>61.75</v>
+        <v>32.27</v>
       </c>
       <c r="H119" t="n">
-        <v>5.6</v>
+        <v>1.11</v>
       </c>
       <c r="I119" t="n">
-        <v>9.970000000000001</v>
+        <v>3.56</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C120" t="n">
         <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E120" t="n">
-        <v>10.756</v>
+        <v>23.145</v>
       </c>
       <c r="F120" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G120" t="n">
-        <v>32.27</v>
+        <v>69.44</v>
       </c>
       <c r="H120" t="n">
-        <v>1.11</v>
+        <v>3.77</v>
       </c>
       <c r="I120" t="n">
-        <v>3.56</v>
+        <v>5.74</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D121" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E121" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F121" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G121" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H121" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I121" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D127" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E127" t="n">
-        <v>39.36</v>
+        <v>103.46</v>
       </c>
       <c r="F127" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G127" t="n">
-        <v>157.44</v>
+        <v>103.46</v>
       </c>
       <c r="H127" t="n">
-        <v>18.42</v>
+        <v>3.37</v>
       </c>
       <c r="I127" t="n">
-        <v>13.25</v>
+        <v>3.37</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E128" t="n">
-        <v>6.868</v>
+        <v>23.17</v>
       </c>
       <c r="F128" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G128" t="n">
-        <v>61.81</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H128" t="n">
-        <v>5.66</v>
+        <v>3.84</v>
       </c>
       <c r="I128" t="n">
-        <v>10.08</v>
+        <v>5.85</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D130" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E130" t="n">
-        <v>23.17</v>
+        <v>39.36</v>
       </c>
       <c r="F130" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G130" t="n">
-        <v>69.51000000000001</v>
+        <v>157.44</v>
       </c>
       <c r="H130" t="n">
-        <v>3.84</v>
+        <v>18.42</v>
       </c>
       <c r="I130" t="n">
-        <v>5.85</v>
+        <v>13.25</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D131" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E131" t="n">
-        <v>103.46</v>
+        <v>6.868</v>
       </c>
       <c r="F131" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G131" t="n">
-        <v>103.46</v>
+        <v>61.81</v>
       </c>
       <c r="H131" t="n">
-        <v>3.37</v>
+        <v>5.66</v>
       </c>
       <c r="I131" t="n">
-        <v>3.37</v>
+        <v>10.08</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D137" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E137" t="n">
-        <v>104.76</v>
+        <v>40.61</v>
       </c>
       <c r="F137" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G137" t="n">
-        <v>104.76</v>
+        <v>162.44</v>
       </c>
       <c r="H137" t="n">
-        <v>4.67</v>
+        <v>23.42</v>
       </c>
       <c r="I137" t="n">
-        <v>4.67</v>
+        <v>16.85</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C138" t="n">
         <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E138" t="n">
-        <v>23.3</v>
+        <v>11.728</v>
       </c>
       <c r="F138" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G138" t="n">
-        <v>69.90000000000001</v>
+        <v>35.18</v>
       </c>
       <c r="H138" t="n">
-        <v>4.23</v>
+        <v>4.02</v>
       </c>
       <c r="I138" t="n">
-        <v>6.44</v>
+        <v>12.9</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D139" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E139" t="n">
-        <v>11.728</v>
+        <v>6.927</v>
       </c>
       <c r="F139" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G139" t="n">
-        <v>35.18</v>
+        <v>62.34</v>
       </c>
       <c r="H139" t="n">
-        <v>4.02</v>
+        <v>6.19</v>
       </c>
       <c r="I139" t="n">
-        <v>12.9</v>
+        <v>11.02</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D140" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E140" t="n">
-        <v>6.927</v>
+        <v>104.76</v>
       </c>
       <c r="F140" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G140" t="n">
-        <v>62.34</v>
+        <v>104.76</v>
       </c>
       <c r="H140" t="n">
-        <v>6.19</v>
+        <v>4.67</v>
       </c>
       <c r="I140" t="n">
-        <v>11.02</v>
+        <v>4.67</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D141" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E141" t="n">
-        <v>40.61</v>
+        <v>23.3</v>
       </c>
       <c r="F141" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G141" t="n">
-        <v>162.44</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H141" t="n">
-        <v>23.42</v>
+        <v>4.23</v>
       </c>
       <c r="I141" t="n">
-        <v>16.85</v>
+        <v>6.44</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D147" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E147" t="n">
-        <v>6.826</v>
+        <v>101.7</v>
       </c>
       <c r="F147" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G147" t="n">
-        <v>61.43</v>
+        <v>101.7</v>
       </c>
       <c r="H147" t="n">
-        <v>5.28</v>
+        <v>1.61</v>
       </c>
       <c r="I147" t="n">
-        <v>9.4</v>
+        <v>1.61</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D148" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E148" t="n">
-        <v>11.162</v>
+        <v>38.955</v>
       </c>
       <c r="F148" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G148" t="n">
-        <v>33.49</v>
+        <v>155.82</v>
       </c>
       <c r="H148" t="n">
-        <v>2.33</v>
+        <v>16.8</v>
       </c>
       <c r="I148" t="n">
-        <v>7.48</v>
+        <v>12.08</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E149" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F149" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G149" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H149" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I149" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D150" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E150" t="n">
-        <v>22.755</v>
+        <v>6.826</v>
       </c>
       <c r="F150" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G150" t="n">
-        <v>68.27</v>
+        <v>61.43</v>
       </c>
       <c r="H150" t="n">
-        <v>2.6</v>
+        <v>5.28</v>
       </c>
       <c r="I150" t="n">
-        <v>3.96</v>
+        <v>9.4</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E151" t="n">
-        <v>101.7</v>
+        <v>11.162</v>
       </c>
       <c r="F151" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G151" t="n">
-        <v>101.7</v>
+        <v>33.49</v>
       </c>
       <c r="H151" t="n">
-        <v>1.61</v>
+        <v>2.33</v>
       </c>
       <c r="I151" t="n">
-        <v>1.61</v>
+        <v>7.48</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5739,6 +5739,176 @@
         <v>10.49</v>
       </c>
       <c r="J156" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>3</v>
+      </c>
+      <c r="D157" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E157" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="F157" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G157" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="H157" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="I157" t="n">
+        <v>5.13</v>
+      </c>
+      <c r="J157" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>4</v>
+      </c>
+      <c r="D158" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E158" t="n">
+        <v>40.015</v>
+      </c>
+      <c r="F158" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G158" t="n">
+        <v>160.06</v>
+      </c>
+      <c r="H158" t="n">
+        <v>21.04</v>
+      </c>
+      <c r="I158" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="J158" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>3</v>
+      </c>
+      <c r="D159" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E159" t="n">
+        <v>23.08</v>
+      </c>
+      <c r="F159" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G159" t="n">
+        <v>69.23999999999999</v>
+      </c>
+      <c r="H159" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="I159" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="J159" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E160" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="F160" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G160" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="H160" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="I160" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="J160" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>9</v>
+      </c>
+      <c r="D161" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E161" t="n">
+        <v>6.913</v>
+      </c>
+      <c r="F161" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G161" t="n">
+        <v>62.22</v>
+      </c>
+      <c r="H161" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="I161" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="J161" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 13/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J161"/>
+  <dimension ref="A1:J166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E22" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F22" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G22" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I22" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E23" t="n">
-        <v>105.78</v>
+        <v>10.536</v>
       </c>
       <c r="F23" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G23" t="n">
-        <v>105.78</v>
+        <v>31.61</v>
       </c>
       <c r="H23" t="n">
-        <v>5.69</v>
+        <v>0.45</v>
       </c>
       <c r="I23" t="n">
-        <v>5.68</v>
+        <v>1.44</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E24" t="n">
-        <v>6.799</v>
+        <v>21.669</v>
       </c>
       <c r="F24" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G24" t="n">
-        <v>61.19</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H24" t="n">
-        <v>5.04</v>
+        <v>-0.66</v>
       </c>
       <c r="I24" t="n">
-        <v>8.98</v>
+        <v>-1.01</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E25" t="n">
-        <v>10.536</v>
+        <v>105.78</v>
       </c>
       <c r="F25" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G25" t="n">
-        <v>31.61</v>
+        <v>105.78</v>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>5.69</v>
       </c>
       <c r="I25" t="n">
-        <v>1.44</v>
+        <v>5.68</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E26" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F26" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G26" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H26" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I26" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E32" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F32" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G32" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H32" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I32" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E33" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F33" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G33" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H33" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I33" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E35" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F35" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G35" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H35" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I35" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E36" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F36" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G36" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H36" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I36" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E42" t="n">
-        <v>22</v>
+        <v>6.629</v>
       </c>
       <c r="F42" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>59.66</v>
       </c>
       <c r="H42" t="n">
-        <v>0.33</v>
+        <v>3.51</v>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>6.25</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>100.06</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>100.06</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.03</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.03</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E45" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F45" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G45" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H45" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I45" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E46" t="n">
-        <v>6.629</v>
+        <v>10.61</v>
       </c>
       <c r="F46" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G46" t="n">
-        <v>59.66</v>
+        <v>31.83</v>
       </c>
       <c r="H46" t="n">
-        <v>3.51</v>
+        <v>0.67</v>
       </c>
       <c r="I46" t="n">
-        <v>6.25</v>
+        <v>2.15</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E52" t="n">
-        <v>100.34</v>
+        <v>21.703</v>
       </c>
       <c r="F52" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G52" t="n">
-        <v>100.34</v>
+        <v>65.11</v>
       </c>
       <c r="H52" t="n">
-        <v>0.25</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I52" t="n">
-        <v>0.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D53" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E53" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F53" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G53" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H53" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I53" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E54" t="n">
-        <v>10.702</v>
+        <v>100.34</v>
       </c>
       <c r="F54" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G54" t="n">
-        <v>32.11</v>
+        <v>100.34</v>
       </c>
       <c r="H54" t="n">
-        <v>0.95</v>
+        <v>0.25</v>
       </c>
       <c r="I54" t="n">
-        <v>3.05</v>
+        <v>0.25</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D55" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E55" t="n">
-        <v>6.629</v>
+        <v>38.544</v>
       </c>
       <c r="F55" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G55" t="n">
-        <v>59.66</v>
+        <v>154.18</v>
       </c>
       <c r="H55" t="n">
-        <v>3.51</v>
+        <v>15.16</v>
       </c>
       <c r="I55" t="n">
-        <v>6.25</v>
+        <v>10.9</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E56" t="n">
-        <v>21.703</v>
+        <v>10.702</v>
       </c>
       <c r="F56" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G56" t="n">
-        <v>65.11</v>
+        <v>32.11</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.85</v>
+        <v>3.05</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E62" t="n">
-        <v>22.7</v>
+        <v>41.064</v>
       </c>
       <c r="F62" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G62" t="n">
-        <v>68.09999999999999</v>
+        <v>164.26</v>
       </c>
       <c r="H62" t="n">
-        <v>2.43</v>
+        <v>25.24</v>
       </c>
       <c r="I62" t="n">
-        <v>3.7</v>
+        <v>18.16</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>105.5</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>105.5</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>5.41</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>5.41</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E65" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F65" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G65" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H65" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I65" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E66" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F66" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G66" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H66" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I66" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E72" t="n">
-        <v>6.811</v>
+        <v>104.22</v>
       </c>
       <c r="F72" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G72" t="n">
-        <v>61.3</v>
+        <v>104.22</v>
       </c>
       <c r="H72" t="n">
-        <v>5.15</v>
+        <v>4.13</v>
       </c>
       <c r="I72" t="n">
-        <v>9.17</v>
+        <v>4.13</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D73" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E73" t="n">
-        <v>23</v>
+        <v>41.15</v>
       </c>
       <c r="F73" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G73" t="n">
-        <v>69</v>
+        <v>164.6</v>
       </c>
       <c r="H73" t="n">
-        <v>3.33</v>
+        <v>25.58</v>
       </c>
       <c r="I73" t="n">
-        <v>5.07</v>
+        <v>18.4</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E75" t="n">
-        <v>41.15</v>
+        <v>6.811</v>
       </c>
       <c r="F75" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G75" t="n">
-        <v>164.6</v>
+        <v>61.3</v>
       </c>
       <c r="H75" t="n">
-        <v>25.58</v>
+        <v>5.15</v>
       </c>
       <c r="I75" t="n">
-        <v>18.4</v>
+        <v>9.17</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E76" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F76" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G76" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H76" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I76" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E82" t="n">
-        <v>10.988</v>
+        <v>106.26</v>
       </c>
       <c r="F82" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G82" t="n">
-        <v>32.96</v>
+        <v>106.26</v>
       </c>
       <c r="H82" t="n">
-        <v>1.8</v>
+        <v>6.17</v>
       </c>
       <c r="I82" t="n">
-        <v>5.78</v>
+        <v>6.16</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D83" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E83" t="n">
-        <v>6.846</v>
+        <v>42.1</v>
       </c>
       <c r="F83" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G83" t="n">
-        <v>61.61</v>
+        <v>168.4</v>
       </c>
       <c r="H83" t="n">
-        <v>5.46</v>
+        <v>29.38</v>
       </c>
       <c r="I83" t="n">
-        <v>9.720000000000001</v>
+        <v>21.13</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D85" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E85" t="n">
-        <v>42.1</v>
+        <v>6.846</v>
       </c>
       <c r="F85" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G85" t="n">
-        <v>168.4</v>
+        <v>61.61</v>
       </c>
       <c r="H85" t="n">
-        <v>29.38</v>
+        <v>5.46</v>
       </c>
       <c r="I85" t="n">
-        <v>21.13</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E86" t="n">
-        <v>106.26</v>
+        <v>10.988</v>
       </c>
       <c r="F86" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G86" t="n">
-        <v>106.26</v>
+        <v>32.96</v>
       </c>
       <c r="H86" t="n">
-        <v>6.17</v>
+        <v>1.8</v>
       </c>
       <c r="I86" t="n">
-        <v>6.16</v>
+        <v>5.78</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D92" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E92" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F92" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G92" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H92" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I92" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C93" t="n">
         <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E93" t="n">
-        <v>23.025</v>
+        <v>10.876</v>
       </c>
       <c r="F93" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G93" t="n">
-        <v>69.06999999999999</v>
+        <v>32.63</v>
       </c>
       <c r="H93" t="n">
-        <v>3.4</v>
+        <v>1.47</v>
       </c>
       <c r="I93" t="n">
-        <v>5.18</v>
+        <v>4.72</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C95" t="n">
         <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E95" t="n">
-        <v>10.876</v>
+        <v>23.025</v>
       </c>
       <c r="F95" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G95" t="n">
-        <v>32.63</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H95" t="n">
-        <v>1.47</v>
+        <v>3.4</v>
       </c>
       <c r="I95" t="n">
-        <v>4.72</v>
+        <v>5.18</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D96" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E96" t="n">
-        <v>40.575</v>
+        <v>6.797</v>
       </c>
       <c r="F96" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G96" t="n">
-        <v>162.3</v>
+        <v>61.17</v>
       </c>
       <c r="H96" t="n">
-        <v>23.28</v>
+        <v>5.02</v>
       </c>
       <c r="I96" t="n">
-        <v>16.75</v>
+        <v>8.94</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D102" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E102" t="n">
-        <v>6.804</v>
+        <v>40.97</v>
       </c>
       <c r="F102" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G102" t="n">
-        <v>61.24</v>
+        <v>163.88</v>
       </c>
       <c r="H102" t="n">
-        <v>5.09</v>
+        <v>24.86</v>
       </c>
       <c r="I102" t="n">
-        <v>9.07</v>
+        <v>17.88</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D103" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E103" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F103" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G103" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H103" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I103" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E105" t="n">
-        <v>103.46</v>
+        <v>23.29</v>
       </c>
       <c r="F105" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G105" t="n">
-        <v>103.46</v>
+        <v>69.87</v>
       </c>
       <c r="H105" t="n">
-        <v>3.37</v>
+        <v>4.2</v>
       </c>
       <c r="I105" t="n">
-        <v>3.37</v>
+        <v>6.4</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D106" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E106" t="n">
-        <v>40.97</v>
+        <v>6.804</v>
       </c>
       <c r="F106" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G106" t="n">
-        <v>163.88</v>
+        <v>61.24</v>
       </c>
       <c r="H106" t="n">
-        <v>24.86</v>
+        <v>5.09</v>
       </c>
       <c r="I106" t="n">
-        <v>17.88</v>
+        <v>9.07</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E112" t="n">
-        <v>103.56</v>
+        <v>40</v>
       </c>
       <c r="F112" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G112" t="n">
-        <v>103.56</v>
+        <v>160</v>
       </c>
       <c r="H112" t="n">
-        <v>3.47</v>
+        <v>20.98</v>
       </c>
       <c r="I112" t="n">
-        <v>3.47</v>
+        <v>15.09</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C113" t="n">
         <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E113" t="n">
-        <v>10.568</v>
+        <v>23.025</v>
       </c>
       <c r="F113" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G113" t="n">
-        <v>31.7</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H113" t="n">
-        <v>0.54</v>
+        <v>3.4</v>
       </c>
       <c r="I113" t="n">
-        <v>1.73</v>
+        <v>5.18</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C115" t="n">
         <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E115" t="n">
-        <v>23.025</v>
+        <v>10.568</v>
       </c>
       <c r="F115" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G115" t="n">
-        <v>69.06999999999999</v>
+        <v>31.7</v>
       </c>
       <c r="H115" t="n">
-        <v>3.4</v>
+        <v>0.54</v>
       </c>
       <c r="I115" t="n">
-        <v>5.18</v>
+        <v>1.73</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D116" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E116" t="n">
-        <v>40</v>
+        <v>103.56</v>
       </c>
       <c r="F116" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G116" t="n">
-        <v>160</v>
+        <v>103.56</v>
       </c>
       <c r="H116" t="n">
-        <v>20.98</v>
+        <v>3.47</v>
       </c>
       <c r="I116" t="n">
-        <v>15.09</v>
+        <v>3.47</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C122" t="n">
         <v>3</v>
       </c>
       <c r="D122" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E122" t="n">
-        <v>11.038</v>
+        <v>23.165</v>
       </c>
       <c r="F122" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G122" t="n">
-        <v>33.11</v>
+        <v>69.5</v>
       </c>
       <c r="H122" t="n">
-        <v>1.95</v>
+        <v>3.83</v>
       </c>
       <c r="I122" t="n">
-        <v>6.26</v>
+        <v>5.83</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D123" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E123" t="n">
-        <v>6.901</v>
+        <v>106</v>
       </c>
       <c r="F123" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G123" t="n">
-        <v>62.11</v>
+        <v>106</v>
       </c>
       <c r="H123" t="n">
-        <v>5.96</v>
+        <v>5.91</v>
       </c>
       <c r="I123" t="n">
-        <v>10.61</v>
+        <v>5.9</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D124" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E124" t="n">
-        <v>106</v>
+        <v>40.395</v>
       </c>
       <c r="F124" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G124" t="n">
-        <v>106</v>
+        <v>161.58</v>
       </c>
       <c r="H124" t="n">
-        <v>5.91</v>
+        <v>22.56</v>
       </c>
       <c r="I124" t="n">
-        <v>5.9</v>
+        <v>16.23</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D125" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E125" t="n">
-        <v>40.395</v>
+        <v>6.901</v>
       </c>
       <c r="F125" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G125" t="n">
-        <v>161.58</v>
+        <v>62.11</v>
       </c>
       <c r="H125" t="n">
-        <v>22.56</v>
+        <v>5.96</v>
       </c>
       <c r="I125" t="n">
-        <v>16.23</v>
+        <v>10.61</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C126" t="n">
         <v>3</v>
       </c>
       <c r="D126" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E126" t="n">
-        <v>23.165</v>
+        <v>11.038</v>
       </c>
       <c r="F126" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G126" t="n">
-        <v>69.5</v>
+        <v>33.11</v>
       </c>
       <c r="H126" t="n">
-        <v>3.83</v>
+        <v>1.95</v>
       </c>
       <c r="I126" t="n">
-        <v>5.83</v>
+        <v>6.26</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E132" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F132" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G132" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H132" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I132" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D133" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E133" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F133" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G133" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H133" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I133" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E135" t="n">
-        <v>6.895</v>
+        <v>40.54</v>
       </c>
       <c r="F135" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G135" t="n">
-        <v>62.05</v>
+        <v>162.16</v>
       </c>
       <c r="H135" t="n">
-        <v>5.9</v>
+        <v>23.14</v>
       </c>
       <c r="I135" t="n">
-        <v>10.51</v>
+        <v>16.65</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D136" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E136" t="n">
-        <v>11.516</v>
+        <v>104.02</v>
       </c>
       <c r="F136" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G136" t="n">
-        <v>34.55</v>
+        <v>104.02</v>
       </c>
       <c r="H136" t="n">
-        <v>3.39</v>
+        <v>3.93</v>
       </c>
       <c r="I136" t="n">
-        <v>10.88</v>
+        <v>3.93</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D142" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E142" t="n">
-        <v>6.878</v>
+        <v>38.89</v>
       </c>
       <c r="F142" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G142" t="n">
-        <v>61.9</v>
+        <v>155.56</v>
       </c>
       <c r="H142" t="n">
-        <v>5.75</v>
+        <v>16.54</v>
       </c>
       <c r="I142" t="n">
-        <v>10.24</v>
+        <v>11.9</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D143" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E143" t="n">
-        <v>23.135</v>
+        <v>102.06</v>
       </c>
       <c r="F143" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G143" t="n">
-        <v>69.41</v>
+        <v>102.06</v>
       </c>
       <c r="H143" t="n">
-        <v>3.74</v>
+        <v>1.97</v>
       </c>
       <c r="I143" t="n">
-        <v>5.7</v>
+        <v>1.97</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5306,29 +5306,29 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C144" t="n">
         <v>3</v>
       </c>
       <c r="D144" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E144" t="n">
-        <v>11.498</v>
+        <v>23.135</v>
       </c>
       <c r="F144" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G144" t="n">
-        <v>34.49</v>
+        <v>69.41</v>
       </c>
       <c r="H144" t="n">
-        <v>3.33</v>
+        <v>3.74</v>
       </c>
       <c r="I144" t="n">
-        <v>10.69</v>
+        <v>5.7</v>
       </c>
       <c r="J144" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D145" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E145" t="n">
-        <v>102.06</v>
+        <v>6.878</v>
       </c>
       <c r="F145" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G145" t="n">
-        <v>102.06</v>
+        <v>61.9</v>
       </c>
       <c r="H145" t="n">
-        <v>1.97</v>
+        <v>5.75</v>
       </c>
       <c r="I145" t="n">
-        <v>1.97</v>
+        <v>10.24</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E146" t="n">
-        <v>38.89</v>
+        <v>11.498</v>
       </c>
       <c r="F146" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G146" t="n">
-        <v>155.56</v>
+        <v>34.49</v>
       </c>
       <c r="H146" t="n">
-        <v>16.54</v>
+        <v>3.33</v>
       </c>
       <c r="I146" t="n">
-        <v>11.9</v>
+        <v>10.69</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E152" t="n">
-        <v>104.12</v>
+        <v>11.034</v>
       </c>
       <c r="F152" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G152" t="n">
-        <v>104.12</v>
+        <v>33.1</v>
       </c>
       <c r="H152" t="n">
-        <v>4.03</v>
+        <v>1.94</v>
       </c>
       <c r="I152" t="n">
-        <v>4.03</v>
+        <v>6.23</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D153" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E153" t="n">
-        <v>11.034</v>
+        <v>104.12</v>
       </c>
       <c r="F153" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G153" t="n">
-        <v>33.1</v>
+        <v>104.12</v>
       </c>
       <c r="H153" t="n">
-        <v>1.94</v>
+        <v>4.03</v>
       </c>
       <c r="I153" t="n">
-        <v>6.23</v>
+        <v>4.03</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D157" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E157" t="n">
-        <v>10.92</v>
+        <v>104.5</v>
       </c>
       <c r="F157" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G157" t="n">
-        <v>32.76</v>
+        <v>104.5</v>
       </c>
       <c r="H157" t="n">
-        <v>1.6</v>
+        <v>4.41</v>
       </c>
       <c r="I157" t="n">
-        <v>5.13</v>
+        <v>4.41</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E158" t="n">
-        <v>40.015</v>
+        <v>23.08</v>
       </c>
       <c r="F158" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G158" t="n">
-        <v>160.06</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H158" t="n">
-        <v>21.04</v>
+        <v>3.57</v>
       </c>
       <c r="I158" t="n">
-        <v>15.13</v>
+        <v>5.44</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D159" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E159" t="n">
-        <v>23.08</v>
+        <v>6.913</v>
       </c>
       <c r="F159" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G159" t="n">
-        <v>69.23999999999999</v>
+        <v>62.22</v>
       </c>
       <c r="H159" t="n">
-        <v>3.57</v>
+        <v>6.07</v>
       </c>
       <c r="I159" t="n">
-        <v>5.44</v>
+        <v>10.81</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E160" t="n">
-        <v>104.5</v>
+        <v>10.92</v>
       </c>
       <c r="F160" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G160" t="n">
-        <v>104.5</v>
+        <v>32.76</v>
       </c>
       <c r="H160" t="n">
-        <v>4.41</v>
+        <v>1.6</v>
       </c>
       <c r="I160" t="n">
-        <v>4.41</v>
+        <v>5.13</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,31 +5884,201 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>4</v>
+      </c>
+      <c r="D161" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E161" t="n">
+        <v>40.015</v>
+      </c>
+      <c r="F161" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G161" t="n">
+        <v>160.06</v>
+      </c>
+      <c r="H161" t="n">
+        <v>21.04</v>
+      </c>
+      <c r="I161" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="J161" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E162" t="n">
+        <v>103.84</v>
+      </c>
+      <c r="F162" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G162" t="n">
+        <v>103.84</v>
+      </c>
+      <c r="H162" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I162" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J162" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>3</v>
+      </c>
+      <c r="D163" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E163" t="n">
+        <v>10.748</v>
+      </c>
+      <c r="F163" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G163" t="n">
+        <v>32.24</v>
+      </c>
+      <c r="H163" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="I163" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="J163" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>4</v>
+      </c>
+      <c r="D164" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E164" t="n">
+        <v>38.845</v>
+      </c>
+      <c r="F164" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G164" t="n">
+        <v>155.38</v>
+      </c>
+      <c r="H164" t="n">
+        <v>16.36</v>
+      </c>
+      <c r="I164" t="n">
+        <v>11.77</v>
+      </c>
+      <c r="J164" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>3</v>
+      </c>
+      <c r="D165" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E165" t="n">
+        <v>23.01</v>
+      </c>
+      <c r="F165" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G165" t="n">
+        <v>69.03</v>
+      </c>
+      <c r="H165" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="I165" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="J165" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="1" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C161" t="n">
+      <c r="C166" t="n">
         <v>9</v>
       </c>
-      <c r="D161" t="n">
+      <c r="D166" t="n">
         <v>6.239</v>
       </c>
-      <c r="E161" t="n">
-        <v>6.913</v>
-      </c>
-      <c r="F161" t="n">
+      <c r="E166" t="n">
+        <v>6.927</v>
+      </c>
+      <c r="F166" t="n">
         <v>56.15</v>
       </c>
-      <c r="G161" t="n">
-        <v>62.22</v>
-      </c>
-      <c r="H161" t="n">
-        <v>6.07</v>
-      </c>
-      <c r="I161" t="n">
-        <v>10.81</v>
-      </c>
-      <c r="J161" t="n">
+      <c r="G166" t="n">
+        <v>62.34</v>
+      </c>
+      <c r="H166" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="I166" t="n">
+        <v>11.02</v>
+      </c>
+      <c r="J166" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 14/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J166"/>
+  <dimension ref="A1:J171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E22" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F22" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G22" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H22" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I22" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E23" t="n">
-        <v>10.536</v>
+        <v>105.78</v>
       </c>
       <c r="F23" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G23" t="n">
-        <v>31.61</v>
+        <v>105.78</v>
       </c>
       <c r="H23" t="n">
-        <v>0.45</v>
+        <v>5.69</v>
       </c>
       <c r="I23" t="n">
-        <v>1.44</v>
+        <v>5.68</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E24" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F24" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G24" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I24" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E25" t="n">
-        <v>105.78</v>
+        <v>10.536</v>
       </c>
       <c r="F25" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G25" t="n">
-        <v>105.78</v>
+        <v>31.61</v>
       </c>
       <c r="H25" t="n">
-        <v>5.69</v>
+        <v>0.45</v>
       </c>
       <c r="I25" t="n">
-        <v>5.68</v>
+        <v>1.44</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E26" t="n">
-        <v>6.799</v>
+        <v>21.669</v>
       </c>
       <c r="F26" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G26" t="n">
-        <v>61.19</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>5.04</v>
+        <v>-0.66</v>
       </c>
       <c r="I26" t="n">
-        <v>8.98</v>
+        <v>-1.01</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E32" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F32" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G32" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H32" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I32" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E33" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F33" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G33" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H33" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I33" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D35" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E35" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F35" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G35" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H35" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I35" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E36" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F36" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G36" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H36" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I36" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E42" t="n">
-        <v>6.629</v>
+        <v>10.61</v>
       </c>
       <c r="F42" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G42" t="n">
-        <v>59.66</v>
+        <v>31.83</v>
       </c>
       <c r="H42" t="n">
-        <v>3.51</v>
+        <v>0.67</v>
       </c>
       <c r="I42" t="n">
-        <v>6.25</v>
+        <v>2.15</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>6.629</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>59.66</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>3.51</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>6.25</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E45" t="n">
-        <v>100.06</v>
+        <v>38.497</v>
       </c>
       <c r="F45" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G45" t="n">
-        <v>100.06</v>
+        <v>153.99</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.03</v>
+        <v>14.97</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03</v>
+        <v>10.77</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E46" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F46" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G46" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H46" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I46" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E52" t="n">
-        <v>21.703</v>
+        <v>10.702</v>
       </c>
       <c r="F52" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G52" t="n">
-        <v>65.11</v>
+        <v>32.11</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.85</v>
+        <v>3.05</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D53" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E53" t="n">
-        <v>6.629</v>
+        <v>38.544</v>
       </c>
       <c r="F53" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G53" t="n">
-        <v>59.66</v>
+        <v>154.18</v>
       </c>
       <c r="H53" t="n">
-        <v>3.51</v>
+        <v>15.16</v>
       </c>
       <c r="I53" t="n">
-        <v>6.25</v>
+        <v>10.9</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E54" t="n">
-        <v>100.34</v>
+        <v>21.703</v>
       </c>
       <c r="F54" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G54" t="n">
-        <v>100.34</v>
+        <v>65.11</v>
       </c>
       <c r="H54" t="n">
-        <v>0.25</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>0.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E55" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F55" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G55" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H55" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I55" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E56" t="n">
-        <v>10.702</v>
+        <v>100.34</v>
       </c>
       <c r="F56" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G56" t="n">
-        <v>32.11</v>
+        <v>100.34</v>
       </c>
       <c r="H56" t="n">
-        <v>0.95</v>
+        <v>0.25</v>
       </c>
       <c r="I56" t="n">
-        <v>3.05</v>
+        <v>0.25</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E62" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F62" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G62" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H62" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I62" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>41.064</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>164.26</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>25.24</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>18.16</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E66" t="n">
-        <v>105.5</v>
+        <v>10.712</v>
       </c>
       <c r="F66" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G66" t="n">
-        <v>105.5</v>
+        <v>32.14</v>
       </c>
       <c r="H66" t="n">
-        <v>5.41</v>
+        <v>0.98</v>
       </c>
       <c r="I66" t="n">
-        <v>5.41</v>
+        <v>3.15</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>41.15</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>164.6</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>25.58</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>18.4</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E75" t="n">
-        <v>6.811</v>
+        <v>104.22</v>
       </c>
       <c r="F75" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G75" t="n">
-        <v>61.3</v>
+        <v>104.22</v>
       </c>
       <c r="H75" t="n">
-        <v>5.15</v>
+        <v>4.13</v>
       </c>
       <c r="I75" t="n">
-        <v>9.17</v>
+        <v>4.13</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D76" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E76" t="n">
-        <v>23</v>
+        <v>41.15</v>
       </c>
       <c r="F76" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G76" t="n">
-        <v>69</v>
+        <v>164.6</v>
       </c>
       <c r="H76" t="n">
-        <v>3.33</v>
+        <v>25.58</v>
       </c>
       <c r="I76" t="n">
-        <v>5.07</v>
+        <v>18.4</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E82" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F82" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G82" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H82" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I82" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E83" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F83" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G83" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H83" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I83" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C84" t="n">
         <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E84" t="n">
-        <v>23.3</v>
+        <v>10.988</v>
       </c>
       <c r="F84" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G84" t="n">
-        <v>69.90000000000001</v>
+        <v>32.96</v>
       </c>
       <c r="H84" t="n">
-        <v>4.23</v>
+        <v>1.8</v>
       </c>
       <c r="I84" t="n">
-        <v>6.44</v>
+        <v>5.78</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E85" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F85" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G85" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H85" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I85" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D86" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E86" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F86" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G86" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H86" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I86" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D92" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E92" t="n">
-        <v>40.575</v>
+        <v>6.797</v>
       </c>
       <c r="F92" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G92" t="n">
-        <v>162.3</v>
+        <v>61.17</v>
       </c>
       <c r="H92" t="n">
-        <v>23.28</v>
+        <v>5.02</v>
       </c>
       <c r="I92" t="n">
-        <v>16.75</v>
+        <v>8.94</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E93" t="n">
-        <v>10.876</v>
+        <v>103.88</v>
       </c>
       <c r="F93" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G93" t="n">
-        <v>32.63</v>
+        <v>103.88</v>
       </c>
       <c r="H93" t="n">
-        <v>1.47</v>
+        <v>3.79</v>
       </c>
       <c r="I93" t="n">
-        <v>4.72</v>
+        <v>3.79</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E94" t="n">
-        <v>103.88</v>
+        <v>23.025</v>
       </c>
       <c r="F94" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G94" t="n">
-        <v>103.88</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H94" t="n">
-        <v>3.79</v>
+        <v>3.4</v>
       </c>
       <c r="I94" t="n">
-        <v>3.79</v>
+        <v>5.18</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D95" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E95" t="n">
-        <v>23.025</v>
+        <v>40.575</v>
       </c>
       <c r="F95" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G95" t="n">
-        <v>69.06999999999999</v>
+        <v>162.3</v>
       </c>
       <c r="H95" t="n">
-        <v>3.4</v>
+        <v>23.28</v>
       </c>
       <c r="I95" t="n">
-        <v>5.18</v>
+        <v>16.75</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D96" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E96" t="n">
-        <v>6.797</v>
+        <v>10.876</v>
       </c>
       <c r="F96" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G96" t="n">
-        <v>61.17</v>
+        <v>32.63</v>
       </c>
       <c r="H96" t="n">
-        <v>5.02</v>
+        <v>1.47</v>
       </c>
       <c r="I96" t="n">
-        <v>8.94</v>
+        <v>4.72</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E102" t="n">
-        <v>40.97</v>
+        <v>23.29</v>
       </c>
       <c r="F102" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G102" t="n">
-        <v>163.88</v>
+        <v>69.87</v>
       </c>
       <c r="H102" t="n">
-        <v>24.86</v>
+        <v>4.2</v>
       </c>
       <c r="I102" t="n">
-        <v>17.88</v>
+        <v>6.4</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E103" t="n">
-        <v>103.46</v>
+        <v>10.556</v>
       </c>
       <c r="F103" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G103" t="n">
-        <v>103.46</v>
+        <v>31.67</v>
       </c>
       <c r="H103" t="n">
-        <v>3.37</v>
+        <v>0.51</v>
       </c>
       <c r="I103" t="n">
-        <v>3.37</v>
+        <v>1.64</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D104" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E104" t="n">
-        <v>10.556</v>
+        <v>6.804</v>
       </c>
       <c r="F104" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G104" t="n">
-        <v>31.67</v>
+        <v>61.24</v>
       </c>
       <c r="H104" t="n">
-        <v>0.51</v>
+        <v>5.09</v>
       </c>
       <c r="I104" t="n">
-        <v>1.64</v>
+        <v>9.07</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D105" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E105" t="n">
-        <v>23.29</v>
+        <v>40.97</v>
       </c>
       <c r="F105" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G105" t="n">
-        <v>69.87</v>
+        <v>163.88</v>
       </c>
       <c r="H105" t="n">
-        <v>4.2</v>
+        <v>24.86</v>
       </c>
       <c r="I105" t="n">
-        <v>6.4</v>
+        <v>17.88</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D106" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E106" t="n">
-        <v>6.804</v>
+        <v>103.46</v>
       </c>
       <c r="F106" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G106" t="n">
-        <v>61.24</v>
+        <v>103.46</v>
       </c>
       <c r="H106" t="n">
-        <v>5.09</v>
+        <v>3.37</v>
       </c>
       <c r="I106" t="n">
-        <v>9.07</v>
+        <v>3.37</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D107" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E107" t="n">
-        <v>40.5</v>
+        <v>103.14</v>
       </c>
       <c r="F107" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G107" t="n">
-        <v>162</v>
+        <v>103.14</v>
       </c>
       <c r="H107" t="n">
-        <v>22.98</v>
+        <v>3.05</v>
       </c>
       <c r="I107" t="n">
-        <v>16.53</v>
+        <v>3.05</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C108" t="n">
         <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E108" t="n">
-        <v>10.456</v>
+        <v>23.33</v>
       </c>
       <c r="F108" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G108" t="n">
-        <v>31.37</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H108" t="n">
-        <v>0.21</v>
+        <v>4.32</v>
       </c>
       <c r="I108" t="n">
-        <v>0.67</v>
+        <v>6.58</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D109" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E109" t="n">
-        <v>6.785</v>
+        <v>40.5</v>
       </c>
       <c r="F109" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G109" t="n">
-        <v>61.06</v>
+        <v>162</v>
       </c>
       <c r="H109" t="n">
-        <v>4.91</v>
+        <v>22.98</v>
       </c>
       <c r="I109" t="n">
-        <v>8.74</v>
+        <v>16.53</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C110" t="n">
         <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E110" t="n">
-        <v>23.33</v>
+        <v>10.456</v>
       </c>
       <c r="F110" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G110" t="n">
-        <v>69.98999999999999</v>
+        <v>31.37</v>
       </c>
       <c r="H110" t="n">
-        <v>4.32</v>
+        <v>0.21</v>
       </c>
       <c r="I110" t="n">
-        <v>6.58</v>
+        <v>0.67</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D111" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E111" t="n">
-        <v>103.14</v>
+        <v>6.785</v>
       </c>
       <c r="F111" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G111" t="n">
-        <v>103.14</v>
+        <v>61.06</v>
       </c>
       <c r="H111" t="n">
-        <v>3.05</v>
+        <v>4.91</v>
       </c>
       <c r="I111" t="n">
-        <v>3.05</v>
+        <v>8.74</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E112" t="n">
-        <v>40</v>
+        <v>10.568</v>
       </c>
       <c r="F112" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G112" t="n">
-        <v>160</v>
+        <v>31.7</v>
       </c>
       <c r="H112" t="n">
-        <v>20.98</v>
+        <v>0.54</v>
       </c>
       <c r="I112" t="n">
-        <v>15.09</v>
+        <v>1.73</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D113" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E113" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F113" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G113" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H113" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I113" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E114" t="n">
-        <v>6.797</v>
+        <v>103.56</v>
       </c>
       <c r="F114" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G114" t="n">
-        <v>61.17</v>
+        <v>103.56</v>
       </c>
       <c r="H114" t="n">
-        <v>5.02</v>
+        <v>3.47</v>
       </c>
       <c r="I114" t="n">
-        <v>8.94</v>
+        <v>3.47</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D115" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E115" t="n">
-        <v>10.568</v>
+        <v>40</v>
       </c>
       <c r="F115" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G115" t="n">
-        <v>31.7</v>
+        <v>160</v>
       </c>
       <c r="H115" t="n">
-        <v>0.54</v>
+        <v>20.98</v>
       </c>
       <c r="I115" t="n">
-        <v>1.73</v>
+        <v>15.09</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E116" t="n">
-        <v>103.56</v>
+        <v>23.025</v>
       </c>
       <c r="F116" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G116" t="n">
-        <v>103.56</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H116" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="I116" t="n">
-        <v>3.47</v>
+        <v>5.18</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C119" t="n">
         <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E119" t="n">
-        <v>10.756</v>
+        <v>23.145</v>
       </c>
       <c r="F119" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G119" t="n">
-        <v>32.27</v>
+        <v>69.44</v>
       </c>
       <c r="H119" t="n">
-        <v>1.11</v>
+        <v>3.77</v>
       </c>
       <c r="I119" t="n">
-        <v>3.56</v>
+        <v>5.74</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E120" t="n">
-        <v>23.145</v>
+        <v>105.96</v>
       </c>
       <c r="F120" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G120" t="n">
-        <v>69.44</v>
+        <v>105.96</v>
       </c>
       <c r="H120" t="n">
-        <v>3.77</v>
+        <v>5.87</v>
       </c>
       <c r="I120" t="n">
-        <v>5.74</v>
+        <v>5.86</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E121" t="n">
-        <v>105.96</v>
+        <v>10.756</v>
       </c>
       <c r="F121" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G121" t="n">
-        <v>105.96</v>
+        <v>32.27</v>
       </c>
       <c r="H121" t="n">
-        <v>5.87</v>
+        <v>1.11</v>
       </c>
       <c r="I121" t="n">
-        <v>5.86</v>
+        <v>3.56</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D127" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E127" t="n">
-        <v>103.46</v>
+        <v>39.36</v>
       </c>
       <c r="F127" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G127" t="n">
-        <v>103.46</v>
+        <v>157.44</v>
       </c>
       <c r="H127" t="n">
-        <v>3.37</v>
+        <v>18.42</v>
       </c>
       <c r="I127" t="n">
-        <v>3.37</v>
+        <v>13.25</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D128" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E128" t="n">
-        <v>23.17</v>
+        <v>6.868</v>
       </c>
       <c r="F128" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G128" t="n">
-        <v>69.51000000000001</v>
+        <v>61.81</v>
       </c>
       <c r="H128" t="n">
-        <v>3.84</v>
+        <v>5.66</v>
       </c>
       <c r="I128" t="n">
-        <v>5.85</v>
+        <v>10.08</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4796,29 +4796,29 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C129" t="n">
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E129" t="n">
-        <v>11.458</v>
+        <v>23.17</v>
       </c>
       <c r="F129" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G129" t="n">
-        <v>34.37</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H129" t="n">
-        <v>3.21</v>
+        <v>3.84</v>
       </c>
       <c r="I129" t="n">
-        <v>10.3</v>
+        <v>5.85</v>
       </c>
       <c r="J129" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D130" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E130" t="n">
-        <v>39.36</v>
+        <v>103.46</v>
       </c>
       <c r="F130" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G130" t="n">
-        <v>157.44</v>
+        <v>103.46</v>
       </c>
       <c r="H130" t="n">
-        <v>18.42</v>
+        <v>3.37</v>
       </c>
       <c r="I130" t="n">
-        <v>13.25</v>
+        <v>3.37</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E131" t="n">
-        <v>6.868</v>
+        <v>11.458</v>
       </c>
       <c r="F131" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G131" t="n">
-        <v>61.81</v>
+        <v>34.37</v>
       </c>
       <c r="H131" t="n">
-        <v>5.66</v>
+        <v>3.21</v>
       </c>
       <c r="I131" t="n">
-        <v>10.08</v>
+        <v>10.3</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D137" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E137" t="n">
-        <v>40.61</v>
+        <v>23.3</v>
       </c>
       <c r="F137" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G137" t="n">
-        <v>162.44</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H137" t="n">
-        <v>23.42</v>
+        <v>4.23</v>
       </c>
       <c r="I137" t="n">
-        <v>16.85</v>
+        <v>6.44</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D138" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E138" t="n">
-        <v>11.728</v>
+        <v>104.76</v>
       </c>
       <c r="F138" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G138" t="n">
-        <v>35.18</v>
+        <v>104.76</v>
       </c>
       <c r="H138" t="n">
-        <v>4.02</v>
+        <v>4.67</v>
       </c>
       <c r="I138" t="n">
-        <v>12.9</v>
+        <v>4.67</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D140" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E140" t="n">
-        <v>104.76</v>
+        <v>40.61</v>
       </c>
       <c r="F140" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G140" t="n">
-        <v>104.76</v>
+        <v>162.44</v>
       </c>
       <c r="H140" t="n">
-        <v>4.67</v>
+        <v>23.42</v>
       </c>
       <c r="I140" t="n">
-        <v>4.67</v>
+        <v>16.85</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C141" t="n">
         <v>3</v>
       </c>
       <c r="D141" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E141" t="n">
-        <v>23.3</v>
+        <v>11.728</v>
       </c>
       <c r="F141" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G141" t="n">
-        <v>69.90000000000001</v>
+        <v>35.18</v>
       </c>
       <c r="H141" t="n">
-        <v>4.23</v>
+        <v>4.02</v>
       </c>
       <c r="I141" t="n">
-        <v>6.44</v>
+        <v>12.9</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E147" t="n">
-        <v>101.7</v>
+        <v>11.162</v>
       </c>
       <c r="F147" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G147" t="n">
-        <v>101.7</v>
+        <v>33.49</v>
       </c>
       <c r="H147" t="n">
-        <v>1.61</v>
+        <v>2.33</v>
       </c>
       <c r="I147" t="n">
-        <v>1.61</v>
+        <v>7.48</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E148" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F148" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G148" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H148" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I148" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D149" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E149" t="n">
-        <v>22.755</v>
+        <v>6.826</v>
       </c>
       <c r="F149" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G149" t="n">
-        <v>68.27</v>
+        <v>61.43</v>
       </c>
       <c r="H149" t="n">
-        <v>2.6</v>
+        <v>5.28</v>
       </c>
       <c r="I149" t="n">
-        <v>3.96</v>
+        <v>9.4</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D150" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E150" t="n">
-        <v>6.826</v>
+        <v>101.7</v>
       </c>
       <c r="F150" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G150" t="n">
-        <v>61.43</v>
+        <v>101.7</v>
       </c>
       <c r="H150" t="n">
-        <v>5.28</v>
+        <v>1.61</v>
       </c>
       <c r="I150" t="n">
-        <v>9.4</v>
+        <v>1.61</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D151" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E151" t="n">
-        <v>11.162</v>
+        <v>38.955</v>
       </c>
       <c r="F151" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G151" t="n">
-        <v>33.49</v>
+        <v>155.82</v>
       </c>
       <c r="H151" t="n">
-        <v>2.33</v>
+        <v>16.8</v>
       </c>
       <c r="I151" t="n">
-        <v>7.48</v>
+        <v>12.08</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D157" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E157" t="n">
-        <v>104.5</v>
+        <v>40.015</v>
       </c>
       <c r="F157" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G157" t="n">
-        <v>104.5</v>
+        <v>160.06</v>
       </c>
       <c r="H157" t="n">
-        <v>4.41</v>
+        <v>21.04</v>
       </c>
       <c r="I157" t="n">
-        <v>4.41</v>
+        <v>15.13</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D158" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E158" t="n">
-        <v>23.08</v>
+        <v>6.913</v>
       </c>
       <c r="F158" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G158" t="n">
-        <v>69.23999999999999</v>
+        <v>62.22</v>
       </c>
       <c r="H158" t="n">
-        <v>3.57</v>
+        <v>6.07</v>
       </c>
       <c r="I158" t="n">
-        <v>5.44</v>
+        <v>10.81</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D159" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E159" t="n">
-        <v>6.913</v>
+        <v>10.92</v>
       </c>
       <c r="F159" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G159" t="n">
-        <v>62.22</v>
+        <v>32.76</v>
       </c>
       <c r="H159" t="n">
-        <v>6.07</v>
+        <v>1.6</v>
       </c>
       <c r="I159" t="n">
-        <v>10.81</v>
+        <v>5.13</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D160" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E160" t="n">
-        <v>10.92</v>
+        <v>104.5</v>
       </c>
       <c r="F160" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G160" t="n">
-        <v>32.76</v>
+        <v>104.5</v>
       </c>
       <c r="H160" t="n">
-        <v>1.6</v>
+        <v>4.41</v>
       </c>
       <c r="I160" t="n">
-        <v>5.13</v>
+        <v>4.41</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D161" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E161" t="n">
-        <v>40.015</v>
+        <v>23.08</v>
       </c>
       <c r="F161" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G161" t="n">
-        <v>160.06</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H161" t="n">
-        <v>21.04</v>
+        <v>3.57</v>
       </c>
       <c r="I161" t="n">
-        <v>15.13</v>
+        <v>5.44</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6079,6 +6079,176 @@
         <v>11.02</v>
       </c>
       <c r="J166" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>3</v>
+      </c>
+      <c r="D167" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E167" t="n">
+        <v>10.726</v>
+      </c>
+      <c r="F167" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G167" t="n">
+        <v>32.18</v>
+      </c>
+      <c r="H167" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="I167" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="J167" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>4</v>
+      </c>
+      <c r="D168" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E168" t="n">
+        <v>38.98</v>
+      </c>
+      <c r="F168" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G168" t="n">
+        <v>155.92</v>
+      </c>
+      <c r="H168" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I168" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="J168" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>3</v>
+      </c>
+      <c r="D169" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E169" t="n">
+        <v>22.92</v>
+      </c>
+      <c r="F169" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G169" t="n">
+        <v>68.76000000000001</v>
+      </c>
+      <c r="H169" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="I169" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="J169" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E170" t="n">
+        <v>103.98</v>
+      </c>
+      <c r="F170" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G170" t="n">
+        <v>103.98</v>
+      </c>
+      <c r="H170" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="I170" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="J170" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="1" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>9</v>
+      </c>
+      <c r="D171" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E171" t="n">
+        <v>6.911</v>
+      </c>
+      <c r="F171" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G171" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="H171" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="I171" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="J171" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 15/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J171"/>
+  <dimension ref="A1:J176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E22" t="n">
-        <v>6.799</v>
+        <v>21.669</v>
       </c>
       <c r="F22" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G22" t="n">
-        <v>61.19</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>5.04</v>
+        <v>-0.66</v>
       </c>
       <c r="I22" t="n">
-        <v>8.98</v>
+        <v>-1.01</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E23" t="n">
-        <v>105.78</v>
+        <v>10.536</v>
       </c>
       <c r="F23" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G23" t="n">
-        <v>105.78</v>
+        <v>31.61</v>
       </c>
       <c r="H23" t="n">
-        <v>5.69</v>
+        <v>0.45</v>
       </c>
       <c r="I23" t="n">
-        <v>5.68</v>
+        <v>1.44</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E24" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F24" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G24" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H24" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I24" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E25" t="n">
-        <v>10.536</v>
+        <v>105.78</v>
       </c>
       <c r="F25" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G25" t="n">
-        <v>31.61</v>
+        <v>105.78</v>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>5.69</v>
       </c>
       <c r="I25" t="n">
-        <v>1.44</v>
+        <v>5.68</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E26" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F26" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G26" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I26" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E32" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F32" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G32" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H32" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I32" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D33" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E33" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F33" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G33" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H33" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I33" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E35" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F35" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G35" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H35" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I35" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E36" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F36" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G36" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H36" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D43" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E43" t="n">
-        <v>100.06</v>
+        <v>6.629</v>
       </c>
       <c r="F43" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G43" t="n">
-        <v>100.06</v>
+        <v>59.66</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.03</v>
+        <v>3.51</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.03</v>
+        <v>6.25</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E44" t="n">
-        <v>6.629</v>
+        <v>38.497</v>
       </c>
       <c r="F44" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G44" t="n">
-        <v>59.66</v>
+        <v>153.99</v>
       </c>
       <c r="H44" t="n">
-        <v>3.51</v>
+        <v>14.97</v>
       </c>
       <c r="I44" t="n">
-        <v>6.25</v>
+        <v>10.77</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>38.497</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>153.99</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>14.97</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>10.77</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E46" t="n">
-        <v>22</v>
+        <v>100.06</v>
       </c>
       <c r="F46" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G46" t="n">
-        <v>66</v>
+        <v>100.06</v>
       </c>
       <c r="H46" t="n">
-        <v>0.33</v>
+        <v>-0.03</v>
       </c>
       <c r="I46" t="n">
-        <v>0.5</v>
+        <v>-0.03</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E52" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F52" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G52" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H52" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I52" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E53" t="n">
-        <v>38.544</v>
+        <v>100.34</v>
       </c>
       <c r="F53" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G53" t="n">
-        <v>154.18</v>
+        <v>100.34</v>
       </c>
       <c r="H53" t="n">
-        <v>15.16</v>
+        <v>0.25</v>
       </c>
       <c r="I53" t="n">
-        <v>10.9</v>
+        <v>0.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E54" t="n">
-        <v>21.703</v>
+        <v>6.629</v>
       </c>
       <c r="F54" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G54" t="n">
-        <v>65.11</v>
+        <v>59.66</v>
       </c>
       <c r="H54" t="n">
-        <v>-0.5600000000000001</v>
+        <v>3.51</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.85</v>
+        <v>6.25</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D55" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E55" t="n">
-        <v>6.629</v>
+        <v>38.544</v>
       </c>
       <c r="F55" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G55" t="n">
-        <v>59.66</v>
+        <v>154.18</v>
       </c>
       <c r="H55" t="n">
-        <v>3.51</v>
+        <v>15.16</v>
       </c>
       <c r="I55" t="n">
-        <v>6.25</v>
+        <v>10.9</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E56" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F56" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G56" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H56" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I56" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E62" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F62" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G62" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H62" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I62" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D63" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E63" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F63" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G63" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H63" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I63" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D64" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E64" t="n">
-        <v>6.817</v>
+        <v>41.064</v>
       </c>
       <c r="F64" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G64" t="n">
-        <v>61.35</v>
+        <v>164.26</v>
       </c>
       <c r="H64" t="n">
-        <v>5.2</v>
+        <v>25.24</v>
       </c>
       <c r="I64" t="n">
-        <v>9.26</v>
+        <v>18.16</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E65" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F65" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G65" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H65" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I65" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E66" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F66" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G66" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H66" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I66" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E72" t="n">
-        <v>23</v>
+        <v>104.22</v>
       </c>
       <c r="F72" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G72" t="n">
-        <v>69</v>
+        <v>104.22</v>
       </c>
       <c r="H72" t="n">
-        <v>3.33</v>
+        <v>4.13</v>
       </c>
       <c r="I72" t="n">
-        <v>5.07</v>
+        <v>4.13</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D74" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E74" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F74" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G74" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H74" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I74" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E75" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F75" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G75" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H75" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I75" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E76" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F76" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G76" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H76" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I76" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E77" t="n">
-        <v>6.836</v>
+        <v>42.25</v>
       </c>
       <c r="F77" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G77" t="n">
-        <v>61.52</v>
+        <v>169</v>
       </c>
       <c r="H77" t="n">
-        <v>5.37</v>
+        <v>29.98</v>
       </c>
       <c r="I77" t="n">
-        <v>9.56</v>
+        <v>21.57</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D78" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E78" t="n">
-        <v>10.958</v>
+        <v>6.836</v>
       </c>
       <c r="F78" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G78" t="n">
-        <v>32.87</v>
+        <v>61.52</v>
       </c>
       <c r="H78" t="n">
-        <v>1.71</v>
+        <v>5.37</v>
       </c>
       <c r="I78" t="n">
-        <v>5.49</v>
+        <v>9.56</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C79" t="n">
         <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E79" t="n">
-        <v>23.4</v>
+        <v>10.958</v>
       </c>
       <c r="F79" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G79" t="n">
-        <v>70.2</v>
+        <v>32.87</v>
       </c>
       <c r="H79" t="n">
-        <v>4.53</v>
+        <v>1.71</v>
       </c>
       <c r="I79" t="n">
-        <v>6.9</v>
+        <v>5.49</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E81" t="n">
-        <v>42.25</v>
+        <v>105.8</v>
       </c>
       <c r="F81" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G81" t="n">
-        <v>169</v>
+        <v>105.8</v>
       </c>
       <c r="H81" t="n">
-        <v>29.98</v>
+        <v>5.71</v>
       </c>
       <c r="I81" t="n">
-        <v>21.57</v>
+        <v>5.7</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E82" t="n">
-        <v>6.846</v>
+        <v>10.988</v>
       </c>
       <c r="F82" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G82" t="n">
-        <v>61.61</v>
+        <v>32.96</v>
       </c>
       <c r="H82" t="n">
-        <v>5.46</v>
+        <v>1.8</v>
       </c>
       <c r="I82" t="n">
-        <v>9.720000000000001</v>
+        <v>5.78</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D83" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E83" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F83" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G83" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H83" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I83" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D84" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E84" t="n">
-        <v>10.988</v>
+        <v>6.846</v>
       </c>
       <c r="F84" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G84" t="n">
-        <v>32.96</v>
+        <v>61.61</v>
       </c>
       <c r="H84" t="n">
-        <v>1.8</v>
+        <v>5.46</v>
       </c>
       <c r="I84" t="n">
-        <v>5.78</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E85" t="n">
-        <v>106.26</v>
+        <v>23.3</v>
       </c>
       <c r="F85" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G85" t="n">
-        <v>106.26</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H85" t="n">
-        <v>6.17</v>
+        <v>4.23</v>
       </c>
       <c r="I85" t="n">
-        <v>6.16</v>
+        <v>6.44</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E87" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F87" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G87" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H87" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I87" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E88" t="n">
-        <v>6.856</v>
+        <v>23.32</v>
       </c>
       <c r="F88" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G88" t="n">
-        <v>61.7</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>5.55</v>
+        <v>4.29</v>
       </c>
       <c r="I88" t="n">
-        <v>9.880000000000001</v>
+        <v>6.53</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E90" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F90" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G90" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H90" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I90" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E91" t="n">
-        <v>43.005</v>
+        <v>10.852</v>
       </c>
       <c r="F91" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G91" t="n">
-        <v>172.02</v>
+        <v>32.56</v>
       </c>
       <c r="H91" t="n">
-        <v>33</v>
+        <v>1.4</v>
       </c>
       <c r="I91" t="n">
-        <v>23.74</v>
+        <v>4.49</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D97" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E97" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F97" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G97" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H97" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I97" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E98" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F98" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G98" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H98" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I98" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C100" t="n">
         <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E100" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F100" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G100" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H100" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I100" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D101" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E101" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F101" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G101" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H101" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I101" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E107" t="n">
-        <v>103.14</v>
+        <v>10.456</v>
       </c>
       <c r="F107" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G107" t="n">
-        <v>103.14</v>
+        <v>31.37</v>
       </c>
       <c r="H107" t="n">
-        <v>3.05</v>
+        <v>0.21</v>
       </c>
       <c r="I107" t="n">
-        <v>3.05</v>
+        <v>0.67</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D108" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E108" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F108" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G108" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H108" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I108" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D109" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E109" t="n">
-        <v>40.5</v>
+        <v>6.785</v>
       </c>
       <c r="F109" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G109" t="n">
-        <v>162</v>
+        <v>61.06</v>
       </c>
       <c r="H109" t="n">
-        <v>22.98</v>
+        <v>4.91</v>
       </c>
       <c r="I109" t="n">
-        <v>16.53</v>
+        <v>8.74</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D110" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E110" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F110" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G110" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H110" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I110" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E111" t="n">
-        <v>6.785</v>
+        <v>23.33</v>
       </c>
       <c r="F111" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G111" t="n">
-        <v>61.06</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H111" t="n">
-        <v>4.91</v>
+        <v>4.32</v>
       </c>
       <c r="I111" t="n">
-        <v>8.74</v>
+        <v>6.58</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D117" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E117" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F117" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G117" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H117" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I117" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E118" t="n">
-        <v>6.861</v>
+        <v>23.145</v>
       </c>
       <c r="F118" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G118" t="n">
-        <v>61.75</v>
+        <v>69.44</v>
       </c>
       <c r="H118" t="n">
-        <v>5.6</v>
+        <v>3.77</v>
       </c>
       <c r="I118" t="n">
-        <v>9.970000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C119" t="n">
         <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E119" t="n">
-        <v>23.145</v>
+        <v>10.756</v>
       </c>
       <c r="F119" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G119" t="n">
-        <v>69.44</v>
+        <v>32.27</v>
       </c>
       <c r="H119" t="n">
-        <v>3.77</v>
+        <v>1.11</v>
       </c>
       <c r="I119" t="n">
-        <v>5.74</v>
+        <v>3.56</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>41</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>164</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>24.98</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>17.97</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D121" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E121" t="n">
-        <v>10.756</v>
+        <v>6.861</v>
       </c>
       <c r="F121" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G121" t="n">
-        <v>32.27</v>
+        <v>61.75</v>
       </c>
       <c r="H121" t="n">
-        <v>1.11</v>
+        <v>5.6</v>
       </c>
       <c r="I121" t="n">
-        <v>3.56</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D132" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E132" t="n">
-        <v>11.516</v>
+        <v>104.02</v>
       </c>
       <c r="F132" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G132" t="n">
-        <v>34.55</v>
+        <v>104.02</v>
       </c>
       <c r="H132" t="n">
-        <v>3.39</v>
+        <v>3.93</v>
       </c>
       <c r="I132" t="n">
-        <v>10.88</v>
+        <v>3.93</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E133" t="n">
-        <v>6.895</v>
+        <v>40.54</v>
       </c>
       <c r="F133" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G133" t="n">
-        <v>62.05</v>
+        <v>162.16</v>
       </c>
       <c r="H133" t="n">
-        <v>5.9</v>
+        <v>23.14</v>
       </c>
       <c r="I133" t="n">
-        <v>10.51</v>
+        <v>16.65</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D134" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E134" t="n">
-        <v>23.18</v>
+        <v>6.895</v>
       </c>
       <c r="F134" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G134" t="n">
-        <v>69.54000000000001</v>
+        <v>62.05</v>
       </c>
       <c r="H134" t="n">
-        <v>3.87</v>
+        <v>5.9</v>
       </c>
       <c r="I134" t="n">
-        <v>5.89</v>
+        <v>10.51</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E135" t="n">
-        <v>40.54</v>
+        <v>23.18</v>
       </c>
       <c r="F135" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G135" t="n">
-        <v>162.16</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H135" t="n">
-        <v>23.14</v>
+        <v>3.87</v>
       </c>
       <c r="I135" t="n">
-        <v>16.65</v>
+        <v>5.89</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E136" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F136" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G136" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H136" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I136" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D142" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E142" t="n">
-        <v>38.89</v>
+        <v>11.498</v>
       </c>
       <c r="F142" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G142" t="n">
-        <v>155.56</v>
+        <v>34.49</v>
       </c>
       <c r="H142" t="n">
-        <v>16.54</v>
+        <v>3.33</v>
       </c>
       <c r="I142" t="n">
-        <v>11.9</v>
+        <v>10.69</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D143" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E143" t="n">
-        <v>102.06</v>
+        <v>6.878</v>
       </c>
       <c r="F143" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G143" t="n">
-        <v>102.06</v>
+        <v>61.9</v>
       </c>
       <c r="H143" t="n">
-        <v>1.97</v>
+        <v>5.75</v>
       </c>
       <c r="I143" t="n">
-        <v>1.97</v>
+        <v>10.24</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E145" t="n">
-        <v>6.878</v>
+        <v>102.06</v>
       </c>
       <c r="F145" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G145" t="n">
-        <v>61.9</v>
+        <v>102.06</v>
       </c>
       <c r="H145" t="n">
-        <v>5.75</v>
+        <v>1.97</v>
       </c>
       <c r="I145" t="n">
-        <v>10.24</v>
+        <v>1.97</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E146" t="n">
-        <v>11.498</v>
+        <v>38.89</v>
       </c>
       <c r="F146" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G146" t="n">
-        <v>34.49</v>
+        <v>155.56</v>
       </c>
       <c r="H146" t="n">
-        <v>3.33</v>
+        <v>16.54</v>
       </c>
       <c r="I146" t="n">
-        <v>10.69</v>
+        <v>11.9</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D152" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E152" t="n">
-        <v>11.034</v>
+        <v>6.893</v>
       </c>
       <c r="F152" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G152" t="n">
-        <v>33.1</v>
+        <v>62.04</v>
       </c>
       <c r="H152" t="n">
-        <v>1.94</v>
+        <v>5.89</v>
       </c>
       <c r="I152" t="n">
-        <v>6.23</v>
+        <v>10.49</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D153" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E153" t="n">
-        <v>104.12</v>
+        <v>23.045</v>
       </c>
       <c r="F153" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G153" t="n">
-        <v>104.12</v>
+        <v>69.14</v>
       </c>
       <c r="H153" t="n">
-        <v>4.03</v>
+        <v>3.47</v>
       </c>
       <c r="I153" t="n">
-        <v>4.03</v>
+        <v>5.28</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5646,29 +5646,29 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D154" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E154" t="n">
-        <v>39.915</v>
+        <v>104.12</v>
       </c>
       <c r="F154" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G154" t="n">
-        <v>159.66</v>
+        <v>104.12</v>
       </c>
       <c r="H154" t="n">
-        <v>20.64</v>
+        <v>4.03</v>
       </c>
       <c r="I154" t="n">
-        <v>14.85</v>
+        <v>4.03</v>
       </c>
       <c r="J154" t="n">
         <v>7.91</v>
@@ -5680,29 +5680,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C155" t="n">
         <v>3</v>
       </c>
       <c r="D155" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E155" t="n">
-        <v>23.045</v>
+        <v>11.034</v>
       </c>
       <c r="F155" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G155" t="n">
-        <v>69.14</v>
+        <v>33.1</v>
       </c>
       <c r="H155" t="n">
-        <v>3.47</v>
+        <v>1.94</v>
       </c>
       <c r="I155" t="n">
-        <v>5.28</v>
+        <v>6.23</v>
       </c>
       <c r="J155" t="n">
         <v>7.91</v>
@@ -5714,29 +5714,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D156" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E156" t="n">
-        <v>6.893</v>
+        <v>39.915</v>
       </c>
       <c r="F156" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G156" t="n">
-        <v>62.04</v>
+        <v>159.66</v>
       </c>
       <c r="H156" t="n">
-        <v>5.89</v>
+        <v>20.64</v>
       </c>
       <c r="I156" t="n">
-        <v>10.49</v>
+        <v>14.85</v>
       </c>
       <c r="J156" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E162" t="n">
-        <v>103.84</v>
+        <v>10.748</v>
       </c>
       <c r="F162" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G162" t="n">
-        <v>103.84</v>
+        <v>32.24</v>
       </c>
       <c r="H162" t="n">
-        <v>3.75</v>
+        <v>1.08</v>
       </c>
       <c r="I162" t="n">
-        <v>3.75</v>
+        <v>3.47</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D163" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E163" t="n">
-        <v>10.748</v>
+        <v>103.84</v>
       </c>
       <c r="F163" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G163" t="n">
-        <v>32.24</v>
+        <v>103.84</v>
       </c>
       <c r="H163" t="n">
-        <v>1.08</v>
+        <v>3.75</v>
       </c>
       <c r="I163" t="n">
-        <v>3.47</v>
+        <v>3.75</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D167" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E167" t="n">
-        <v>10.726</v>
+        <v>103.98</v>
       </c>
       <c r="F167" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G167" t="n">
-        <v>32.18</v>
+        <v>103.98</v>
       </c>
       <c r="H167" t="n">
-        <v>1.02</v>
+        <v>3.89</v>
       </c>
       <c r="I167" t="n">
-        <v>3.27</v>
+        <v>3.89</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D168" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E168" t="n">
-        <v>38.98</v>
+        <v>22.92</v>
       </c>
       <c r="F168" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G168" t="n">
-        <v>155.92</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H168" t="n">
-        <v>16.9</v>
+        <v>3.09</v>
       </c>
       <c r="I168" t="n">
-        <v>12.16</v>
+        <v>4.71</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6156,29 +6156,29 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D169" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E169" t="n">
-        <v>22.92</v>
+        <v>6.911</v>
       </c>
       <c r="F169" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G169" t="n">
-        <v>68.76000000000001</v>
+        <v>62.2</v>
       </c>
       <c r="H169" t="n">
-        <v>3.09</v>
+        <v>6.05</v>
       </c>
       <c r="I169" t="n">
-        <v>4.71</v>
+        <v>10.77</v>
       </c>
       <c r="J169" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D170" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E170" t="n">
-        <v>103.98</v>
+        <v>10.726</v>
       </c>
       <c r="F170" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G170" t="n">
-        <v>103.98</v>
+        <v>32.18</v>
       </c>
       <c r="H170" t="n">
-        <v>3.89</v>
+        <v>1.02</v>
       </c>
       <c r="I170" t="n">
-        <v>3.89</v>
+        <v>3.27</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,31 +6224,201 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>4</v>
+      </c>
+      <c r="D171" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E171" t="n">
+        <v>38.98</v>
+      </c>
+      <c r="F171" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G171" t="n">
+        <v>155.92</v>
+      </c>
+      <c r="H171" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="I171" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="J171" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E172" t="n">
+        <v>103.22</v>
+      </c>
+      <c r="F172" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G172" t="n">
+        <v>103.22</v>
+      </c>
+      <c r="H172" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="I172" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="J172" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>3</v>
+      </c>
+      <c r="D173" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E173" t="n">
+        <v>10.712</v>
+      </c>
+      <c r="F173" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G173" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="H173" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I173" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="J173" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>4</v>
+      </c>
+      <c r="D174" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E174" t="n">
+        <v>38.74</v>
+      </c>
+      <c r="F174" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G174" t="n">
+        <v>154.96</v>
+      </c>
+      <c r="H174" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="I174" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="J174" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>3</v>
+      </c>
+      <c r="D175" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E175" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="F175" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G175" t="n">
+        <v>68.84999999999999</v>
+      </c>
+      <c r="H175" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I175" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="J175" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="1" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C171" t="n">
+      <c r="C176" t="n">
         <v>9</v>
       </c>
-      <c r="D171" t="n">
+      <c r="D176" t="n">
         <v>6.239</v>
       </c>
-      <c r="E171" t="n">
-        <v>6.911</v>
-      </c>
-      <c r="F171" t="n">
+      <c r="E176" t="n">
+        <v>6.926</v>
+      </c>
+      <c r="F176" t="n">
         <v>56.15</v>
       </c>
-      <c r="G171" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="H171" t="n">
-        <v>6.05</v>
-      </c>
-      <c r="I171" t="n">
-        <v>10.77</v>
-      </c>
-      <c r="J171" t="n">
+      <c r="G176" t="n">
+        <v>62.33</v>
+      </c>
+      <c r="H176" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="I176" t="n">
+        <v>11.01</v>
+      </c>
+      <c r="J176" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 16/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J176"/>
+  <dimension ref="A1:J181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E22" t="n">
-        <v>21.669</v>
+        <v>41.336</v>
       </c>
       <c r="F22" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G22" t="n">
-        <v>65.01000000000001</v>
+        <v>165.34</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.66</v>
+        <v>26.32</v>
       </c>
       <c r="I22" t="n">
-        <v>-1.01</v>
+        <v>18.93</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E23" t="n">
-        <v>10.536</v>
+        <v>105.78</v>
       </c>
       <c r="F23" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G23" t="n">
-        <v>31.61</v>
+        <v>105.78</v>
       </c>
       <c r="H23" t="n">
-        <v>0.45</v>
+        <v>5.69</v>
       </c>
       <c r="I23" t="n">
-        <v>1.44</v>
+        <v>5.68</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E24" t="n">
-        <v>6.799</v>
+        <v>21.669</v>
       </c>
       <c r="F24" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G24" t="n">
-        <v>61.19</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H24" t="n">
-        <v>5.04</v>
+        <v>-0.66</v>
       </c>
       <c r="I24" t="n">
-        <v>8.98</v>
+        <v>-1.01</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E25" t="n">
-        <v>105.78</v>
+        <v>10.536</v>
       </c>
       <c r="F25" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G25" t="n">
-        <v>105.78</v>
+        <v>31.61</v>
       </c>
       <c r="H25" t="n">
-        <v>5.69</v>
+        <v>0.45</v>
       </c>
       <c r="I25" t="n">
-        <v>5.68</v>
+        <v>1.44</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D26" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E26" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F26" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G26" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H26" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I26" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E32" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F32" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G32" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I32" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D33" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E33" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F33" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G33" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H33" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I33" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E35" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F35" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G35" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H35" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I35" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D36" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E36" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F36" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G36" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H36" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I36" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E42" t="n">
-        <v>22</v>
+        <v>100.06</v>
       </c>
       <c r="F42" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>100.06</v>
       </c>
       <c r="H42" t="n">
-        <v>0.33</v>
+        <v>-0.03</v>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>-0.03</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>6.629</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>59.66</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>3.51</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>6.25</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E44" t="n">
-        <v>38.497</v>
+        <v>10.61</v>
       </c>
       <c r="F44" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G44" t="n">
-        <v>153.99</v>
+        <v>31.83</v>
       </c>
       <c r="H44" t="n">
-        <v>14.97</v>
+        <v>0.67</v>
       </c>
       <c r="I44" t="n">
-        <v>10.77</v>
+        <v>2.15</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E45" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F45" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G45" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H45" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I45" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E46" t="n">
-        <v>100.06</v>
+        <v>6.629</v>
       </c>
       <c r="F46" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G46" t="n">
-        <v>100.06</v>
+        <v>59.66</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.03</v>
+        <v>3.51</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03</v>
+        <v>6.25</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D52" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E52" t="n">
-        <v>21.703</v>
+        <v>6.629</v>
       </c>
       <c r="F52" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G52" t="n">
-        <v>65.11</v>
+        <v>59.66</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.5600000000000001</v>
+        <v>3.51</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.85</v>
+        <v>6.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E53" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F53" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G53" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H53" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I53" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E54" t="n">
-        <v>6.629</v>
+        <v>38.544</v>
       </c>
       <c r="F54" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G54" t="n">
-        <v>59.66</v>
+        <v>154.18</v>
       </c>
       <c r="H54" t="n">
-        <v>3.51</v>
+        <v>15.16</v>
       </c>
       <c r="I54" t="n">
-        <v>6.25</v>
+        <v>10.9</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E55" t="n">
-        <v>38.544</v>
+        <v>100.34</v>
       </c>
       <c r="F55" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G55" t="n">
-        <v>154.18</v>
+        <v>100.34</v>
       </c>
       <c r="H55" t="n">
-        <v>15.16</v>
+        <v>0.25</v>
       </c>
       <c r="I55" t="n">
-        <v>10.9</v>
+        <v>0.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E56" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F56" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G56" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H56" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I56" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E62" t="n">
-        <v>10.712</v>
+        <v>105.5</v>
       </c>
       <c r="F62" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G62" t="n">
-        <v>32.14</v>
+        <v>105.5</v>
       </c>
       <c r="H62" t="n">
-        <v>0.98</v>
+        <v>5.41</v>
       </c>
       <c r="I62" t="n">
-        <v>3.15</v>
+        <v>5.41</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E63" t="n">
-        <v>6.817</v>
+        <v>41.064</v>
       </c>
       <c r="F63" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G63" t="n">
-        <v>61.35</v>
+        <v>164.26</v>
       </c>
       <c r="H63" t="n">
-        <v>5.2</v>
+        <v>25.24</v>
       </c>
       <c r="I63" t="n">
-        <v>9.26</v>
+        <v>18.16</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E64" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F64" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G64" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H64" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I64" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D66" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E66" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F66" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G66" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H66" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I66" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>23</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>69</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>3.33</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>5.07</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E73" t="n">
-        <v>41.15</v>
+        <v>10.892</v>
       </c>
       <c r="F73" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G73" t="n">
-        <v>164.6</v>
+        <v>32.68</v>
       </c>
       <c r="H73" t="n">
-        <v>25.58</v>
+        <v>1.52</v>
       </c>
       <c r="I73" t="n">
-        <v>18.4</v>
+        <v>4.88</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D74" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E74" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F74" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G74" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H74" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I74" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E75" t="n">
-        <v>23</v>
+        <v>104.22</v>
       </c>
       <c r="F75" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G75" t="n">
-        <v>69</v>
+        <v>104.22</v>
       </c>
       <c r="H75" t="n">
-        <v>3.33</v>
+        <v>4.13</v>
       </c>
       <c r="I75" t="n">
-        <v>5.07</v>
+        <v>4.13</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D76" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E76" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F76" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G76" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H76" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I76" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E77" t="n">
-        <v>42.25</v>
+        <v>105.8</v>
       </c>
       <c r="F77" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G77" t="n">
-        <v>169</v>
+        <v>105.8</v>
       </c>
       <c r="H77" t="n">
-        <v>29.98</v>
+        <v>5.71</v>
       </c>
       <c r="I77" t="n">
-        <v>21.57</v>
+        <v>5.7</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D78" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E78" t="n">
-        <v>6.836</v>
+        <v>42.25</v>
       </c>
       <c r="F78" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G78" t="n">
-        <v>61.52</v>
+        <v>169</v>
       </c>
       <c r="H78" t="n">
-        <v>5.37</v>
+        <v>29.98</v>
       </c>
       <c r="I78" t="n">
-        <v>9.56</v>
+        <v>21.57</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D79" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E79" t="n">
-        <v>10.958</v>
+        <v>6.836</v>
       </c>
       <c r="F79" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G79" t="n">
-        <v>32.87</v>
+        <v>61.52</v>
       </c>
       <c r="H79" t="n">
-        <v>1.71</v>
+        <v>5.37</v>
       </c>
       <c r="I79" t="n">
-        <v>5.49</v>
+        <v>9.56</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C80" t="n">
         <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E80" t="n">
-        <v>23.4</v>
+        <v>10.958</v>
       </c>
       <c r="F80" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G80" t="n">
-        <v>70.2</v>
+        <v>32.87</v>
       </c>
       <c r="H80" t="n">
-        <v>4.53</v>
+        <v>1.71</v>
       </c>
       <c r="I80" t="n">
-        <v>6.9</v>
+        <v>5.49</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E81" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F81" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G81" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H81" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I81" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E82" t="n">
-        <v>10.988</v>
+        <v>6.846</v>
       </c>
       <c r="F82" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G82" t="n">
-        <v>32.96</v>
+        <v>61.61</v>
       </c>
       <c r="H82" t="n">
-        <v>1.8</v>
+        <v>5.46</v>
       </c>
       <c r="I82" t="n">
-        <v>5.78</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E83" t="n">
-        <v>106.26</v>
+        <v>23.3</v>
       </c>
       <c r="F83" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G83" t="n">
-        <v>106.26</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H83" t="n">
-        <v>6.17</v>
+        <v>4.23</v>
       </c>
       <c r="I83" t="n">
-        <v>6.16</v>
+        <v>6.44</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E84" t="n">
-        <v>6.846</v>
+        <v>10.988</v>
       </c>
       <c r="F84" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G84" t="n">
-        <v>61.61</v>
+        <v>32.96</v>
       </c>
       <c r="H84" t="n">
-        <v>5.46</v>
+        <v>1.8</v>
       </c>
       <c r="I84" t="n">
-        <v>9.720000000000001</v>
+        <v>5.78</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E85" t="n">
-        <v>23.3</v>
+        <v>106.26</v>
       </c>
       <c r="F85" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G85" t="n">
-        <v>69.90000000000001</v>
+        <v>106.26</v>
       </c>
       <c r="H85" t="n">
-        <v>4.23</v>
+        <v>6.17</v>
       </c>
       <c r="I85" t="n">
-        <v>6.44</v>
+        <v>6.16</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D87" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E87" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F87" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G87" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H87" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I87" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E88" t="n">
-        <v>23.32</v>
+        <v>106.28</v>
       </c>
       <c r="F88" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G88" t="n">
-        <v>69.95999999999999</v>
+        <v>106.28</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>6.19</v>
       </c>
       <c r="I88" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E89" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F89" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G89" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H89" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I89" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D90" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E90" t="n">
-        <v>6.856</v>
+        <v>43.005</v>
       </c>
       <c r="F90" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G90" t="n">
-        <v>61.7</v>
+        <v>172.02</v>
       </c>
       <c r="H90" t="n">
-        <v>5.55</v>
+        <v>33</v>
       </c>
       <c r="I90" t="n">
-        <v>9.880000000000001</v>
+        <v>23.74</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C91" t="n">
         <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E91" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F91" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G91" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H91" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I91" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D97" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E97" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F97" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G97" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H97" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I97" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E98" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F98" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G98" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H98" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I98" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C100" t="n">
         <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E100" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F100" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G100" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H100" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I100" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D101" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E101" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F101" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G101" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H101" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I101" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D107" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E107" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F107" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G107" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H107" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I107" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D108" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E108" t="n">
-        <v>40.5</v>
+        <v>6.785</v>
       </c>
       <c r="F108" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G108" t="n">
-        <v>162</v>
+        <v>61.06</v>
       </c>
       <c r="H108" t="n">
-        <v>22.98</v>
+        <v>4.91</v>
       </c>
       <c r="I108" t="n">
-        <v>16.53</v>
+        <v>8.74</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D109" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E109" t="n">
-        <v>6.785</v>
+        <v>23.33</v>
       </c>
       <c r="F109" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G109" t="n">
-        <v>61.06</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H109" t="n">
-        <v>4.91</v>
+        <v>4.32</v>
       </c>
       <c r="I109" t="n">
-        <v>8.74</v>
+        <v>6.58</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E110" t="n">
-        <v>103.14</v>
+        <v>10.456</v>
       </c>
       <c r="F110" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G110" t="n">
-        <v>103.14</v>
+        <v>31.37</v>
       </c>
       <c r="H110" t="n">
-        <v>3.05</v>
+        <v>0.21</v>
       </c>
       <c r="I110" t="n">
-        <v>3.05</v>
+        <v>0.67</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D111" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E111" t="n">
-        <v>23.33</v>
+        <v>40.5</v>
       </c>
       <c r="F111" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G111" t="n">
-        <v>69.98999999999999</v>
+        <v>162</v>
       </c>
       <c r="H111" t="n">
-        <v>4.32</v>
+        <v>22.98</v>
       </c>
       <c r="I111" t="n">
-        <v>6.58</v>
+        <v>16.53</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E117" t="n">
-        <v>105.96</v>
+        <v>41</v>
       </c>
       <c r="F117" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G117" t="n">
-        <v>105.96</v>
+        <v>164</v>
       </c>
       <c r="H117" t="n">
-        <v>5.87</v>
+        <v>24.98</v>
       </c>
       <c r="I117" t="n">
-        <v>5.86</v>
+        <v>17.97</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C118" t="n">
         <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E118" t="n">
-        <v>23.145</v>
+        <v>10.756</v>
       </c>
       <c r="F118" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G118" t="n">
-        <v>69.44</v>
+        <v>32.27</v>
       </c>
       <c r="H118" t="n">
-        <v>3.77</v>
+        <v>1.11</v>
       </c>
       <c r="I118" t="n">
-        <v>5.74</v>
+        <v>3.56</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D119" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E119" t="n">
-        <v>10.756</v>
+        <v>6.861</v>
       </c>
       <c r="F119" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G119" t="n">
-        <v>32.27</v>
+        <v>61.75</v>
       </c>
       <c r="H119" t="n">
-        <v>1.11</v>
+        <v>5.6</v>
       </c>
       <c r="I119" t="n">
-        <v>3.56</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E120" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F120" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G120" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H120" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I120" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E121" t="n">
-        <v>6.861</v>
+        <v>23.145</v>
       </c>
       <c r="F121" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G121" t="n">
-        <v>61.75</v>
+        <v>69.44</v>
       </c>
       <c r="H121" t="n">
-        <v>5.6</v>
+        <v>3.77</v>
       </c>
       <c r="I121" t="n">
-        <v>9.970000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E132" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F132" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G132" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H132" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I132" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D133" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E133" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F133" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G133" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H133" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I133" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E134" t="n">
-        <v>6.895</v>
+        <v>23.18</v>
       </c>
       <c r="F134" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G134" t="n">
-        <v>62.05</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H134" t="n">
-        <v>5.9</v>
+        <v>3.87</v>
       </c>
       <c r="I134" t="n">
-        <v>10.51</v>
+        <v>5.89</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D135" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E135" t="n">
-        <v>23.18</v>
+        <v>104.02</v>
       </c>
       <c r="F135" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G135" t="n">
-        <v>69.54000000000001</v>
+        <v>104.02</v>
       </c>
       <c r="H135" t="n">
-        <v>3.87</v>
+        <v>3.93</v>
       </c>
       <c r="I135" t="n">
-        <v>5.89</v>
+        <v>3.93</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D136" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E136" t="n">
-        <v>11.516</v>
+        <v>40.54</v>
       </c>
       <c r="F136" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G136" t="n">
-        <v>34.55</v>
+        <v>162.16</v>
       </c>
       <c r="H136" t="n">
-        <v>3.39</v>
+        <v>23.14</v>
       </c>
       <c r="I136" t="n">
-        <v>10.88</v>
+        <v>16.65</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D142" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E142" t="n">
-        <v>11.498</v>
+        <v>102.06</v>
       </c>
       <c r="F142" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G142" t="n">
-        <v>34.49</v>
+        <v>102.06</v>
       </c>
       <c r="H142" t="n">
-        <v>3.33</v>
+        <v>1.97</v>
       </c>
       <c r="I142" t="n">
-        <v>10.69</v>
+        <v>1.97</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E143" t="n">
-        <v>6.878</v>
+        <v>23.135</v>
       </c>
       <c r="F143" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G143" t="n">
-        <v>61.9</v>
+        <v>69.41</v>
       </c>
       <c r="H143" t="n">
-        <v>5.75</v>
+        <v>3.74</v>
       </c>
       <c r="I143" t="n">
-        <v>10.24</v>
+        <v>5.7</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5306,29 +5306,29 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D144" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E144" t="n">
-        <v>23.135</v>
+        <v>38.89</v>
       </c>
       <c r="F144" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G144" t="n">
-        <v>69.41</v>
+        <v>155.56</v>
       </c>
       <c r="H144" t="n">
-        <v>3.74</v>
+        <v>16.54</v>
       </c>
       <c r="I144" t="n">
-        <v>5.7</v>
+        <v>11.9</v>
       </c>
       <c r="J144" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D145" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E145" t="n">
-        <v>102.06</v>
+        <v>11.498</v>
       </c>
       <c r="F145" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G145" t="n">
-        <v>102.06</v>
+        <v>34.49</v>
       </c>
       <c r="H145" t="n">
-        <v>1.97</v>
+        <v>3.33</v>
       </c>
       <c r="I145" t="n">
-        <v>1.97</v>
+        <v>10.69</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D146" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E146" t="n">
-        <v>38.89</v>
+        <v>6.878</v>
       </c>
       <c r="F146" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G146" t="n">
-        <v>155.56</v>
+        <v>61.9</v>
       </c>
       <c r="H146" t="n">
-        <v>16.54</v>
+        <v>5.75</v>
       </c>
       <c r="I146" t="n">
-        <v>11.9</v>
+        <v>10.24</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C147" t="n">
         <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E147" t="n">
-        <v>11.162</v>
+        <v>22.755</v>
       </c>
       <c r="F147" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G147" t="n">
-        <v>33.49</v>
+        <v>68.27</v>
       </c>
       <c r="H147" t="n">
-        <v>2.33</v>
+        <v>2.6</v>
       </c>
       <c r="I147" t="n">
-        <v>7.48</v>
+        <v>3.96</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D148" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E148" t="n">
-        <v>22.755</v>
+        <v>6.826</v>
       </c>
       <c r="F148" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G148" t="n">
-        <v>68.27</v>
+        <v>61.43</v>
       </c>
       <c r="H148" t="n">
-        <v>2.6</v>
+        <v>5.28</v>
       </c>
       <c r="I148" t="n">
-        <v>3.96</v>
+        <v>9.4</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D149" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E149" t="n">
-        <v>6.826</v>
+        <v>101.7</v>
       </c>
       <c r="F149" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G149" t="n">
-        <v>61.43</v>
+        <v>101.7</v>
       </c>
       <c r="H149" t="n">
-        <v>5.28</v>
+        <v>1.61</v>
       </c>
       <c r="I149" t="n">
-        <v>9.4</v>
+        <v>1.61</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D150" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E150" t="n">
-        <v>101.7</v>
+        <v>38.955</v>
       </c>
       <c r="F150" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G150" t="n">
-        <v>101.7</v>
+        <v>155.82</v>
       </c>
       <c r="H150" t="n">
-        <v>1.61</v>
+        <v>16.8</v>
       </c>
       <c r="I150" t="n">
-        <v>1.61</v>
+        <v>12.08</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E151" t="n">
-        <v>38.955</v>
+        <v>11.162</v>
       </c>
       <c r="F151" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G151" t="n">
-        <v>155.82</v>
+        <v>33.49</v>
       </c>
       <c r="H151" t="n">
-        <v>16.8</v>
+        <v>2.33</v>
       </c>
       <c r="I151" t="n">
-        <v>12.08</v>
+        <v>7.48</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D157" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E157" t="n">
-        <v>40.015</v>
+        <v>104.5</v>
       </c>
       <c r="F157" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G157" t="n">
-        <v>160.06</v>
+        <v>104.5</v>
       </c>
       <c r="H157" t="n">
-        <v>21.04</v>
+        <v>4.41</v>
       </c>
       <c r="I157" t="n">
-        <v>15.13</v>
+        <v>4.41</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E158" t="n">
-        <v>6.913</v>
+        <v>23.08</v>
       </c>
       <c r="F158" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G158" t="n">
-        <v>62.22</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H158" t="n">
-        <v>6.07</v>
+        <v>3.57</v>
       </c>
       <c r="I158" t="n">
-        <v>10.81</v>
+        <v>5.44</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D159" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E159" t="n">
-        <v>10.92</v>
+        <v>6.913</v>
       </c>
       <c r="F159" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G159" t="n">
-        <v>32.76</v>
+        <v>62.22</v>
       </c>
       <c r="H159" t="n">
-        <v>1.6</v>
+        <v>6.07</v>
       </c>
       <c r="I159" t="n">
-        <v>5.13</v>
+        <v>10.81</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D160" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E160" t="n">
-        <v>104.5</v>
+        <v>40.015</v>
       </c>
       <c r="F160" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G160" t="n">
-        <v>104.5</v>
+        <v>160.06</v>
       </c>
       <c r="H160" t="n">
-        <v>4.41</v>
+        <v>21.04</v>
       </c>
       <c r="I160" t="n">
-        <v>4.41</v>
+        <v>15.13</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C161" t="n">
         <v>3</v>
       </c>
       <c r="D161" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E161" t="n">
-        <v>23.08</v>
+        <v>10.92</v>
       </c>
       <c r="F161" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G161" t="n">
-        <v>69.23999999999999</v>
+        <v>32.76</v>
       </c>
       <c r="H161" t="n">
-        <v>3.57</v>
+        <v>1.6</v>
       </c>
       <c r="I161" t="n">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E167" t="n">
-        <v>103.98</v>
+        <v>38.98</v>
       </c>
       <c r="F167" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G167" t="n">
-        <v>103.98</v>
+        <v>155.92</v>
       </c>
       <c r="H167" t="n">
-        <v>3.89</v>
+        <v>16.9</v>
       </c>
       <c r="I167" t="n">
-        <v>3.89</v>
+        <v>12.16</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D168" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E168" t="n">
-        <v>22.92</v>
+        <v>6.911</v>
       </c>
       <c r="F168" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G168" t="n">
-        <v>68.76000000000001</v>
+        <v>62.2</v>
       </c>
       <c r="H168" t="n">
-        <v>3.09</v>
+        <v>6.05</v>
       </c>
       <c r="I168" t="n">
-        <v>4.71</v>
+        <v>10.77</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6156,29 +6156,29 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D169" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E169" t="n">
-        <v>6.911</v>
+        <v>10.726</v>
       </c>
       <c r="F169" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G169" t="n">
-        <v>62.2</v>
+        <v>32.18</v>
       </c>
       <c r="H169" t="n">
-        <v>6.05</v>
+        <v>1.02</v>
       </c>
       <c r="I169" t="n">
-        <v>10.77</v>
+        <v>3.27</v>
       </c>
       <c r="J169" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D170" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E170" t="n">
-        <v>10.726</v>
+        <v>103.98</v>
       </c>
       <c r="F170" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G170" t="n">
-        <v>32.18</v>
+        <v>103.98</v>
       </c>
       <c r="H170" t="n">
-        <v>1.02</v>
+        <v>3.89</v>
       </c>
       <c r="I170" t="n">
-        <v>3.27</v>
+        <v>3.89</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,29 +6224,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D171" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E171" t="n">
-        <v>38.98</v>
+        <v>22.92</v>
       </c>
       <c r="F171" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G171" t="n">
-        <v>155.92</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H171" t="n">
-        <v>16.9</v>
+        <v>3.09</v>
       </c>
       <c r="I171" t="n">
-        <v>12.16</v>
+        <v>4.71</v>
       </c>
       <c r="J171" t="n">
         <v>7.91</v>
@@ -6419,6 +6419,176 @@
         <v>11.01</v>
       </c>
       <c r="J176" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>3</v>
+      </c>
+      <c r="D177" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E177" t="n">
+        <v>10.642</v>
+      </c>
+      <c r="F177" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G177" t="n">
+        <v>31.93</v>
+      </c>
+      <c r="H177" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I177" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="J177" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>4</v>
+      </c>
+      <c r="D178" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E178" t="n">
+        <v>38.245</v>
+      </c>
+      <c r="F178" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G178" t="n">
+        <v>152.98</v>
+      </c>
+      <c r="H178" t="n">
+        <v>13.96</v>
+      </c>
+      <c r="I178" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="J178" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>3</v>
+      </c>
+      <c r="D179" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E179" t="n">
+        <v>22.95</v>
+      </c>
+      <c r="F179" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G179" t="n">
+        <v>68.84999999999999</v>
+      </c>
+      <c r="H179" t="n">
+        <v>3.18</v>
+      </c>
+      <c r="I179" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="J179" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>1</v>
+      </c>
+      <c r="D180" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E180" t="n">
+        <v>102.54</v>
+      </c>
+      <c r="F180" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G180" t="n">
+        <v>102.54</v>
+      </c>
+      <c r="H180" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="I180" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="J180" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="1" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>9</v>
+      </c>
+      <c r="D181" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E181" t="n">
+        <v>6.922</v>
+      </c>
+      <c r="F181" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G181" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="H181" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="I181" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="J181" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 17/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E22" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F22" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G22" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H22" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I22" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E23" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F23" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G23" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I23" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C24" t="n">
         <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E24" t="n">
-        <v>21.669</v>
+        <v>10.536</v>
       </c>
       <c r="F24" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G24" t="n">
-        <v>65.01000000000001</v>
+        <v>31.61</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.66</v>
+        <v>0.45</v>
       </c>
       <c r="I24" t="n">
-        <v>-1.01</v>
+        <v>1.44</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E25" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F25" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G25" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H25" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I25" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E26" t="n">
-        <v>6.799</v>
+        <v>105.78</v>
       </c>
       <c r="F26" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G26" t="n">
-        <v>61.19</v>
+        <v>105.78</v>
       </c>
       <c r="H26" t="n">
-        <v>5.04</v>
+        <v>5.69</v>
       </c>
       <c r="I26" t="n">
-        <v>8.98</v>
+        <v>5.68</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E32" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F32" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G32" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H32" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I32" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E33" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F33" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G33" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H33" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I33" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E34" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F34" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G34" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H34" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I34" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>3</v>
       </c>
       <c r="D35" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E35" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F35" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G35" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H35" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I35" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E36" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F36" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G36" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H36" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I36" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E42" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F42" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G42" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E44" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F44" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G44" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H44" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I44" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D47" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E47" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F47" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G47" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E48" t="n">
-        <v>38.312</v>
+        <v>10.562</v>
       </c>
       <c r="F48" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G48" t="n">
-        <v>153.25</v>
+        <v>31.69</v>
       </c>
       <c r="H48" t="n">
-        <v>14.23</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="n">
-        <v>10.24</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E49" t="n">
-        <v>99.83</v>
+        <v>21.778</v>
       </c>
       <c r="F49" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G49" t="n">
-        <v>99.83</v>
+        <v>65.33</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.26</v>
+        <v>-0.34</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.26</v>
+        <v>-0.52</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E50" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F50" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G50" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I50" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E51" t="n">
-        <v>6.622</v>
+        <v>99.83</v>
       </c>
       <c r="F51" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G51" t="n">
-        <v>59.6</v>
+        <v>99.83</v>
       </c>
       <c r="H51" t="n">
-        <v>3.45</v>
+        <v>-0.26</v>
       </c>
       <c r="I51" t="n">
-        <v>6.14</v>
+        <v>-0.26</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E60" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F60" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G60" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H60" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I60" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E67" t="n">
-        <v>6.807</v>
+        <v>22.797</v>
       </c>
       <c r="F67" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G67" t="n">
-        <v>61.26</v>
+        <v>68.39</v>
       </c>
       <c r="H67" t="n">
-        <v>5.11</v>
+        <v>2.72</v>
       </c>
       <c r="I67" t="n">
-        <v>9.1</v>
+        <v>4.14</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E68" t="n">
-        <v>40.567</v>
+        <v>104.58</v>
       </c>
       <c r="F68" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G68" t="n">
-        <v>162.27</v>
+        <v>104.58</v>
       </c>
       <c r="H68" t="n">
-        <v>23.25</v>
+        <v>4.49</v>
       </c>
       <c r="I68" t="n">
-        <v>16.72</v>
+        <v>4.49</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E69" t="n">
-        <v>104.58</v>
+        <v>10.796</v>
       </c>
       <c r="F69" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G69" t="n">
-        <v>104.58</v>
+        <v>32.39</v>
       </c>
       <c r="H69" t="n">
-        <v>4.49</v>
+        <v>1.23</v>
       </c>
       <c r="I69" t="n">
-        <v>4.49</v>
+        <v>3.95</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E70" t="n">
-        <v>22.797</v>
+        <v>6.807</v>
       </c>
       <c r="F70" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G70" t="n">
-        <v>68.39</v>
+        <v>61.26</v>
       </c>
       <c r="H70" t="n">
-        <v>2.72</v>
+        <v>5.11</v>
       </c>
       <c r="I70" t="n">
-        <v>4.14</v>
+        <v>9.1</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D71" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E71" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F71" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G71" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H71" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I71" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D77" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E77" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F77" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G77" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H77" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I77" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D78" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E78" t="n">
-        <v>42.25</v>
+        <v>6.836</v>
       </c>
       <c r="F78" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G78" t="n">
-        <v>169</v>
+        <v>61.52</v>
       </c>
       <c r="H78" t="n">
-        <v>29.98</v>
+        <v>5.37</v>
       </c>
       <c r="I78" t="n">
-        <v>21.57</v>
+        <v>9.56</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E79" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F79" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G79" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H79" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I79" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E80" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F80" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G80" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H80" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I80" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D81" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E81" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F81" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G81" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H81" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I81" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E92" t="n">
-        <v>6.797</v>
+        <v>10.876</v>
       </c>
       <c r="F92" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G92" t="n">
-        <v>61.17</v>
+        <v>32.63</v>
       </c>
       <c r="H92" t="n">
-        <v>5.02</v>
+        <v>1.47</v>
       </c>
       <c r="I92" t="n">
-        <v>8.94</v>
+        <v>4.72</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D93" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E93" t="n">
-        <v>103.88</v>
+        <v>40.575</v>
       </c>
       <c r="F93" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G93" t="n">
-        <v>103.88</v>
+        <v>162.3</v>
       </c>
       <c r="H93" t="n">
-        <v>3.79</v>
+        <v>23.28</v>
       </c>
       <c r="I93" t="n">
-        <v>3.79</v>
+        <v>16.75</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E95" t="n">
-        <v>40.575</v>
+        <v>103.88</v>
       </c>
       <c r="F95" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G95" t="n">
-        <v>162.3</v>
+        <v>103.88</v>
       </c>
       <c r="H95" t="n">
-        <v>23.28</v>
+        <v>3.79</v>
       </c>
       <c r="I95" t="n">
-        <v>16.75</v>
+        <v>3.79</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D96" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E96" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F96" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G96" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H96" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I96" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D102" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E102" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F102" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G102" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H102" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I102" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D103" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E103" t="n">
-        <v>10.556</v>
+        <v>40.97</v>
       </c>
       <c r="F103" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G103" t="n">
-        <v>31.67</v>
+        <v>163.88</v>
       </c>
       <c r="H103" t="n">
-        <v>0.51</v>
+        <v>24.86</v>
       </c>
       <c r="I103" t="n">
-        <v>1.64</v>
+        <v>17.88</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E105" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F105" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G105" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H105" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I105" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D106" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E106" t="n">
-        <v>103.46</v>
+        <v>23.29</v>
       </c>
       <c r="F106" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G106" t="n">
-        <v>103.46</v>
+        <v>69.87</v>
       </c>
       <c r="H106" t="n">
-        <v>3.37</v>
+        <v>4.2</v>
       </c>
       <c r="I106" t="n">
-        <v>3.37</v>
+        <v>6.4</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E112" t="n">
-        <v>10.568</v>
+        <v>40</v>
       </c>
       <c r="F112" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G112" t="n">
-        <v>31.7</v>
+        <v>160</v>
       </c>
       <c r="H112" t="n">
-        <v>0.54</v>
+        <v>20.98</v>
       </c>
       <c r="I112" t="n">
-        <v>1.73</v>
+        <v>15.09</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D113" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E113" t="n">
-        <v>6.797</v>
+        <v>103.56</v>
       </c>
       <c r="F113" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G113" t="n">
-        <v>61.17</v>
+        <v>103.56</v>
       </c>
       <c r="H113" t="n">
-        <v>5.02</v>
+        <v>3.47</v>
       </c>
       <c r="I113" t="n">
-        <v>8.94</v>
+        <v>3.47</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E114" t="n">
-        <v>103.56</v>
+        <v>23.025</v>
       </c>
       <c r="F114" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G114" t="n">
-        <v>103.56</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H114" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="I114" t="n">
-        <v>3.47</v>
+        <v>5.18</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E115" t="n">
-        <v>40</v>
+        <v>10.568</v>
       </c>
       <c r="F115" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G115" t="n">
-        <v>160</v>
+        <v>31.7</v>
       </c>
       <c r="H115" t="n">
-        <v>20.98</v>
+        <v>0.54</v>
       </c>
       <c r="I115" t="n">
-        <v>15.09</v>
+        <v>1.73</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D116" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E116" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F116" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G116" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H116" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I116" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D122" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E122" t="n">
-        <v>23.165</v>
+        <v>6.901</v>
       </c>
       <c r="F122" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G122" t="n">
-        <v>69.5</v>
+        <v>62.11</v>
       </c>
       <c r="H122" t="n">
-        <v>3.83</v>
+        <v>5.96</v>
       </c>
       <c r="I122" t="n">
-        <v>5.83</v>
+        <v>10.61</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D123" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E123" t="n">
-        <v>106</v>
+        <v>40.395</v>
       </c>
       <c r="F123" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G123" t="n">
-        <v>106</v>
+        <v>161.58</v>
       </c>
       <c r="H123" t="n">
-        <v>5.91</v>
+        <v>22.56</v>
       </c>
       <c r="I123" t="n">
-        <v>5.9</v>
+        <v>16.23</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E124" t="n">
-        <v>40.395</v>
+        <v>11.038</v>
       </c>
       <c r="F124" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G124" t="n">
-        <v>161.58</v>
+        <v>33.11</v>
       </c>
       <c r="H124" t="n">
-        <v>22.56</v>
+        <v>1.95</v>
       </c>
       <c r="I124" t="n">
-        <v>16.23</v>
+        <v>6.26</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D125" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E125" t="n">
-        <v>6.901</v>
+        <v>23.165</v>
       </c>
       <c r="F125" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G125" t="n">
-        <v>62.11</v>
+        <v>69.5</v>
       </c>
       <c r="H125" t="n">
-        <v>5.96</v>
+        <v>3.83</v>
       </c>
       <c r="I125" t="n">
-        <v>10.61</v>
+        <v>5.83</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D126" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E126" t="n">
-        <v>11.038</v>
+        <v>106</v>
       </c>
       <c r="F126" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G126" t="n">
-        <v>33.11</v>
+        <v>106</v>
       </c>
       <c r="H126" t="n">
-        <v>1.95</v>
+        <v>5.91</v>
       </c>
       <c r="I126" t="n">
-        <v>6.26</v>
+        <v>5.9</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C137" t="n">
         <v>3</v>
       </c>
       <c r="D137" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E137" t="n">
-        <v>23.3</v>
+        <v>11.728</v>
       </c>
       <c r="F137" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G137" t="n">
-        <v>69.90000000000001</v>
+        <v>35.18</v>
       </c>
       <c r="H137" t="n">
-        <v>4.23</v>
+        <v>4.02</v>
       </c>
       <c r="I137" t="n">
-        <v>6.44</v>
+        <v>12.9</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D138" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E138" t="n">
-        <v>104.76</v>
+        <v>6.927</v>
       </c>
       <c r="F138" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G138" t="n">
-        <v>104.76</v>
+        <v>62.34</v>
       </c>
       <c r="H138" t="n">
-        <v>4.67</v>
+        <v>6.19</v>
       </c>
       <c r="I138" t="n">
-        <v>4.67</v>
+        <v>11.02</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D139" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E139" t="n">
-        <v>6.927</v>
+        <v>40.61</v>
       </c>
       <c r="F139" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G139" t="n">
-        <v>62.34</v>
+        <v>162.44</v>
       </c>
       <c r="H139" t="n">
-        <v>6.19</v>
+        <v>23.42</v>
       </c>
       <c r="I139" t="n">
-        <v>11.02</v>
+        <v>16.85</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D140" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E140" t="n">
-        <v>40.61</v>
+        <v>104.76</v>
       </c>
       <c r="F140" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G140" t="n">
-        <v>162.44</v>
+        <v>104.76</v>
       </c>
       <c r="H140" t="n">
-        <v>23.42</v>
+        <v>4.67</v>
       </c>
       <c r="I140" t="n">
-        <v>16.85</v>
+        <v>4.67</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C141" t="n">
         <v>3</v>
       </c>
       <c r="D141" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E141" t="n">
-        <v>11.728</v>
+        <v>23.3</v>
       </c>
       <c r="F141" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G141" t="n">
-        <v>35.18</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H141" t="n">
-        <v>4.02</v>
+        <v>4.23</v>
       </c>
       <c r="I141" t="n">
-        <v>12.9</v>
+        <v>6.44</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D147" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E147" t="n">
-        <v>22.755</v>
+        <v>38.955</v>
       </c>
       <c r="F147" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G147" t="n">
-        <v>68.27</v>
+        <v>155.82</v>
       </c>
       <c r="H147" t="n">
-        <v>2.6</v>
+        <v>16.8</v>
       </c>
       <c r="I147" t="n">
-        <v>3.96</v>
+        <v>12.08</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D148" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E148" t="n">
-        <v>6.826</v>
+        <v>101.7</v>
       </c>
       <c r="F148" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G148" t="n">
-        <v>61.43</v>
+        <v>101.7</v>
       </c>
       <c r="H148" t="n">
-        <v>5.28</v>
+        <v>1.61</v>
       </c>
       <c r="I148" t="n">
-        <v>9.4</v>
+        <v>1.61</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E149" t="n">
-        <v>101.7</v>
+        <v>11.162</v>
       </c>
       <c r="F149" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G149" t="n">
-        <v>101.7</v>
+        <v>33.49</v>
       </c>
       <c r="H149" t="n">
-        <v>1.61</v>
+        <v>2.33</v>
       </c>
       <c r="I149" t="n">
-        <v>1.61</v>
+        <v>7.48</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D150" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E150" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F150" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G150" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H150" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I150" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D151" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E151" t="n">
-        <v>11.162</v>
+        <v>6.826</v>
       </c>
       <c r="F151" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G151" t="n">
-        <v>33.49</v>
+        <v>61.43</v>
       </c>
       <c r="H151" t="n">
-        <v>2.33</v>
+        <v>5.28</v>
       </c>
       <c r="I151" t="n">
-        <v>7.48</v>
+        <v>9.4</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C162" t="n">
         <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E162" t="n">
-        <v>10.748</v>
+        <v>23.01</v>
       </c>
       <c r="F162" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G162" t="n">
-        <v>32.24</v>
+        <v>69.03</v>
       </c>
       <c r="H162" t="n">
-        <v>1.08</v>
+        <v>3.36</v>
       </c>
       <c r="I162" t="n">
-        <v>3.47</v>
+        <v>5.12</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D163" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E163" t="n">
-        <v>103.84</v>
+        <v>6.927</v>
       </c>
       <c r="F163" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G163" t="n">
-        <v>103.84</v>
+        <v>62.34</v>
       </c>
       <c r="H163" t="n">
-        <v>3.75</v>
+        <v>6.19</v>
       </c>
       <c r="I163" t="n">
-        <v>3.75</v>
+        <v>11.02</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -5986,29 +5986,29 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D164" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E164" t="n">
-        <v>38.845</v>
+        <v>103.84</v>
       </c>
       <c r="F164" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G164" t="n">
-        <v>155.38</v>
+        <v>103.84</v>
       </c>
       <c r="H164" t="n">
-        <v>16.36</v>
+        <v>3.75</v>
       </c>
       <c r="I164" t="n">
-        <v>11.77</v>
+        <v>3.75</v>
       </c>
       <c r="J164" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C165" t="n">
         <v>3</v>
       </c>
       <c r="D165" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E165" t="n">
-        <v>23.01</v>
+        <v>10.748</v>
       </c>
       <c r="F165" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G165" t="n">
-        <v>69.03</v>
+        <v>32.24</v>
       </c>
       <c r="H165" t="n">
-        <v>3.36</v>
+        <v>1.08</v>
       </c>
       <c r="I165" t="n">
-        <v>5.12</v>
+        <v>3.47</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D166" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E166" t="n">
-        <v>6.927</v>
+        <v>38.845</v>
       </c>
       <c r="F166" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G166" t="n">
-        <v>62.34</v>
+        <v>155.38</v>
       </c>
       <c r="H166" t="n">
-        <v>6.19</v>
+        <v>16.36</v>
       </c>
       <c r="I166" t="n">
-        <v>11.02</v>
+        <v>11.77</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6258,29 +6258,29 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D172" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E172" t="n">
-        <v>103.22</v>
+        <v>6.926</v>
       </c>
       <c r="F172" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G172" t="n">
-        <v>103.22</v>
+        <v>62.33</v>
       </c>
       <c r="H172" t="n">
-        <v>3.13</v>
+        <v>6.18</v>
       </c>
       <c r="I172" t="n">
-        <v>3.13</v>
+        <v>11.01</v>
       </c>
       <c r="J172" t="n">
         <v>7.91</v>
@@ -6292,29 +6292,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C173" t="n">
         <v>3</v>
       </c>
       <c r="D173" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E173" t="n">
-        <v>10.712</v>
+        <v>22.95</v>
       </c>
       <c r="F173" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G173" t="n">
-        <v>32.14</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H173" t="n">
-        <v>0.98</v>
+        <v>3.18</v>
       </c>
       <c r="I173" t="n">
-        <v>3.15</v>
+        <v>4.84</v>
       </c>
       <c r="J173" t="n">
         <v>7.91</v>
@@ -6326,29 +6326,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D174" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E174" t="n">
-        <v>38.74</v>
+        <v>10.712</v>
       </c>
       <c r="F174" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G174" t="n">
-        <v>154.96</v>
+        <v>32.14</v>
       </c>
       <c r="H174" t="n">
-        <v>15.94</v>
+        <v>0.98</v>
       </c>
       <c r="I174" t="n">
-        <v>11.47</v>
+        <v>3.15</v>
       </c>
       <c r="J174" t="n">
         <v>7.91</v>
@@ -6360,29 +6360,29 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D175" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E175" t="n">
-        <v>22.95</v>
+        <v>103.22</v>
       </c>
       <c r="F175" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G175" t="n">
-        <v>68.84999999999999</v>
+        <v>103.22</v>
       </c>
       <c r="H175" t="n">
-        <v>3.18</v>
+        <v>3.13</v>
       </c>
       <c r="I175" t="n">
-        <v>4.84</v>
+        <v>3.13</v>
       </c>
       <c r="J175" t="n">
         <v>7.91</v>
@@ -6394,29 +6394,29 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E176" t="n">
-        <v>6.926</v>
+        <v>38.74</v>
       </c>
       <c r="F176" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G176" t="n">
-        <v>62.33</v>
+        <v>154.96</v>
       </c>
       <c r="H176" t="n">
-        <v>6.18</v>
+        <v>15.94</v>
       </c>
       <c r="I176" t="n">
-        <v>11.01</v>
+        <v>11.47</v>
       </c>
       <c r="J176" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D177" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E177" t="n">
-        <v>10.642</v>
+        <v>6.922</v>
       </c>
       <c r="F177" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G177" t="n">
-        <v>31.93</v>
+        <v>62.3</v>
       </c>
       <c r="H177" t="n">
-        <v>0.77</v>
+        <v>6.15</v>
       </c>
       <c r="I177" t="n">
-        <v>2.47</v>
+        <v>10.95</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D178" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E178" t="n">
-        <v>38.245</v>
+        <v>10.642</v>
       </c>
       <c r="F178" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G178" t="n">
-        <v>152.98</v>
+        <v>31.93</v>
       </c>
       <c r="H178" t="n">
-        <v>13.96</v>
+        <v>0.77</v>
       </c>
       <c r="I178" t="n">
-        <v>10.04</v>
+        <v>2.47</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D179" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E179" t="n">
-        <v>22.95</v>
+        <v>38.245</v>
       </c>
       <c r="F179" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G179" t="n">
-        <v>68.84999999999999</v>
+        <v>152.98</v>
       </c>
       <c r="H179" t="n">
-        <v>3.18</v>
+        <v>13.96</v>
       </c>
       <c r="I179" t="n">
-        <v>4.84</v>
+        <v>10.04</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D180" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E180" t="n">
-        <v>102.54</v>
+        <v>22.95</v>
       </c>
       <c r="F180" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G180" t="n">
-        <v>102.54</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H180" t="n">
-        <v>2.45</v>
+        <v>3.18</v>
       </c>
       <c r="I180" t="n">
-        <v>2.45</v>
+        <v>4.84</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,31 +6564,201 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E181" t="n">
+        <v>102.54</v>
+      </c>
+      <c r="F181" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G181" t="n">
+        <v>102.54</v>
+      </c>
+      <c r="H181" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="I181" t="n">
+        <v>2.45</v>
+      </c>
+      <c r="J181" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E182" t="n">
+        <v>100.14</v>
+      </c>
+      <c r="F182" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G182" t="n">
+        <v>100.14</v>
+      </c>
+      <c r="H182" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I182" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J182" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>3</v>
+      </c>
+      <c r="D183" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E183" t="n">
+        <v>10.776</v>
+      </c>
+      <c r="F183" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G183" t="n">
+        <v>32.33</v>
+      </c>
+      <c r="H183" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="I183" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="J183" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>4</v>
+      </c>
+      <c r="D184" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E184" t="n">
+        <v>37.235</v>
+      </c>
+      <c r="F184" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G184" t="n">
+        <v>148.94</v>
+      </c>
+      <c r="H184" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="I184" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="J184" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>3</v>
+      </c>
+      <c r="D185" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E185" t="n">
+        <v>22.835</v>
+      </c>
+      <c r="F185" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G185" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="H185" t="n">
+        <v>2.83</v>
+      </c>
+      <c r="I185" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="J185" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="1" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C181" t="n">
+      <c r="C186" t="n">
         <v>9</v>
       </c>
-      <c r="D181" t="n">
+      <c r="D186" t="n">
         <v>6.239</v>
       </c>
-      <c r="E181" t="n">
-        <v>6.922</v>
-      </c>
-      <c r="F181" t="n">
+      <c r="E186" t="n">
+        <v>6.848</v>
+      </c>
+      <c r="F186" t="n">
         <v>56.15</v>
       </c>
-      <c r="G181" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="H181" t="n">
-        <v>6.15</v>
-      </c>
-      <c r="I181" t="n">
-        <v>10.95</v>
-      </c>
-      <c r="J181" t="n">
+      <c r="G186" t="n">
+        <v>61.63</v>
+      </c>
+      <c r="H186" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="I186" t="n">
+        <v>9.76</v>
+      </c>
+      <c r="J186" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 20/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
         <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E22" t="n">
-        <v>6.799</v>
+        <v>105.78</v>
       </c>
       <c r="F22" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G22" t="n">
-        <v>61.19</v>
+        <v>105.78</v>
       </c>
       <c r="H22" t="n">
-        <v>5.04</v>
+        <v>5.69</v>
       </c>
       <c r="I22" t="n">
-        <v>8.98</v>
+        <v>5.68</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C23" t="n">
         <v>3</v>
       </c>
       <c r="D23" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E23" t="n">
-        <v>21.669</v>
+        <v>10.536</v>
       </c>
       <c r="F23" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G23" t="n">
-        <v>65.01000000000001</v>
+        <v>31.61</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.66</v>
+        <v>0.45</v>
       </c>
       <c r="I23" t="n">
-        <v>-1.01</v>
+        <v>1.44</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E24" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F24" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G24" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H24" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I24" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D25" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E25" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F25" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G25" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H25" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I25" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E26" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F26" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G26" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H26" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I26" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E32" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F32" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G32" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H32" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I32" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E33" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F33" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G33" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H33" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I33" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E34" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F34" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G34" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H34" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I34" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D35" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E35" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F35" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G35" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H35" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I35" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E36" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F36" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G36" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H36" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I36" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E42" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F42" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H42" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E43" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F43" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G43" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E44" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F44" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G44" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H44" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I44" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E45" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F45" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G45" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H45" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I45" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E47" t="n">
-        <v>6.622</v>
+        <v>99.83</v>
       </c>
       <c r="F47" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G47" t="n">
-        <v>59.6</v>
+        <v>99.83</v>
       </c>
       <c r="H47" t="n">
-        <v>3.45</v>
+        <v>-0.26</v>
       </c>
       <c r="I47" t="n">
-        <v>6.14</v>
+        <v>-0.26</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E48" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F48" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G48" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D49" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E49" t="n">
-        <v>21.778</v>
+        <v>6.622</v>
       </c>
       <c r="F49" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G49" t="n">
-        <v>65.33</v>
+        <v>59.6</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.34</v>
+        <v>3.45</v>
       </c>
       <c r="I49" t="n">
-        <v>-0.52</v>
+        <v>6.14</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E50" t="n">
-        <v>38.312</v>
+        <v>10.562</v>
       </c>
       <c r="F50" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G50" t="n">
-        <v>153.25</v>
+        <v>31.69</v>
       </c>
       <c r="H50" t="n">
-        <v>14.23</v>
+        <v>0.53</v>
       </c>
       <c r="I50" t="n">
-        <v>10.24</v>
+        <v>1.7</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E51" t="n">
-        <v>99.83</v>
+        <v>21.778</v>
       </c>
       <c r="F51" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G51" t="n">
-        <v>99.83</v>
+        <v>65.33</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.26</v>
+        <v>-0.34</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.26</v>
+        <v>-0.52</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>102.86</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>102.86</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>2.77</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>2.77</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E60" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F60" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G60" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H60" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I60" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E61" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F61" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G61" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I61" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E67" t="n">
-        <v>22.797</v>
+        <v>6.807</v>
       </c>
       <c r="F67" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G67" t="n">
-        <v>68.39</v>
+        <v>61.26</v>
       </c>
       <c r="H67" t="n">
-        <v>2.72</v>
+        <v>5.11</v>
       </c>
       <c r="I67" t="n">
-        <v>4.14</v>
+        <v>9.1</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E68" t="n">
-        <v>104.58</v>
+        <v>10.796</v>
       </c>
       <c r="F68" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G68" t="n">
-        <v>104.58</v>
+        <v>32.39</v>
       </c>
       <c r="H68" t="n">
-        <v>4.49</v>
+        <v>1.23</v>
       </c>
       <c r="I68" t="n">
-        <v>4.49</v>
+        <v>3.95</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D69" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E69" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F69" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G69" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H69" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I69" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E70" t="n">
-        <v>6.807</v>
+        <v>22.797</v>
       </c>
       <c r="F70" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G70" t="n">
-        <v>61.26</v>
+        <v>68.39</v>
       </c>
       <c r="H70" t="n">
-        <v>5.11</v>
+        <v>2.72</v>
       </c>
       <c r="I70" t="n">
-        <v>9.1</v>
+        <v>4.14</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E71" t="n">
-        <v>40.567</v>
+        <v>104.58</v>
       </c>
       <c r="F71" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G71" t="n">
-        <v>162.27</v>
+        <v>104.58</v>
       </c>
       <c r="H71" t="n">
-        <v>23.25</v>
+        <v>4.49</v>
       </c>
       <c r="I71" t="n">
-        <v>16.72</v>
+        <v>4.49</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E77" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F77" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G77" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H77" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I77" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E78" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F78" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G78" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H78" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I78" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D79" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E79" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F79" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G79" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H79" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I79" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D81" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E81" t="n">
-        <v>42.25</v>
+        <v>6.836</v>
       </c>
       <c r="F81" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G81" t="n">
-        <v>169</v>
+        <v>61.52</v>
       </c>
       <c r="H81" t="n">
-        <v>29.98</v>
+        <v>5.37</v>
       </c>
       <c r="I81" t="n">
-        <v>21.57</v>
+        <v>9.56</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D92" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E92" t="n">
-        <v>10.876</v>
+        <v>103.88</v>
       </c>
       <c r="F92" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G92" t="n">
-        <v>32.63</v>
+        <v>103.88</v>
       </c>
       <c r="H92" t="n">
-        <v>1.47</v>
+        <v>3.79</v>
       </c>
       <c r="I92" t="n">
-        <v>4.72</v>
+        <v>3.79</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E93" t="n">
-        <v>40.575</v>
+        <v>23.025</v>
       </c>
       <c r="F93" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G93" t="n">
-        <v>162.3</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H93" t="n">
-        <v>23.28</v>
+        <v>3.4</v>
       </c>
       <c r="I93" t="n">
-        <v>16.75</v>
+        <v>5.18</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D94" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E94" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F94" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G94" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H94" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I94" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E95" t="n">
-        <v>103.88</v>
+        <v>10.876</v>
       </c>
       <c r="F95" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G95" t="n">
-        <v>103.88</v>
+        <v>32.63</v>
       </c>
       <c r="H95" t="n">
-        <v>3.79</v>
+        <v>1.47</v>
       </c>
       <c r="I95" t="n">
-        <v>3.79</v>
+        <v>4.72</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D96" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E96" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F96" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G96" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H96" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I96" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D107" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E107" t="n">
-        <v>103.14</v>
+        <v>40.5</v>
       </c>
       <c r="F107" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G107" t="n">
-        <v>103.14</v>
+        <v>162</v>
       </c>
       <c r="H107" t="n">
-        <v>3.05</v>
+        <v>22.98</v>
       </c>
       <c r="I107" t="n">
-        <v>3.05</v>
+        <v>16.53</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E108" t="n">
-        <v>6.785</v>
+        <v>10.456</v>
       </c>
       <c r="F108" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G108" t="n">
-        <v>61.06</v>
+        <v>31.37</v>
       </c>
       <c r="H108" t="n">
-        <v>4.91</v>
+        <v>0.21</v>
       </c>
       <c r="I108" t="n">
-        <v>8.74</v>
+        <v>0.67</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D109" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E109" t="n">
-        <v>23.33</v>
+        <v>103.14</v>
       </c>
       <c r="F109" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G109" t="n">
-        <v>69.98999999999999</v>
+        <v>103.14</v>
       </c>
       <c r="H109" t="n">
-        <v>4.32</v>
+        <v>3.05</v>
       </c>
       <c r="I109" t="n">
-        <v>6.58</v>
+        <v>3.05</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D110" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E110" t="n">
-        <v>10.456</v>
+        <v>6.785</v>
       </c>
       <c r="F110" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G110" t="n">
-        <v>31.37</v>
+        <v>61.06</v>
       </c>
       <c r="H110" t="n">
-        <v>0.21</v>
+        <v>4.91</v>
       </c>
       <c r="I110" t="n">
-        <v>0.67</v>
+        <v>8.74</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E111" t="n">
-        <v>40.5</v>
+        <v>23.33</v>
       </c>
       <c r="F111" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G111" t="n">
-        <v>162</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H111" t="n">
-        <v>22.98</v>
+        <v>4.32</v>
       </c>
       <c r="I111" t="n">
-        <v>16.53</v>
+        <v>6.58</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D112" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E112" t="n">
-        <v>40</v>
+        <v>6.797</v>
       </c>
       <c r="F112" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G112" t="n">
-        <v>160</v>
+        <v>61.17</v>
       </c>
       <c r="H112" t="n">
-        <v>20.98</v>
+        <v>5.02</v>
       </c>
       <c r="I112" t="n">
-        <v>15.09</v>
+        <v>8.94</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D113" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E113" t="n">
-        <v>103.56</v>
+        <v>40</v>
       </c>
       <c r="F113" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G113" t="n">
-        <v>103.56</v>
+        <v>160</v>
       </c>
       <c r="H113" t="n">
-        <v>3.47</v>
+        <v>20.98</v>
       </c>
       <c r="I113" t="n">
-        <v>3.47</v>
+        <v>15.09</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E114" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F114" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G114" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H114" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I114" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C115" t="n">
         <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E115" t="n">
-        <v>10.568</v>
+        <v>23.025</v>
       </c>
       <c r="F115" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G115" t="n">
-        <v>31.7</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H115" t="n">
-        <v>0.54</v>
+        <v>3.4</v>
       </c>
       <c r="I115" t="n">
-        <v>1.73</v>
+        <v>5.18</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E116" t="n">
-        <v>6.797</v>
+        <v>10.568</v>
       </c>
       <c r="F116" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G116" t="n">
-        <v>61.17</v>
+        <v>31.7</v>
       </c>
       <c r="H116" t="n">
-        <v>5.02</v>
+        <v>0.54</v>
       </c>
       <c r="I116" t="n">
-        <v>8.94</v>
+        <v>1.73</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E117" t="n">
-        <v>41</v>
+        <v>23.145</v>
       </c>
       <c r="F117" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G117" t="n">
-        <v>164</v>
+        <v>69.44</v>
       </c>
       <c r="H117" t="n">
-        <v>24.98</v>
+        <v>3.77</v>
       </c>
       <c r="I117" t="n">
-        <v>17.97</v>
+        <v>5.74</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E118" t="n">
-        <v>10.756</v>
+        <v>105.96</v>
       </c>
       <c r="F118" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G118" t="n">
-        <v>32.27</v>
+        <v>105.96</v>
       </c>
       <c r="H118" t="n">
-        <v>1.11</v>
+        <v>5.87</v>
       </c>
       <c r="I118" t="n">
-        <v>3.56</v>
+        <v>5.86</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>10.756</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>32.27</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>1.11</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>3.56</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D121" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E121" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F121" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G121" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H121" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I121" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D127" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E127" t="n">
-        <v>39.36</v>
+        <v>103.46</v>
       </c>
       <c r="F127" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G127" t="n">
-        <v>157.44</v>
+        <v>103.46</v>
       </c>
       <c r="H127" t="n">
-        <v>18.42</v>
+        <v>3.37</v>
       </c>
       <c r="I127" t="n">
-        <v>13.25</v>
+        <v>3.37</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E128" t="n">
-        <v>6.868</v>
+        <v>23.17</v>
       </c>
       <c r="F128" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G128" t="n">
-        <v>61.81</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H128" t="n">
-        <v>5.66</v>
+        <v>3.84</v>
       </c>
       <c r="I128" t="n">
-        <v>10.08</v>
+        <v>5.85</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4796,29 +4796,29 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C129" t="n">
         <v>3</v>
       </c>
       <c r="D129" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E129" t="n">
-        <v>23.17</v>
+        <v>11.458</v>
       </c>
       <c r="F129" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G129" t="n">
-        <v>69.51000000000001</v>
+        <v>34.37</v>
       </c>
       <c r="H129" t="n">
-        <v>3.84</v>
+        <v>3.21</v>
       </c>
       <c r="I129" t="n">
-        <v>5.85</v>
+        <v>10.3</v>
       </c>
       <c r="J129" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D130" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E130" t="n">
-        <v>103.46</v>
+        <v>39.36</v>
       </c>
       <c r="F130" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G130" t="n">
-        <v>103.46</v>
+        <v>157.44</v>
       </c>
       <c r="H130" t="n">
-        <v>3.37</v>
+        <v>18.42</v>
       </c>
       <c r="I130" t="n">
-        <v>3.37</v>
+        <v>13.25</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D131" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E131" t="n">
-        <v>11.458</v>
+        <v>6.868</v>
       </c>
       <c r="F131" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G131" t="n">
-        <v>34.37</v>
+        <v>61.81</v>
       </c>
       <c r="H131" t="n">
-        <v>3.21</v>
+        <v>5.66</v>
       </c>
       <c r="I131" t="n">
-        <v>10.3</v>
+        <v>10.08</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D142" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E142" t="n">
-        <v>102.06</v>
+        <v>6.878</v>
       </c>
       <c r="F142" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G142" t="n">
-        <v>102.06</v>
+        <v>61.9</v>
       </c>
       <c r="H142" t="n">
-        <v>1.97</v>
+        <v>5.75</v>
       </c>
       <c r="I142" t="n">
-        <v>1.97</v>
+        <v>10.24</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C143" t="n">
         <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E143" t="n">
-        <v>23.135</v>
+        <v>11.498</v>
       </c>
       <c r="F143" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G143" t="n">
-        <v>69.41</v>
+        <v>34.49</v>
       </c>
       <c r="H143" t="n">
-        <v>3.74</v>
+        <v>3.33</v>
       </c>
       <c r="I143" t="n">
-        <v>5.7</v>
+        <v>10.69</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5306,29 +5306,29 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D144" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E144" t="n">
-        <v>38.89</v>
+        <v>23.135</v>
       </c>
       <c r="F144" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G144" t="n">
-        <v>155.56</v>
+        <v>69.41</v>
       </c>
       <c r="H144" t="n">
-        <v>16.54</v>
+        <v>3.74</v>
       </c>
       <c r="I144" t="n">
-        <v>11.9</v>
+        <v>5.7</v>
       </c>
       <c r="J144" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E145" t="n">
-        <v>11.498</v>
+        <v>102.06</v>
       </c>
       <c r="F145" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G145" t="n">
-        <v>34.49</v>
+        <v>102.06</v>
       </c>
       <c r="H145" t="n">
-        <v>3.33</v>
+        <v>1.97</v>
       </c>
       <c r="I145" t="n">
-        <v>10.69</v>
+        <v>1.97</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E146" t="n">
-        <v>6.878</v>
+        <v>38.89</v>
       </c>
       <c r="F146" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G146" t="n">
-        <v>61.9</v>
+        <v>155.56</v>
       </c>
       <c r="H146" t="n">
-        <v>5.75</v>
+        <v>16.54</v>
       </c>
       <c r="I146" t="n">
-        <v>10.24</v>
+        <v>11.9</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E152" t="n">
-        <v>6.893</v>
+        <v>11.034</v>
       </c>
       <c r="F152" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G152" t="n">
-        <v>62.04</v>
+        <v>33.1</v>
       </c>
       <c r="H152" t="n">
-        <v>5.89</v>
+        <v>1.94</v>
       </c>
       <c r="I152" t="n">
-        <v>10.49</v>
+        <v>6.23</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D153" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E153" t="n">
-        <v>23.045</v>
+        <v>104.12</v>
       </c>
       <c r="F153" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G153" t="n">
-        <v>69.14</v>
+        <v>104.12</v>
       </c>
       <c r="H153" t="n">
-        <v>3.47</v>
+        <v>4.03</v>
       </c>
       <c r="I153" t="n">
-        <v>5.28</v>
+        <v>4.03</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5646,29 +5646,29 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D154" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E154" t="n">
-        <v>104.12</v>
+        <v>39.915</v>
       </c>
       <c r="F154" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G154" t="n">
-        <v>104.12</v>
+        <v>159.66</v>
       </c>
       <c r="H154" t="n">
-        <v>4.03</v>
+        <v>20.64</v>
       </c>
       <c r="I154" t="n">
-        <v>4.03</v>
+        <v>14.85</v>
       </c>
       <c r="J154" t="n">
         <v>7.91</v>
@@ -5680,29 +5680,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D155" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E155" t="n">
-        <v>11.034</v>
+        <v>6.893</v>
       </c>
       <c r="F155" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G155" t="n">
-        <v>33.1</v>
+        <v>62.04</v>
       </c>
       <c r="H155" t="n">
-        <v>1.94</v>
+        <v>5.89</v>
       </c>
       <c r="I155" t="n">
-        <v>6.23</v>
+        <v>10.49</v>
       </c>
       <c r="J155" t="n">
         <v>7.91</v>
@@ -5714,29 +5714,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D156" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E156" t="n">
-        <v>39.915</v>
+        <v>23.045</v>
       </c>
       <c r="F156" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G156" t="n">
-        <v>159.66</v>
+        <v>69.14</v>
       </c>
       <c r="H156" t="n">
-        <v>20.64</v>
+        <v>3.47</v>
       </c>
       <c r="I156" t="n">
-        <v>14.85</v>
+        <v>5.28</v>
       </c>
       <c r="J156" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D157" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E157" t="n">
-        <v>104.5</v>
+        <v>23.08</v>
       </c>
       <c r="F157" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G157" t="n">
-        <v>104.5</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H157" t="n">
-        <v>4.41</v>
+        <v>3.57</v>
       </c>
       <c r="I157" t="n">
-        <v>4.41</v>
+        <v>5.44</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D158" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E158" t="n">
-        <v>23.08</v>
+        <v>6.913</v>
       </c>
       <c r="F158" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G158" t="n">
-        <v>69.23999999999999</v>
+        <v>62.22</v>
       </c>
       <c r="H158" t="n">
-        <v>3.57</v>
+        <v>6.07</v>
       </c>
       <c r="I158" t="n">
-        <v>5.44</v>
+        <v>10.81</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D159" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E159" t="n">
-        <v>6.913</v>
+        <v>40.015</v>
       </c>
       <c r="F159" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G159" t="n">
-        <v>62.22</v>
+        <v>160.06</v>
       </c>
       <c r="H159" t="n">
-        <v>6.07</v>
+        <v>21.04</v>
       </c>
       <c r="I159" t="n">
-        <v>10.81</v>
+        <v>15.13</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E160" t="n">
-        <v>40.015</v>
+        <v>10.92</v>
       </c>
       <c r="F160" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G160" t="n">
-        <v>160.06</v>
+        <v>32.76</v>
       </c>
       <c r="H160" t="n">
-        <v>21.04</v>
+        <v>1.6</v>
       </c>
       <c r="I160" t="n">
-        <v>15.13</v>
+        <v>5.13</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D161" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E161" t="n">
-        <v>10.92</v>
+        <v>104.5</v>
       </c>
       <c r="F161" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G161" t="n">
-        <v>32.76</v>
+        <v>104.5</v>
       </c>
       <c r="H161" t="n">
-        <v>1.6</v>
+        <v>4.41</v>
       </c>
       <c r="I161" t="n">
-        <v>5.13</v>
+        <v>4.41</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D167" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E167" t="n">
-        <v>38.98</v>
+        <v>103.98</v>
       </c>
       <c r="F167" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G167" t="n">
-        <v>155.92</v>
+        <v>103.98</v>
       </c>
       <c r="H167" t="n">
-        <v>16.9</v>
+        <v>3.89</v>
       </c>
       <c r="I167" t="n">
-        <v>12.16</v>
+        <v>3.89</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D168" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E168" t="n">
-        <v>6.911</v>
+        <v>22.92</v>
       </c>
       <c r="F168" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G168" t="n">
-        <v>62.2</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H168" t="n">
-        <v>6.05</v>
+        <v>3.09</v>
       </c>
       <c r="I168" t="n">
-        <v>10.77</v>
+        <v>4.71</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6156,29 +6156,29 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D169" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E169" t="n">
-        <v>10.726</v>
+        <v>6.911</v>
       </c>
       <c r="F169" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G169" t="n">
-        <v>32.18</v>
+        <v>62.2</v>
       </c>
       <c r="H169" t="n">
-        <v>1.02</v>
+        <v>6.05</v>
       </c>
       <c r="I169" t="n">
-        <v>3.27</v>
+        <v>10.77</v>
       </c>
       <c r="J169" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D170" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E170" t="n">
-        <v>103.98</v>
+        <v>38.98</v>
       </c>
       <c r="F170" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G170" t="n">
-        <v>103.98</v>
+        <v>155.92</v>
       </c>
       <c r="H170" t="n">
-        <v>3.89</v>
+        <v>16.9</v>
       </c>
       <c r="I170" t="n">
-        <v>3.89</v>
+        <v>12.16</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,29 +6224,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C171" t="n">
         <v>3</v>
       </c>
       <c r="D171" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E171" t="n">
-        <v>22.92</v>
+        <v>10.726</v>
       </c>
       <c r="F171" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G171" t="n">
-        <v>68.76000000000001</v>
+        <v>32.18</v>
       </c>
       <c r="H171" t="n">
-        <v>3.09</v>
+        <v>1.02</v>
       </c>
       <c r="I171" t="n">
-        <v>4.71</v>
+        <v>3.27</v>
       </c>
       <c r="J171" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D177" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E177" t="n">
-        <v>6.922</v>
+        <v>102.54</v>
       </c>
       <c r="F177" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G177" t="n">
-        <v>62.3</v>
+        <v>102.54</v>
       </c>
       <c r="H177" t="n">
-        <v>6.15</v>
+        <v>2.45</v>
       </c>
       <c r="I177" t="n">
-        <v>10.95</v>
+        <v>2.45</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D178" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E178" t="n">
-        <v>10.642</v>
+        <v>38.245</v>
       </c>
       <c r="F178" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G178" t="n">
-        <v>31.93</v>
+        <v>152.98</v>
       </c>
       <c r="H178" t="n">
-        <v>0.77</v>
+        <v>13.96</v>
       </c>
       <c r="I178" t="n">
-        <v>2.47</v>
+        <v>10.04</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D179" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E179" t="n">
-        <v>38.245</v>
+        <v>22.95</v>
       </c>
       <c r="F179" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G179" t="n">
-        <v>152.98</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H179" t="n">
-        <v>13.96</v>
+        <v>3.18</v>
       </c>
       <c r="I179" t="n">
-        <v>10.04</v>
+        <v>4.84</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D180" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E180" t="n">
-        <v>22.95</v>
+        <v>6.922</v>
       </c>
       <c r="F180" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G180" t="n">
-        <v>68.84999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="H180" t="n">
-        <v>3.18</v>
+        <v>6.15</v>
       </c>
       <c r="I180" t="n">
-        <v>4.84</v>
+        <v>10.95</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,29 +6564,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D181" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E181" t="n">
-        <v>102.54</v>
+        <v>10.642</v>
       </c>
       <c r="F181" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G181" t="n">
-        <v>102.54</v>
+        <v>31.93</v>
       </c>
       <c r="H181" t="n">
-        <v>2.45</v>
+        <v>0.77</v>
       </c>
       <c r="I181" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="J181" t="n">
         <v>7.91</v>
@@ -6759,6 +6759,176 @@
         <v>9.76</v>
       </c>
       <c r="J186" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>3</v>
+      </c>
+      <c r="D187" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E187" t="n">
+        <v>10.708</v>
+      </c>
+      <c r="F187" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G187" t="n">
+        <v>32.12</v>
+      </c>
+      <c r="H187" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="I187" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="J187" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>4</v>
+      </c>
+      <c r="D188" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E188" t="n">
+        <v>37.85</v>
+      </c>
+      <c r="F188" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G188" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="H188" t="n">
+        <v>12.38</v>
+      </c>
+      <c r="I188" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="J188" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>3</v>
+      </c>
+      <c r="D189" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E189" t="n">
+        <v>22.845</v>
+      </c>
+      <c r="F189" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G189" t="n">
+        <v>68.53</v>
+      </c>
+      <c r="H189" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="I189" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="J189" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E190" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="F190" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G190" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="H190" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="I190" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J190" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="1" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>9</v>
+      </c>
+      <c r="D191" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E191" t="n">
+        <v>6.862</v>
+      </c>
+      <c r="F191" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G191" t="n">
+        <v>61.76</v>
+      </c>
+      <c r="H191" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="I191" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="J191" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 21/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J191"/>
+  <dimension ref="A1:J196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
         <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E22" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F22" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G22" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I22" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E23" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F23" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G23" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H23" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I23" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D24" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E24" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F24" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G24" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H24" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I24" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E25" t="n">
-        <v>6.799</v>
+        <v>105.78</v>
       </c>
       <c r="F25" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G25" t="n">
-        <v>61.19</v>
+        <v>105.78</v>
       </c>
       <c r="H25" t="n">
-        <v>5.04</v>
+        <v>5.69</v>
       </c>
       <c r="I25" t="n">
-        <v>8.98</v>
+        <v>5.68</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C26" t="n">
         <v>3</v>
       </c>
       <c r="D26" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E26" t="n">
-        <v>21.669</v>
+        <v>10.536</v>
       </c>
       <c r="F26" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G26" t="n">
-        <v>65.01000000000001</v>
+        <v>31.61</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.66</v>
+        <v>0.45</v>
       </c>
       <c r="I26" t="n">
-        <v>-1.01</v>
+        <v>1.44</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D32" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E32" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F32" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G32" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H32" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I32" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E33" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F33" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G33" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H33" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I33" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E34" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F34" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G34" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H34" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I34" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D35" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E35" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F35" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G35" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H35" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I35" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E36" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F36" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G36" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H36" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I36" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C43" t="n">
         <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E43" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F43" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G43" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H43" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I43" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E45" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F45" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G45" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H45" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I45" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E47" t="n">
-        <v>99.83</v>
+        <v>21.778</v>
       </c>
       <c r="F47" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G47" t="n">
-        <v>99.83</v>
+        <v>65.33</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.26</v>
+        <v>-0.34</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.26</v>
+        <v>-0.52</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E48" t="n">
-        <v>38.312</v>
+        <v>6.622</v>
       </c>
       <c r="F48" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G48" t="n">
-        <v>153.25</v>
+        <v>59.6</v>
       </c>
       <c r="H48" t="n">
-        <v>14.23</v>
+        <v>3.45</v>
       </c>
       <c r="I48" t="n">
-        <v>10.24</v>
+        <v>6.14</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E49" t="n">
-        <v>6.622</v>
+        <v>10.562</v>
       </c>
       <c r="F49" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G49" t="n">
-        <v>59.6</v>
+        <v>31.69</v>
       </c>
       <c r="H49" t="n">
-        <v>3.45</v>
+        <v>0.53</v>
       </c>
       <c r="I49" t="n">
-        <v>6.14</v>
+        <v>1.7</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D50" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E50" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F50" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G50" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H50" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I50" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E51" t="n">
-        <v>21.778</v>
+        <v>99.83</v>
       </c>
       <c r="F51" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G51" t="n">
-        <v>65.33</v>
+        <v>99.83</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.34</v>
+        <v>-0.26</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.52</v>
+        <v>-0.26</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D62" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E62" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F62" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G62" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H62" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>41.064</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>164.26</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>25.24</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>18.16</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E64" t="n">
-        <v>22.7</v>
+        <v>105.5</v>
       </c>
       <c r="F64" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G64" t="n">
-        <v>68.09999999999999</v>
+        <v>105.5</v>
       </c>
       <c r="H64" t="n">
-        <v>2.43</v>
+        <v>5.41</v>
       </c>
       <c r="I64" t="n">
-        <v>3.7</v>
+        <v>5.41</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D65" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E65" t="n">
-        <v>10.712</v>
+        <v>41.064</v>
       </c>
       <c r="F65" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G65" t="n">
-        <v>32.14</v>
+        <v>164.26</v>
       </c>
       <c r="H65" t="n">
-        <v>0.98</v>
+        <v>25.24</v>
       </c>
       <c r="I65" t="n">
-        <v>3.15</v>
+        <v>18.16</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E66" t="n">
-        <v>6.817</v>
+        <v>22.7</v>
       </c>
       <c r="F66" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G66" t="n">
-        <v>61.35</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H66" t="n">
-        <v>5.2</v>
+        <v>2.43</v>
       </c>
       <c r="I66" t="n">
-        <v>9.26</v>
+        <v>3.7</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E72" t="n">
-        <v>23</v>
+        <v>104.22</v>
       </c>
       <c r="F72" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G72" t="n">
-        <v>69</v>
+        <v>104.22</v>
       </c>
       <c r="H72" t="n">
-        <v>3.33</v>
+        <v>4.13</v>
       </c>
       <c r="I72" t="n">
-        <v>5.07</v>
+        <v>4.13</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E75" t="n">
-        <v>104.22</v>
+        <v>10.892</v>
       </c>
       <c r="F75" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G75" t="n">
-        <v>104.22</v>
+        <v>32.68</v>
       </c>
       <c r="H75" t="n">
-        <v>4.13</v>
+        <v>1.52</v>
       </c>
       <c r="I75" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D76" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E76" t="n">
-        <v>6.811</v>
+        <v>23</v>
       </c>
       <c r="F76" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G76" t="n">
-        <v>61.3</v>
+        <v>69</v>
       </c>
       <c r="H76" t="n">
-        <v>5.15</v>
+        <v>3.33</v>
       </c>
       <c r="I76" t="n">
-        <v>9.17</v>
+        <v>5.07</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E82" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F82" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G82" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H82" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I82" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C83" t="n">
         <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E83" t="n">
-        <v>23.3</v>
+        <v>10.988</v>
       </c>
       <c r="F83" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G83" t="n">
-        <v>69.90000000000001</v>
+        <v>32.96</v>
       </c>
       <c r="H83" t="n">
-        <v>4.23</v>
+        <v>1.8</v>
       </c>
       <c r="I83" t="n">
-        <v>6.44</v>
+        <v>5.78</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E84" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F84" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G84" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H84" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I84" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D85" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E85" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F85" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G85" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H85" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I85" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E86" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F86" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G86" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H86" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I86" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E92" t="n">
-        <v>103.88</v>
+        <v>10.876</v>
       </c>
       <c r="F92" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G92" t="n">
-        <v>103.88</v>
+        <v>32.63</v>
       </c>
       <c r="H92" t="n">
-        <v>3.79</v>
+        <v>1.47</v>
       </c>
       <c r="I92" t="n">
-        <v>3.79</v>
+        <v>4.72</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E93" t="n">
-        <v>23.025</v>
+        <v>103.88</v>
       </c>
       <c r="F93" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G93" t="n">
-        <v>69.06999999999999</v>
+        <v>103.88</v>
       </c>
       <c r="H93" t="n">
-        <v>3.4</v>
+        <v>3.79</v>
       </c>
       <c r="I93" t="n">
-        <v>5.18</v>
+        <v>3.79</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E94" t="n">
-        <v>6.797</v>
+        <v>23.025</v>
       </c>
       <c r="F94" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G94" t="n">
-        <v>61.17</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H94" t="n">
-        <v>5.02</v>
+        <v>3.4</v>
       </c>
       <c r="I94" t="n">
-        <v>8.94</v>
+        <v>5.18</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D95" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E95" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F95" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G95" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H95" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I95" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D97" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E97" t="n">
-        <v>40.65</v>
+        <v>6.839</v>
       </c>
       <c r="F97" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G97" t="n">
-        <v>162.6</v>
+        <v>61.55</v>
       </c>
       <c r="H97" t="n">
-        <v>23.58</v>
+        <v>5.4</v>
       </c>
       <c r="I97" t="n">
-        <v>16.96</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E98" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F98" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G98" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H98" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I98" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C100" t="n">
         <v>3</v>
       </c>
       <c r="D100" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E100" t="n">
-        <v>10.642</v>
+        <v>23.35</v>
       </c>
       <c r="F100" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G100" t="n">
-        <v>31.93</v>
+        <v>70.05</v>
       </c>
       <c r="H100" t="n">
-        <v>0.77</v>
+        <v>4.38</v>
       </c>
       <c r="I100" t="n">
-        <v>2.47</v>
+        <v>6.67</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D101" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E101" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F101" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G101" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H101" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I101" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D107" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E107" t="n">
-        <v>40.5</v>
+        <v>6.785</v>
       </c>
       <c r="F107" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G107" t="n">
-        <v>162</v>
+        <v>61.06</v>
       </c>
       <c r="H107" t="n">
-        <v>22.98</v>
+        <v>4.91</v>
       </c>
       <c r="I107" t="n">
-        <v>16.53</v>
+        <v>8.74</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E108" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F108" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G108" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H108" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I108" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D109" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E109" t="n">
-        <v>103.14</v>
+        <v>23.33</v>
       </c>
       <c r="F109" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G109" t="n">
-        <v>103.14</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H109" t="n">
-        <v>3.05</v>
+        <v>4.32</v>
       </c>
       <c r="I109" t="n">
-        <v>3.05</v>
+        <v>6.58</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D110" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E110" t="n">
-        <v>6.785</v>
+        <v>40.5</v>
       </c>
       <c r="F110" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G110" t="n">
-        <v>61.06</v>
+        <v>162</v>
       </c>
       <c r="H110" t="n">
-        <v>4.91</v>
+        <v>22.98</v>
       </c>
       <c r="I110" t="n">
-        <v>8.74</v>
+        <v>16.53</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C111" t="n">
         <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E111" t="n">
-        <v>23.33</v>
+        <v>10.456</v>
       </c>
       <c r="F111" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G111" t="n">
-        <v>69.98999999999999</v>
+        <v>31.37</v>
       </c>
       <c r="H111" t="n">
-        <v>4.32</v>
+        <v>0.21</v>
       </c>
       <c r="I111" t="n">
-        <v>6.58</v>
+        <v>0.67</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E122" t="n">
-        <v>6.901</v>
+        <v>106</v>
       </c>
       <c r="F122" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G122" t="n">
-        <v>62.11</v>
+        <v>106</v>
       </c>
       <c r="H122" t="n">
-        <v>5.96</v>
+        <v>5.91</v>
       </c>
       <c r="I122" t="n">
-        <v>10.61</v>
+        <v>5.9</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E123" t="n">
-        <v>40.395</v>
+        <v>23.165</v>
       </c>
       <c r="F123" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G123" t="n">
-        <v>161.58</v>
+        <v>69.5</v>
       </c>
       <c r="H123" t="n">
-        <v>22.56</v>
+        <v>3.83</v>
       </c>
       <c r="I123" t="n">
-        <v>16.23</v>
+        <v>5.83</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D125" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E125" t="n">
-        <v>23.165</v>
+        <v>40.395</v>
       </c>
       <c r="F125" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G125" t="n">
-        <v>69.5</v>
+        <v>161.58</v>
       </c>
       <c r="H125" t="n">
-        <v>3.83</v>
+        <v>22.56</v>
       </c>
       <c r="I125" t="n">
-        <v>5.83</v>
+        <v>16.23</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D126" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E126" t="n">
-        <v>106</v>
+        <v>6.901</v>
       </c>
       <c r="F126" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G126" t="n">
-        <v>106</v>
+        <v>62.11</v>
       </c>
       <c r="H126" t="n">
-        <v>5.91</v>
+        <v>5.96</v>
       </c>
       <c r="I126" t="n">
-        <v>5.9</v>
+        <v>10.61</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D132" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E132" t="n">
-        <v>11.516</v>
+        <v>104.02</v>
       </c>
       <c r="F132" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G132" t="n">
-        <v>34.55</v>
+        <v>104.02</v>
       </c>
       <c r="H132" t="n">
-        <v>3.39</v>
+        <v>3.93</v>
       </c>
       <c r="I132" t="n">
-        <v>10.88</v>
+        <v>3.93</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E133" t="n">
-        <v>6.895</v>
+        <v>23.18</v>
       </c>
       <c r="F133" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G133" t="n">
-        <v>62.05</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H133" t="n">
-        <v>5.9</v>
+        <v>3.87</v>
       </c>
       <c r="I133" t="n">
-        <v>10.51</v>
+        <v>5.89</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D134" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E134" t="n">
-        <v>23.18</v>
+        <v>40.54</v>
       </c>
       <c r="F134" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G134" t="n">
-        <v>69.54000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="H134" t="n">
-        <v>3.87</v>
+        <v>23.14</v>
       </c>
       <c r="I134" t="n">
-        <v>5.89</v>
+        <v>16.65</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E135" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F135" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G135" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H135" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I135" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D136" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E136" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F136" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G136" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H136" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I136" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D147" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E147" t="n">
-        <v>38.955</v>
+        <v>6.826</v>
       </c>
       <c r="F147" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G147" t="n">
-        <v>155.82</v>
+        <v>61.43</v>
       </c>
       <c r="H147" t="n">
-        <v>16.8</v>
+        <v>5.28</v>
       </c>
       <c r="I147" t="n">
-        <v>12.08</v>
+        <v>9.4</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E148" t="n">
-        <v>101.7</v>
+        <v>22.755</v>
       </c>
       <c r="F148" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G148" t="n">
-        <v>101.7</v>
+        <v>68.27</v>
       </c>
       <c r="H148" t="n">
-        <v>1.61</v>
+        <v>2.6</v>
       </c>
       <c r="I148" t="n">
-        <v>1.61</v>
+        <v>3.96</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D149" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E149" t="n">
-        <v>11.162</v>
+        <v>101.7</v>
       </c>
       <c r="F149" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G149" t="n">
-        <v>33.49</v>
+        <v>101.7</v>
       </c>
       <c r="H149" t="n">
-        <v>2.33</v>
+        <v>1.61</v>
       </c>
       <c r="I149" t="n">
-        <v>7.48</v>
+        <v>1.61</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C150" t="n">
         <v>3</v>
       </c>
       <c r="D150" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E150" t="n">
-        <v>22.755</v>
+        <v>11.162</v>
       </c>
       <c r="F150" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G150" t="n">
-        <v>68.27</v>
+        <v>33.49</v>
       </c>
       <c r="H150" t="n">
-        <v>2.6</v>
+        <v>2.33</v>
       </c>
       <c r="I150" t="n">
-        <v>3.96</v>
+        <v>7.48</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D151" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E151" t="n">
-        <v>6.826</v>
+        <v>38.955</v>
       </c>
       <c r="F151" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G151" t="n">
-        <v>61.43</v>
+        <v>155.82</v>
       </c>
       <c r="H151" t="n">
-        <v>5.28</v>
+        <v>16.8</v>
       </c>
       <c r="I151" t="n">
-        <v>9.4</v>
+        <v>12.08</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C157" t="n">
         <v>3</v>
       </c>
       <c r="D157" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E157" t="n">
-        <v>23.08</v>
+        <v>10.92</v>
       </c>
       <c r="F157" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G157" t="n">
-        <v>69.23999999999999</v>
+        <v>32.76</v>
       </c>
       <c r="H157" t="n">
-        <v>3.57</v>
+        <v>1.6</v>
       </c>
       <c r="I157" t="n">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D158" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E158" t="n">
-        <v>6.913</v>
+        <v>40.015</v>
       </c>
       <c r="F158" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G158" t="n">
-        <v>62.22</v>
+        <v>160.06</v>
       </c>
       <c r="H158" t="n">
-        <v>6.07</v>
+        <v>21.04</v>
       </c>
       <c r="I158" t="n">
-        <v>10.81</v>
+        <v>15.13</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D159" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E159" t="n">
-        <v>40.015</v>
+        <v>104.5</v>
       </c>
       <c r="F159" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G159" t="n">
-        <v>160.06</v>
+        <v>104.5</v>
       </c>
       <c r="H159" t="n">
-        <v>21.04</v>
+        <v>4.41</v>
       </c>
       <c r="I159" t="n">
-        <v>15.13</v>
+        <v>4.41</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C160" t="n">
         <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E160" t="n">
-        <v>10.92</v>
+        <v>23.08</v>
       </c>
       <c r="F160" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G160" t="n">
-        <v>32.76</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H160" t="n">
-        <v>1.6</v>
+        <v>3.57</v>
       </c>
       <c r="I160" t="n">
-        <v>5.13</v>
+        <v>5.44</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D161" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E161" t="n">
-        <v>104.5</v>
+        <v>6.913</v>
       </c>
       <c r="F161" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G161" t="n">
-        <v>104.5</v>
+        <v>62.22</v>
       </c>
       <c r="H161" t="n">
-        <v>4.41</v>
+        <v>6.07</v>
       </c>
       <c r="I161" t="n">
-        <v>4.41</v>
+        <v>10.81</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6258,29 +6258,29 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D172" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E172" t="n">
-        <v>6.926</v>
+        <v>103.22</v>
       </c>
       <c r="F172" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G172" t="n">
-        <v>62.33</v>
+        <v>103.22</v>
       </c>
       <c r="H172" t="n">
-        <v>6.18</v>
+        <v>3.13</v>
       </c>
       <c r="I172" t="n">
-        <v>11.01</v>
+        <v>3.13</v>
       </c>
       <c r="J172" t="n">
         <v>7.91</v>
@@ -6292,29 +6292,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E173" t="n">
-        <v>22.95</v>
+        <v>38.74</v>
       </c>
       <c r="F173" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G173" t="n">
-        <v>68.84999999999999</v>
+        <v>154.96</v>
       </c>
       <c r="H173" t="n">
-        <v>3.18</v>
+        <v>15.94</v>
       </c>
       <c r="I173" t="n">
-        <v>4.84</v>
+        <v>11.47</v>
       </c>
       <c r="J173" t="n">
         <v>7.91</v>
@@ -6326,29 +6326,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C174" t="n">
         <v>3</v>
       </c>
       <c r="D174" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E174" t="n">
-        <v>10.712</v>
+        <v>22.95</v>
       </c>
       <c r="F174" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G174" t="n">
-        <v>32.14</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H174" t="n">
-        <v>0.98</v>
+        <v>3.18</v>
       </c>
       <c r="I174" t="n">
-        <v>3.15</v>
+        <v>4.84</v>
       </c>
       <c r="J174" t="n">
         <v>7.91</v>
@@ -6360,29 +6360,29 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D175" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E175" t="n">
-        <v>103.22</v>
+        <v>6.926</v>
       </c>
       <c r="F175" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G175" t="n">
-        <v>103.22</v>
+        <v>62.33</v>
       </c>
       <c r="H175" t="n">
-        <v>3.13</v>
+        <v>6.18</v>
       </c>
       <c r="I175" t="n">
-        <v>3.13</v>
+        <v>11.01</v>
       </c>
       <c r="J175" t="n">
         <v>7.91</v>
@@ -6394,29 +6394,29 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D176" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E176" t="n">
-        <v>38.74</v>
+        <v>10.712</v>
       </c>
       <c r="F176" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G176" t="n">
-        <v>154.96</v>
+        <v>32.14</v>
       </c>
       <c r="H176" t="n">
-        <v>15.94</v>
+        <v>0.98</v>
       </c>
       <c r="I176" t="n">
-        <v>11.47</v>
+        <v>3.15</v>
       </c>
       <c r="J176" t="n">
         <v>7.91</v>
@@ -6598,29 +6598,29 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D182" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E182" t="n">
-        <v>100.14</v>
+        <v>6.848</v>
       </c>
       <c r="F182" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G182" t="n">
-        <v>100.14</v>
+        <v>61.63</v>
       </c>
       <c r="H182" t="n">
-        <v>0.05</v>
+        <v>5.48</v>
       </c>
       <c r="I182" t="n">
-        <v>0.05</v>
+        <v>9.76</v>
       </c>
       <c r="J182" t="n">
         <v>7.91</v>
@@ -6632,29 +6632,29 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C183" t="n">
         <v>3</v>
       </c>
       <c r="D183" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E183" t="n">
-        <v>10.776</v>
+        <v>22.835</v>
       </c>
       <c r="F183" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G183" t="n">
-        <v>32.33</v>
+        <v>68.5</v>
       </c>
       <c r="H183" t="n">
-        <v>1.17</v>
+        <v>2.83</v>
       </c>
       <c r="I183" t="n">
-        <v>3.75</v>
+        <v>4.31</v>
       </c>
       <c r="J183" t="n">
         <v>7.91</v>
@@ -6666,29 +6666,29 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D184" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E184" t="n">
-        <v>37.235</v>
+        <v>10.776</v>
       </c>
       <c r="F184" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G184" t="n">
-        <v>148.94</v>
+        <v>32.33</v>
       </c>
       <c r="H184" t="n">
-        <v>9.92</v>
+        <v>1.17</v>
       </c>
       <c r="I184" t="n">
-        <v>7.14</v>
+        <v>3.75</v>
       </c>
       <c r="J184" t="n">
         <v>7.91</v>
@@ -6700,29 +6700,29 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D185" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E185" t="n">
-        <v>22.835</v>
+        <v>100.14</v>
       </c>
       <c r="F185" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G185" t="n">
-        <v>68.5</v>
+        <v>100.14</v>
       </c>
       <c r="H185" t="n">
-        <v>2.83</v>
+        <v>0.05</v>
       </c>
       <c r="I185" t="n">
-        <v>4.31</v>
+        <v>0.05</v>
       </c>
       <c r="J185" t="n">
         <v>7.91</v>
@@ -6734,29 +6734,29 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E186" t="n">
-        <v>6.848</v>
+        <v>37.235</v>
       </c>
       <c r="F186" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G186" t="n">
-        <v>61.63</v>
+        <v>148.94</v>
       </c>
       <c r="H186" t="n">
-        <v>5.48</v>
+        <v>9.92</v>
       </c>
       <c r="I186" t="n">
-        <v>9.76</v>
+        <v>7.14</v>
       </c>
       <c r="J186" t="n">
         <v>7.91</v>
@@ -6768,29 +6768,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D187" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E187" t="n">
-        <v>10.708</v>
+        <v>6.862</v>
       </c>
       <c r="F187" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G187" t="n">
-        <v>32.12</v>
+        <v>61.76</v>
       </c>
       <c r="H187" t="n">
-        <v>0.96</v>
+        <v>5.61</v>
       </c>
       <c r="I187" t="n">
-        <v>3.08</v>
+        <v>9.99</v>
       </c>
       <c r="J187" t="n">
         <v>7.91</v>
@@ -6802,29 +6802,29 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D188" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E188" t="n">
-        <v>37.85</v>
+        <v>10.708</v>
       </c>
       <c r="F188" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G188" t="n">
-        <v>151.4</v>
+        <v>32.12</v>
       </c>
       <c r="H188" t="n">
-        <v>12.38</v>
+        <v>0.96</v>
       </c>
       <c r="I188" t="n">
-        <v>8.91</v>
+        <v>3.08</v>
       </c>
       <c r="J188" t="n">
         <v>7.91</v>
@@ -6836,29 +6836,29 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D189" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E189" t="n">
-        <v>22.845</v>
+        <v>37.85</v>
       </c>
       <c r="F189" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G189" t="n">
-        <v>68.53</v>
+        <v>151.4</v>
       </c>
       <c r="H189" t="n">
-        <v>2.86</v>
+        <v>12.38</v>
       </c>
       <c r="I189" t="n">
-        <v>4.36</v>
+        <v>8.91</v>
       </c>
       <c r="J189" t="n">
         <v>7.91</v>
@@ -6870,29 +6870,29 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D190" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E190" t="n">
-        <v>101.44</v>
+        <v>22.845</v>
       </c>
       <c r="F190" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G190" t="n">
-        <v>101.44</v>
+        <v>68.53</v>
       </c>
       <c r="H190" t="n">
-        <v>1.35</v>
+        <v>2.86</v>
       </c>
       <c r="I190" t="n">
-        <v>1.35</v>
+        <v>4.36</v>
       </c>
       <c r="J190" t="n">
         <v>7.91</v>
@@ -6904,31 +6904,201 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E191" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="F191" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G191" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="H191" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="I191" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="J191" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E192" t="n">
+        <v>102.46</v>
+      </c>
+      <c r="F192" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G192" t="n">
+        <v>102.46</v>
+      </c>
+      <c r="H192" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="I192" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="J192" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>3</v>
+      </c>
+      <c r="D193" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E193" t="n">
+        <v>10.792</v>
+      </c>
+      <c r="F193" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G193" t="n">
+        <v>32.38</v>
+      </c>
+      <c r="H193" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="I193" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="J193" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>4</v>
+      </c>
+      <c r="D194" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E194" t="n">
+        <v>38.755</v>
+      </c>
+      <c r="F194" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G194" t="n">
+        <v>155.02</v>
+      </c>
+      <c r="H194" t="n">
+        <v>16</v>
+      </c>
+      <c r="I194" t="n">
+        <v>11.51</v>
+      </c>
+      <c r="J194" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>3</v>
+      </c>
+      <c r="D195" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E195" t="n">
+        <v>22.82</v>
+      </c>
+      <c r="F195" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G195" t="n">
+        <v>68.45999999999999</v>
+      </c>
+      <c r="H195" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="I195" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J195" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="1" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C191" t="n">
+      <c r="C196" t="n">
         <v>9</v>
       </c>
-      <c r="D191" t="n">
+      <c r="D196" t="n">
         <v>6.239</v>
       </c>
-      <c r="E191" t="n">
-        <v>6.862</v>
-      </c>
-      <c r="F191" t="n">
+      <c r="E196" t="n">
+        <v>6.894</v>
+      </c>
+      <c r="F196" t="n">
         <v>56.15</v>
       </c>
-      <c r="G191" t="n">
-        <v>61.76</v>
-      </c>
-      <c r="H191" t="n">
-        <v>5.61</v>
-      </c>
-      <c r="I191" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="J191" t="n">
+      <c r="G196" t="n">
+        <v>62.05</v>
+      </c>
+      <c r="H196" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I196" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="J196" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 22/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J196"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
         <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1158,29 +1158,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C22" t="n">
         <v>3</v>
       </c>
       <c r="D22" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E22" t="n">
-        <v>21.669</v>
+        <v>10.536</v>
       </c>
       <c r="F22" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G22" t="n">
-        <v>65.01000000000001</v>
+        <v>31.61</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.66</v>
+        <v>0.45</v>
       </c>
       <c r="I22" t="n">
-        <v>-1.01</v>
+        <v>1.44</v>
       </c>
       <c r="J22" t="n">
         <v>7.91</v>
@@ -1192,29 +1192,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D23" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E23" t="n">
-        <v>41.336</v>
+        <v>6.799</v>
       </c>
       <c r="F23" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G23" t="n">
-        <v>165.34</v>
+        <v>61.19</v>
       </c>
       <c r="H23" t="n">
-        <v>26.32</v>
+        <v>5.04</v>
       </c>
       <c r="I23" t="n">
-        <v>18.93</v>
+        <v>8.98</v>
       </c>
       <c r="J23" t="n">
         <v>7.91</v>
@@ -1226,29 +1226,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E24" t="n">
-        <v>6.799</v>
+        <v>105.78</v>
       </c>
       <c r="F24" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G24" t="n">
-        <v>61.19</v>
+        <v>105.78</v>
       </c>
       <c r="H24" t="n">
-        <v>5.04</v>
+        <v>5.69</v>
       </c>
       <c r="I24" t="n">
-        <v>8.98</v>
+        <v>5.68</v>
       </c>
       <c r="J24" t="n">
         <v>7.91</v>
@@ -1260,29 +1260,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E25" t="n">
-        <v>105.78</v>
+        <v>21.669</v>
       </c>
       <c r="F25" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G25" t="n">
-        <v>105.78</v>
+        <v>65.01000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>5.69</v>
+        <v>-0.66</v>
       </c>
       <c r="I25" t="n">
-        <v>5.68</v>
+        <v>-1.01</v>
       </c>
       <c r="J25" t="n">
         <v>7.91</v>
@@ -1294,29 +1294,29 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E26" t="n">
-        <v>10.536</v>
+        <v>41.336</v>
       </c>
       <c r="F26" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G26" t="n">
-        <v>31.61</v>
+        <v>165.34</v>
       </c>
       <c r="H26" t="n">
-        <v>0.45</v>
+        <v>26.32</v>
       </c>
       <c r="I26" t="n">
-        <v>1.44</v>
+        <v>18.93</v>
       </c>
       <c r="J26" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E32" t="n">
-        <v>103.08</v>
+        <v>22.053</v>
       </c>
       <c r="F32" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G32" t="n">
-        <v>103.08</v>
+        <v>66.16</v>
       </c>
       <c r="H32" t="n">
-        <v>2.99</v>
+        <v>0.49</v>
       </c>
       <c r="I32" t="n">
-        <v>2.99</v>
+        <v>0.75</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D33" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E33" t="n">
-        <v>10.714</v>
+        <v>6.762</v>
       </c>
       <c r="F33" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G33" t="n">
-        <v>32.14</v>
+        <v>60.86</v>
       </c>
       <c r="H33" t="n">
-        <v>0.98</v>
+        <v>4.71</v>
       </c>
       <c r="I33" t="n">
-        <v>3.15</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D34" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E34" t="n">
-        <v>6.762</v>
+        <v>38.849</v>
       </c>
       <c r="F34" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G34" t="n">
-        <v>60.86</v>
+        <v>155.4</v>
       </c>
       <c r="H34" t="n">
-        <v>4.71</v>
+        <v>16.38</v>
       </c>
       <c r="I34" t="n">
-        <v>8.390000000000001</v>
+        <v>11.78</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E35" t="n">
-        <v>38.849</v>
+        <v>103.08</v>
       </c>
       <c r="F35" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G35" t="n">
-        <v>155.4</v>
+        <v>103.08</v>
       </c>
       <c r="H35" t="n">
-        <v>16.38</v>
+        <v>2.99</v>
       </c>
       <c r="I35" t="n">
-        <v>11.78</v>
+        <v>2.99</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C36" t="n">
         <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E36" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F36" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G36" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H36" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I36" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E42" t="n">
-        <v>38.497</v>
+        <v>100.06</v>
       </c>
       <c r="F42" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G42" t="n">
-        <v>153.99</v>
+        <v>100.06</v>
       </c>
       <c r="H42" t="n">
-        <v>14.97</v>
+        <v>-0.03</v>
       </c>
       <c r="I42" t="n">
-        <v>10.77</v>
+        <v>-0.03</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D43" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E43" t="n">
-        <v>10.61</v>
+        <v>38.497</v>
       </c>
       <c r="F43" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G43" t="n">
-        <v>31.83</v>
+        <v>153.99</v>
       </c>
       <c r="H43" t="n">
-        <v>0.67</v>
+        <v>14.97</v>
       </c>
       <c r="I43" t="n">
-        <v>2.15</v>
+        <v>10.77</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>10.61</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>31.83</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>2.15</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E45" t="n">
-        <v>100.06</v>
+        <v>22</v>
       </c>
       <c r="F45" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G45" t="n">
-        <v>100.06</v>
+        <v>66</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.03</v>
+        <v>0.33</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03</v>
+        <v>0.5</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E47" t="n">
-        <v>21.778</v>
+        <v>99.83</v>
       </c>
       <c r="F47" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G47" t="n">
-        <v>65.33</v>
+        <v>99.83</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.34</v>
+        <v>-0.26</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.52</v>
+        <v>-0.26</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D48" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E48" t="n">
-        <v>6.622</v>
+        <v>10.562</v>
       </c>
       <c r="F48" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G48" t="n">
-        <v>59.6</v>
+        <v>31.69</v>
       </c>
       <c r="H48" t="n">
-        <v>3.45</v>
+        <v>0.53</v>
       </c>
       <c r="I48" t="n">
-        <v>6.14</v>
+        <v>1.7</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2076,29 +2076,29 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E49" t="n">
-        <v>10.562</v>
+        <v>38.312</v>
       </c>
       <c r="F49" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G49" t="n">
-        <v>31.69</v>
+        <v>153.25</v>
       </c>
       <c r="H49" t="n">
-        <v>0.53</v>
+        <v>14.23</v>
       </c>
       <c r="I49" t="n">
-        <v>1.7</v>
+        <v>10.24</v>
       </c>
       <c r="J49" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D50" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E50" t="n">
-        <v>38.312</v>
+        <v>6.622</v>
       </c>
       <c r="F50" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G50" t="n">
-        <v>153.25</v>
+        <v>59.6</v>
       </c>
       <c r="H50" t="n">
-        <v>14.23</v>
+        <v>3.45</v>
       </c>
       <c r="I50" t="n">
-        <v>10.24</v>
+        <v>6.14</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E51" t="n">
-        <v>99.83</v>
+        <v>21.778</v>
       </c>
       <c r="F51" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G51" t="n">
-        <v>99.83</v>
+        <v>65.33</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.26</v>
+        <v>-0.34</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.26</v>
+        <v>-0.52</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E62" t="n">
-        <v>6.817</v>
+        <v>22.7</v>
       </c>
       <c r="F62" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G62" t="n">
-        <v>61.35</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H62" t="n">
-        <v>5.2</v>
+        <v>2.43</v>
       </c>
       <c r="I62" t="n">
-        <v>9.26</v>
+        <v>3.7</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>41.064</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>164.26</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>25.24</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>18.16</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D64" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E64" t="n">
-        <v>105.5</v>
+        <v>6.817</v>
       </c>
       <c r="F64" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G64" t="n">
-        <v>105.5</v>
+        <v>61.35</v>
       </c>
       <c r="H64" t="n">
-        <v>5.41</v>
+        <v>5.2</v>
       </c>
       <c r="I64" t="n">
-        <v>5.41</v>
+        <v>9.26</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>41.064</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>164.26</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>25.24</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>18.16</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E66" t="n">
-        <v>22.7</v>
+        <v>105.5</v>
       </c>
       <c r="F66" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G66" t="n">
-        <v>68.09999999999999</v>
+        <v>105.5</v>
       </c>
       <c r="H66" t="n">
-        <v>2.43</v>
+        <v>5.41</v>
       </c>
       <c r="I66" t="n">
-        <v>3.7</v>
+        <v>5.41</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>10.892</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>32.68</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>1.52</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>23</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>69</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>3.33</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>5.07</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E75" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F75" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G75" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H75" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I75" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E76" t="n">
-        <v>23</v>
+        <v>104.22</v>
       </c>
       <c r="F76" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G76" t="n">
-        <v>69</v>
+        <v>104.22</v>
       </c>
       <c r="H76" t="n">
-        <v>3.33</v>
+        <v>4.13</v>
       </c>
       <c r="I76" t="n">
-        <v>5.07</v>
+        <v>4.13</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E82" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F82" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G82" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H82" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I82" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D83" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E83" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F83" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G83" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H83" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I83" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E84" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F84" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G84" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H84" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I84" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E85" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F85" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G85" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H85" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I85" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C86" t="n">
         <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E86" t="n">
-        <v>23.3</v>
+        <v>10.988</v>
       </c>
       <c r="F86" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G86" t="n">
-        <v>69.90000000000001</v>
+        <v>32.96</v>
       </c>
       <c r="H86" t="n">
-        <v>4.23</v>
+        <v>1.8</v>
       </c>
       <c r="I86" t="n">
-        <v>6.44</v>
+        <v>5.78</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D92" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E92" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F92" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G92" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H92" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I92" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E93" t="n">
-        <v>103.88</v>
+        <v>10.876</v>
       </c>
       <c r="F93" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G93" t="n">
-        <v>103.88</v>
+        <v>32.63</v>
       </c>
       <c r="H93" t="n">
-        <v>3.79</v>
+        <v>1.47</v>
       </c>
       <c r="I93" t="n">
-        <v>3.79</v>
+        <v>4.72</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D94" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E94" t="n">
-        <v>23.025</v>
+        <v>103.88</v>
       </c>
       <c r="F94" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G94" t="n">
-        <v>69.06999999999999</v>
+        <v>103.88</v>
       </c>
       <c r="H94" t="n">
-        <v>3.4</v>
+        <v>3.79</v>
       </c>
       <c r="I94" t="n">
-        <v>5.18</v>
+        <v>3.79</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E95" t="n">
-        <v>6.797</v>
+        <v>23.025</v>
       </c>
       <c r="F95" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G95" t="n">
-        <v>61.17</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H95" t="n">
-        <v>5.02</v>
+        <v>3.4</v>
       </c>
       <c r="I95" t="n">
-        <v>8.94</v>
+        <v>5.18</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E97" t="n">
-        <v>6.839</v>
+        <v>23.35</v>
       </c>
       <c r="F97" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G97" t="n">
-        <v>61.55</v>
+        <v>70.05</v>
       </c>
       <c r="H97" t="n">
-        <v>5.4</v>
+        <v>4.38</v>
       </c>
       <c r="I97" t="n">
-        <v>9.619999999999999</v>
+        <v>6.67</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E98" t="n">
-        <v>10.642</v>
+        <v>104.22</v>
       </c>
       <c r="F98" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G98" t="n">
-        <v>31.93</v>
+        <v>104.22</v>
       </c>
       <c r="H98" t="n">
-        <v>0.77</v>
+        <v>4.13</v>
       </c>
       <c r="I98" t="n">
-        <v>2.47</v>
+        <v>4.13</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D99" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E99" t="n">
-        <v>104.22</v>
+        <v>40.65</v>
       </c>
       <c r="F99" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G99" t="n">
-        <v>104.22</v>
+        <v>162.6</v>
       </c>
       <c r="H99" t="n">
-        <v>4.13</v>
+        <v>23.58</v>
       </c>
       <c r="I99" t="n">
-        <v>4.13</v>
+        <v>16.96</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D100" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E100" t="n">
-        <v>23.35</v>
+        <v>6.839</v>
       </c>
       <c r="F100" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G100" t="n">
-        <v>70.05</v>
+        <v>61.55</v>
       </c>
       <c r="H100" t="n">
-        <v>4.38</v>
+        <v>5.4</v>
       </c>
       <c r="I100" t="n">
-        <v>6.67</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E101" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F101" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G101" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H101" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I101" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D107" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E107" t="n">
-        <v>6.785</v>
+        <v>40.5</v>
       </c>
       <c r="F107" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G107" t="n">
-        <v>61.06</v>
+        <v>162</v>
       </c>
       <c r="H107" t="n">
-        <v>4.91</v>
+        <v>22.98</v>
       </c>
       <c r="I107" t="n">
-        <v>8.74</v>
+        <v>16.53</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E108" t="n">
-        <v>103.14</v>
+        <v>23.33</v>
       </c>
       <c r="F108" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G108" t="n">
-        <v>103.14</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H108" t="n">
-        <v>3.05</v>
+        <v>4.32</v>
       </c>
       <c r="I108" t="n">
-        <v>3.05</v>
+        <v>6.58</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C109" t="n">
         <v>3</v>
       </c>
       <c r="D109" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E109" t="n">
-        <v>23.33</v>
+        <v>10.456</v>
       </c>
       <c r="F109" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G109" t="n">
-        <v>69.98999999999999</v>
+        <v>31.37</v>
       </c>
       <c r="H109" t="n">
-        <v>4.32</v>
+        <v>0.21</v>
       </c>
       <c r="I109" t="n">
-        <v>6.58</v>
+        <v>0.67</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D110" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E110" t="n">
-        <v>40.5</v>
+        <v>6.785</v>
       </c>
       <c r="F110" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G110" t="n">
-        <v>162</v>
+        <v>61.06</v>
       </c>
       <c r="H110" t="n">
-        <v>22.98</v>
+        <v>4.91</v>
       </c>
       <c r="I110" t="n">
-        <v>16.53</v>
+        <v>8.74</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D111" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E111" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F111" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G111" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H111" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I111" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D112" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E112" t="n">
-        <v>6.797</v>
+        <v>40</v>
       </c>
       <c r="F112" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G112" t="n">
-        <v>61.17</v>
+        <v>160</v>
       </c>
       <c r="H112" t="n">
-        <v>5.02</v>
+        <v>20.98</v>
       </c>
       <c r="I112" t="n">
-        <v>8.94</v>
+        <v>15.09</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D113" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E113" t="n">
-        <v>40</v>
+        <v>103.56</v>
       </c>
       <c r="F113" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G113" t="n">
-        <v>160</v>
+        <v>103.56</v>
       </c>
       <c r="H113" t="n">
-        <v>20.98</v>
+        <v>3.47</v>
       </c>
       <c r="I113" t="n">
-        <v>15.09</v>
+        <v>3.47</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E114" t="n">
-        <v>103.56</v>
+        <v>23.025</v>
       </c>
       <c r="F114" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G114" t="n">
-        <v>103.56</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H114" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="I114" t="n">
-        <v>3.47</v>
+        <v>5.18</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C115" t="n">
         <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E115" t="n">
-        <v>23.025</v>
+        <v>10.568</v>
       </c>
       <c r="F115" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G115" t="n">
-        <v>69.06999999999999</v>
+        <v>31.7</v>
       </c>
       <c r="H115" t="n">
-        <v>3.4</v>
+        <v>0.54</v>
       </c>
       <c r="I115" t="n">
-        <v>5.18</v>
+        <v>1.73</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D116" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E116" t="n">
-        <v>10.568</v>
+        <v>6.797</v>
       </c>
       <c r="F116" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G116" t="n">
-        <v>31.7</v>
+        <v>61.17</v>
       </c>
       <c r="H116" t="n">
-        <v>0.54</v>
+        <v>5.02</v>
       </c>
       <c r="I116" t="n">
-        <v>1.73</v>
+        <v>8.94</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D122" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E122" t="n">
-        <v>106</v>
+        <v>40.395</v>
       </c>
       <c r="F122" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G122" t="n">
-        <v>106</v>
+        <v>161.58</v>
       </c>
       <c r="H122" t="n">
-        <v>5.91</v>
+        <v>22.56</v>
       </c>
       <c r="I122" t="n">
-        <v>5.9</v>
+        <v>16.23</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D123" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E123" t="n">
-        <v>23.165</v>
+        <v>6.901</v>
       </c>
       <c r="F123" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G123" t="n">
-        <v>69.5</v>
+        <v>62.11</v>
       </c>
       <c r="H123" t="n">
-        <v>3.83</v>
+        <v>5.96</v>
       </c>
       <c r="I123" t="n">
-        <v>5.83</v>
+        <v>10.61</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D125" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E125" t="n">
-        <v>40.395</v>
+        <v>106</v>
       </c>
       <c r="F125" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G125" t="n">
-        <v>161.58</v>
+        <v>106</v>
       </c>
       <c r="H125" t="n">
-        <v>22.56</v>
+        <v>5.91</v>
       </c>
       <c r="I125" t="n">
-        <v>16.23</v>
+        <v>5.9</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D126" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E126" t="n">
-        <v>6.901</v>
+        <v>23.165</v>
       </c>
       <c r="F126" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G126" t="n">
-        <v>62.11</v>
+        <v>69.5</v>
       </c>
       <c r="H126" t="n">
-        <v>5.96</v>
+        <v>3.83</v>
       </c>
       <c r="I126" t="n">
-        <v>10.61</v>
+        <v>5.83</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E132" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F132" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G132" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H132" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I132" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E133" t="n">
-        <v>23.18</v>
+        <v>40.54</v>
       </c>
       <c r="F133" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G133" t="n">
-        <v>69.54000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="H133" t="n">
-        <v>3.87</v>
+        <v>23.14</v>
       </c>
       <c r="I133" t="n">
-        <v>5.89</v>
+        <v>16.65</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D134" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E134" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F134" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G134" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H134" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I134" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D135" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E135" t="n">
-        <v>11.516</v>
+        <v>104.02</v>
       </c>
       <c r="F135" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G135" t="n">
-        <v>34.55</v>
+        <v>104.02</v>
       </c>
       <c r="H135" t="n">
-        <v>3.39</v>
+        <v>3.93</v>
       </c>
       <c r="I135" t="n">
-        <v>10.88</v>
+        <v>3.93</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E136" t="n">
-        <v>6.895</v>
+        <v>23.18</v>
       </c>
       <c r="F136" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G136" t="n">
-        <v>62.05</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H136" t="n">
-        <v>5.9</v>
+        <v>3.87</v>
       </c>
       <c r="I136" t="n">
-        <v>10.51</v>
+        <v>5.89</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D147" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E147" t="n">
-        <v>6.826</v>
+        <v>38.955</v>
       </c>
       <c r="F147" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G147" t="n">
-        <v>61.43</v>
+        <v>155.82</v>
       </c>
       <c r="H147" t="n">
-        <v>5.28</v>
+        <v>16.8</v>
       </c>
       <c r="I147" t="n">
-        <v>9.4</v>
+        <v>12.08</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D148" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E148" t="n">
-        <v>22.755</v>
+        <v>101.7</v>
       </c>
       <c r="F148" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G148" t="n">
-        <v>68.27</v>
+        <v>101.7</v>
       </c>
       <c r="H148" t="n">
-        <v>2.6</v>
+        <v>1.61</v>
       </c>
       <c r="I148" t="n">
-        <v>3.96</v>
+        <v>1.61</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5476,29 +5476,29 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E149" t="n">
-        <v>101.7</v>
+        <v>11.162</v>
       </c>
       <c r="F149" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G149" t="n">
-        <v>101.7</v>
+        <v>33.49</v>
       </c>
       <c r="H149" t="n">
-        <v>1.61</v>
+        <v>2.33</v>
       </c>
       <c r="I149" t="n">
-        <v>1.61</v>
+        <v>7.48</v>
       </c>
       <c r="J149" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D150" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E150" t="n">
-        <v>11.162</v>
+        <v>6.826</v>
       </c>
       <c r="F150" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G150" t="n">
-        <v>33.49</v>
+        <v>61.43</v>
       </c>
       <c r="H150" t="n">
-        <v>2.33</v>
+        <v>5.28</v>
       </c>
       <c r="I150" t="n">
-        <v>7.48</v>
+        <v>9.4</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E151" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F151" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G151" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H151" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I151" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C157" t="n">
         <v>3</v>
       </c>
       <c r="D157" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E157" t="n">
-        <v>10.92</v>
+        <v>23.08</v>
       </c>
       <c r="F157" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G157" t="n">
-        <v>32.76</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H157" t="n">
-        <v>1.6</v>
+        <v>3.57</v>
       </c>
       <c r="I157" t="n">
-        <v>5.13</v>
+        <v>5.44</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D158" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E158" t="n">
-        <v>40.015</v>
+        <v>104.5</v>
       </c>
       <c r="F158" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G158" t="n">
-        <v>160.06</v>
+        <v>104.5</v>
       </c>
       <c r="H158" t="n">
-        <v>21.04</v>
+        <v>4.41</v>
       </c>
       <c r="I158" t="n">
-        <v>15.13</v>
+        <v>4.41</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D159" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E159" t="n">
-        <v>104.5</v>
+        <v>6.913</v>
       </c>
       <c r="F159" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G159" t="n">
-        <v>104.5</v>
+        <v>62.22</v>
       </c>
       <c r="H159" t="n">
-        <v>4.41</v>
+        <v>6.07</v>
       </c>
       <c r="I159" t="n">
-        <v>4.41</v>
+        <v>10.81</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C160" t="n">
         <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E160" t="n">
-        <v>23.08</v>
+        <v>10.92</v>
       </c>
       <c r="F160" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G160" t="n">
-        <v>69.23999999999999</v>
+        <v>32.76</v>
       </c>
       <c r="H160" t="n">
-        <v>3.57</v>
+        <v>1.6</v>
       </c>
       <c r="I160" t="n">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D161" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E161" t="n">
-        <v>6.913</v>
+        <v>40.015</v>
       </c>
       <c r="F161" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G161" t="n">
-        <v>62.22</v>
+        <v>160.06</v>
       </c>
       <c r="H161" t="n">
-        <v>6.07</v>
+        <v>21.04</v>
       </c>
       <c r="I161" t="n">
-        <v>10.81</v>
+        <v>15.13</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6258,29 +6258,29 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D172" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E172" t="n">
-        <v>103.22</v>
+        <v>10.712</v>
       </c>
       <c r="F172" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G172" t="n">
-        <v>103.22</v>
+        <v>32.14</v>
       </c>
       <c r="H172" t="n">
-        <v>3.13</v>
+        <v>0.98</v>
       </c>
       <c r="I172" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
       <c r="J172" t="n">
         <v>7.91</v>
@@ -6292,29 +6292,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D173" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E173" t="n">
-        <v>38.74</v>
+        <v>22.95</v>
       </c>
       <c r="F173" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G173" t="n">
-        <v>154.96</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H173" t="n">
-        <v>15.94</v>
+        <v>3.18</v>
       </c>
       <c r="I173" t="n">
-        <v>11.47</v>
+        <v>4.84</v>
       </c>
       <c r="J173" t="n">
         <v>7.91</v>
@@ -6326,29 +6326,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D174" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E174" t="n">
-        <v>22.95</v>
+        <v>6.926</v>
       </c>
       <c r="F174" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G174" t="n">
-        <v>68.84999999999999</v>
+        <v>62.33</v>
       </c>
       <c r="H174" t="n">
-        <v>3.18</v>
+        <v>6.18</v>
       </c>
       <c r="I174" t="n">
-        <v>4.84</v>
+        <v>11.01</v>
       </c>
       <c r="J174" t="n">
         <v>7.91</v>
@@ -6360,29 +6360,29 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D175" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E175" t="n">
-        <v>6.926</v>
+        <v>103.22</v>
       </c>
       <c r="F175" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G175" t="n">
-        <v>62.33</v>
+        <v>103.22</v>
       </c>
       <c r="H175" t="n">
-        <v>6.18</v>
+        <v>3.13</v>
       </c>
       <c r="I175" t="n">
-        <v>11.01</v>
+        <v>3.13</v>
       </c>
       <c r="J175" t="n">
         <v>7.91</v>
@@ -6394,29 +6394,29 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E176" t="n">
-        <v>10.712</v>
+        <v>38.74</v>
       </c>
       <c r="F176" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G176" t="n">
-        <v>32.14</v>
+        <v>154.96</v>
       </c>
       <c r="H176" t="n">
-        <v>0.98</v>
+        <v>15.94</v>
       </c>
       <c r="I176" t="n">
-        <v>3.15</v>
+        <v>11.47</v>
       </c>
       <c r="J176" t="n">
         <v>7.91</v>
@@ -6768,29 +6768,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D187" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E187" t="n">
-        <v>6.862</v>
+        <v>101.44</v>
       </c>
       <c r="F187" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G187" t="n">
-        <v>61.76</v>
+        <v>101.44</v>
       </c>
       <c r="H187" t="n">
-        <v>5.61</v>
+        <v>1.35</v>
       </c>
       <c r="I187" t="n">
-        <v>9.99</v>
+        <v>1.35</v>
       </c>
       <c r="J187" t="n">
         <v>7.91</v>
@@ -6802,29 +6802,29 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C188" t="n">
         <v>3</v>
       </c>
       <c r="D188" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E188" t="n">
-        <v>10.708</v>
+        <v>22.845</v>
       </c>
       <c r="F188" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G188" t="n">
-        <v>32.12</v>
+        <v>68.53</v>
       </c>
       <c r="H188" t="n">
-        <v>0.96</v>
+        <v>2.86</v>
       </c>
       <c r="I188" t="n">
-        <v>3.08</v>
+        <v>4.36</v>
       </c>
       <c r="J188" t="n">
         <v>7.91</v>
@@ -6836,29 +6836,29 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D189" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E189" t="n">
-        <v>37.85</v>
+        <v>10.708</v>
       </c>
       <c r="F189" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G189" t="n">
-        <v>151.4</v>
+        <v>32.12</v>
       </c>
       <c r="H189" t="n">
-        <v>12.38</v>
+        <v>0.96</v>
       </c>
       <c r="I189" t="n">
-        <v>8.91</v>
+        <v>3.08</v>
       </c>
       <c r="J189" t="n">
         <v>7.91</v>
@@ -6870,29 +6870,29 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D190" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E190" t="n">
-        <v>22.845</v>
+        <v>6.862</v>
       </c>
       <c r="F190" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G190" t="n">
-        <v>68.53</v>
+        <v>61.76</v>
       </c>
       <c r="H190" t="n">
-        <v>2.86</v>
+        <v>5.61</v>
       </c>
       <c r="I190" t="n">
-        <v>4.36</v>
+        <v>9.99</v>
       </c>
       <c r="J190" t="n">
         <v>7.91</v>
@@ -6904,29 +6904,29 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D191" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E191" t="n">
-        <v>101.44</v>
+        <v>37.85</v>
       </c>
       <c r="F191" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G191" t="n">
-        <v>101.44</v>
+        <v>151.4</v>
       </c>
       <c r="H191" t="n">
-        <v>1.35</v>
+        <v>12.38</v>
       </c>
       <c r="I191" t="n">
-        <v>1.35</v>
+        <v>8.91</v>
       </c>
       <c r="J191" t="n">
         <v>7.91</v>
@@ -7099,6 +7099,176 @@
         <v>10.51</v>
       </c>
       <c r="J196" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>3</v>
+      </c>
+      <c r="D197" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E197" t="n">
+        <v>11.022</v>
+      </c>
+      <c r="F197" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G197" t="n">
+        <v>33.07</v>
+      </c>
+      <c r="H197" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="I197" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="J197" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>4</v>
+      </c>
+      <c r="D198" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E198" t="n">
+        <v>38.565</v>
+      </c>
+      <c r="F198" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G198" t="n">
+        <v>154.26</v>
+      </c>
+      <c r="H198" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="I198" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="J198" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>3</v>
+      </c>
+      <c r="D199" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E199" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="F199" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G199" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="H199" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="I199" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="J199" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>1</v>
+      </c>
+      <c r="D200" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E200" t="n">
+        <v>102.48</v>
+      </c>
+      <c r="F200" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G200" t="n">
+        <v>102.48</v>
+      </c>
+      <c r="H200" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="I200" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="J200" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="1" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>9</v>
+      </c>
+      <c r="D201" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E201" t="n">
+        <v>6.909</v>
+      </c>
+      <c r="F201" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G201" t="n">
+        <v>62.18</v>
+      </c>
+      <c r="H201" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="I201" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="J201" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 23/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E28" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F28" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G28" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H28" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I28" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E29" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F29" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G29" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H29" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I29" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E31" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F31" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G31" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H31" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I31" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D37" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E37" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F37" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G37" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H37" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I37" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E38" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F38" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G38" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E39" t="n">
-        <v>10.67</v>
+        <v>102.8</v>
       </c>
       <c r="F39" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G39" t="n">
-        <v>32.01</v>
+        <v>102.8</v>
       </c>
       <c r="H39" t="n">
-        <v>0.85</v>
+        <v>2.71</v>
       </c>
       <c r="I39" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E40" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F40" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G40" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H40" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I40" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E41" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F41" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G41" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H41" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I41" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E52" t="n">
-        <v>6.629</v>
+        <v>21.703</v>
       </c>
       <c r="F52" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G52" t="n">
-        <v>59.66</v>
+        <v>65.11</v>
       </c>
       <c r="H52" t="n">
-        <v>3.51</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I52" t="n">
-        <v>6.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E53" t="n">
-        <v>10.702</v>
+        <v>100.34</v>
       </c>
       <c r="F53" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G53" t="n">
-        <v>32.11</v>
+        <v>100.34</v>
       </c>
       <c r="H53" t="n">
-        <v>0.95</v>
+        <v>0.25</v>
       </c>
       <c r="I53" t="n">
-        <v>3.05</v>
+        <v>0.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D54" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E54" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F54" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G54" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H54" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I54" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D55" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E55" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F55" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G55" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H55" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I55" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D56" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E56" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F56" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G56" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I56" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E62" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F62" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G62" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H62" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I62" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D63" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E63" t="n">
-        <v>41.064</v>
+        <v>6.817</v>
       </c>
       <c r="F63" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G63" t="n">
-        <v>164.26</v>
+        <v>61.35</v>
       </c>
       <c r="H63" t="n">
-        <v>25.24</v>
+        <v>5.2</v>
       </c>
       <c r="I63" t="n">
-        <v>18.16</v>
+        <v>9.26</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E64" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F64" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G64" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H64" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I64" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E65" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F65" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G65" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H65" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I65" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D66" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E66" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F66" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G66" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H66" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I66" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E67" t="n">
-        <v>6.807</v>
+        <v>10.796</v>
       </c>
       <c r="F67" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G67" t="n">
-        <v>61.26</v>
+        <v>32.39</v>
       </c>
       <c r="H67" t="n">
-        <v>5.11</v>
+        <v>1.23</v>
       </c>
       <c r="I67" t="n">
-        <v>9.1</v>
+        <v>3.95</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D68" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E68" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F68" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G68" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H68" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I68" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E69" t="n">
-        <v>40.567</v>
+        <v>22.797</v>
       </c>
       <c r="F69" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G69" t="n">
-        <v>162.27</v>
+        <v>68.39</v>
       </c>
       <c r="H69" t="n">
-        <v>23.25</v>
+        <v>2.72</v>
       </c>
       <c r="I69" t="n">
-        <v>16.72</v>
+        <v>4.14</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E70" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F70" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G70" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H70" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I70" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D71" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E71" t="n">
-        <v>104.58</v>
+        <v>6.807</v>
       </c>
       <c r="F71" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G71" t="n">
-        <v>104.58</v>
+        <v>61.26</v>
       </c>
       <c r="H71" t="n">
-        <v>4.49</v>
+        <v>5.11</v>
       </c>
       <c r="I71" t="n">
-        <v>4.49</v>
+        <v>9.1</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D77" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E77" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F77" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G77" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H77" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I77" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D78" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E78" t="n">
-        <v>23.4</v>
+        <v>6.836</v>
       </c>
       <c r="F78" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G78" t="n">
-        <v>70.2</v>
+        <v>61.52</v>
       </c>
       <c r="H78" t="n">
-        <v>4.53</v>
+        <v>5.37</v>
       </c>
       <c r="I78" t="n">
-        <v>6.9</v>
+        <v>9.56</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E80" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F80" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G80" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H80" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I80" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E81" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F81" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G81" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H81" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I81" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E87" t="n">
-        <v>6.856</v>
+        <v>43.005</v>
       </c>
       <c r="F87" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G87" t="n">
-        <v>61.7</v>
+        <v>172.02</v>
       </c>
       <c r="H87" t="n">
-        <v>5.55</v>
+        <v>33</v>
       </c>
       <c r="I87" t="n">
-        <v>9.880000000000001</v>
+        <v>23.74</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E88" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F88" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G88" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H88" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I88" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C89" t="n">
         <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E89" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F89" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G89" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H89" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I89" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D90" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E90" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F90" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G90" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H90" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I90" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E91" t="n">
-        <v>23.32</v>
+        <v>106.28</v>
       </c>
       <c r="F91" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G91" t="n">
-        <v>69.95999999999999</v>
+        <v>106.28</v>
       </c>
       <c r="H91" t="n">
-        <v>4.29</v>
+        <v>6.19</v>
       </c>
       <c r="I91" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E102" t="n">
-        <v>103.46</v>
+        <v>23.29</v>
       </c>
       <c r="F102" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G102" t="n">
-        <v>103.46</v>
+        <v>69.87</v>
       </c>
       <c r="H102" t="n">
-        <v>3.37</v>
+        <v>4.2</v>
       </c>
       <c r="I102" t="n">
-        <v>3.37</v>
+        <v>6.4</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E103" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F103" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G103" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H103" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I103" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D105" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E105" t="n">
-        <v>10.556</v>
+        <v>40.97</v>
       </c>
       <c r="F105" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G105" t="n">
-        <v>31.67</v>
+        <v>163.88</v>
       </c>
       <c r="H105" t="n">
-        <v>0.51</v>
+        <v>24.86</v>
       </c>
       <c r="I105" t="n">
-        <v>1.64</v>
+        <v>17.88</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D106" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E106" t="n">
-        <v>23.29</v>
+        <v>103.46</v>
       </c>
       <c r="F106" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G106" t="n">
-        <v>69.87</v>
+        <v>103.46</v>
       </c>
       <c r="H106" t="n">
-        <v>4.2</v>
+        <v>3.37</v>
       </c>
       <c r="I106" t="n">
-        <v>6.4</v>
+        <v>3.37</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E112" t="n">
-        <v>40</v>
+        <v>10.568</v>
       </c>
       <c r="F112" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G112" t="n">
-        <v>160</v>
+        <v>31.7</v>
       </c>
       <c r="H112" t="n">
-        <v>20.98</v>
+        <v>0.54</v>
       </c>
       <c r="I112" t="n">
-        <v>15.09</v>
+        <v>1.73</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E113" t="n">
-        <v>103.56</v>
+        <v>23.025</v>
       </c>
       <c r="F113" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G113" t="n">
-        <v>103.56</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H113" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="I113" t="n">
-        <v>3.47</v>
+        <v>5.18</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D114" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E114" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F114" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G114" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H114" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I114" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D115" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E115" t="n">
-        <v>10.568</v>
+        <v>40</v>
       </c>
       <c r="F115" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G115" t="n">
-        <v>31.7</v>
+        <v>160</v>
       </c>
       <c r="H115" t="n">
-        <v>0.54</v>
+        <v>20.98</v>
       </c>
       <c r="I115" t="n">
-        <v>1.73</v>
+        <v>15.09</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D116" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E116" t="n">
-        <v>6.797</v>
+        <v>103.56</v>
       </c>
       <c r="F116" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G116" t="n">
-        <v>61.17</v>
+        <v>103.56</v>
       </c>
       <c r="H116" t="n">
-        <v>5.02</v>
+        <v>3.47</v>
       </c>
       <c r="I116" t="n">
-        <v>8.94</v>
+        <v>3.47</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D127" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E127" t="n">
-        <v>103.46</v>
+        <v>6.868</v>
       </c>
       <c r="F127" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G127" t="n">
-        <v>103.46</v>
+        <v>61.81</v>
       </c>
       <c r="H127" t="n">
-        <v>3.37</v>
+        <v>5.66</v>
       </c>
       <c r="I127" t="n">
-        <v>3.37</v>
+        <v>10.08</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D128" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E128" t="n">
-        <v>23.17</v>
+        <v>39.36</v>
       </c>
       <c r="F128" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G128" t="n">
-        <v>69.51000000000001</v>
+        <v>157.44</v>
       </c>
       <c r="H128" t="n">
-        <v>3.84</v>
+        <v>18.42</v>
       </c>
       <c r="I128" t="n">
-        <v>5.85</v>
+        <v>13.25</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E130" t="n">
-        <v>39.36</v>
+        <v>23.17</v>
       </c>
       <c r="F130" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G130" t="n">
-        <v>157.44</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H130" t="n">
-        <v>18.42</v>
+        <v>3.84</v>
       </c>
       <c r="I130" t="n">
-        <v>13.25</v>
+        <v>5.85</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D131" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E131" t="n">
-        <v>6.868</v>
+        <v>103.46</v>
       </c>
       <c r="F131" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G131" t="n">
-        <v>61.81</v>
+        <v>103.46</v>
       </c>
       <c r="H131" t="n">
-        <v>5.66</v>
+        <v>3.37</v>
       </c>
       <c r="I131" t="n">
-        <v>10.08</v>
+        <v>3.37</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D137" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E137" t="n">
-        <v>11.728</v>
+        <v>104.76</v>
       </c>
       <c r="F137" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G137" t="n">
-        <v>35.18</v>
+        <v>104.76</v>
       </c>
       <c r="H137" t="n">
-        <v>4.02</v>
+        <v>4.67</v>
       </c>
       <c r="I137" t="n">
-        <v>12.9</v>
+        <v>4.67</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D138" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E138" t="n">
-        <v>6.927</v>
+        <v>40.61</v>
       </c>
       <c r="F138" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G138" t="n">
-        <v>62.34</v>
+        <v>162.44</v>
       </c>
       <c r="H138" t="n">
-        <v>6.19</v>
+        <v>23.42</v>
       </c>
       <c r="I138" t="n">
-        <v>11.02</v>
+        <v>16.85</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D139" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E139" t="n">
-        <v>40.61</v>
+        <v>23.3</v>
       </c>
       <c r="F139" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G139" t="n">
-        <v>162.44</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H139" t="n">
-        <v>23.42</v>
+        <v>4.23</v>
       </c>
       <c r="I139" t="n">
-        <v>16.85</v>
+        <v>6.44</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E140" t="n">
-        <v>104.76</v>
+        <v>11.728</v>
       </c>
       <c r="F140" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G140" t="n">
-        <v>104.76</v>
+        <v>35.18</v>
       </c>
       <c r="H140" t="n">
-        <v>4.67</v>
+        <v>4.02</v>
       </c>
       <c r="I140" t="n">
-        <v>4.67</v>
+        <v>12.9</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D141" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E141" t="n">
-        <v>23.3</v>
+        <v>6.927</v>
       </c>
       <c r="F141" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G141" t="n">
-        <v>69.90000000000001</v>
+        <v>62.34</v>
       </c>
       <c r="H141" t="n">
-        <v>4.23</v>
+        <v>6.19</v>
       </c>
       <c r="I141" t="n">
-        <v>6.44</v>
+        <v>11.02</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C152" t="n">
         <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E152" t="n">
-        <v>11.034</v>
+        <v>23.045</v>
       </c>
       <c r="F152" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G152" t="n">
-        <v>33.1</v>
+        <v>69.14</v>
       </c>
       <c r="H152" t="n">
-        <v>1.94</v>
+        <v>3.47</v>
       </c>
       <c r="I152" t="n">
-        <v>6.23</v>
+        <v>5.28</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D153" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E153" t="n">
-        <v>104.12</v>
+        <v>39.915</v>
       </c>
       <c r="F153" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G153" t="n">
-        <v>104.12</v>
+        <v>159.66</v>
       </c>
       <c r="H153" t="n">
-        <v>4.03</v>
+        <v>20.64</v>
       </c>
       <c r="I153" t="n">
-        <v>4.03</v>
+        <v>14.85</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5646,29 +5646,29 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D154" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E154" t="n">
-        <v>39.915</v>
+        <v>6.893</v>
       </c>
       <c r="F154" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G154" t="n">
-        <v>159.66</v>
+        <v>62.04</v>
       </c>
       <c r="H154" t="n">
-        <v>20.64</v>
+        <v>5.89</v>
       </c>
       <c r="I154" t="n">
-        <v>14.85</v>
+        <v>10.49</v>
       </c>
       <c r="J154" t="n">
         <v>7.91</v>
@@ -5680,29 +5680,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E155" t="n">
-        <v>6.893</v>
+        <v>104.12</v>
       </c>
       <c r="F155" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G155" t="n">
-        <v>62.04</v>
+        <v>104.12</v>
       </c>
       <c r="H155" t="n">
-        <v>5.89</v>
+        <v>4.03</v>
       </c>
       <c r="I155" t="n">
-        <v>10.49</v>
+        <v>4.03</v>
       </c>
       <c r="J155" t="n">
         <v>7.91</v>
@@ -5714,29 +5714,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C156" t="n">
         <v>3</v>
       </c>
       <c r="D156" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E156" t="n">
-        <v>23.045</v>
+        <v>11.034</v>
       </c>
       <c r="F156" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G156" t="n">
-        <v>69.14</v>
+        <v>33.1</v>
       </c>
       <c r="H156" t="n">
-        <v>3.47</v>
+        <v>1.94</v>
       </c>
       <c r="I156" t="n">
-        <v>5.28</v>
+        <v>6.23</v>
       </c>
       <c r="J156" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C162" t="n">
         <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E162" t="n">
-        <v>23.01</v>
+        <v>10.748</v>
       </c>
       <c r="F162" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G162" t="n">
-        <v>69.03</v>
+        <v>32.24</v>
       </c>
       <c r="H162" t="n">
-        <v>3.36</v>
+        <v>1.08</v>
       </c>
       <c r="I162" t="n">
-        <v>5.12</v>
+        <v>3.47</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D163" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E163" t="n">
-        <v>6.927</v>
+        <v>103.84</v>
       </c>
       <c r="F163" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G163" t="n">
-        <v>62.34</v>
+        <v>103.84</v>
       </c>
       <c r="H163" t="n">
-        <v>6.19</v>
+        <v>3.75</v>
       </c>
       <c r="I163" t="n">
-        <v>11.02</v>
+        <v>3.75</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -5986,29 +5986,29 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D164" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E164" t="n">
-        <v>103.84</v>
+        <v>38.845</v>
       </c>
       <c r="F164" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G164" t="n">
-        <v>103.84</v>
+        <v>155.38</v>
       </c>
       <c r="H164" t="n">
-        <v>3.75</v>
+        <v>16.36</v>
       </c>
       <c r="I164" t="n">
-        <v>3.75</v>
+        <v>11.77</v>
       </c>
       <c r="J164" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C165" t="n">
         <v>3</v>
       </c>
       <c r="D165" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E165" t="n">
-        <v>10.748</v>
+        <v>23.01</v>
       </c>
       <c r="F165" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G165" t="n">
-        <v>32.24</v>
+        <v>69.03</v>
       </c>
       <c r="H165" t="n">
-        <v>1.08</v>
+        <v>3.36</v>
       </c>
       <c r="I165" t="n">
-        <v>3.47</v>
+        <v>5.12</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D166" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E166" t="n">
-        <v>38.845</v>
+        <v>6.927</v>
       </c>
       <c r="F166" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G166" t="n">
-        <v>155.38</v>
+        <v>62.34</v>
       </c>
       <c r="H166" t="n">
-        <v>16.36</v>
+        <v>6.19</v>
       </c>
       <c r="I166" t="n">
-        <v>11.77</v>
+        <v>11.02</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D177" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E177" t="n">
-        <v>102.54</v>
+        <v>10.642</v>
       </c>
       <c r="F177" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G177" t="n">
-        <v>102.54</v>
+        <v>31.93</v>
       </c>
       <c r="H177" t="n">
-        <v>2.45</v>
+        <v>0.77</v>
       </c>
       <c r="I177" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D178" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E178" t="n">
-        <v>38.245</v>
+        <v>6.922</v>
       </c>
       <c r="F178" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G178" t="n">
-        <v>152.98</v>
+        <v>62.3</v>
       </c>
       <c r="H178" t="n">
-        <v>13.96</v>
+        <v>6.15</v>
       </c>
       <c r="I178" t="n">
-        <v>10.04</v>
+        <v>10.95</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D179" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E179" t="n">
-        <v>22.95</v>
+        <v>38.245</v>
       </c>
       <c r="F179" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G179" t="n">
-        <v>68.84999999999999</v>
+        <v>152.98</v>
       </c>
       <c r="H179" t="n">
-        <v>3.18</v>
+        <v>13.96</v>
       </c>
       <c r="I179" t="n">
-        <v>4.84</v>
+        <v>10.04</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D180" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E180" t="n">
-        <v>6.922</v>
+        <v>102.54</v>
       </c>
       <c r="F180" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G180" t="n">
-        <v>62.3</v>
+        <v>102.54</v>
       </c>
       <c r="H180" t="n">
-        <v>6.15</v>
+        <v>2.45</v>
       </c>
       <c r="I180" t="n">
-        <v>10.95</v>
+        <v>2.45</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,29 +6564,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C181" t="n">
         <v>3</v>
       </c>
       <c r="D181" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E181" t="n">
-        <v>10.642</v>
+        <v>22.95</v>
       </c>
       <c r="F181" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G181" t="n">
-        <v>31.93</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H181" t="n">
-        <v>0.77</v>
+        <v>3.18</v>
       </c>
       <c r="I181" t="n">
-        <v>2.47</v>
+        <v>4.84</v>
       </c>
       <c r="J181" t="n">
         <v>7.91</v>
@@ -6768,29 +6768,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E187" t="n">
-        <v>101.44</v>
+        <v>37.85</v>
       </c>
       <c r="F187" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G187" t="n">
-        <v>101.44</v>
+        <v>151.4</v>
       </c>
       <c r="H187" t="n">
-        <v>1.35</v>
+        <v>12.38</v>
       </c>
       <c r="I187" t="n">
-        <v>1.35</v>
+        <v>8.91</v>
       </c>
       <c r="J187" t="n">
         <v>7.91</v>
@@ -6802,29 +6802,29 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D188" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E188" t="n">
-        <v>22.845</v>
+        <v>6.862</v>
       </c>
       <c r="F188" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G188" t="n">
-        <v>68.53</v>
+        <v>61.76</v>
       </c>
       <c r="H188" t="n">
-        <v>2.86</v>
+        <v>5.61</v>
       </c>
       <c r="I188" t="n">
-        <v>4.36</v>
+        <v>9.99</v>
       </c>
       <c r="J188" t="n">
         <v>7.91</v>
@@ -6870,29 +6870,29 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D190" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E190" t="n">
-        <v>6.862</v>
+        <v>22.845</v>
       </c>
       <c r="F190" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G190" t="n">
-        <v>61.76</v>
+        <v>68.53</v>
       </c>
       <c r="H190" t="n">
-        <v>5.61</v>
+        <v>2.86</v>
       </c>
       <c r="I190" t="n">
-        <v>9.99</v>
+        <v>4.36</v>
       </c>
       <c r="J190" t="n">
         <v>7.91</v>
@@ -6904,29 +6904,29 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D191" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E191" t="n">
-        <v>37.85</v>
+        <v>101.44</v>
       </c>
       <c r="F191" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G191" t="n">
-        <v>151.4</v>
+        <v>101.44</v>
       </c>
       <c r="H191" t="n">
-        <v>12.38</v>
+        <v>1.35</v>
       </c>
       <c r="I191" t="n">
-        <v>8.91</v>
+        <v>1.35</v>
       </c>
       <c r="J191" t="n">
         <v>7.91</v>
@@ -7108,29 +7108,29 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D197" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E197" t="n">
-        <v>11.022</v>
+        <v>102.48</v>
       </c>
       <c r="F197" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G197" t="n">
-        <v>33.07</v>
+        <v>102.48</v>
       </c>
       <c r="H197" t="n">
-        <v>1.91</v>
+        <v>2.39</v>
       </c>
       <c r="I197" t="n">
-        <v>6.13</v>
+        <v>2.39</v>
       </c>
       <c r="J197" t="n">
         <v>7.91</v>
@@ -7142,29 +7142,29 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D198" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E198" t="n">
-        <v>38.565</v>
+        <v>22.6</v>
       </c>
       <c r="F198" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G198" t="n">
-        <v>154.26</v>
+        <v>67.8</v>
       </c>
       <c r="H198" t="n">
-        <v>15.24</v>
+        <v>2.13</v>
       </c>
       <c r="I198" t="n">
-        <v>10.96</v>
+        <v>3.24</v>
       </c>
       <c r="J198" t="n">
         <v>7.91</v>
@@ -7176,29 +7176,29 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D199" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E199" t="n">
-        <v>22.6</v>
+        <v>6.909</v>
       </c>
       <c r="F199" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G199" t="n">
-        <v>67.8</v>
+        <v>62.18</v>
       </c>
       <c r="H199" t="n">
-        <v>2.13</v>
+        <v>6.03</v>
       </c>
       <c r="I199" t="n">
-        <v>3.24</v>
+        <v>10.74</v>
       </c>
       <c r="J199" t="n">
         <v>7.91</v>
@@ -7210,29 +7210,29 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D200" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E200" t="n">
-        <v>102.48</v>
+        <v>11.022</v>
       </c>
       <c r="F200" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G200" t="n">
-        <v>102.48</v>
+        <v>33.07</v>
       </c>
       <c r="H200" t="n">
-        <v>2.39</v>
+        <v>1.91</v>
       </c>
       <c r="I200" t="n">
-        <v>2.39</v>
+        <v>6.13</v>
       </c>
       <c r="J200" t="n">
         <v>7.91</v>
@@ -7244,31 +7244,201 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>4</v>
+      </c>
+      <c r="D201" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E201" t="n">
+        <v>38.565</v>
+      </c>
+      <c r="F201" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G201" t="n">
+        <v>154.26</v>
+      </c>
+      <c r="H201" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="I201" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="J201" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E202" t="n">
+        <v>100.08</v>
+      </c>
+      <c r="F202" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G202" t="n">
+        <v>100.08</v>
+      </c>
+      <c r="H202" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="I202" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="J202" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>3</v>
+      </c>
+      <c r="D203" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E203" t="n">
+        <v>11.044</v>
+      </c>
+      <c r="F203" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G203" t="n">
+        <v>33.13</v>
+      </c>
+      <c r="H203" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="I203" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="J203" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>4</v>
+      </c>
+      <c r="D204" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E204" t="n">
+        <v>38.04</v>
+      </c>
+      <c r="F204" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G204" t="n">
+        <v>152.16</v>
+      </c>
+      <c r="H204" t="n">
+        <v>13.14</v>
+      </c>
+      <c r="I204" t="n">
+        <v>9.449999999999999</v>
+      </c>
+      <c r="J204" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>3</v>
+      </c>
+      <c r="D205" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E205" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="F205" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G205" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="H205" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="I205" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="J205" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C201" t="n">
+      <c r="C206" t="n">
         <v>9</v>
       </c>
-      <c r="D201" t="n">
+      <c r="D206" t="n">
         <v>6.239</v>
       </c>
-      <c r="E201" t="n">
-        <v>6.909</v>
-      </c>
-      <c r="F201" t="n">
+      <c r="E206" t="n">
+        <v>6.822</v>
+      </c>
+      <c r="F206" t="n">
         <v>56.15</v>
       </c>
-      <c r="G201" t="n">
-        <v>62.18</v>
-      </c>
-      <c r="H201" t="n">
-        <v>6.03</v>
-      </c>
-      <c r="I201" t="n">
-        <v>10.74</v>
-      </c>
-      <c r="J201" t="n">
+      <c r="G206" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="H206" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="I206" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="J206" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 24/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J206"/>
+  <dimension ref="A1:J211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E27" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F27" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G27" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H27" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I27" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E28" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F28" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G28" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H28" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I28" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E31" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F31" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G31" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H31" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I31" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E37" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F37" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G37" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H37" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I37" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E38" t="n">
-        <v>10.67</v>
+        <v>102.8</v>
       </c>
       <c r="F38" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G38" t="n">
-        <v>32.01</v>
+        <v>102.8</v>
       </c>
       <c r="H38" t="n">
-        <v>0.85</v>
+        <v>2.71</v>
       </c>
       <c r="I38" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E39" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F39" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G39" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H39" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I39" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E40" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F40" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G40" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H40" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I40" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C41" t="n">
         <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E41" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F41" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G41" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I41" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E52" t="n">
-        <v>21.703</v>
+        <v>38.544</v>
       </c>
       <c r="F52" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G52" t="n">
-        <v>65.11</v>
+        <v>154.18</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.5600000000000001</v>
+        <v>15.16</v>
       </c>
       <c r="I52" t="n">
-        <v>-0.85</v>
+        <v>10.9</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E53" t="n">
-        <v>100.34</v>
+        <v>10.702</v>
       </c>
       <c r="F53" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G53" t="n">
-        <v>100.34</v>
+        <v>32.11</v>
       </c>
       <c r="H53" t="n">
-        <v>0.25</v>
+        <v>0.95</v>
       </c>
       <c r="I53" t="n">
-        <v>0.25</v>
+        <v>3.05</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E54" t="n">
-        <v>6.629</v>
+        <v>21.703</v>
       </c>
       <c r="F54" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G54" t="n">
-        <v>59.66</v>
+        <v>65.11</v>
       </c>
       <c r="H54" t="n">
-        <v>3.51</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I54" t="n">
-        <v>6.25</v>
+        <v>-0.85</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E55" t="n">
-        <v>10.702</v>
+        <v>100.34</v>
       </c>
       <c r="F55" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G55" t="n">
-        <v>32.11</v>
+        <v>100.34</v>
       </c>
       <c r="H55" t="n">
-        <v>0.95</v>
+        <v>0.25</v>
       </c>
       <c r="I55" t="n">
-        <v>3.05</v>
+        <v>0.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D56" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E56" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F56" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G56" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H56" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I56" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>3</v>
       </c>
       <c r="D62" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E62" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F62" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G62" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H62" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I62" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E63" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F63" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G63" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H63" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I63" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D64" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E64" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F64" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G64" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H64" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I64" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D66" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E66" t="n">
-        <v>41.064</v>
+        <v>6.817</v>
       </c>
       <c r="F66" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G66" t="n">
-        <v>164.26</v>
+        <v>61.35</v>
       </c>
       <c r="H66" t="n">
-        <v>25.24</v>
+        <v>5.2</v>
       </c>
       <c r="I66" t="n">
-        <v>18.16</v>
+        <v>9.26</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E67" t="n">
-        <v>10.796</v>
+        <v>40.567</v>
       </c>
       <c r="F67" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G67" t="n">
-        <v>32.39</v>
+        <v>162.27</v>
       </c>
       <c r="H67" t="n">
-        <v>1.23</v>
+        <v>23.25</v>
       </c>
       <c r="I67" t="n">
-        <v>3.95</v>
+        <v>16.72</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E68" t="n">
-        <v>40.567</v>
+        <v>22.797</v>
       </c>
       <c r="F68" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G68" t="n">
-        <v>162.27</v>
+        <v>68.39</v>
       </c>
       <c r="H68" t="n">
-        <v>23.25</v>
+        <v>2.72</v>
       </c>
       <c r="I68" t="n">
-        <v>16.72</v>
+        <v>4.14</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E69" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F69" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G69" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H69" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I69" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E70" t="n">
-        <v>104.58</v>
+        <v>6.807</v>
       </c>
       <c r="F70" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G70" t="n">
-        <v>104.58</v>
+        <v>61.26</v>
       </c>
       <c r="H70" t="n">
-        <v>4.49</v>
+        <v>5.11</v>
       </c>
       <c r="I70" t="n">
-        <v>4.49</v>
+        <v>9.1</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E71" t="n">
-        <v>6.807</v>
+        <v>10.796</v>
       </c>
       <c r="F71" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G71" t="n">
-        <v>61.26</v>
+        <v>32.39</v>
       </c>
       <c r="H71" t="n">
-        <v>5.11</v>
+        <v>1.23</v>
       </c>
       <c r="I71" t="n">
-        <v>9.1</v>
+        <v>3.95</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E77" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F77" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G77" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H77" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I77" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E78" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F78" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G78" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H78" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I78" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>10.958</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>32.87</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>1.71</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>5.49</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D81" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E81" t="n">
-        <v>23.4</v>
+        <v>6.836</v>
       </c>
       <c r="F81" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G81" t="n">
-        <v>70.2</v>
+        <v>61.52</v>
       </c>
       <c r="H81" t="n">
-        <v>4.53</v>
+        <v>5.37</v>
       </c>
       <c r="I81" t="n">
-        <v>6.9</v>
+        <v>9.56</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D87" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E87" t="n">
-        <v>43.005</v>
+        <v>6.856</v>
       </c>
       <c r="F87" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G87" t="n">
-        <v>172.02</v>
+        <v>61.7</v>
       </c>
       <c r="H87" t="n">
-        <v>33</v>
+        <v>5.55</v>
       </c>
       <c r="I87" t="n">
-        <v>23.74</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E88" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F88" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G88" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I88" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D89" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E89" t="n">
-        <v>23.32</v>
+        <v>106.28</v>
       </c>
       <c r="F89" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G89" t="n">
-        <v>69.95999999999999</v>
+        <v>106.28</v>
       </c>
       <c r="H89" t="n">
-        <v>4.29</v>
+        <v>6.19</v>
       </c>
       <c r="I89" t="n">
-        <v>6.53</v>
+        <v>6.18</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D90" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E90" t="n">
-        <v>6.856</v>
+        <v>43.005</v>
       </c>
       <c r="F90" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G90" t="n">
-        <v>61.7</v>
+        <v>172.02</v>
       </c>
       <c r="H90" t="n">
-        <v>5.55</v>
+        <v>33</v>
       </c>
       <c r="I90" t="n">
-        <v>9.880000000000001</v>
+        <v>23.74</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E91" t="n">
-        <v>106.28</v>
+        <v>10.852</v>
       </c>
       <c r="F91" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G91" t="n">
-        <v>106.28</v>
+        <v>32.56</v>
       </c>
       <c r="H91" t="n">
-        <v>6.19</v>
+        <v>1.4</v>
       </c>
       <c r="I91" t="n">
-        <v>6.18</v>
+        <v>4.49</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D102" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E102" t="n">
-        <v>23.29</v>
+        <v>40.97</v>
       </c>
       <c r="F102" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G102" t="n">
-        <v>69.87</v>
+        <v>163.88</v>
       </c>
       <c r="H102" t="n">
-        <v>4.2</v>
+        <v>24.86</v>
       </c>
       <c r="I102" t="n">
-        <v>6.4</v>
+        <v>17.88</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D103" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E103" t="n">
-        <v>10.556</v>
+        <v>6.804</v>
       </c>
       <c r="F103" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G103" t="n">
-        <v>31.67</v>
+        <v>61.24</v>
       </c>
       <c r="H103" t="n">
-        <v>0.51</v>
+        <v>5.09</v>
       </c>
       <c r="I103" t="n">
-        <v>1.64</v>
+        <v>9.07</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E104" t="n">
-        <v>6.804</v>
+        <v>103.46</v>
       </c>
       <c r="F104" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G104" t="n">
-        <v>61.24</v>
+        <v>103.46</v>
       </c>
       <c r="H104" t="n">
-        <v>5.09</v>
+        <v>3.37</v>
       </c>
       <c r="I104" t="n">
-        <v>9.07</v>
+        <v>3.37</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E105" t="n">
-        <v>40.97</v>
+        <v>23.29</v>
       </c>
       <c r="F105" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G105" t="n">
-        <v>163.88</v>
+        <v>69.87</v>
       </c>
       <c r="H105" t="n">
-        <v>24.86</v>
+        <v>4.2</v>
       </c>
       <c r="I105" t="n">
-        <v>17.88</v>
+        <v>6.4</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D106" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E106" t="n">
-        <v>103.46</v>
+        <v>10.556</v>
       </c>
       <c r="F106" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G106" t="n">
-        <v>103.46</v>
+        <v>31.67</v>
       </c>
       <c r="H106" t="n">
-        <v>3.37</v>
+        <v>0.51</v>
       </c>
       <c r="I106" t="n">
-        <v>3.37</v>
+        <v>1.64</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E117" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F117" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G117" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H117" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I117" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E118" t="n">
-        <v>105.96</v>
+        <v>10.756</v>
       </c>
       <c r="F118" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G118" t="n">
-        <v>105.96</v>
+        <v>32.27</v>
       </c>
       <c r="H118" t="n">
-        <v>5.87</v>
+        <v>1.11</v>
       </c>
       <c r="I118" t="n">
-        <v>5.86</v>
+        <v>3.56</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E119" t="n">
-        <v>6.861</v>
+        <v>23.145</v>
       </c>
       <c r="F119" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G119" t="n">
-        <v>61.75</v>
+        <v>69.44</v>
       </c>
       <c r="H119" t="n">
-        <v>5.6</v>
+        <v>3.77</v>
       </c>
       <c r="I119" t="n">
-        <v>9.970000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E120" t="n">
-        <v>10.756</v>
+        <v>105.96</v>
       </c>
       <c r="F120" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G120" t="n">
-        <v>32.27</v>
+        <v>105.96</v>
       </c>
       <c r="H120" t="n">
-        <v>1.11</v>
+        <v>5.87</v>
       </c>
       <c r="I120" t="n">
-        <v>3.56</v>
+        <v>5.86</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D121" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E121" t="n">
-        <v>41</v>
+        <v>6.861</v>
       </c>
       <c r="F121" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G121" t="n">
-        <v>164</v>
+        <v>61.75</v>
       </c>
       <c r="H121" t="n">
-        <v>24.98</v>
+        <v>5.6</v>
       </c>
       <c r="I121" t="n">
-        <v>17.97</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D127" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E127" t="n">
-        <v>6.868</v>
+        <v>23.17</v>
       </c>
       <c r="F127" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G127" t="n">
-        <v>61.81</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H127" t="n">
-        <v>5.66</v>
+        <v>3.84</v>
       </c>
       <c r="I127" t="n">
-        <v>10.08</v>
+        <v>5.85</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D128" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E128" t="n">
-        <v>39.36</v>
+        <v>11.458</v>
       </c>
       <c r="F128" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G128" t="n">
-        <v>157.44</v>
+        <v>34.37</v>
       </c>
       <c r="H128" t="n">
-        <v>18.42</v>
+        <v>3.21</v>
       </c>
       <c r="I128" t="n">
-        <v>13.25</v>
+        <v>10.3</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4796,29 +4796,29 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D129" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E129" t="n">
-        <v>11.458</v>
+        <v>103.46</v>
       </c>
       <c r="F129" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G129" t="n">
-        <v>34.37</v>
+        <v>103.46</v>
       </c>
       <c r="H129" t="n">
-        <v>3.21</v>
+        <v>3.37</v>
       </c>
       <c r="I129" t="n">
-        <v>10.3</v>
+        <v>3.37</v>
       </c>
       <c r="J129" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D130" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E130" t="n">
-        <v>23.17</v>
+        <v>6.868</v>
       </c>
       <c r="F130" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G130" t="n">
-        <v>69.51000000000001</v>
+        <v>61.81</v>
       </c>
       <c r="H130" t="n">
-        <v>3.84</v>
+        <v>5.66</v>
       </c>
       <c r="I130" t="n">
-        <v>5.85</v>
+        <v>10.08</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E131" t="n">
-        <v>103.46</v>
+        <v>39.36</v>
       </c>
       <c r="F131" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G131" t="n">
-        <v>103.46</v>
+        <v>157.44</v>
       </c>
       <c r="H131" t="n">
-        <v>3.37</v>
+        <v>18.42</v>
       </c>
       <c r="I131" t="n">
-        <v>3.37</v>
+        <v>13.25</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C132" t="n">
         <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E132" t="n">
-        <v>11.516</v>
+        <v>23.18</v>
       </c>
       <c r="F132" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G132" t="n">
-        <v>34.55</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H132" t="n">
-        <v>3.39</v>
+        <v>3.87</v>
       </c>
       <c r="I132" t="n">
-        <v>10.88</v>
+        <v>5.89</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D133" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E133" t="n">
-        <v>40.54</v>
+        <v>104.02</v>
       </c>
       <c r="F133" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G133" t="n">
-        <v>162.16</v>
+        <v>104.02</v>
       </c>
       <c r="H133" t="n">
-        <v>23.14</v>
+        <v>3.93</v>
       </c>
       <c r="I133" t="n">
-        <v>16.65</v>
+        <v>3.93</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E134" t="n">
-        <v>6.895</v>
+        <v>11.516</v>
       </c>
       <c r="F134" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G134" t="n">
-        <v>62.05</v>
+        <v>34.55</v>
       </c>
       <c r="H134" t="n">
-        <v>5.9</v>
+        <v>3.39</v>
       </c>
       <c r="I134" t="n">
-        <v>10.51</v>
+        <v>10.88</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E135" t="n">
-        <v>104.02</v>
+        <v>40.54</v>
       </c>
       <c r="F135" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G135" t="n">
-        <v>104.02</v>
+        <v>162.16</v>
       </c>
       <c r="H135" t="n">
-        <v>3.93</v>
+        <v>23.14</v>
       </c>
       <c r="I135" t="n">
-        <v>3.93</v>
+        <v>16.65</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D136" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E136" t="n">
-        <v>23.18</v>
+        <v>6.895</v>
       </c>
       <c r="F136" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G136" t="n">
-        <v>69.54000000000001</v>
+        <v>62.05</v>
       </c>
       <c r="H136" t="n">
-        <v>3.87</v>
+        <v>5.9</v>
       </c>
       <c r="I136" t="n">
-        <v>5.89</v>
+        <v>10.51</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D142" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E142" t="n">
-        <v>6.878</v>
+        <v>102.06</v>
       </c>
       <c r="F142" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G142" t="n">
-        <v>61.9</v>
+        <v>102.06</v>
       </c>
       <c r="H142" t="n">
-        <v>5.75</v>
+        <v>1.97</v>
       </c>
       <c r="I142" t="n">
-        <v>10.24</v>
+        <v>1.97</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E143" t="n">
-        <v>11.498</v>
+        <v>38.89</v>
       </c>
       <c r="F143" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G143" t="n">
-        <v>34.49</v>
+        <v>155.56</v>
       </c>
       <c r="H143" t="n">
-        <v>3.33</v>
+        <v>16.54</v>
       </c>
       <c r="I143" t="n">
-        <v>10.69</v>
+        <v>11.9</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5306,29 +5306,29 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D144" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E144" t="n">
-        <v>23.135</v>
+        <v>6.878</v>
       </c>
       <c r="F144" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G144" t="n">
-        <v>69.41</v>
+        <v>61.9</v>
       </c>
       <c r="H144" t="n">
-        <v>3.74</v>
+        <v>5.75</v>
       </c>
       <c r="I144" t="n">
-        <v>5.7</v>
+        <v>10.24</v>
       </c>
       <c r="J144" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D145" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E145" t="n">
-        <v>102.06</v>
+        <v>11.498</v>
       </c>
       <c r="F145" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G145" t="n">
-        <v>102.06</v>
+        <v>34.49</v>
       </c>
       <c r="H145" t="n">
-        <v>1.97</v>
+        <v>3.33</v>
       </c>
       <c r="I145" t="n">
-        <v>1.97</v>
+        <v>10.69</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D146" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E146" t="n">
-        <v>38.89</v>
+        <v>23.135</v>
       </c>
       <c r="F146" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G146" t="n">
-        <v>155.56</v>
+        <v>69.41</v>
       </c>
       <c r="H146" t="n">
-        <v>16.54</v>
+        <v>3.74</v>
       </c>
       <c r="I146" t="n">
-        <v>11.9</v>
+        <v>5.7</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C157" t="n">
         <v>3</v>
       </c>
       <c r="D157" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E157" t="n">
-        <v>23.08</v>
+        <v>10.92</v>
       </c>
       <c r="F157" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G157" t="n">
-        <v>69.23999999999999</v>
+        <v>32.76</v>
       </c>
       <c r="H157" t="n">
-        <v>3.57</v>
+        <v>1.6</v>
       </c>
       <c r="I157" t="n">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D158" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E158" t="n">
-        <v>104.5</v>
+        <v>40.015</v>
       </c>
       <c r="F158" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G158" t="n">
-        <v>104.5</v>
+        <v>160.06</v>
       </c>
       <c r="H158" t="n">
-        <v>4.41</v>
+        <v>21.04</v>
       </c>
       <c r="I158" t="n">
-        <v>4.41</v>
+        <v>15.13</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D159" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E159" t="n">
-        <v>6.913</v>
+        <v>104.5</v>
       </c>
       <c r="F159" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G159" t="n">
-        <v>62.22</v>
+        <v>104.5</v>
       </c>
       <c r="H159" t="n">
-        <v>6.07</v>
+        <v>4.41</v>
       </c>
       <c r="I159" t="n">
-        <v>10.81</v>
+        <v>4.41</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C160" t="n">
         <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E160" t="n">
-        <v>10.92</v>
+        <v>23.08</v>
       </c>
       <c r="F160" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G160" t="n">
-        <v>32.76</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H160" t="n">
-        <v>1.6</v>
+        <v>3.57</v>
       </c>
       <c r="I160" t="n">
-        <v>5.13</v>
+        <v>5.44</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D161" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E161" t="n">
-        <v>40.015</v>
+        <v>6.913</v>
       </c>
       <c r="F161" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G161" t="n">
-        <v>160.06</v>
+        <v>62.22</v>
       </c>
       <c r="H161" t="n">
-        <v>21.04</v>
+        <v>6.07</v>
       </c>
       <c r="I161" t="n">
-        <v>15.13</v>
+        <v>10.81</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E167" t="n">
-        <v>103.98</v>
+        <v>38.98</v>
       </c>
       <c r="F167" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G167" t="n">
-        <v>103.98</v>
+        <v>155.92</v>
       </c>
       <c r="H167" t="n">
-        <v>3.89</v>
+        <v>16.9</v>
       </c>
       <c r="I167" t="n">
-        <v>3.89</v>
+        <v>12.16</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D168" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E168" t="n">
-        <v>22.92</v>
+        <v>6.911</v>
       </c>
       <c r="F168" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G168" t="n">
-        <v>68.76000000000001</v>
+        <v>62.2</v>
       </c>
       <c r="H168" t="n">
-        <v>3.09</v>
+        <v>6.05</v>
       </c>
       <c r="I168" t="n">
-        <v>4.71</v>
+        <v>10.77</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6156,29 +6156,29 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D169" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E169" t="n">
-        <v>6.911</v>
+        <v>10.726</v>
       </c>
       <c r="F169" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G169" t="n">
-        <v>62.2</v>
+        <v>32.18</v>
       </c>
       <c r="H169" t="n">
-        <v>6.05</v>
+        <v>1.02</v>
       </c>
       <c r="I169" t="n">
-        <v>10.77</v>
+        <v>3.27</v>
       </c>
       <c r="J169" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D170" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E170" t="n">
-        <v>38.98</v>
+        <v>103.98</v>
       </c>
       <c r="F170" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G170" t="n">
-        <v>155.92</v>
+        <v>103.98</v>
       </c>
       <c r="H170" t="n">
-        <v>16.9</v>
+        <v>3.89</v>
       </c>
       <c r="I170" t="n">
-        <v>12.16</v>
+        <v>3.89</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,29 +6224,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C171" t="n">
         <v>3</v>
       </c>
       <c r="D171" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E171" t="n">
-        <v>10.726</v>
+        <v>22.92</v>
       </c>
       <c r="F171" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G171" t="n">
-        <v>32.18</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H171" t="n">
-        <v>1.02</v>
+        <v>3.09</v>
       </c>
       <c r="I171" t="n">
-        <v>3.27</v>
+        <v>4.71</v>
       </c>
       <c r="J171" t="n">
         <v>7.91</v>
@@ -6598,29 +6598,29 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D182" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E182" t="n">
-        <v>6.848</v>
+        <v>37.235</v>
       </c>
       <c r="F182" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G182" t="n">
-        <v>61.63</v>
+        <v>148.94</v>
       </c>
       <c r="H182" t="n">
-        <v>5.48</v>
+        <v>9.92</v>
       </c>
       <c r="I182" t="n">
-        <v>9.76</v>
+        <v>7.14</v>
       </c>
       <c r="J182" t="n">
         <v>7.91</v>
@@ -6632,29 +6632,29 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C183" t="n">
         <v>3</v>
       </c>
       <c r="D183" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E183" t="n">
-        <v>22.835</v>
+        <v>10.776</v>
       </c>
       <c r="F183" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G183" t="n">
-        <v>68.5</v>
+        <v>32.33</v>
       </c>
       <c r="H183" t="n">
-        <v>2.83</v>
+        <v>1.17</v>
       </c>
       <c r="I183" t="n">
-        <v>4.31</v>
+        <v>3.75</v>
       </c>
       <c r="J183" t="n">
         <v>7.91</v>
@@ -6666,29 +6666,29 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D184" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E184" t="n">
-        <v>10.776</v>
+        <v>100.14</v>
       </c>
       <c r="F184" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G184" t="n">
-        <v>32.33</v>
+        <v>100.14</v>
       </c>
       <c r="H184" t="n">
-        <v>1.17</v>
+        <v>0.05</v>
       </c>
       <c r="I184" t="n">
-        <v>3.75</v>
+        <v>0.05</v>
       </c>
       <c r="J184" t="n">
         <v>7.91</v>
@@ -6700,29 +6700,29 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D185" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E185" t="n">
-        <v>100.14</v>
+        <v>6.848</v>
       </c>
       <c r="F185" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G185" t="n">
-        <v>100.14</v>
+        <v>61.63</v>
       </c>
       <c r="H185" t="n">
-        <v>0.05</v>
+        <v>5.48</v>
       </c>
       <c r="I185" t="n">
-        <v>0.05</v>
+        <v>9.76</v>
       </c>
       <c r="J185" t="n">
         <v>7.91</v>
@@ -6734,29 +6734,29 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D186" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E186" t="n">
-        <v>37.235</v>
+        <v>22.835</v>
       </c>
       <c r="F186" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G186" t="n">
-        <v>148.94</v>
+        <v>68.5</v>
       </c>
       <c r="H186" t="n">
-        <v>9.92</v>
+        <v>2.83</v>
       </c>
       <c r="I186" t="n">
-        <v>7.14</v>
+        <v>4.31</v>
       </c>
       <c r="J186" t="n">
         <v>7.91</v>
@@ -7108,29 +7108,29 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D197" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E197" t="n">
-        <v>102.48</v>
+        <v>38.565</v>
       </c>
       <c r="F197" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G197" t="n">
-        <v>102.48</v>
+        <v>154.26</v>
       </c>
       <c r="H197" t="n">
-        <v>2.39</v>
+        <v>15.24</v>
       </c>
       <c r="I197" t="n">
-        <v>2.39</v>
+        <v>10.96</v>
       </c>
       <c r="J197" t="n">
         <v>7.91</v>
@@ -7142,29 +7142,29 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C198" t="n">
         <v>3</v>
       </c>
       <c r="D198" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E198" t="n">
-        <v>22.6</v>
+        <v>11.022</v>
       </c>
       <c r="F198" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G198" t="n">
-        <v>67.8</v>
+        <v>33.07</v>
       </c>
       <c r="H198" t="n">
-        <v>2.13</v>
+        <v>1.91</v>
       </c>
       <c r="I198" t="n">
-        <v>3.24</v>
+        <v>6.13</v>
       </c>
       <c r="J198" t="n">
         <v>7.91</v>
@@ -7176,29 +7176,29 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D199" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E199" t="n">
-        <v>6.909</v>
+        <v>22.6</v>
       </c>
       <c r="F199" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G199" t="n">
-        <v>62.18</v>
+        <v>67.8</v>
       </c>
       <c r="H199" t="n">
-        <v>6.03</v>
+        <v>2.13</v>
       </c>
       <c r="I199" t="n">
-        <v>10.74</v>
+        <v>3.24</v>
       </c>
       <c r="J199" t="n">
         <v>7.91</v>
@@ -7210,29 +7210,29 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D200" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E200" t="n">
-        <v>11.022</v>
+        <v>102.48</v>
       </c>
       <c r="F200" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G200" t="n">
-        <v>33.07</v>
+        <v>102.48</v>
       </c>
       <c r="H200" t="n">
-        <v>1.91</v>
+        <v>2.39</v>
       </c>
       <c r="I200" t="n">
-        <v>6.13</v>
+        <v>2.39</v>
       </c>
       <c r="J200" t="n">
         <v>7.91</v>
@@ -7244,29 +7244,29 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D201" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E201" t="n">
-        <v>38.565</v>
+        <v>6.909</v>
       </c>
       <c r="F201" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G201" t="n">
-        <v>154.26</v>
+        <v>62.18</v>
       </c>
       <c r="H201" t="n">
-        <v>15.24</v>
+        <v>6.03</v>
       </c>
       <c r="I201" t="n">
-        <v>10.96</v>
+        <v>10.74</v>
       </c>
       <c r="J201" t="n">
         <v>7.91</v>
@@ -7439,6 +7439,176 @@
         <v>9.35</v>
       </c>
       <c r="J206" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>3</v>
+      </c>
+      <c r="D207" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E207" t="n">
+        <v>11.172</v>
+      </c>
+      <c r="F207" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G207" t="n">
+        <v>33.52</v>
+      </c>
+      <c r="H207" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="I207" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="J207" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>4</v>
+      </c>
+      <c r="D208" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E208" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="F208" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G208" t="n">
+        <v>151.28</v>
+      </c>
+      <c r="H208" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="I208" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="J208" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>3</v>
+      </c>
+      <c r="D209" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E209" t="n">
+        <v>22.725</v>
+      </c>
+      <c r="F209" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G209" t="n">
+        <v>68.18000000000001</v>
+      </c>
+      <c r="H209" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="I209" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="J209" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>1</v>
+      </c>
+      <c r="D210" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E210" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="F210" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G210" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="H210" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="I210" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="J210" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="1" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>9</v>
+      </c>
+      <c r="D211" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E211" t="n">
+        <v>6.865</v>
+      </c>
+      <c r="F211" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G211" t="n">
+        <v>61.79</v>
+      </c>
+      <c r="H211" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="I211" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="J211" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 27/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J211"/>
+  <dimension ref="A1:J216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E28" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F28" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G28" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H28" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I28" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E29" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F29" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G29" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H29" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I29" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D37" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E37" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F37" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G37" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H37" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I37" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E38" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F38" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G38" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H38" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I38" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>3</v>
       </c>
       <c r="D39" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E39" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F39" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G39" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H39" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I39" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D40" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E40" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F40" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G40" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H40" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I40" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D41" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E41" t="n">
-        <v>10.67</v>
+        <v>102.8</v>
       </c>
       <c r="F41" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G41" t="n">
-        <v>32.01</v>
+        <v>102.8</v>
       </c>
       <c r="H41" t="n">
-        <v>0.85</v>
+        <v>2.71</v>
       </c>
       <c r="I41" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D52" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E52" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F52" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G52" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H52" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I52" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>3</v>
       </c>
       <c r="D53" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E53" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F53" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G53" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H53" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E54" t="n">
-        <v>21.703</v>
+        <v>100.34</v>
       </c>
       <c r="F54" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G54" t="n">
-        <v>65.11</v>
+        <v>100.34</v>
       </c>
       <c r="H54" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="I54" t="n">
-        <v>-0.85</v>
+        <v>0.25</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D55" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E55" t="n">
-        <v>100.34</v>
+        <v>38.544</v>
       </c>
       <c r="F55" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G55" t="n">
-        <v>100.34</v>
+        <v>154.18</v>
       </c>
       <c r="H55" t="n">
-        <v>0.25</v>
+        <v>15.16</v>
       </c>
       <c r="I55" t="n">
-        <v>0.25</v>
+        <v>10.9</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E56" t="n">
-        <v>6.629</v>
+        <v>10.702</v>
       </c>
       <c r="F56" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G56" t="n">
-        <v>59.66</v>
+        <v>32.11</v>
       </c>
       <c r="H56" t="n">
-        <v>3.51</v>
+        <v>0.95</v>
       </c>
       <c r="I56" t="n">
-        <v>6.25</v>
+        <v>3.05</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D62" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E62" t="n">
-        <v>22.7</v>
+        <v>6.817</v>
       </c>
       <c r="F62" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G62" t="n">
-        <v>68.09999999999999</v>
+        <v>61.35</v>
       </c>
       <c r="H62" t="n">
-        <v>2.43</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>3.7</v>
+        <v>9.26</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D63" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E63" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F63" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G63" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H63" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I63" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E64" t="n">
-        <v>41.064</v>
+        <v>10.712</v>
       </c>
       <c r="F64" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G64" t="n">
-        <v>164.26</v>
+        <v>32.14</v>
       </c>
       <c r="H64" t="n">
-        <v>25.24</v>
+        <v>0.98</v>
       </c>
       <c r="I64" t="n">
-        <v>18.16</v>
+        <v>3.15</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E65" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F65" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G65" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H65" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I65" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E66" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F66" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G66" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H66" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I66" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D72" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E72" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F72" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G72" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H72" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I72" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C73" t="n">
         <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E73" t="n">
-        <v>23</v>
+        <v>10.892</v>
       </c>
       <c r="F73" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G73" t="n">
-        <v>69</v>
+        <v>32.68</v>
       </c>
       <c r="H73" t="n">
-        <v>3.33</v>
+        <v>1.52</v>
       </c>
       <c r="I73" t="n">
-        <v>5.07</v>
+        <v>4.88</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E74" t="n">
-        <v>41.15</v>
+        <v>23</v>
       </c>
       <c r="F74" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G74" t="n">
-        <v>164.6</v>
+        <v>69</v>
       </c>
       <c r="H74" t="n">
-        <v>25.58</v>
+        <v>3.33</v>
       </c>
       <c r="I74" t="n">
-        <v>18.4</v>
+        <v>5.07</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D75" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E75" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F75" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G75" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H75" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I75" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D77" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E77" t="n">
-        <v>105.8</v>
+        <v>6.836</v>
       </c>
       <c r="F77" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G77" t="n">
-        <v>105.8</v>
+        <v>61.52</v>
       </c>
       <c r="H77" t="n">
-        <v>5.71</v>
+        <v>5.37</v>
       </c>
       <c r="I77" t="n">
-        <v>5.7</v>
+        <v>9.56</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D78" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E78" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F78" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G78" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H78" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I78" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E79" t="n">
-        <v>42.25</v>
+        <v>10.958</v>
       </c>
       <c r="F79" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G79" t="n">
-        <v>169</v>
+        <v>32.87</v>
       </c>
       <c r="H79" t="n">
-        <v>29.98</v>
+        <v>1.71</v>
       </c>
       <c r="I79" t="n">
-        <v>21.57</v>
+        <v>5.49</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E80" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F80" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G80" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H80" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I80" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D81" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E81" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F81" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G81" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H81" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I81" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D87" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E87" t="n">
-        <v>6.856</v>
+        <v>10.852</v>
       </c>
       <c r="F87" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G87" t="n">
-        <v>61.7</v>
+        <v>32.56</v>
       </c>
       <c r="H87" t="n">
-        <v>5.55</v>
+        <v>1.4</v>
       </c>
       <c r="I87" t="n">
-        <v>9.880000000000001</v>
+        <v>4.49</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D88" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E88" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F88" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G88" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I88" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D89" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E89" t="n">
-        <v>106.28</v>
+        <v>23.32</v>
       </c>
       <c r="F89" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G89" t="n">
-        <v>106.28</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H89" t="n">
-        <v>6.19</v>
+        <v>4.29</v>
       </c>
       <c r="I89" t="n">
-        <v>6.18</v>
+        <v>6.53</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D90" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E90" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F90" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G90" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H90" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I90" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E91" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F91" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G91" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H91" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I91" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D92" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E92" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F92" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G92" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H92" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I92" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C93" t="n">
         <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E93" t="n">
-        <v>10.876</v>
+        <v>23.025</v>
       </c>
       <c r="F93" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G93" t="n">
-        <v>32.63</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H93" t="n">
-        <v>1.47</v>
+        <v>3.4</v>
       </c>
       <c r="I93" t="n">
-        <v>4.72</v>
+        <v>5.18</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E94" t="n">
-        <v>103.88</v>
+        <v>10.876</v>
       </c>
       <c r="F94" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G94" t="n">
-        <v>103.88</v>
+        <v>32.63</v>
       </c>
       <c r="H94" t="n">
-        <v>3.79</v>
+        <v>1.47</v>
       </c>
       <c r="I94" t="n">
-        <v>3.79</v>
+        <v>4.72</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D95" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E95" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F95" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G95" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H95" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I95" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D96" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E96" t="n">
-        <v>40.575</v>
+        <v>103.88</v>
       </c>
       <c r="F96" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G96" t="n">
-        <v>162.3</v>
+        <v>103.88</v>
       </c>
       <c r="H96" t="n">
-        <v>23.28</v>
+        <v>3.79</v>
       </c>
       <c r="I96" t="n">
-        <v>16.75</v>
+        <v>3.79</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C97" t="n">
         <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E97" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F97" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G97" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H97" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I97" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E98" t="n">
-        <v>104.22</v>
+        <v>23.35</v>
       </c>
       <c r="F98" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G98" t="n">
-        <v>104.22</v>
+        <v>70.05</v>
       </c>
       <c r="H98" t="n">
-        <v>4.13</v>
+        <v>4.38</v>
       </c>
       <c r="I98" t="n">
-        <v>4.13</v>
+        <v>6.67</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D99" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E99" t="n">
-        <v>40.65</v>
+        <v>104.22</v>
       </c>
       <c r="F99" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G99" t="n">
-        <v>162.6</v>
+        <v>104.22</v>
       </c>
       <c r="H99" t="n">
-        <v>23.58</v>
+        <v>4.13</v>
       </c>
       <c r="I99" t="n">
-        <v>16.96</v>
+        <v>4.13</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E100" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F100" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G100" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H100" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I100" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D101" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E101" t="n">
-        <v>10.642</v>
+        <v>6.839</v>
       </c>
       <c r="F101" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G101" t="n">
-        <v>31.93</v>
+        <v>61.55</v>
       </c>
       <c r="H101" t="n">
-        <v>0.77</v>
+        <v>5.4</v>
       </c>
       <c r="I101" t="n">
-        <v>2.47</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D102" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E102" t="n">
-        <v>40.97</v>
+        <v>103.46</v>
       </c>
       <c r="F102" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G102" t="n">
-        <v>163.88</v>
+        <v>103.46</v>
       </c>
       <c r="H102" t="n">
-        <v>24.86</v>
+        <v>3.37</v>
       </c>
       <c r="I102" t="n">
-        <v>17.88</v>
+        <v>3.37</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E103" t="n">
-        <v>6.804</v>
+        <v>23.29</v>
       </c>
       <c r="F103" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G103" t="n">
-        <v>61.24</v>
+        <v>69.87</v>
       </c>
       <c r="H103" t="n">
-        <v>5.09</v>
+        <v>4.2</v>
       </c>
       <c r="I103" t="n">
-        <v>9.07</v>
+        <v>6.4</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D104" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E104" t="n">
-        <v>103.46</v>
+        <v>40.97</v>
       </c>
       <c r="F104" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G104" t="n">
-        <v>103.46</v>
+        <v>163.88</v>
       </c>
       <c r="H104" t="n">
-        <v>3.37</v>
+        <v>24.86</v>
       </c>
       <c r="I104" t="n">
-        <v>3.37</v>
+        <v>17.88</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D105" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E105" t="n">
-        <v>23.29</v>
+        <v>6.804</v>
       </c>
       <c r="F105" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G105" t="n">
-        <v>69.87</v>
+        <v>61.24</v>
       </c>
       <c r="H105" t="n">
-        <v>4.2</v>
+        <v>5.09</v>
       </c>
       <c r="I105" t="n">
-        <v>6.4</v>
+        <v>9.07</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D107" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E107" t="n">
-        <v>40.5</v>
+        <v>103.14</v>
       </c>
       <c r="F107" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G107" t="n">
-        <v>162</v>
+        <v>103.14</v>
       </c>
       <c r="H107" t="n">
-        <v>22.98</v>
+        <v>3.05</v>
       </c>
       <c r="I107" t="n">
-        <v>16.53</v>
+        <v>3.05</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D108" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E108" t="n">
-        <v>23.33</v>
+        <v>6.785</v>
       </c>
       <c r="F108" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G108" t="n">
-        <v>69.98999999999999</v>
+        <v>61.06</v>
       </c>
       <c r="H108" t="n">
-        <v>4.32</v>
+        <v>4.91</v>
       </c>
       <c r="I108" t="n">
-        <v>6.58</v>
+        <v>8.74</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E110" t="n">
-        <v>6.785</v>
+        <v>23.33</v>
       </c>
       <c r="F110" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G110" t="n">
-        <v>61.06</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H110" t="n">
-        <v>4.91</v>
+        <v>4.32</v>
       </c>
       <c r="I110" t="n">
-        <v>8.74</v>
+        <v>6.58</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D111" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E111" t="n">
-        <v>103.14</v>
+        <v>40.5</v>
       </c>
       <c r="F111" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G111" t="n">
-        <v>103.14</v>
+        <v>162</v>
       </c>
       <c r="H111" t="n">
-        <v>3.05</v>
+        <v>22.98</v>
       </c>
       <c r="I111" t="n">
-        <v>3.05</v>
+        <v>16.53</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D117" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E117" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F117" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G117" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H117" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I117" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C118" t="n">
         <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E118" t="n">
-        <v>10.756</v>
+        <v>23.145</v>
       </c>
       <c r="F118" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G118" t="n">
-        <v>32.27</v>
+        <v>69.44</v>
       </c>
       <c r="H118" t="n">
-        <v>1.11</v>
+        <v>3.77</v>
       </c>
       <c r="I118" t="n">
-        <v>3.56</v>
+        <v>5.74</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D119" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E119" t="n">
-        <v>23.145</v>
+        <v>6.861</v>
       </c>
       <c r="F119" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G119" t="n">
-        <v>69.44</v>
+        <v>61.75</v>
       </c>
       <c r="H119" t="n">
-        <v>3.77</v>
+        <v>5.6</v>
       </c>
       <c r="I119" t="n">
-        <v>5.74</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>41</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>164</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>24.98</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>17.97</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E121" t="n">
-        <v>6.861</v>
+        <v>10.756</v>
       </c>
       <c r="F121" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G121" t="n">
-        <v>61.75</v>
+        <v>32.27</v>
       </c>
       <c r="H121" t="n">
-        <v>5.6</v>
+        <v>1.11</v>
       </c>
       <c r="I121" t="n">
-        <v>9.970000000000001</v>
+        <v>3.56</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D132" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E132" t="n">
-        <v>23.18</v>
+        <v>40.54</v>
       </c>
       <c r="F132" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G132" t="n">
-        <v>69.54000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="H132" t="n">
-        <v>3.87</v>
+        <v>23.14</v>
       </c>
       <c r="I132" t="n">
-        <v>5.89</v>
+        <v>16.65</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D133" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E133" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F133" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G133" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H133" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I133" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D134" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E134" t="n">
-        <v>11.516</v>
+        <v>6.895</v>
       </c>
       <c r="F134" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G134" t="n">
-        <v>34.55</v>
+        <v>62.05</v>
       </c>
       <c r="H134" t="n">
-        <v>3.39</v>
+        <v>5.9</v>
       </c>
       <c r="I134" t="n">
-        <v>10.88</v>
+        <v>10.51</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D135" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E135" t="n">
-        <v>40.54</v>
+        <v>23.18</v>
       </c>
       <c r="F135" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G135" t="n">
-        <v>162.16</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H135" t="n">
-        <v>23.14</v>
+        <v>3.87</v>
       </c>
       <c r="I135" t="n">
-        <v>16.65</v>
+        <v>5.89</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D136" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E136" t="n">
-        <v>6.895</v>
+        <v>104.02</v>
       </c>
       <c r="F136" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G136" t="n">
-        <v>62.05</v>
+        <v>104.02</v>
       </c>
       <c r="H136" t="n">
-        <v>5.9</v>
+        <v>3.93</v>
       </c>
       <c r="I136" t="n">
-        <v>10.51</v>
+        <v>3.93</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D147" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E147" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F147" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G147" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H147" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I147" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D148" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E148" t="n">
-        <v>101.7</v>
+        <v>6.826</v>
       </c>
       <c r="F148" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G148" t="n">
-        <v>101.7</v>
+        <v>61.43</v>
       </c>
       <c r="H148" t="n">
-        <v>1.61</v>
+        <v>5.28</v>
       </c>
       <c r="I148" t="n">
-        <v>1.61</v>
+        <v>9.4</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D150" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E150" t="n">
-        <v>6.826</v>
+        <v>38.955</v>
       </c>
       <c r="F150" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G150" t="n">
-        <v>61.43</v>
+        <v>155.82</v>
       </c>
       <c r="H150" t="n">
-        <v>5.28</v>
+        <v>16.8</v>
       </c>
       <c r="I150" t="n">
-        <v>9.4</v>
+        <v>12.08</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D151" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E151" t="n">
-        <v>22.755</v>
+        <v>101.7</v>
       </c>
       <c r="F151" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G151" t="n">
-        <v>68.27</v>
+        <v>101.7</v>
       </c>
       <c r="H151" t="n">
-        <v>2.6</v>
+        <v>1.61</v>
       </c>
       <c r="I151" t="n">
-        <v>3.96</v>
+        <v>1.61</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D162" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E162" t="n">
-        <v>10.748</v>
+        <v>6.927</v>
       </c>
       <c r="F162" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G162" t="n">
-        <v>32.24</v>
+        <v>62.34</v>
       </c>
       <c r="H162" t="n">
-        <v>1.08</v>
+        <v>6.19</v>
       </c>
       <c r="I162" t="n">
-        <v>3.47</v>
+        <v>11.02</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D163" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E163" t="n">
-        <v>103.84</v>
+        <v>23.01</v>
       </c>
       <c r="F163" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G163" t="n">
-        <v>103.84</v>
+        <v>69.03</v>
       </c>
       <c r="H163" t="n">
-        <v>3.75</v>
+        <v>3.36</v>
       </c>
       <c r="I163" t="n">
-        <v>3.75</v>
+        <v>5.12</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -5986,29 +5986,29 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D164" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E164" t="n">
-        <v>38.845</v>
+        <v>103.84</v>
       </c>
       <c r="F164" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G164" t="n">
-        <v>155.38</v>
+        <v>103.84</v>
       </c>
       <c r="H164" t="n">
-        <v>16.36</v>
+        <v>3.75</v>
       </c>
       <c r="I164" t="n">
-        <v>11.77</v>
+        <v>3.75</v>
       </c>
       <c r="J164" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D165" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E165" t="n">
-        <v>23.01</v>
+        <v>38.845</v>
       </c>
       <c r="F165" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G165" t="n">
-        <v>69.03</v>
+        <v>155.38</v>
       </c>
       <c r="H165" t="n">
-        <v>3.36</v>
+        <v>16.36</v>
       </c>
       <c r="I165" t="n">
-        <v>5.12</v>
+        <v>11.77</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D166" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E166" t="n">
-        <v>6.927</v>
+        <v>10.748</v>
       </c>
       <c r="F166" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G166" t="n">
-        <v>62.34</v>
+        <v>32.24</v>
       </c>
       <c r="H166" t="n">
-        <v>6.19</v>
+        <v>1.08</v>
       </c>
       <c r="I166" t="n">
-        <v>11.02</v>
+        <v>3.47</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6258,29 +6258,29 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D172" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E172" t="n">
-        <v>10.712</v>
+        <v>103.22</v>
       </c>
       <c r="F172" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G172" t="n">
-        <v>32.14</v>
+        <v>103.22</v>
       </c>
       <c r="H172" t="n">
-        <v>0.98</v>
+        <v>3.13</v>
       </c>
       <c r="I172" t="n">
-        <v>3.15</v>
+        <v>3.13</v>
       </c>
       <c r="J172" t="n">
         <v>7.91</v>
@@ -6292,29 +6292,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D173" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E173" t="n">
-        <v>22.95</v>
+        <v>6.926</v>
       </c>
       <c r="F173" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G173" t="n">
-        <v>68.84999999999999</v>
+        <v>62.33</v>
       </c>
       <c r="H173" t="n">
-        <v>3.18</v>
+        <v>6.18</v>
       </c>
       <c r="I173" t="n">
-        <v>4.84</v>
+        <v>11.01</v>
       </c>
       <c r="J173" t="n">
         <v>7.91</v>
@@ -6326,29 +6326,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D174" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E174" t="n">
-        <v>6.926</v>
+        <v>38.74</v>
       </c>
       <c r="F174" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G174" t="n">
-        <v>62.33</v>
+        <v>154.96</v>
       </c>
       <c r="H174" t="n">
-        <v>6.18</v>
+        <v>15.94</v>
       </c>
       <c r="I174" t="n">
-        <v>11.01</v>
+        <v>11.47</v>
       </c>
       <c r="J174" t="n">
         <v>7.91</v>
@@ -6360,29 +6360,29 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D175" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E175" t="n">
-        <v>103.22</v>
+        <v>10.712</v>
       </c>
       <c r="F175" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G175" t="n">
-        <v>103.22</v>
+        <v>32.14</v>
       </c>
       <c r="H175" t="n">
-        <v>3.13</v>
+        <v>0.98</v>
       </c>
       <c r="I175" t="n">
-        <v>3.13</v>
+        <v>3.15</v>
       </c>
       <c r="J175" t="n">
         <v>7.91</v>
@@ -6394,29 +6394,29 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D176" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E176" t="n">
-        <v>38.74</v>
+        <v>22.95</v>
       </c>
       <c r="F176" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G176" t="n">
-        <v>154.96</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H176" t="n">
-        <v>15.94</v>
+        <v>3.18</v>
       </c>
       <c r="I176" t="n">
-        <v>11.47</v>
+        <v>4.84</v>
       </c>
       <c r="J176" t="n">
         <v>7.91</v>
@@ -6768,29 +6768,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D187" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E187" t="n">
-        <v>37.85</v>
+        <v>101.44</v>
       </c>
       <c r="F187" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G187" t="n">
-        <v>151.4</v>
+        <v>101.44</v>
       </c>
       <c r="H187" t="n">
-        <v>12.38</v>
+        <v>1.35</v>
       </c>
       <c r="I187" t="n">
-        <v>8.91</v>
+        <v>1.35</v>
       </c>
       <c r="J187" t="n">
         <v>7.91</v>
@@ -6802,29 +6802,29 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D188" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E188" t="n">
-        <v>6.862</v>
+        <v>22.845</v>
       </c>
       <c r="F188" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G188" t="n">
-        <v>61.76</v>
+        <v>68.53</v>
       </c>
       <c r="H188" t="n">
-        <v>5.61</v>
+        <v>2.86</v>
       </c>
       <c r="I188" t="n">
-        <v>9.99</v>
+        <v>4.36</v>
       </c>
       <c r="J188" t="n">
         <v>7.91</v>
@@ -6836,29 +6836,29 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D189" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E189" t="n">
-        <v>10.708</v>
+        <v>6.862</v>
       </c>
       <c r="F189" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G189" t="n">
-        <v>32.12</v>
+        <v>61.76</v>
       </c>
       <c r="H189" t="n">
-        <v>0.96</v>
+        <v>5.61</v>
       </c>
       <c r="I189" t="n">
-        <v>3.08</v>
+        <v>9.99</v>
       </c>
       <c r="J189" t="n">
         <v>7.91</v>
@@ -6870,29 +6870,29 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E190" t="n">
-        <v>22.845</v>
+        <v>37.85</v>
       </c>
       <c r="F190" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G190" t="n">
-        <v>68.53</v>
+        <v>151.4</v>
       </c>
       <c r="H190" t="n">
-        <v>2.86</v>
+        <v>12.38</v>
       </c>
       <c r="I190" t="n">
-        <v>4.36</v>
+        <v>8.91</v>
       </c>
       <c r="J190" t="n">
         <v>7.91</v>
@@ -6904,29 +6904,29 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D191" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E191" t="n">
-        <v>101.44</v>
+        <v>10.708</v>
       </c>
       <c r="F191" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G191" t="n">
-        <v>101.44</v>
+        <v>32.12</v>
       </c>
       <c r="H191" t="n">
-        <v>1.35</v>
+        <v>0.96</v>
       </c>
       <c r="I191" t="n">
-        <v>1.35</v>
+        <v>3.08</v>
       </c>
       <c r="J191" t="n">
         <v>7.91</v>
@@ -7108,29 +7108,29 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D197" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E197" t="n">
-        <v>38.565</v>
+        <v>6.909</v>
       </c>
       <c r="F197" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G197" t="n">
-        <v>154.26</v>
+        <v>62.18</v>
       </c>
       <c r="H197" t="n">
-        <v>15.24</v>
+        <v>6.03</v>
       </c>
       <c r="I197" t="n">
-        <v>10.96</v>
+        <v>10.74</v>
       </c>
       <c r="J197" t="n">
         <v>7.91</v>
@@ -7142,29 +7142,29 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D198" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E198" t="n">
-        <v>11.022</v>
+        <v>102.48</v>
       </c>
       <c r="F198" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G198" t="n">
-        <v>33.07</v>
+        <v>102.48</v>
       </c>
       <c r="H198" t="n">
-        <v>1.91</v>
+        <v>2.39</v>
       </c>
       <c r="I198" t="n">
-        <v>6.13</v>
+        <v>2.39</v>
       </c>
       <c r="J198" t="n">
         <v>7.91</v>
@@ -7210,29 +7210,29 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D200" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E200" t="n">
-        <v>102.48</v>
+        <v>11.022</v>
       </c>
       <c r="F200" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G200" t="n">
-        <v>102.48</v>
+        <v>33.07</v>
       </c>
       <c r="H200" t="n">
-        <v>2.39</v>
+        <v>1.91</v>
       </c>
       <c r="I200" t="n">
-        <v>2.39</v>
+        <v>6.13</v>
       </c>
       <c r="J200" t="n">
         <v>7.91</v>
@@ -7244,29 +7244,29 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D201" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E201" t="n">
-        <v>6.909</v>
+        <v>38.565</v>
       </c>
       <c r="F201" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G201" t="n">
-        <v>62.18</v>
+        <v>154.26</v>
       </c>
       <c r="H201" t="n">
-        <v>6.03</v>
+        <v>15.24</v>
       </c>
       <c r="I201" t="n">
-        <v>10.74</v>
+        <v>10.96</v>
       </c>
       <c r="J201" t="n">
         <v>7.91</v>
@@ -7448,29 +7448,29 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D207" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E207" t="n">
-        <v>11.172</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F207" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G207" t="n">
-        <v>33.52</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H207" t="n">
-        <v>2.36</v>
+        <v>-0.19</v>
       </c>
       <c r="I207" t="n">
-        <v>7.57</v>
+        <v>-0.19</v>
       </c>
       <c r="J207" t="n">
         <v>7.91</v>
@@ -7482,29 +7482,29 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D208" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E208" t="n">
-        <v>37.82</v>
+        <v>22.725</v>
       </c>
       <c r="F208" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G208" t="n">
-        <v>151.28</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H208" t="n">
-        <v>12.26</v>
+        <v>2.51</v>
       </c>
       <c r="I208" t="n">
-        <v>8.82</v>
+        <v>3.82</v>
       </c>
       <c r="J208" t="n">
         <v>7.91</v>
@@ -7516,29 +7516,29 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D209" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E209" t="n">
-        <v>22.725</v>
+        <v>6.865</v>
       </c>
       <c r="F209" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G209" t="n">
-        <v>68.18000000000001</v>
+        <v>61.79</v>
       </c>
       <c r="H209" t="n">
-        <v>2.51</v>
+        <v>5.64</v>
       </c>
       <c r="I209" t="n">
-        <v>3.82</v>
+        <v>10.04</v>
       </c>
       <c r="J209" t="n">
         <v>7.91</v>
@@ -7550,29 +7550,29 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D210" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E210" t="n">
-        <v>99.90000000000001</v>
+        <v>11.172</v>
       </c>
       <c r="F210" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G210" t="n">
-        <v>99.90000000000001</v>
+        <v>33.52</v>
       </c>
       <c r="H210" t="n">
-        <v>-0.19</v>
+        <v>2.36</v>
       </c>
       <c r="I210" t="n">
-        <v>-0.19</v>
+        <v>7.57</v>
       </c>
       <c r="J210" t="n">
         <v>7.91</v>
@@ -7584,31 +7584,201 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>4</v>
+      </c>
+      <c r="D211" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E211" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="F211" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G211" t="n">
+        <v>151.28</v>
+      </c>
+      <c r="H211" t="n">
+        <v>12.26</v>
+      </c>
+      <c r="I211" t="n">
+        <v>8.82</v>
+      </c>
+      <c r="J211" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>1</v>
+      </c>
+      <c r="D212" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E212" t="n">
+        <v>98.29000000000001</v>
+      </c>
+      <c r="F212" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G212" t="n">
+        <v>98.29000000000001</v>
+      </c>
+      <c r="H212" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="I212" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="J212" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>3</v>
+      </c>
+      <c r="D213" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E213" t="n">
+        <v>11.338</v>
+      </c>
+      <c r="F213" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G213" t="n">
+        <v>34.01</v>
+      </c>
+      <c r="H213" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="I213" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="J213" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>4</v>
+      </c>
+      <c r="D214" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E214" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="F214" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G214" t="n">
+        <v>149</v>
+      </c>
+      <c r="H214" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="I214" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="J214" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>3</v>
+      </c>
+      <c r="D215" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E215" t="n">
+        <v>22.885</v>
+      </c>
+      <c r="F215" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G215" t="n">
+        <v>68.66</v>
+      </c>
+      <c r="H215" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="I215" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="J215" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="1" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C211" t="n">
+      <c r="C216" t="n">
         <v>9</v>
       </c>
-      <c r="D211" t="n">
+      <c r="D216" t="n">
         <v>6.239</v>
       </c>
-      <c r="E211" t="n">
-        <v>6.865</v>
-      </c>
-      <c r="F211" t="n">
+      <c r="E216" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="F216" t="n">
         <v>56.15</v>
       </c>
-      <c r="G211" t="n">
-        <v>61.79</v>
-      </c>
-      <c r="H211" t="n">
-        <v>5.64</v>
-      </c>
-      <c r="I211" t="n">
-        <v>10.04</v>
-      </c>
-      <c r="J211" t="n">
+      <c r="G216" t="n">
+        <v>61.56</v>
+      </c>
+      <c r="H216" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="I216" t="n">
+        <v>9.630000000000001</v>
+      </c>
+      <c r="J216" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 28/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J216"/>
+  <dimension ref="A1:J221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E12" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F12" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G12" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H12" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I12" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E13" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F13" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G13" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H13" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I13" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D14" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E14" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F14" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G14" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H14" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E15" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F15" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G15" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H15" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I15" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D16" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E16" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F16" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G16" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H16" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I16" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>6.795</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>61.16</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>5.01</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>8.92</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E28" t="n">
-        <v>10.66</v>
+        <v>104.9</v>
       </c>
       <c r="F28" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G28" t="n">
-        <v>31.98</v>
+        <v>104.9</v>
       </c>
       <c r="H28" t="n">
-        <v>0.82</v>
+        <v>4.81</v>
       </c>
       <c r="I28" t="n">
-        <v>2.63</v>
+        <v>4.81</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E29" t="n">
-        <v>40.532</v>
+        <v>21.98</v>
       </c>
       <c r="F29" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G29" t="n">
-        <v>162.13</v>
+        <v>65.94</v>
       </c>
       <c r="H29" t="n">
-        <v>23.11</v>
+        <v>0.27</v>
       </c>
       <c r="I29" t="n">
-        <v>16.62</v>
+        <v>0.41</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>10.66</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>31.98</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>0.82</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>2.63</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D31" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E31" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F31" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G31" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H31" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I31" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1668,29 +1668,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E37" t="n">
-        <v>6.728</v>
+        <v>38.879</v>
       </c>
       <c r="F37" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G37" t="n">
-        <v>60.55</v>
+        <v>155.52</v>
       </c>
       <c r="H37" t="n">
-        <v>4.4</v>
+        <v>16.5</v>
       </c>
       <c r="I37" t="n">
-        <v>7.84</v>
+        <v>11.87</v>
       </c>
       <c r="J37" t="n">
         <v>7.91</v>
@@ -1702,29 +1702,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>3</v>
       </c>
       <c r="D38" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E38" t="n">
-        <v>21.839</v>
+        <v>10.67</v>
       </c>
       <c r="F38" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G38" t="n">
-        <v>65.52</v>
+        <v>32.01</v>
       </c>
       <c r="H38" t="n">
-        <v>-0.15</v>
+        <v>0.85</v>
       </c>
       <c r="I38" t="n">
-        <v>-0.23</v>
+        <v>2.73</v>
       </c>
       <c r="J38" t="n">
         <v>7.91</v>
@@ -1736,29 +1736,29 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D39" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E39" t="n">
-        <v>10.67</v>
+        <v>102.8</v>
       </c>
       <c r="F39" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G39" t="n">
-        <v>32.01</v>
+        <v>102.8</v>
       </c>
       <c r="H39" t="n">
-        <v>0.85</v>
+        <v>2.71</v>
       </c>
       <c r="I39" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="J39" t="n">
         <v>7.91</v>
@@ -1770,29 +1770,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D40" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E40" t="n">
-        <v>38.879</v>
+        <v>6.728</v>
       </c>
       <c r="F40" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G40" t="n">
-        <v>155.52</v>
+        <v>60.55</v>
       </c>
       <c r="H40" t="n">
-        <v>16.5</v>
+        <v>4.4</v>
       </c>
       <c r="I40" t="n">
-        <v>11.87</v>
+        <v>7.84</v>
       </c>
       <c r="J40" t="n">
         <v>7.91</v>
@@ -1804,29 +1804,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E41" t="n">
-        <v>102.8</v>
+        <v>21.839</v>
       </c>
       <c r="F41" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G41" t="n">
-        <v>102.8</v>
+        <v>65.52</v>
       </c>
       <c r="H41" t="n">
-        <v>2.71</v>
+        <v>-0.15</v>
       </c>
       <c r="I41" t="n">
-        <v>2.71</v>
+        <v>-0.23</v>
       </c>
       <c r="J41" t="n">
         <v>7.91</v>
@@ -2178,29 +2178,29 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E52" t="n">
-        <v>6.629</v>
+        <v>10.702</v>
       </c>
       <c r="F52" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G52" t="n">
-        <v>59.66</v>
+        <v>32.11</v>
       </c>
       <c r="H52" t="n">
-        <v>3.51</v>
+        <v>0.95</v>
       </c>
       <c r="I52" t="n">
-        <v>6.25</v>
+        <v>3.05</v>
       </c>
       <c r="J52" t="n">
         <v>7.91</v>
@@ -2212,29 +2212,29 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E53" t="n">
-        <v>21.703</v>
+        <v>100.34</v>
       </c>
       <c r="F53" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G53" t="n">
-        <v>65.11</v>
+        <v>100.34</v>
       </c>
       <c r="H53" t="n">
-        <v>-0.5600000000000001</v>
+        <v>0.25</v>
       </c>
       <c r="I53" t="n">
-        <v>-0.85</v>
+        <v>0.25</v>
       </c>
       <c r="J53" t="n">
         <v>7.91</v>
@@ -2246,29 +2246,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E54" t="n">
-        <v>100.34</v>
+        <v>38.544</v>
       </c>
       <c r="F54" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G54" t="n">
-        <v>100.34</v>
+        <v>154.18</v>
       </c>
       <c r="H54" t="n">
-        <v>0.25</v>
+        <v>15.16</v>
       </c>
       <c r="I54" t="n">
-        <v>0.25</v>
+        <v>10.9</v>
       </c>
       <c r="J54" t="n">
         <v>7.91</v>
@@ -2280,29 +2280,29 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D55" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E55" t="n">
-        <v>38.544</v>
+        <v>6.629</v>
       </c>
       <c r="F55" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G55" t="n">
-        <v>154.18</v>
+        <v>59.66</v>
       </c>
       <c r="H55" t="n">
-        <v>15.16</v>
+        <v>3.51</v>
       </c>
       <c r="I55" t="n">
-        <v>10.9</v>
+        <v>6.25</v>
       </c>
       <c r="J55" t="n">
         <v>7.91</v>
@@ -2314,29 +2314,29 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C56" t="n">
         <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E56" t="n">
-        <v>10.702</v>
+        <v>21.703</v>
       </c>
       <c r="F56" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G56" t="n">
-        <v>32.11</v>
+        <v>65.11</v>
       </c>
       <c r="H56" t="n">
-        <v>0.95</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="I56" t="n">
-        <v>3.05</v>
+        <v>-0.85</v>
       </c>
       <c r="J56" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E62" t="n">
-        <v>6.817</v>
+        <v>105.5</v>
       </c>
       <c r="F62" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G62" t="n">
-        <v>61.35</v>
+        <v>105.5</v>
       </c>
       <c r="H62" t="n">
-        <v>5.2</v>
+        <v>5.41</v>
       </c>
       <c r="I62" t="n">
-        <v>9.26</v>
+        <v>5.41</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D63" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E63" t="n">
-        <v>41.064</v>
+        <v>10.712</v>
       </c>
       <c r="F63" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G63" t="n">
-        <v>164.26</v>
+        <v>32.14</v>
       </c>
       <c r="H63" t="n">
-        <v>25.24</v>
+        <v>0.98</v>
       </c>
       <c r="I63" t="n">
-        <v>18.16</v>
+        <v>3.15</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E64" t="n">
-        <v>10.712</v>
+        <v>22.7</v>
       </c>
       <c r="F64" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G64" t="n">
-        <v>32.14</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H64" t="n">
-        <v>0.98</v>
+        <v>2.43</v>
       </c>
       <c r="I64" t="n">
-        <v>3.15</v>
+        <v>3.7</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D65" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E65" t="n">
-        <v>22.7</v>
+        <v>6.817</v>
       </c>
       <c r="F65" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G65" t="n">
-        <v>68.09999999999999</v>
+        <v>61.35</v>
       </c>
       <c r="H65" t="n">
-        <v>2.43</v>
+        <v>5.2</v>
       </c>
       <c r="I65" t="n">
-        <v>3.7</v>
+        <v>9.26</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D66" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E66" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F66" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G66" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H66" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I66" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E72" t="n">
-        <v>6.811</v>
+        <v>41.15</v>
       </c>
       <c r="F72" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G72" t="n">
-        <v>61.3</v>
+        <v>164.6</v>
       </c>
       <c r="H72" t="n">
-        <v>5.15</v>
+        <v>25.58</v>
       </c>
       <c r="I72" t="n">
-        <v>9.17</v>
+        <v>18.4</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>10.892</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>32.68</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>1.52</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>4.88</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2926,29 +2926,29 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>3</v>
       </c>
       <c r="D74" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E74" t="n">
-        <v>23</v>
+        <v>10.892</v>
       </c>
       <c r="F74" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G74" t="n">
-        <v>69</v>
+        <v>32.68</v>
       </c>
       <c r="H74" t="n">
-        <v>3.33</v>
+        <v>1.52</v>
       </c>
       <c r="I74" t="n">
-        <v>5.07</v>
+        <v>4.88</v>
       </c>
       <c r="J74" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E75" t="n">
-        <v>41.15</v>
+        <v>23</v>
       </c>
       <c r="F75" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G75" t="n">
-        <v>164.6</v>
+        <v>69</v>
       </c>
       <c r="H75" t="n">
-        <v>25.58</v>
+        <v>3.33</v>
       </c>
       <c r="I75" t="n">
-        <v>18.4</v>
+        <v>5.07</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D77" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E77" t="n">
-        <v>6.836</v>
+        <v>23.4</v>
       </c>
       <c r="F77" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G77" t="n">
-        <v>61.52</v>
+        <v>70.2</v>
       </c>
       <c r="H77" t="n">
-        <v>5.37</v>
+        <v>4.53</v>
       </c>
       <c r="I77" t="n">
-        <v>9.56</v>
+        <v>6.9</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D78" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E78" t="n">
-        <v>42.25</v>
+        <v>10.958</v>
       </c>
       <c r="F78" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G78" t="n">
-        <v>169</v>
+        <v>32.87</v>
       </c>
       <c r="H78" t="n">
-        <v>29.98</v>
+        <v>1.71</v>
       </c>
       <c r="I78" t="n">
-        <v>21.57</v>
+        <v>5.49</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E79" t="n">
-        <v>10.958</v>
+        <v>105.8</v>
       </c>
       <c r="F79" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G79" t="n">
-        <v>32.87</v>
+        <v>105.8</v>
       </c>
       <c r="H79" t="n">
-        <v>1.71</v>
+        <v>5.71</v>
       </c>
       <c r="I79" t="n">
-        <v>5.49</v>
+        <v>5.7</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D80" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E80" t="n">
-        <v>105.8</v>
+        <v>6.836</v>
       </c>
       <c r="F80" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G80" t="n">
-        <v>105.8</v>
+        <v>61.52</v>
       </c>
       <c r="H80" t="n">
-        <v>5.71</v>
+        <v>5.37</v>
       </c>
       <c r="I80" t="n">
-        <v>5.7</v>
+        <v>9.56</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D81" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E81" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F81" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G81" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H81" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I81" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E87" t="n">
-        <v>10.852</v>
+        <v>43.005</v>
       </c>
       <c r="F87" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G87" t="n">
-        <v>32.56</v>
+        <v>172.02</v>
       </c>
       <c r="H87" t="n">
-        <v>1.4</v>
+        <v>33</v>
       </c>
       <c r="I87" t="n">
-        <v>4.49</v>
+        <v>23.74</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E88" t="n">
-        <v>6.856</v>
+        <v>10.852</v>
       </c>
       <c r="F88" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G88" t="n">
-        <v>61.7</v>
+        <v>32.56</v>
       </c>
       <c r="H88" t="n">
-        <v>5.55</v>
+        <v>1.4</v>
       </c>
       <c r="I88" t="n">
-        <v>9.880000000000001</v>
+        <v>4.49</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3436,29 +3436,29 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D89" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E89" t="n">
-        <v>23.32</v>
+        <v>6.856</v>
       </c>
       <c r="F89" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G89" t="n">
-        <v>69.95999999999999</v>
+        <v>61.7</v>
       </c>
       <c r="H89" t="n">
-        <v>4.29</v>
+        <v>5.55</v>
       </c>
       <c r="I89" t="n">
-        <v>6.53</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="J89" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E90" t="n">
-        <v>106.28</v>
+        <v>23.32</v>
       </c>
       <c r="F90" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G90" t="n">
-        <v>106.28</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H90" t="n">
-        <v>6.19</v>
+        <v>4.29</v>
       </c>
       <c r="I90" t="n">
-        <v>6.18</v>
+        <v>6.53</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E91" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F91" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G91" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H91" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I91" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D92" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E92" t="n">
-        <v>40.575</v>
+        <v>103.88</v>
       </c>
       <c r="F92" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G92" t="n">
-        <v>162.3</v>
+        <v>103.88</v>
       </c>
       <c r="H92" t="n">
-        <v>23.28</v>
+        <v>3.79</v>
       </c>
       <c r="I92" t="n">
-        <v>16.75</v>
+        <v>3.79</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D93" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E93" t="n">
-        <v>23.025</v>
+        <v>6.797</v>
       </c>
       <c r="F93" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G93" t="n">
-        <v>69.06999999999999</v>
+        <v>61.17</v>
       </c>
       <c r="H93" t="n">
-        <v>3.4</v>
+        <v>5.02</v>
       </c>
       <c r="I93" t="n">
-        <v>5.18</v>
+        <v>8.94</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3606,29 +3606,29 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C94" t="n">
         <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E94" t="n">
-        <v>10.876</v>
+        <v>23.025</v>
       </c>
       <c r="F94" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G94" t="n">
-        <v>32.63</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H94" t="n">
-        <v>1.47</v>
+        <v>3.4</v>
       </c>
       <c r="I94" t="n">
-        <v>4.72</v>
+        <v>5.18</v>
       </c>
       <c r="J94" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D95" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E95" t="n">
-        <v>6.797</v>
+        <v>40.575</v>
       </c>
       <c r="F95" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G95" t="n">
-        <v>61.17</v>
+        <v>162.3</v>
       </c>
       <c r="H95" t="n">
-        <v>5.02</v>
+        <v>23.28</v>
       </c>
       <c r="I95" t="n">
-        <v>8.94</v>
+        <v>16.75</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D96" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E96" t="n">
-        <v>103.88</v>
+        <v>10.876</v>
       </c>
       <c r="F96" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G96" t="n">
-        <v>103.88</v>
+        <v>32.63</v>
       </c>
       <c r="H96" t="n">
-        <v>3.79</v>
+        <v>1.47</v>
       </c>
       <c r="I96" t="n">
-        <v>3.79</v>
+        <v>4.72</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D97" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E97" t="n">
-        <v>10.642</v>
+        <v>6.839</v>
       </c>
       <c r="F97" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G97" t="n">
-        <v>31.93</v>
+        <v>61.55</v>
       </c>
       <c r="H97" t="n">
-        <v>0.77</v>
+        <v>5.4</v>
       </c>
       <c r="I97" t="n">
-        <v>2.47</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C98" t="n">
         <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E98" t="n">
-        <v>23.35</v>
+        <v>10.642</v>
       </c>
       <c r="F98" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G98" t="n">
-        <v>70.05</v>
+        <v>31.93</v>
       </c>
       <c r="H98" t="n">
-        <v>4.38</v>
+        <v>0.77</v>
       </c>
       <c r="I98" t="n">
-        <v>6.67</v>
+        <v>2.47</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3776,29 +3776,29 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D99" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E99" t="n">
-        <v>104.22</v>
+        <v>23.35</v>
       </c>
       <c r="F99" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G99" t="n">
-        <v>104.22</v>
+        <v>70.05</v>
       </c>
       <c r="H99" t="n">
-        <v>4.13</v>
+        <v>4.38</v>
       </c>
       <c r="I99" t="n">
-        <v>4.13</v>
+        <v>6.67</v>
       </c>
       <c r="J99" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E100" t="n">
-        <v>40.65</v>
+        <v>104.22</v>
       </c>
       <c r="F100" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G100" t="n">
-        <v>162.6</v>
+        <v>104.22</v>
       </c>
       <c r="H100" t="n">
-        <v>23.58</v>
+        <v>4.13</v>
       </c>
       <c r="I100" t="n">
-        <v>16.96</v>
+        <v>4.13</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D101" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E101" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F101" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G101" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H101" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I101" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D102" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E102" t="n">
-        <v>103.46</v>
+        <v>40.97</v>
       </c>
       <c r="F102" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G102" t="n">
-        <v>103.46</v>
+        <v>163.88</v>
       </c>
       <c r="H102" t="n">
-        <v>3.37</v>
+        <v>24.86</v>
       </c>
       <c r="I102" t="n">
-        <v>3.37</v>
+        <v>17.88</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D103" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E103" t="n">
-        <v>23.29</v>
+        <v>6.804</v>
       </c>
       <c r="F103" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G103" t="n">
-        <v>69.87</v>
+        <v>61.24</v>
       </c>
       <c r="H103" t="n">
-        <v>4.2</v>
+        <v>5.09</v>
       </c>
       <c r="I103" t="n">
-        <v>6.4</v>
+        <v>9.07</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E104" t="n">
-        <v>40.97</v>
+        <v>103.46</v>
       </c>
       <c r="F104" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G104" t="n">
-        <v>163.88</v>
+        <v>103.46</v>
       </c>
       <c r="H104" t="n">
-        <v>24.86</v>
+        <v>3.37</v>
       </c>
       <c r="I104" t="n">
-        <v>17.88</v>
+        <v>3.37</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E105" t="n">
-        <v>6.804</v>
+        <v>23.29</v>
       </c>
       <c r="F105" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G105" t="n">
-        <v>61.24</v>
+        <v>69.87</v>
       </c>
       <c r="H105" t="n">
-        <v>5.09</v>
+        <v>4.2</v>
       </c>
       <c r="I105" t="n">
-        <v>9.07</v>
+        <v>6.4</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D107" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E107" t="n">
-        <v>103.14</v>
+        <v>23.33</v>
       </c>
       <c r="F107" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G107" t="n">
-        <v>103.14</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H107" t="n">
-        <v>3.05</v>
+        <v>4.32</v>
       </c>
       <c r="I107" t="n">
-        <v>3.05</v>
+        <v>6.58</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D108" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E108" t="n">
-        <v>6.785</v>
+        <v>10.456</v>
       </c>
       <c r="F108" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G108" t="n">
-        <v>61.06</v>
+        <v>31.37</v>
       </c>
       <c r="H108" t="n">
-        <v>4.91</v>
+        <v>0.21</v>
       </c>
       <c r="I108" t="n">
-        <v>8.74</v>
+        <v>0.67</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4116,29 +4116,29 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D109" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E109" t="n">
-        <v>10.456</v>
+        <v>40.5</v>
       </c>
       <c r="F109" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G109" t="n">
-        <v>31.37</v>
+        <v>162</v>
       </c>
       <c r="H109" t="n">
-        <v>0.21</v>
+        <v>22.98</v>
       </c>
       <c r="I109" t="n">
-        <v>0.67</v>
+        <v>16.53</v>
       </c>
       <c r="J109" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D110" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E110" t="n">
-        <v>23.33</v>
+        <v>103.14</v>
       </c>
       <c r="F110" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G110" t="n">
-        <v>69.98999999999999</v>
+        <v>103.14</v>
       </c>
       <c r="H110" t="n">
-        <v>4.32</v>
+        <v>3.05</v>
       </c>
       <c r="I110" t="n">
-        <v>6.58</v>
+        <v>3.05</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D111" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E111" t="n">
-        <v>40.5</v>
+        <v>6.785</v>
       </c>
       <c r="F111" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G111" t="n">
-        <v>162</v>
+        <v>61.06</v>
       </c>
       <c r="H111" t="n">
-        <v>22.98</v>
+        <v>4.91</v>
       </c>
       <c r="I111" t="n">
-        <v>16.53</v>
+        <v>8.74</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E117" t="n">
-        <v>105.96</v>
+        <v>41</v>
       </c>
       <c r="F117" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G117" t="n">
-        <v>105.96</v>
+        <v>164</v>
       </c>
       <c r="H117" t="n">
-        <v>5.87</v>
+        <v>24.98</v>
       </c>
       <c r="I117" t="n">
-        <v>5.86</v>
+        <v>17.97</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D118" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E118" t="n">
-        <v>23.145</v>
+        <v>6.861</v>
       </c>
       <c r="F118" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G118" t="n">
-        <v>69.44</v>
+        <v>61.75</v>
       </c>
       <c r="H118" t="n">
-        <v>3.77</v>
+        <v>5.6</v>
       </c>
       <c r="I118" t="n">
-        <v>5.74</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D119" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E119" t="n">
-        <v>6.861</v>
+        <v>10.756</v>
       </c>
       <c r="F119" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G119" t="n">
-        <v>61.75</v>
+        <v>32.27</v>
       </c>
       <c r="H119" t="n">
-        <v>5.6</v>
+        <v>1.11</v>
       </c>
       <c r="I119" t="n">
-        <v>9.970000000000001</v>
+        <v>3.56</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E120" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F120" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G120" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H120" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I120" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C121" t="n">
         <v>3</v>
       </c>
       <c r="D121" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E121" t="n">
-        <v>10.756</v>
+        <v>23.145</v>
       </c>
       <c r="F121" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G121" t="n">
-        <v>32.27</v>
+        <v>69.44</v>
       </c>
       <c r="H121" t="n">
-        <v>1.11</v>
+        <v>3.77</v>
       </c>
       <c r="I121" t="n">
-        <v>3.56</v>
+        <v>5.74</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E132" t="n">
-        <v>40.54</v>
+        <v>23.18</v>
       </c>
       <c r="F132" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G132" t="n">
-        <v>162.16</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H132" t="n">
-        <v>23.14</v>
+        <v>3.87</v>
       </c>
       <c r="I132" t="n">
-        <v>16.65</v>
+        <v>5.89</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D133" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E133" t="n">
-        <v>11.516</v>
+        <v>6.895</v>
       </c>
       <c r="F133" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G133" t="n">
-        <v>34.55</v>
+        <v>62.05</v>
       </c>
       <c r="H133" t="n">
-        <v>3.39</v>
+        <v>5.9</v>
       </c>
       <c r="I133" t="n">
-        <v>10.88</v>
+        <v>10.51</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D134" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E134" t="n">
-        <v>6.895</v>
+        <v>104.02</v>
       </c>
       <c r="F134" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G134" t="n">
-        <v>62.05</v>
+        <v>104.02</v>
       </c>
       <c r="H134" t="n">
-        <v>5.9</v>
+        <v>3.93</v>
       </c>
       <c r="I134" t="n">
-        <v>10.51</v>
+        <v>3.93</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E135" t="n">
-        <v>23.18</v>
+        <v>40.54</v>
       </c>
       <c r="F135" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G135" t="n">
-        <v>69.54000000000001</v>
+        <v>162.16</v>
       </c>
       <c r="H135" t="n">
-        <v>3.87</v>
+        <v>23.14</v>
       </c>
       <c r="I135" t="n">
-        <v>5.89</v>
+        <v>16.65</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E136" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F136" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G136" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H136" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I136" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D147" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E147" t="n">
-        <v>22.755</v>
+        <v>101.7</v>
       </c>
       <c r="F147" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G147" t="n">
-        <v>68.27</v>
+        <v>101.7</v>
       </c>
       <c r="H147" t="n">
-        <v>2.6</v>
+        <v>1.61</v>
       </c>
       <c r="I147" t="n">
-        <v>3.96</v>
+        <v>1.61</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D148" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E148" t="n">
-        <v>6.826</v>
+        <v>38.955</v>
       </c>
       <c r="F148" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G148" t="n">
-        <v>61.43</v>
+        <v>155.82</v>
       </c>
       <c r="H148" t="n">
-        <v>5.28</v>
+        <v>16.8</v>
       </c>
       <c r="I148" t="n">
-        <v>9.4</v>
+        <v>12.08</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D150" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E150" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F150" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G150" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H150" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I150" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D151" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E151" t="n">
-        <v>101.7</v>
+        <v>6.826</v>
       </c>
       <c r="F151" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G151" t="n">
-        <v>101.7</v>
+        <v>61.43</v>
       </c>
       <c r="H151" t="n">
-        <v>1.61</v>
+        <v>5.28</v>
       </c>
       <c r="I151" t="n">
-        <v>1.61</v>
+        <v>9.4</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E162" t="n">
-        <v>6.927</v>
+        <v>10.748</v>
       </c>
       <c r="F162" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G162" t="n">
-        <v>62.34</v>
+        <v>32.24</v>
       </c>
       <c r="H162" t="n">
-        <v>6.19</v>
+        <v>1.08</v>
       </c>
       <c r="I162" t="n">
-        <v>11.02</v>
+        <v>3.47</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D163" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E163" t="n">
-        <v>23.01</v>
+        <v>103.84</v>
       </c>
       <c r="F163" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G163" t="n">
-        <v>69.03</v>
+        <v>103.84</v>
       </c>
       <c r="H163" t="n">
-        <v>3.36</v>
+        <v>3.75</v>
       </c>
       <c r="I163" t="n">
-        <v>5.12</v>
+        <v>3.75</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -5986,29 +5986,29 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D164" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E164" t="n">
-        <v>103.84</v>
+        <v>38.845</v>
       </c>
       <c r="F164" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G164" t="n">
-        <v>103.84</v>
+        <v>155.38</v>
       </c>
       <c r="H164" t="n">
-        <v>3.75</v>
+        <v>16.36</v>
       </c>
       <c r="I164" t="n">
-        <v>3.75</v>
+        <v>11.77</v>
       </c>
       <c r="J164" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D165" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E165" t="n">
-        <v>38.845</v>
+        <v>6.927</v>
       </c>
       <c r="F165" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G165" t="n">
-        <v>155.38</v>
+        <v>62.34</v>
       </c>
       <c r="H165" t="n">
-        <v>16.36</v>
+        <v>6.19</v>
       </c>
       <c r="I165" t="n">
-        <v>11.77</v>
+        <v>11.02</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C166" t="n">
         <v>3</v>
       </c>
       <c r="D166" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E166" t="n">
-        <v>10.748</v>
+        <v>23.01</v>
       </c>
       <c r="F166" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G166" t="n">
-        <v>32.24</v>
+        <v>69.03</v>
       </c>
       <c r="H166" t="n">
-        <v>1.08</v>
+        <v>3.36</v>
       </c>
       <c r="I166" t="n">
-        <v>3.47</v>
+        <v>5.12</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C177" t="n">
         <v>3</v>
       </c>
       <c r="D177" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E177" t="n">
-        <v>10.642</v>
+        <v>22.95</v>
       </c>
       <c r="F177" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G177" t="n">
-        <v>31.93</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H177" t="n">
-        <v>0.77</v>
+        <v>3.18</v>
       </c>
       <c r="I177" t="n">
-        <v>2.47</v>
+        <v>4.84</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D178" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E178" t="n">
-        <v>6.922</v>
+        <v>102.54</v>
       </c>
       <c r="F178" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G178" t="n">
-        <v>62.3</v>
+        <v>102.54</v>
       </c>
       <c r="H178" t="n">
-        <v>6.15</v>
+        <v>2.45</v>
       </c>
       <c r="I178" t="n">
-        <v>10.95</v>
+        <v>2.45</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D179" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E179" t="n">
-        <v>38.245</v>
+        <v>10.642</v>
       </c>
       <c r="F179" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G179" t="n">
-        <v>152.98</v>
+        <v>31.93</v>
       </c>
       <c r="H179" t="n">
-        <v>13.96</v>
+        <v>0.77</v>
       </c>
       <c r="I179" t="n">
-        <v>10.04</v>
+        <v>2.47</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D180" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E180" t="n">
-        <v>102.54</v>
+        <v>6.922</v>
       </c>
       <c r="F180" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G180" t="n">
-        <v>102.54</v>
+        <v>62.3</v>
       </c>
       <c r="H180" t="n">
-        <v>2.45</v>
+        <v>6.15</v>
       </c>
       <c r="I180" t="n">
-        <v>2.45</v>
+        <v>10.95</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,29 +6564,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D181" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E181" t="n">
-        <v>22.95</v>
+        <v>38.245</v>
       </c>
       <c r="F181" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G181" t="n">
-        <v>68.84999999999999</v>
+        <v>152.98</v>
       </c>
       <c r="H181" t="n">
-        <v>3.18</v>
+        <v>13.96</v>
       </c>
       <c r="I181" t="n">
-        <v>4.84</v>
+        <v>10.04</v>
       </c>
       <c r="J181" t="n">
         <v>7.91</v>
@@ -6938,29 +6938,29 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D192" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E192" t="n">
-        <v>102.46</v>
+        <v>22.82</v>
       </c>
       <c r="F192" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G192" t="n">
-        <v>102.46</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="H192" t="n">
-        <v>2.37</v>
+        <v>2.79</v>
       </c>
       <c r="I192" t="n">
-        <v>2.37</v>
+        <v>4.25</v>
       </c>
       <c r="J192" t="n">
         <v>7.91</v>
@@ -6972,29 +6972,29 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D193" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E193" t="n">
-        <v>10.792</v>
+        <v>6.894</v>
       </c>
       <c r="F193" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G193" t="n">
-        <v>32.38</v>
+        <v>62.05</v>
       </c>
       <c r="H193" t="n">
-        <v>1.22</v>
+        <v>5.9</v>
       </c>
       <c r="I193" t="n">
-        <v>3.92</v>
+        <v>10.51</v>
       </c>
       <c r="J193" t="n">
         <v>7.91</v>
@@ -7006,29 +7006,29 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D194" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E194" t="n">
-        <v>38.755</v>
+        <v>10.792</v>
       </c>
       <c r="F194" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G194" t="n">
-        <v>155.02</v>
+        <v>32.38</v>
       </c>
       <c r="H194" t="n">
-        <v>16</v>
+        <v>1.22</v>
       </c>
       <c r="I194" t="n">
-        <v>11.51</v>
+        <v>3.92</v>
       </c>
       <c r="J194" t="n">
         <v>7.91</v>
@@ -7040,29 +7040,29 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D195" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E195" t="n">
-        <v>22.82</v>
+        <v>102.46</v>
       </c>
       <c r="F195" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G195" t="n">
-        <v>68.45999999999999</v>
+        <v>102.46</v>
       </c>
       <c r="H195" t="n">
-        <v>2.79</v>
+        <v>2.37</v>
       </c>
       <c r="I195" t="n">
-        <v>4.25</v>
+        <v>2.37</v>
       </c>
       <c r="J195" t="n">
         <v>7.91</v>
@@ -7074,29 +7074,29 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D196" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E196" t="n">
-        <v>6.894</v>
+        <v>38.755</v>
       </c>
       <c r="F196" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G196" t="n">
-        <v>62.05</v>
+        <v>155.02</v>
       </c>
       <c r="H196" t="n">
-        <v>5.9</v>
+        <v>16</v>
       </c>
       <c r="I196" t="n">
-        <v>10.51</v>
+        <v>11.51</v>
       </c>
       <c r="J196" t="n">
         <v>7.91</v>
@@ -7448,29 +7448,29 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D207" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E207" t="n">
-        <v>99.90000000000001</v>
+        <v>37.82</v>
       </c>
       <c r="F207" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G207" t="n">
-        <v>99.90000000000001</v>
+        <v>151.28</v>
       </c>
       <c r="H207" t="n">
-        <v>-0.19</v>
+        <v>12.26</v>
       </c>
       <c r="I207" t="n">
-        <v>-0.19</v>
+        <v>8.82</v>
       </c>
       <c r="J207" t="n">
         <v>7.91</v>
@@ -7482,29 +7482,29 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C208" t="n">
         <v>3</v>
       </c>
       <c r="D208" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E208" t="n">
-        <v>22.725</v>
+        <v>11.172</v>
       </c>
       <c r="F208" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G208" t="n">
-        <v>68.18000000000001</v>
+        <v>33.52</v>
       </c>
       <c r="H208" t="n">
-        <v>2.51</v>
+        <v>2.36</v>
       </c>
       <c r="I208" t="n">
-        <v>3.82</v>
+        <v>7.57</v>
       </c>
       <c r="J208" t="n">
         <v>7.91</v>
@@ -7516,29 +7516,29 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D209" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E209" t="n">
-        <v>6.865</v>
+        <v>22.725</v>
       </c>
       <c r="F209" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G209" t="n">
-        <v>61.79</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H209" t="n">
-        <v>5.64</v>
+        <v>2.51</v>
       </c>
       <c r="I209" t="n">
-        <v>10.04</v>
+        <v>3.82</v>
       </c>
       <c r="J209" t="n">
         <v>7.91</v>
@@ -7550,29 +7550,29 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D210" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E210" t="n">
-        <v>11.172</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F210" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G210" t="n">
-        <v>33.52</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H210" t="n">
-        <v>2.36</v>
+        <v>-0.19</v>
       </c>
       <c r="I210" t="n">
-        <v>7.57</v>
+        <v>-0.19</v>
       </c>
       <c r="J210" t="n">
         <v>7.91</v>
@@ -7584,29 +7584,29 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D211" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E211" t="n">
-        <v>37.82</v>
+        <v>6.865</v>
       </c>
       <c r="F211" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G211" t="n">
-        <v>151.28</v>
+        <v>61.79</v>
       </c>
       <c r="H211" t="n">
-        <v>12.26</v>
+        <v>5.64</v>
       </c>
       <c r="I211" t="n">
-        <v>8.82</v>
+        <v>10.04</v>
       </c>
       <c r="J211" t="n">
         <v>7.91</v>
@@ -7779,6 +7779,176 @@
         <v>9.630000000000001</v>
       </c>
       <c r="J216" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>3</v>
+      </c>
+      <c r="D217" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E217" t="n">
+        <v>11.546</v>
+      </c>
+      <c r="F217" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G217" t="n">
+        <v>34.64</v>
+      </c>
+      <c r="H217" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="I217" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="J217" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>4</v>
+      </c>
+      <c r="D218" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E218" t="n">
+        <v>36.75</v>
+      </c>
+      <c r="F218" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G218" t="n">
+        <v>147</v>
+      </c>
+      <c r="H218" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="I218" t="n">
+        <v>5.74</v>
+      </c>
+      <c r="J218" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>3</v>
+      </c>
+      <c r="D219" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E219" t="n">
+        <v>23.175</v>
+      </c>
+      <c r="F219" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G219" t="n">
+        <v>69.53</v>
+      </c>
+      <c r="H219" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="I219" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="J219" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C220" t="n">
+        <v>1</v>
+      </c>
+      <c r="D220" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E220" t="n">
+        <v>98.02</v>
+      </c>
+      <c r="F220" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G220" t="n">
+        <v>98.02</v>
+      </c>
+      <c r="H220" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="I220" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="J220" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>9</v>
+      </c>
+      <c r="D221" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E221" t="n">
+        <v>6.864</v>
+      </c>
+      <c r="F221" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G221" t="n">
+        <v>61.78</v>
+      </c>
+      <c r="H221" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="I221" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="J221" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 29/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J221"/>
+  <dimension ref="A1:J226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D12" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E12" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F12" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G12" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H12" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I12" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D13" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E13" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F13" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G13" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H13" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I13" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E14" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F14" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G14" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H14" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I14" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E15" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F15" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G15" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H15" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I15" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E16" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F16" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G16" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H16" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I16" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D27" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E27" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F27" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G27" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H27" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I27" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E28" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F28" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G28" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H28" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I28" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C29" t="n">
         <v>3</v>
       </c>
       <c r="D29" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E29" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F29" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G29" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H29" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I29" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D30" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E30" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F30" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G30" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H30" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I30" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E31" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F31" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G31" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H31" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I31" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E42" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F42" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G42" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I42" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D43" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E43" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F43" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G43" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H43" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I43" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E44" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F44" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G44" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H44" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I44" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E45" t="n">
-        <v>22</v>
+        <v>38.497</v>
       </c>
       <c r="F45" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G45" t="n">
-        <v>66</v>
+        <v>153.99</v>
       </c>
       <c r="H45" t="n">
-        <v>0.33</v>
+        <v>14.97</v>
       </c>
       <c r="I45" t="n">
-        <v>0.5</v>
+        <v>10.77</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E46" t="n">
-        <v>6.629</v>
+        <v>100.06</v>
       </c>
       <c r="F46" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G46" t="n">
-        <v>59.66</v>
+        <v>100.06</v>
       </c>
       <c r="H46" t="n">
-        <v>3.51</v>
+        <v>-0.03</v>
       </c>
       <c r="I46" t="n">
-        <v>6.25</v>
+        <v>-0.03</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>3</v>
       </c>
       <c r="D59" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E59" t="n">
-        <v>10.75</v>
+        <v>22.289</v>
       </c>
       <c r="F59" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G59" t="n">
-        <v>32.25</v>
+        <v>66.87</v>
       </c>
       <c r="H59" t="n">
-        <v>1.09</v>
+        <v>1.2</v>
       </c>
       <c r="I59" t="n">
-        <v>3.5</v>
+        <v>1.83</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E60" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F60" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G60" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H60" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I60" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E61" t="n">
-        <v>102.86</v>
+        <v>10.75</v>
       </c>
       <c r="F61" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G61" t="n">
-        <v>102.86</v>
+        <v>32.25</v>
       </c>
       <c r="H61" t="n">
-        <v>2.77</v>
+        <v>1.09</v>
       </c>
       <c r="I61" t="n">
-        <v>2.77</v>
+        <v>3.5</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E67" t="n">
-        <v>40.567</v>
+        <v>6.807</v>
       </c>
       <c r="F67" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G67" t="n">
-        <v>162.27</v>
+        <v>61.26</v>
       </c>
       <c r="H67" t="n">
-        <v>23.25</v>
+        <v>5.11</v>
       </c>
       <c r="I67" t="n">
-        <v>16.72</v>
+        <v>9.1</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D68" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E68" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F68" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G68" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H68" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I68" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E69" t="n">
-        <v>104.58</v>
+        <v>10.796</v>
       </c>
       <c r="F69" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G69" t="n">
-        <v>104.58</v>
+        <v>32.39</v>
       </c>
       <c r="H69" t="n">
-        <v>4.49</v>
+        <v>1.23</v>
       </c>
       <c r="I69" t="n">
-        <v>4.49</v>
+        <v>3.95</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D70" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E70" t="n">
-        <v>6.807</v>
+        <v>40.567</v>
       </c>
       <c r="F70" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G70" t="n">
-        <v>61.26</v>
+        <v>162.27</v>
       </c>
       <c r="H70" t="n">
-        <v>5.11</v>
+        <v>23.25</v>
       </c>
       <c r="I70" t="n">
-        <v>9.1</v>
+        <v>16.72</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C71" t="n">
         <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E71" t="n">
-        <v>10.796</v>
+        <v>22.797</v>
       </c>
       <c r="F71" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G71" t="n">
-        <v>32.39</v>
+        <v>68.39</v>
       </c>
       <c r="H71" t="n">
-        <v>1.23</v>
+        <v>2.72</v>
       </c>
       <c r="I71" t="n">
-        <v>3.95</v>
+        <v>4.14</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E82" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F82" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G82" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H82" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I82" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E83" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F83" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G83" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H83" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I83" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C84" t="n">
         <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E84" t="n">
-        <v>23.3</v>
+        <v>10.988</v>
       </c>
       <c r="F84" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G84" t="n">
-        <v>69.90000000000001</v>
+        <v>32.96</v>
       </c>
       <c r="H84" t="n">
-        <v>4.23</v>
+        <v>1.8</v>
       </c>
       <c r="I84" t="n">
-        <v>6.44</v>
+        <v>5.78</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D85" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E85" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F85" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G85" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H85" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I85" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D86" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E86" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F86" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G86" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H86" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I86" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D97" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E97" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F97" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G97" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H97" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I97" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E98" t="n">
-        <v>10.642</v>
+        <v>104.22</v>
       </c>
       <c r="F98" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G98" t="n">
-        <v>31.93</v>
+        <v>104.22</v>
       </c>
       <c r="H98" t="n">
-        <v>0.77</v>
+        <v>4.13</v>
       </c>
       <c r="I98" t="n">
-        <v>2.47</v>
+        <v>4.13</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D100" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E100" t="n">
-        <v>104.22</v>
+        <v>6.839</v>
       </c>
       <c r="F100" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G100" t="n">
-        <v>104.22</v>
+        <v>61.55</v>
       </c>
       <c r="H100" t="n">
-        <v>4.13</v>
+        <v>5.4</v>
       </c>
       <c r="I100" t="n">
-        <v>4.13</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D101" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E101" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F101" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G101" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H101" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I101" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D112" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E112" t="n">
-        <v>10.568</v>
+        <v>103.56</v>
       </c>
       <c r="F112" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G112" t="n">
-        <v>31.7</v>
+        <v>103.56</v>
       </c>
       <c r="H112" t="n">
-        <v>0.54</v>
+        <v>3.47</v>
       </c>
       <c r="I112" t="n">
-        <v>1.73</v>
+        <v>3.47</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D113" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E113" t="n">
-        <v>23.025</v>
+        <v>40</v>
       </c>
       <c r="F113" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G113" t="n">
-        <v>69.06999999999999</v>
+        <v>160</v>
       </c>
       <c r="H113" t="n">
-        <v>3.4</v>
+        <v>20.98</v>
       </c>
       <c r="I113" t="n">
-        <v>5.18</v>
+        <v>15.09</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E115" t="n">
-        <v>40</v>
+        <v>23.025</v>
       </c>
       <c r="F115" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G115" t="n">
-        <v>160</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H115" t="n">
-        <v>20.98</v>
+        <v>3.4</v>
       </c>
       <c r="I115" t="n">
-        <v>15.09</v>
+        <v>5.18</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E116" t="n">
-        <v>103.56</v>
+        <v>10.568</v>
       </c>
       <c r="F116" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G116" t="n">
-        <v>103.56</v>
+        <v>31.7</v>
       </c>
       <c r="H116" t="n">
-        <v>3.47</v>
+        <v>0.54</v>
       </c>
       <c r="I116" t="n">
-        <v>3.47</v>
+        <v>1.73</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D122" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E122" t="n">
-        <v>40.395</v>
+        <v>106</v>
       </c>
       <c r="F122" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G122" t="n">
-        <v>161.58</v>
+        <v>106</v>
       </c>
       <c r="H122" t="n">
-        <v>22.56</v>
+        <v>5.91</v>
       </c>
       <c r="I122" t="n">
-        <v>16.23</v>
+        <v>5.9</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D123" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E123" t="n">
-        <v>6.901</v>
+        <v>11.038</v>
       </c>
       <c r="F123" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G123" t="n">
-        <v>62.11</v>
+        <v>33.11</v>
       </c>
       <c r="H123" t="n">
-        <v>5.96</v>
+        <v>1.95</v>
       </c>
       <c r="I123" t="n">
-        <v>10.61</v>
+        <v>6.26</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4626,29 +4626,29 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C124" t="n">
         <v>3</v>
       </c>
       <c r="D124" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E124" t="n">
-        <v>11.038</v>
+        <v>23.165</v>
       </c>
       <c r="F124" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G124" t="n">
-        <v>33.11</v>
+        <v>69.5</v>
       </c>
       <c r="H124" t="n">
-        <v>1.95</v>
+        <v>3.83</v>
       </c>
       <c r="I124" t="n">
-        <v>6.26</v>
+        <v>5.83</v>
       </c>
       <c r="J124" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D125" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E125" t="n">
-        <v>106</v>
+        <v>40.395</v>
       </c>
       <c r="F125" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G125" t="n">
-        <v>106</v>
+        <v>161.58</v>
       </c>
       <c r="H125" t="n">
-        <v>5.91</v>
+        <v>22.56</v>
       </c>
       <c r="I125" t="n">
-        <v>5.9</v>
+        <v>16.23</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D126" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E126" t="n">
-        <v>23.165</v>
+        <v>6.901</v>
       </c>
       <c r="F126" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G126" t="n">
-        <v>69.5</v>
+        <v>62.11</v>
       </c>
       <c r="H126" t="n">
-        <v>3.83</v>
+        <v>5.96</v>
       </c>
       <c r="I126" t="n">
-        <v>5.83</v>
+        <v>10.61</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D137" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E137" t="n">
-        <v>104.76</v>
+        <v>11.728</v>
       </c>
       <c r="F137" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G137" t="n">
-        <v>104.76</v>
+        <v>35.18</v>
       </c>
       <c r="H137" t="n">
-        <v>4.67</v>
+        <v>4.02</v>
       </c>
       <c r="I137" t="n">
-        <v>4.67</v>
+        <v>12.9</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D138" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E138" t="n">
-        <v>40.61</v>
+        <v>23.3</v>
       </c>
       <c r="F138" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G138" t="n">
-        <v>162.44</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H138" t="n">
-        <v>23.42</v>
+        <v>4.23</v>
       </c>
       <c r="I138" t="n">
-        <v>16.85</v>
+        <v>6.44</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5136,29 +5136,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D139" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E139" t="n">
-        <v>23.3</v>
+        <v>6.927</v>
       </c>
       <c r="F139" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G139" t="n">
-        <v>69.90000000000001</v>
+        <v>62.34</v>
       </c>
       <c r="H139" t="n">
-        <v>4.23</v>
+        <v>6.19</v>
       </c>
       <c r="I139" t="n">
-        <v>6.44</v>
+        <v>11.02</v>
       </c>
       <c r="J139" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D140" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E140" t="n">
-        <v>11.728</v>
+        <v>104.76</v>
       </c>
       <c r="F140" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G140" t="n">
-        <v>35.18</v>
+        <v>104.76</v>
       </c>
       <c r="H140" t="n">
-        <v>4.02</v>
+        <v>4.67</v>
       </c>
       <c r="I140" t="n">
-        <v>12.9</v>
+        <v>4.67</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D141" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E141" t="n">
-        <v>6.927</v>
+        <v>40.61</v>
       </c>
       <c r="F141" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G141" t="n">
-        <v>62.34</v>
+        <v>162.44</v>
       </c>
       <c r="H141" t="n">
-        <v>6.19</v>
+        <v>23.42</v>
       </c>
       <c r="I141" t="n">
-        <v>11.02</v>
+        <v>16.85</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C152" t="n">
         <v>3</v>
       </c>
       <c r="D152" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E152" t="n">
-        <v>23.045</v>
+        <v>11.034</v>
       </c>
       <c r="F152" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G152" t="n">
-        <v>69.14</v>
+        <v>33.1</v>
       </c>
       <c r="H152" t="n">
-        <v>3.47</v>
+        <v>1.94</v>
       </c>
       <c r="I152" t="n">
-        <v>5.28</v>
+        <v>6.23</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D153" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E153" t="n">
-        <v>39.915</v>
+        <v>104.12</v>
       </c>
       <c r="F153" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G153" t="n">
-        <v>159.66</v>
+        <v>104.12</v>
       </c>
       <c r="H153" t="n">
-        <v>20.64</v>
+        <v>4.03</v>
       </c>
       <c r="I153" t="n">
-        <v>14.85</v>
+        <v>4.03</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5680,29 +5680,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D155" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E155" t="n">
-        <v>104.12</v>
+        <v>23.045</v>
       </c>
       <c r="F155" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G155" t="n">
-        <v>104.12</v>
+        <v>69.14</v>
       </c>
       <c r="H155" t="n">
-        <v>4.03</v>
+        <v>3.47</v>
       </c>
       <c r="I155" t="n">
-        <v>4.03</v>
+        <v>5.28</v>
       </c>
       <c r="J155" t="n">
         <v>7.91</v>
@@ -5714,29 +5714,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D156" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E156" t="n">
-        <v>11.034</v>
+        <v>39.915</v>
       </c>
       <c r="F156" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G156" t="n">
-        <v>33.1</v>
+        <v>159.66</v>
       </c>
       <c r="H156" t="n">
-        <v>1.94</v>
+        <v>20.64</v>
       </c>
       <c r="I156" t="n">
-        <v>6.23</v>
+        <v>14.85</v>
       </c>
       <c r="J156" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D167" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E167" t="n">
-        <v>38.98</v>
+        <v>22.92</v>
       </c>
       <c r="F167" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G167" t="n">
-        <v>155.92</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H167" t="n">
-        <v>16.9</v>
+        <v>3.09</v>
       </c>
       <c r="I167" t="n">
-        <v>12.16</v>
+        <v>4.71</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D168" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E168" t="n">
-        <v>6.911</v>
+        <v>10.726</v>
       </c>
       <c r="F168" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G168" t="n">
-        <v>62.2</v>
+        <v>32.18</v>
       </c>
       <c r="H168" t="n">
-        <v>6.05</v>
+        <v>1.02</v>
       </c>
       <c r="I168" t="n">
-        <v>10.77</v>
+        <v>3.27</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6156,29 +6156,29 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D169" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E169" t="n">
-        <v>10.726</v>
+        <v>103.98</v>
       </c>
       <c r="F169" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G169" t="n">
-        <v>32.18</v>
+        <v>103.98</v>
       </c>
       <c r="H169" t="n">
-        <v>1.02</v>
+        <v>3.89</v>
       </c>
       <c r="I169" t="n">
-        <v>3.27</v>
+        <v>3.89</v>
       </c>
       <c r="J169" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D170" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E170" t="n">
-        <v>103.98</v>
+        <v>6.911</v>
       </c>
       <c r="F170" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G170" t="n">
-        <v>103.98</v>
+        <v>62.2</v>
       </c>
       <c r="H170" t="n">
-        <v>3.89</v>
+        <v>6.05</v>
       </c>
       <c r="I170" t="n">
-        <v>3.89</v>
+        <v>10.77</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,29 +6224,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D171" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E171" t="n">
-        <v>22.92</v>
+        <v>38.98</v>
       </c>
       <c r="F171" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G171" t="n">
-        <v>68.76000000000001</v>
+        <v>155.92</v>
       </c>
       <c r="H171" t="n">
-        <v>3.09</v>
+        <v>16.9</v>
       </c>
       <c r="I171" t="n">
-        <v>4.71</v>
+        <v>12.16</v>
       </c>
       <c r="J171" t="n">
         <v>7.91</v>
@@ -6598,29 +6598,29 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D182" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E182" t="n">
-        <v>37.235</v>
+        <v>22.835</v>
       </c>
       <c r="F182" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G182" t="n">
-        <v>148.94</v>
+        <v>68.5</v>
       </c>
       <c r="H182" t="n">
-        <v>9.92</v>
+        <v>2.83</v>
       </c>
       <c r="I182" t="n">
-        <v>7.14</v>
+        <v>4.31</v>
       </c>
       <c r="J182" t="n">
         <v>7.91</v>
@@ -6632,29 +6632,29 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D183" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E183" t="n">
-        <v>10.776</v>
+        <v>6.848</v>
       </c>
       <c r="F183" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G183" t="n">
-        <v>32.33</v>
+        <v>61.63</v>
       </c>
       <c r="H183" t="n">
-        <v>1.17</v>
+        <v>5.48</v>
       </c>
       <c r="I183" t="n">
-        <v>3.75</v>
+        <v>9.76</v>
       </c>
       <c r="J183" t="n">
         <v>7.91</v>
@@ -6700,29 +6700,29 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D185" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E185" t="n">
-        <v>6.848</v>
+        <v>10.776</v>
       </c>
       <c r="F185" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G185" t="n">
-        <v>61.63</v>
+        <v>32.33</v>
       </c>
       <c r="H185" t="n">
-        <v>5.48</v>
+        <v>1.17</v>
       </c>
       <c r="I185" t="n">
-        <v>9.76</v>
+        <v>3.75</v>
       </c>
       <c r="J185" t="n">
         <v>7.91</v>
@@ -6734,29 +6734,29 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E186" t="n">
-        <v>22.835</v>
+        <v>37.235</v>
       </c>
       <c r="F186" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G186" t="n">
-        <v>68.5</v>
+        <v>148.94</v>
       </c>
       <c r="H186" t="n">
-        <v>2.83</v>
+        <v>9.92</v>
       </c>
       <c r="I186" t="n">
-        <v>4.31</v>
+        <v>7.14</v>
       </c>
       <c r="J186" t="n">
         <v>7.91</v>
@@ -7108,29 +7108,29 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D197" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E197" t="n">
-        <v>6.909</v>
+        <v>38.565</v>
       </c>
       <c r="F197" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G197" t="n">
-        <v>62.18</v>
+        <v>154.26</v>
       </c>
       <c r="H197" t="n">
-        <v>6.03</v>
+        <v>15.24</v>
       </c>
       <c r="I197" t="n">
-        <v>10.74</v>
+        <v>10.96</v>
       </c>
       <c r="J197" t="n">
         <v>7.91</v>
@@ -7142,29 +7142,29 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D198" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E198" t="n">
-        <v>102.48</v>
+        <v>11.022</v>
       </c>
       <c r="F198" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G198" t="n">
-        <v>102.48</v>
+        <v>33.07</v>
       </c>
       <c r="H198" t="n">
-        <v>2.39</v>
+        <v>1.91</v>
       </c>
       <c r="I198" t="n">
-        <v>2.39</v>
+        <v>6.13</v>
       </c>
       <c r="J198" t="n">
         <v>7.91</v>
@@ -7176,29 +7176,29 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D199" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E199" t="n">
-        <v>22.6</v>
+        <v>102.48</v>
       </c>
       <c r="F199" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G199" t="n">
-        <v>67.8</v>
+        <v>102.48</v>
       </c>
       <c r="H199" t="n">
-        <v>2.13</v>
+        <v>2.39</v>
       </c>
       <c r="I199" t="n">
-        <v>3.24</v>
+        <v>2.39</v>
       </c>
       <c r="J199" t="n">
         <v>7.91</v>
@@ -7210,29 +7210,29 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D200" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E200" t="n">
-        <v>11.022</v>
+        <v>6.909</v>
       </c>
       <c r="F200" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G200" t="n">
-        <v>33.07</v>
+        <v>62.18</v>
       </c>
       <c r="H200" t="n">
-        <v>1.91</v>
+        <v>6.03</v>
       </c>
       <c r="I200" t="n">
-        <v>6.13</v>
+        <v>10.74</v>
       </c>
       <c r="J200" t="n">
         <v>7.91</v>
@@ -7244,29 +7244,29 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D201" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E201" t="n">
-        <v>38.565</v>
+        <v>22.6</v>
       </c>
       <c r="F201" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G201" t="n">
-        <v>154.26</v>
+        <v>67.8</v>
       </c>
       <c r="H201" t="n">
-        <v>15.24</v>
+        <v>2.13</v>
       </c>
       <c r="I201" t="n">
-        <v>10.96</v>
+        <v>3.24</v>
       </c>
       <c r="J201" t="n">
         <v>7.91</v>
@@ -7448,29 +7448,29 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D207" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E207" t="n">
-        <v>37.82</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F207" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G207" t="n">
-        <v>151.28</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H207" t="n">
-        <v>12.26</v>
+        <v>-0.19</v>
       </c>
       <c r="I207" t="n">
-        <v>8.82</v>
+        <v>-0.19</v>
       </c>
       <c r="J207" t="n">
         <v>7.91</v>
@@ -7482,29 +7482,29 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C208" t="n">
         <v>3</v>
       </c>
       <c r="D208" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E208" t="n">
-        <v>11.172</v>
+        <v>22.725</v>
       </c>
       <c r="F208" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G208" t="n">
-        <v>33.52</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H208" t="n">
-        <v>2.36</v>
+        <v>2.51</v>
       </c>
       <c r="I208" t="n">
-        <v>7.57</v>
+        <v>3.82</v>
       </c>
       <c r="J208" t="n">
         <v>7.91</v>
@@ -7516,29 +7516,29 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D209" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E209" t="n">
-        <v>22.725</v>
+        <v>6.865</v>
       </c>
       <c r="F209" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G209" t="n">
-        <v>68.18000000000001</v>
+        <v>61.79</v>
       </c>
       <c r="H209" t="n">
-        <v>2.51</v>
+        <v>5.64</v>
       </c>
       <c r="I209" t="n">
-        <v>3.82</v>
+        <v>10.04</v>
       </c>
       <c r="J209" t="n">
         <v>7.91</v>
@@ -7550,29 +7550,29 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D210" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E210" t="n">
-        <v>99.90000000000001</v>
+        <v>37.82</v>
       </c>
       <c r="F210" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G210" t="n">
-        <v>99.90000000000001</v>
+        <v>151.28</v>
       </c>
       <c r="H210" t="n">
-        <v>-0.19</v>
+        <v>12.26</v>
       </c>
       <c r="I210" t="n">
-        <v>-0.19</v>
+        <v>8.82</v>
       </c>
       <c r="J210" t="n">
         <v>7.91</v>
@@ -7584,29 +7584,29 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D211" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E211" t="n">
-        <v>6.865</v>
+        <v>11.172</v>
       </c>
       <c r="F211" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G211" t="n">
-        <v>61.79</v>
+        <v>33.52</v>
       </c>
       <c r="H211" t="n">
-        <v>5.64</v>
+        <v>2.36</v>
       </c>
       <c r="I211" t="n">
-        <v>10.04</v>
+        <v>7.57</v>
       </c>
       <c r="J211" t="n">
         <v>7.91</v>
@@ -7788,29 +7788,29 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D217" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E217" t="n">
-        <v>11.546</v>
+        <v>6.864</v>
       </c>
       <c r="F217" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G217" t="n">
-        <v>34.64</v>
+        <v>61.78</v>
       </c>
       <c r="H217" t="n">
-        <v>3.48</v>
+        <v>5.63</v>
       </c>
       <c r="I217" t="n">
-        <v>11.17</v>
+        <v>10.03</v>
       </c>
       <c r="J217" t="n">
         <v>7.91</v>
@@ -7822,29 +7822,29 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D218" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E218" t="n">
-        <v>36.75</v>
+        <v>11.546</v>
       </c>
       <c r="F218" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G218" t="n">
-        <v>147</v>
+        <v>34.64</v>
       </c>
       <c r="H218" t="n">
-        <v>7.98</v>
+        <v>3.48</v>
       </c>
       <c r="I218" t="n">
-        <v>5.74</v>
+        <v>11.17</v>
       </c>
       <c r="J218" t="n">
         <v>7.91</v>
@@ -7856,29 +7856,29 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D219" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E219" t="n">
-        <v>23.175</v>
+        <v>36.75</v>
       </c>
       <c r="F219" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G219" t="n">
-        <v>69.53</v>
+        <v>147</v>
       </c>
       <c r="H219" t="n">
-        <v>3.86</v>
+        <v>7.98</v>
       </c>
       <c r="I219" t="n">
-        <v>5.88</v>
+        <v>5.74</v>
       </c>
       <c r="J219" t="n">
         <v>7.91</v>
@@ -7890,29 +7890,29 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D220" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E220" t="n">
-        <v>98.02</v>
+        <v>23.175</v>
       </c>
       <c r="F220" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G220" t="n">
-        <v>98.02</v>
+        <v>69.53</v>
       </c>
       <c r="H220" t="n">
-        <v>-2.07</v>
+        <v>3.86</v>
       </c>
       <c r="I220" t="n">
-        <v>-2.07</v>
+        <v>5.88</v>
       </c>
       <c r="J220" t="n">
         <v>7.91</v>
@@ -7924,31 +7924,201 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E221" t="n">
+        <v>98.02</v>
+      </c>
+      <c r="F221" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G221" t="n">
+        <v>98.02</v>
+      </c>
+      <c r="H221" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="I221" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="J221" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>1</v>
+      </c>
+      <c r="D222" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E222" t="n">
+        <v>96.67</v>
+      </c>
+      <c r="F222" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G222" t="n">
+        <v>96.67</v>
+      </c>
+      <c r="H222" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="I222" t="n">
+        <v>-3.42</v>
+      </c>
+      <c r="J222" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>3</v>
+      </c>
+      <c r="D223" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E223" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F223" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G223" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H223" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="I223" t="n">
+        <v>10.72</v>
+      </c>
+      <c r="J223" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>4</v>
+      </c>
+      <c r="D224" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E224" t="n">
+        <v>35.89</v>
+      </c>
+      <c r="F224" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G224" t="n">
+        <v>143.56</v>
+      </c>
+      <c r="H224" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="I224" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="J224" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>3</v>
+      </c>
+      <c r="D225" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E225" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="F225" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G225" t="n">
+        <v>69.36</v>
+      </c>
+      <c r="H225" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="I225" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="J225" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="1" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C221" t="n">
+      <c r="C226" t="n">
         <v>9</v>
       </c>
-      <c r="D221" t="n">
+      <c r="D226" t="n">
         <v>6.239</v>
       </c>
-      <c r="E221" t="n">
-        <v>6.864</v>
-      </c>
-      <c r="F221" t="n">
+      <c r="E226" t="n">
+        <v>6.818</v>
+      </c>
+      <c r="F226" t="n">
         <v>56.15</v>
       </c>
-      <c r="G221" t="n">
-        <v>61.78</v>
-      </c>
-      <c r="H221" t="n">
-        <v>5.63</v>
-      </c>
-      <c r="I221" t="n">
-        <v>10.03</v>
-      </c>
-      <c r="J221" t="n">
+      <c r="G226" t="n">
+        <v>61.36</v>
+      </c>
+      <c r="H226" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="I226" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="J226" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 30/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J226"/>
+  <dimension ref="A1:J231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E12" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F12" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G12" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H12" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I12" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E13" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F13" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G13" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H13" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I13" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E14" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F14" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G14" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H14" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I14" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D15" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E15" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F15" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G15" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H15" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E16" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F16" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G16" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H16" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I16" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E27" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F27" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G27" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H27" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I27" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C28" t="n">
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E28" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F28" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G28" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H28" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I28" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E29" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F29" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G29" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H29" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I29" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D30" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E30" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F30" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G30" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H30" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I30" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E31" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F31" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G31" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H31" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I31" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E42" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F42" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G42" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H42" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I42" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E43" t="n">
-        <v>6.629</v>
+        <v>100.06</v>
       </c>
       <c r="F43" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G43" t="n">
-        <v>59.66</v>
+        <v>100.06</v>
       </c>
       <c r="H43" t="n">
-        <v>3.51</v>
+        <v>-0.03</v>
       </c>
       <c r="I43" t="n">
-        <v>6.25</v>
+        <v>-0.03</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D44" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E44" t="n">
-        <v>22</v>
+        <v>38.497</v>
       </c>
       <c r="F44" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G44" t="n">
-        <v>66</v>
+        <v>153.99</v>
       </c>
       <c r="H44" t="n">
-        <v>0.33</v>
+        <v>14.97</v>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>10.77</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D45" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E45" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F45" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G45" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H45" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I45" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E46" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F46" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G46" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H46" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E57" t="n">
-        <v>102.86</v>
+        <v>10.75</v>
       </c>
       <c r="F57" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G57" t="n">
-        <v>102.86</v>
+        <v>32.25</v>
       </c>
       <c r="H57" t="n">
-        <v>2.77</v>
+        <v>1.09</v>
       </c>
       <c r="I57" t="n">
-        <v>2.77</v>
+        <v>3.5</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D58" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E58" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F58" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G58" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H58" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I58" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E59" t="n">
-        <v>22.289</v>
+        <v>102.86</v>
       </c>
       <c r="F59" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G59" t="n">
-        <v>66.87</v>
+        <v>102.86</v>
       </c>
       <c r="H59" t="n">
-        <v>1.2</v>
+        <v>2.77</v>
       </c>
       <c r="I59" t="n">
-        <v>1.83</v>
+        <v>2.77</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D60" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E60" t="n">
-        <v>39.845</v>
+        <v>6.736</v>
       </c>
       <c r="F60" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G60" t="n">
-        <v>159.38</v>
+        <v>60.62</v>
       </c>
       <c r="H60" t="n">
-        <v>20.36</v>
+        <v>4.47</v>
       </c>
       <c r="I60" t="n">
-        <v>14.65</v>
+        <v>7.96</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>10.75</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>32.25</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>1.09</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>3.5</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2688,29 +2688,29 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D67" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E67" t="n">
-        <v>6.807</v>
+        <v>40.567</v>
       </c>
       <c r="F67" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G67" t="n">
-        <v>61.26</v>
+        <v>162.27</v>
       </c>
       <c r="H67" t="n">
-        <v>5.11</v>
+        <v>23.25</v>
       </c>
       <c r="I67" t="n">
-        <v>9.1</v>
+        <v>16.72</v>
       </c>
       <c r="J67" t="n">
         <v>7.91</v>
@@ -2722,29 +2722,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E68" t="n">
-        <v>104.58</v>
+        <v>10.796</v>
       </c>
       <c r="F68" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G68" t="n">
-        <v>104.58</v>
+        <v>32.39</v>
       </c>
       <c r="H68" t="n">
-        <v>4.49</v>
+        <v>1.23</v>
       </c>
       <c r="I68" t="n">
-        <v>4.49</v>
+        <v>3.95</v>
       </c>
       <c r="J68" t="n">
         <v>7.91</v>
@@ -2756,29 +2756,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C69" t="n">
         <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E69" t="n">
-        <v>10.796</v>
+        <v>22.797</v>
       </c>
       <c r="F69" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G69" t="n">
-        <v>32.39</v>
+        <v>68.39</v>
       </c>
       <c r="H69" t="n">
-        <v>1.23</v>
+        <v>2.72</v>
       </c>
       <c r="I69" t="n">
-        <v>3.95</v>
+        <v>4.14</v>
       </c>
       <c r="J69" t="n">
         <v>7.91</v>
@@ -2790,29 +2790,29 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D70" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E70" t="n">
-        <v>40.567</v>
+        <v>6.807</v>
       </c>
       <c r="F70" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G70" t="n">
-        <v>162.27</v>
+        <v>61.26</v>
       </c>
       <c r="H70" t="n">
-        <v>23.25</v>
+        <v>5.11</v>
       </c>
       <c r="I70" t="n">
-        <v>16.72</v>
+        <v>9.1</v>
       </c>
       <c r="J70" t="n">
         <v>7.91</v>
@@ -2824,29 +2824,29 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E71" t="n">
-        <v>22.797</v>
+        <v>104.58</v>
       </c>
       <c r="F71" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G71" t="n">
-        <v>68.39</v>
+        <v>104.58</v>
       </c>
       <c r="H71" t="n">
-        <v>2.72</v>
+        <v>4.49</v>
       </c>
       <c r="I71" t="n">
-        <v>4.14</v>
+        <v>4.49</v>
       </c>
       <c r="J71" t="n">
         <v>7.91</v>
@@ -3198,29 +3198,29 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D82" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E82" t="n">
-        <v>106.26</v>
+        <v>6.846</v>
       </c>
       <c r="F82" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G82" t="n">
-        <v>106.26</v>
+        <v>61.61</v>
       </c>
       <c r="H82" t="n">
-        <v>6.17</v>
+        <v>5.46</v>
       </c>
       <c r="I82" t="n">
-        <v>6.16</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J82" t="n">
         <v>7.91</v>
@@ -3232,29 +3232,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C83" t="n">
         <v>3</v>
       </c>
       <c r="D83" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E83" t="n">
-        <v>23.3</v>
+        <v>10.988</v>
       </c>
       <c r="F83" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G83" t="n">
-        <v>69.90000000000001</v>
+        <v>32.96</v>
       </c>
       <c r="H83" t="n">
-        <v>4.23</v>
+        <v>1.8</v>
       </c>
       <c r="I83" t="n">
-        <v>6.44</v>
+        <v>5.78</v>
       </c>
       <c r="J83" t="n">
         <v>7.91</v>
@@ -3266,29 +3266,29 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D84" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E84" t="n">
-        <v>10.988</v>
+        <v>42.1</v>
       </c>
       <c r="F84" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G84" t="n">
-        <v>32.96</v>
+        <v>168.4</v>
       </c>
       <c r="H84" t="n">
-        <v>1.8</v>
+        <v>29.38</v>
       </c>
       <c r="I84" t="n">
-        <v>5.78</v>
+        <v>21.13</v>
       </c>
       <c r="J84" t="n">
         <v>7.91</v>
@@ -3300,29 +3300,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D85" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E85" t="n">
-        <v>6.846</v>
+        <v>106.26</v>
       </c>
       <c r="F85" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G85" t="n">
-        <v>61.61</v>
+        <v>106.26</v>
       </c>
       <c r="H85" t="n">
-        <v>5.46</v>
+        <v>6.17</v>
       </c>
       <c r="I85" t="n">
-        <v>9.720000000000001</v>
+        <v>6.16</v>
       </c>
       <c r="J85" t="n">
         <v>7.91</v>
@@ -3334,29 +3334,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E86" t="n">
-        <v>42.1</v>
+        <v>23.3</v>
       </c>
       <c r="F86" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G86" t="n">
-        <v>168.4</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H86" t="n">
-        <v>29.38</v>
+        <v>4.23</v>
       </c>
       <c r="I86" t="n">
-        <v>21.13</v>
+        <v>6.44</v>
       </c>
       <c r="J86" t="n">
         <v>7.91</v>
@@ -3708,29 +3708,29 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E97" t="n">
-        <v>40.65</v>
+        <v>10.642</v>
       </c>
       <c r="F97" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G97" t="n">
-        <v>162.6</v>
+        <v>31.93</v>
       </c>
       <c r="H97" t="n">
-        <v>23.58</v>
+        <v>0.77</v>
       </c>
       <c r="I97" t="n">
-        <v>16.96</v>
+        <v>2.47</v>
       </c>
       <c r="J97" t="n">
         <v>7.91</v>
@@ -3742,29 +3742,29 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D98" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E98" t="n">
-        <v>104.22</v>
+        <v>6.839</v>
       </c>
       <c r="F98" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G98" t="n">
-        <v>104.22</v>
+        <v>61.55</v>
       </c>
       <c r="H98" t="n">
-        <v>4.13</v>
+        <v>5.4</v>
       </c>
       <c r="I98" t="n">
-        <v>4.13</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="J98" t="n">
         <v>7.91</v>
@@ -3810,29 +3810,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D100" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E100" t="n">
-        <v>6.839</v>
+        <v>40.65</v>
       </c>
       <c r="F100" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G100" t="n">
-        <v>61.55</v>
+        <v>162.6</v>
       </c>
       <c r="H100" t="n">
-        <v>5.4</v>
+        <v>23.58</v>
       </c>
       <c r="I100" t="n">
-        <v>9.619999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="J100" t="n">
         <v>7.91</v>
@@ -3844,29 +3844,29 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D101" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E101" t="n">
-        <v>10.642</v>
+        <v>104.22</v>
       </c>
       <c r="F101" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G101" t="n">
-        <v>31.93</v>
+        <v>104.22</v>
       </c>
       <c r="H101" t="n">
-        <v>0.77</v>
+        <v>4.13</v>
       </c>
       <c r="I101" t="n">
-        <v>2.47</v>
+        <v>4.13</v>
       </c>
       <c r="J101" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E112" t="n">
-        <v>103.56</v>
+        <v>23.025</v>
       </c>
       <c r="F112" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G112" t="n">
-        <v>103.56</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H112" t="n">
-        <v>3.47</v>
+        <v>3.4</v>
       </c>
       <c r="I112" t="n">
-        <v>3.47</v>
+        <v>5.18</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D113" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E113" t="n">
-        <v>40</v>
+        <v>6.797</v>
       </c>
       <c r="F113" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G113" t="n">
-        <v>160</v>
+        <v>61.17</v>
       </c>
       <c r="H113" t="n">
-        <v>20.98</v>
+        <v>5.02</v>
       </c>
       <c r="I113" t="n">
-        <v>15.09</v>
+        <v>8.94</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E114" t="n">
-        <v>6.797</v>
+        <v>10.568</v>
       </c>
       <c r="F114" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G114" t="n">
-        <v>61.17</v>
+        <v>31.7</v>
       </c>
       <c r="H114" t="n">
-        <v>5.02</v>
+        <v>0.54</v>
       </c>
       <c r="I114" t="n">
-        <v>8.94</v>
+        <v>1.73</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E115" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F115" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G115" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H115" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I115" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4354,29 +4354,29 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D116" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E116" t="n">
-        <v>10.568</v>
+        <v>40</v>
       </c>
       <c r="F116" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G116" t="n">
-        <v>31.7</v>
+        <v>160</v>
       </c>
       <c r="H116" t="n">
-        <v>0.54</v>
+        <v>20.98</v>
       </c>
       <c r="I116" t="n">
-        <v>1.73</v>
+        <v>15.09</v>
       </c>
       <c r="J116" t="n">
         <v>7.91</v>
@@ -4728,29 +4728,29 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D127" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E127" t="n">
-        <v>23.17</v>
+        <v>39.36</v>
       </c>
       <c r="F127" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G127" t="n">
-        <v>69.51000000000001</v>
+        <v>157.44</v>
       </c>
       <c r="H127" t="n">
-        <v>3.84</v>
+        <v>18.42</v>
       </c>
       <c r="I127" t="n">
-        <v>5.85</v>
+        <v>13.25</v>
       </c>
       <c r="J127" t="n">
         <v>7.91</v>
@@ -4762,29 +4762,29 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D128" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E128" t="n">
-        <v>11.458</v>
+        <v>6.868</v>
       </c>
       <c r="F128" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G128" t="n">
-        <v>34.37</v>
+        <v>61.81</v>
       </c>
       <c r="H128" t="n">
-        <v>3.21</v>
+        <v>5.66</v>
       </c>
       <c r="I128" t="n">
-        <v>10.3</v>
+        <v>10.08</v>
       </c>
       <c r="J128" t="n">
         <v>7.91</v>
@@ -4830,29 +4830,29 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D130" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E130" t="n">
-        <v>6.868</v>
+        <v>11.458</v>
       </c>
       <c r="F130" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G130" t="n">
-        <v>61.81</v>
+        <v>34.37</v>
       </c>
       <c r="H130" t="n">
-        <v>5.66</v>
+        <v>3.21</v>
       </c>
       <c r="I130" t="n">
-        <v>10.08</v>
+        <v>10.3</v>
       </c>
       <c r="J130" t="n">
         <v>7.91</v>
@@ -4864,29 +4864,29 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D131" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E131" t="n">
-        <v>39.36</v>
+        <v>23.17</v>
       </c>
       <c r="F131" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G131" t="n">
-        <v>157.44</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H131" t="n">
-        <v>18.42</v>
+        <v>3.84</v>
       </c>
       <c r="I131" t="n">
-        <v>13.25</v>
+        <v>5.85</v>
       </c>
       <c r="J131" t="n">
         <v>7.91</v>
@@ -5238,29 +5238,29 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D142" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E142" t="n">
-        <v>102.06</v>
+        <v>23.135</v>
       </c>
       <c r="F142" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G142" t="n">
-        <v>102.06</v>
+        <v>69.41</v>
       </c>
       <c r="H142" t="n">
-        <v>1.97</v>
+        <v>3.74</v>
       </c>
       <c r="I142" t="n">
-        <v>1.97</v>
+        <v>5.7</v>
       </c>
       <c r="J142" t="n">
         <v>7.91</v>
@@ -5272,29 +5272,29 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D143" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E143" t="n">
-        <v>38.89</v>
+        <v>11.498</v>
       </c>
       <c r="F143" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G143" t="n">
-        <v>155.56</v>
+        <v>34.49</v>
       </c>
       <c r="H143" t="n">
-        <v>16.54</v>
+        <v>3.33</v>
       </c>
       <c r="I143" t="n">
-        <v>11.9</v>
+        <v>10.69</v>
       </c>
       <c r="J143" t="n">
         <v>7.91</v>
@@ -5340,29 +5340,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D145" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E145" t="n">
-        <v>11.498</v>
+        <v>102.06</v>
       </c>
       <c r="F145" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G145" t="n">
-        <v>34.49</v>
+        <v>102.06</v>
       </c>
       <c r="H145" t="n">
-        <v>3.33</v>
+        <v>1.97</v>
       </c>
       <c r="I145" t="n">
-        <v>10.69</v>
+        <v>1.97</v>
       </c>
       <c r="J145" t="n">
         <v>7.91</v>
@@ -5374,29 +5374,29 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E146" t="n">
-        <v>23.135</v>
+        <v>38.89</v>
       </c>
       <c r="F146" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G146" t="n">
-        <v>69.41</v>
+        <v>155.56</v>
       </c>
       <c r="H146" t="n">
-        <v>3.74</v>
+        <v>16.54</v>
       </c>
       <c r="I146" t="n">
-        <v>5.7</v>
+        <v>11.9</v>
       </c>
       <c r="J146" t="n">
         <v>7.91</v>
@@ -5748,29 +5748,29 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D157" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E157" t="n">
-        <v>10.92</v>
+        <v>6.913</v>
       </c>
       <c r="F157" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G157" t="n">
-        <v>32.76</v>
+        <v>62.22</v>
       </c>
       <c r="H157" t="n">
-        <v>1.6</v>
+        <v>6.07</v>
       </c>
       <c r="I157" t="n">
-        <v>5.13</v>
+        <v>10.81</v>
       </c>
       <c r="J157" t="n">
         <v>7.91</v>
@@ -5782,29 +5782,29 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E158" t="n">
-        <v>40.015</v>
+        <v>23.08</v>
       </c>
       <c r="F158" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G158" t="n">
-        <v>160.06</v>
+        <v>69.23999999999999</v>
       </c>
       <c r="H158" t="n">
-        <v>21.04</v>
+        <v>3.57</v>
       </c>
       <c r="I158" t="n">
-        <v>15.13</v>
+        <v>5.44</v>
       </c>
       <c r="J158" t="n">
         <v>7.91</v>
@@ -5816,29 +5816,29 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D159" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E159" t="n">
-        <v>104.5</v>
+        <v>40.015</v>
       </c>
       <c r="F159" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G159" t="n">
-        <v>104.5</v>
+        <v>160.06</v>
       </c>
       <c r="H159" t="n">
-        <v>4.41</v>
+        <v>21.04</v>
       </c>
       <c r="I159" t="n">
-        <v>4.41</v>
+        <v>15.13</v>
       </c>
       <c r="J159" t="n">
         <v>7.91</v>
@@ -5850,29 +5850,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C160" t="n">
         <v>3</v>
       </c>
       <c r="D160" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E160" t="n">
-        <v>23.08</v>
+        <v>10.92</v>
       </c>
       <c r="F160" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G160" t="n">
-        <v>69.23999999999999</v>
+        <v>32.76</v>
       </c>
       <c r="H160" t="n">
-        <v>3.57</v>
+        <v>1.6</v>
       </c>
       <c r="I160" t="n">
-        <v>5.44</v>
+        <v>5.13</v>
       </c>
       <c r="J160" t="n">
         <v>7.91</v>
@@ -5884,29 +5884,29 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D161" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E161" t="n">
-        <v>6.913</v>
+        <v>104.5</v>
       </c>
       <c r="F161" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G161" t="n">
-        <v>62.22</v>
+        <v>104.5</v>
       </c>
       <c r="H161" t="n">
-        <v>6.07</v>
+        <v>4.41</v>
       </c>
       <c r="I161" t="n">
-        <v>10.81</v>
+        <v>4.41</v>
       </c>
       <c r="J161" t="n">
         <v>7.91</v>
@@ -6258,29 +6258,29 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D172" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E172" t="n">
-        <v>103.22</v>
+        <v>22.95</v>
       </c>
       <c r="F172" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G172" t="n">
-        <v>103.22</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H172" t="n">
-        <v>3.13</v>
+        <v>3.18</v>
       </c>
       <c r="I172" t="n">
-        <v>3.13</v>
+        <v>4.84</v>
       </c>
       <c r="J172" t="n">
         <v>7.91</v>
@@ -6292,29 +6292,29 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D173" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E173" t="n">
-        <v>6.926</v>
+        <v>10.712</v>
       </c>
       <c r="F173" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G173" t="n">
-        <v>62.33</v>
+        <v>32.14</v>
       </c>
       <c r="H173" t="n">
-        <v>6.18</v>
+        <v>0.98</v>
       </c>
       <c r="I173" t="n">
-        <v>11.01</v>
+        <v>3.15</v>
       </c>
       <c r="J173" t="n">
         <v>7.91</v>
@@ -6326,29 +6326,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D174" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E174" t="n">
-        <v>38.74</v>
+        <v>6.926</v>
       </c>
       <c r="F174" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G174" t="n">
-        <v>154.96</v>
+        <v>62.33</v>
       </c>
       <c r="H174" t="n">
-        <v>15.94</v>
+        <v>6.18</v>
       </c>
       <c r="I174" t="n">
-        <v>11.47</v>
+        <v>11.01</v>
       </c>
       <c r="J174" t="n">
         <v>7.91</v>
@@ -6360,29 +6360,29 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D175" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E175" t="n">
-        <v>10.712</v>
+        <v>103.22</v>
       </c>
       <c r="F175" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G175" t="n">
-        <v>32.14</v>
+        <v>103.22</v>
       </c>
       <c r="H175" t="n">
-        <v>0.98</v>
+        <v>3.13</v>
       </c>
       <c r="I175" t="n">
-        <v>3.15</v>
+        <v>3.13</v>
       </c>
       <c r="J175" t="n">
         <v>7.91</v>
@@ -6394,29 +6394,29 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E176" t="n">
-        <v>22.95</v>
+        <v>38.74</v>
       </c>
       <c r="F176" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G176" t="n">
-        <v>68.84999999999999</v>
+        <v>154.96</v>
       </c>
       <c r="H176" t="n">
-        <v>3.18</v>
+        <v>15.94</v>
       </c>
       <c r="I176" t="n">
-        <v>4.84</v>
+        <v>11.47</v>
       </c>
       <c r="J176" t="n">
         <v>7.91</v>
@@ -6768,29 +6768,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D187" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E187" t="n">
-        <v>101.44</v>
+        <v>10.708</v>
       </c>
       <c r="F187" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G187" t="n">
-        <v>101.44</v>
+        <v>32.12</v>
       </c>
       <c r="H187" t="n">
-        <v>1.35</v>
+        <v>0.96</v>
       </c>
       <c r="I187" t="n">
-        <v>1.35</v>
+        <v>3.08</v>
       </c>
       <c r="J187" t="n">
         <v>7.91</v>
@@ -6802,29 +6802,29 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E188" t="n">
-        <v>22.845</v>
+        <v>37.85</v>
       </c>
       <c r="F188" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G188" t="n">
-        <v>68.53</v>
+        <v>151.4</v>
       </c>
       <c r="H188" t="n">
-        <v>2.86</v>
+        <v>12.38</v>
       </c>
       <c r="I188" t="n">
-        <v>4.36</v>
+        <v>8.91</v>
       </c>
       <c r="J188" t="n">
         <v>7.91</v>
@@ -6836,29 +6836,29 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D189" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E189" t="n">
-        <v>6.862</v>
+        <v>101.44</v>
       </c>
       <c r="F189" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G189" t="n">
-        <v>61.76</v>
+        <v>101.44</v>
       </c>
       <c r="H189" t="n">
-        <v>5.61</v>
+        <v>1.35</v>
       </c>
       <c r="I189" t="n">
-        <v>9.99</v>
+        <v>1.35</v>
       </c>
       <c r="J189" t="n">
         <v>7.91</v>
@@ -6870,29 +6870,29 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D190" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E190" t="n">
-        <v>37.85</v>
+        <v>22.845</v>
       </c>
       <c r="F190" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G190" t="n">
-        <v>151.4</v>
+        <v>68.53</v>
       </c>
       <c r="H190" t="n">
-        <v>12.38</v>
+        <v>2.86</v>
       </c>
       <c r="I190" t="n">
-        <v>8.91</v>
+        <v>4.36</v>
       </c>
       <c r="J190" t="n">
         <v>7.91</v>
@@ -6904,29 +6904,29 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D191" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E191" t="n">
-        <v>10.708</v>
+        <v>6.862</v>
       </c>
       <c r="F191" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G191" t="n">
-        <v>32.12</v>
+        <v>61.76</v>
       </c>
       <c r="H191" t="n">
-        <v>0.96</v>
+        <v>5.61</v>
       </c>
       <c r="I191" t="n">
-        <v>3.08</v>
+        <v>9.99</v>
       </c>
       <c r="J191" t="n">
         <v>7.91</v>
@@ -7278,29 +7278,29 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D202" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E202" t="n">
-        <v>100.08</v>
+        <v>22.4</v>
       </c>
       <c r="F202" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G202" t="n">
-        <v>100.08</v>
+        <v>67.2</v>
       </c>
       <c r="H202" t="n">
-        <v>-0.01</v>
+        <v>1.53</v>
       </c>
       <c r="I202" t="n">
-        <v>-0.01</v>
+        <v>2.33</v>
       </c>
       <c r="J202" t="n">
         <v>7.91</v>
@@ -7312,29 +7312,29 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D203" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E203" t="n">
-        <v>11.044</v>
+        <v>6.822</v>
       </c>
       <c r="F203" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G203" t="n">
-        <v>33.13</v>
+        <v>61.4</v>
       </c>
       <c r="H203" t="n">
-        <v>1.97</v>
+        <v>5.25</v>
       </c>
       <c r="I203" t="n">
-        <v>6.32</v>
+        <v>9.35</v>
       </c>
       <c r="J203" t="n">
         <v>7.91</v>
@@ -7346,29 +7346,29 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D204" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E204" t="n">
-        <v>38.04</v>
+        <v>11.044</v>
       </c>
       <c r="F204" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G204" t="n">
-        <v>152.16</v>
+        <v>33.13</v>
       </c>
       <c r="H204" t="n">
-        <v>13.14</v>
+        <v>1.97</v>
       </c>
       <c r="I204" t="n">
-        <v>9.449999999999999</v>
+        <v>6.32</v>
       </c>
       <c r="J204" t="n">
         <v>7.91</v>
@@ -7380,29 +7380,29 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D205" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E205" t="n">
-        <v>22.4</v>
+        <v>100.08</v>
       </c>
       <c r="F205" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G205" t="n">
-        <v>67.2</v>
+        <v>100.08</v>
       </c>
       <c r="H205" t="n">
-        <v>1.53</v>
+        <v>-0.01</v>
       </c>
       <c r="I205" t="n">
-        <v>2.33</v>
+        <v>-0.01</v>
       </c>
       <c r="J205" t="n">
         <v>7.91</v>
@@ -7414,29 +7414,29 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D206" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E206" t="n">
-        <v>6.822</v>
+        <v>38.04</v>
       </c>
       <c r="F206" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G206" t="n">
-        <v>61.4</v>
+        <v>152.16</v>
       </c>
       <c r="H206" t="n">
-        <v>5.25</v>
+        <v>13.14</v>
       </c>
       <c r="I206" t="n">
-        <v>9.35</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="J206" t="n">
         <v>7.91</v>
@@ -7788,29 +7788,29 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D217" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E217" t="n">
-        <v>6.864</v>
+        <v>98.02</v>
       </c>
       <c r="F217" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G217" t="n">
-        <v>61.78</v>
+        <v>98.02</v>
       </c>
       <c r="H217" t="n">
-        <v>5.63</v>
+        <v>-2.07</v>
       </c>
       <c r="I217" t="n">
-        <v>10.03</v>
+        <v>-2.07</v>
       </c>
       <c r="J217" t="n">
         <v>7.91</v>
@@ -7822,29 +7822,29 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C218" t="n">
         <v>3</v>
       </c>
       <c r="D218" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E218" t="n">
-        <v>11.546</v>
+        <v>23.175</v>
       </c>
       <c r="F218" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G218" t="n">
-        <v>34.64</v>
+        <v>69.53</v>
       </c>
       <c r="H218" t="n">
-        <v>3.48</v>
+        <v>3.86</v>
       </c>
       <c r="I218" t="n">
-        <v>11.17</v>
+        <v>5.88</v>
       </c>
       <c r="J218" t="n">
         <v>7.91</v>
@@ -7856,29 +7856,29 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D219" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E219" t="n">
-        <v>36.75</v>
+        <v>11.546</v>
       </c>
       <c r="F219" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G219" t="n">
-        <v>147</v>
+        <v>34.64</v>
       </c>
       <c r="H219" t="n">
-        <v>7.98</v>
+        <v>3.48</v>
       </c>
       <c r="I219" t="n">
-        <v>5.74</v>
+        <v>11.17</v>
       </c>
       <c r="J219" t="n">
         <v>7.91</v>
@@ -7890,29 +7890,29 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D220" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E220" t="n">
-        <v>23.175</v>
+        <v>6.864</v>
       </c>
       <c r="F220" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G220" t="n">
-        <v>69.53</v>
+        <v>61.78</v>
       </c>
       <c r="H220" t="n">
-        <v>3.86</v>
+        <v>5.63</v>
       </c>
       <c r="I220" t="n">
-        <v>5.88</v>
+        <v>10.03</v>
       </c>
       <c r="J220" t="n">
         <v>7.91</v>
@@ -7924,29 +7924,29 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D221" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E221" t="n">
-        <v>98.02</v>
+        <v>36.75</v>
       </c>
       <c r="F221" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G221" t="n">
-        <v>98.02</v>
+        <v>147</v>
       </c>
       <c r="H221" t="n">
-        <v>-2.07</v>
+        <v>7.98</v>
       </c>
       <c r="I221" t="n">
-        <v>-2.07</v>
+        <v>5.74</v>
       </c>
       <c r="J221" t="n">
         <v>7.91</v>
@@ -8119,6 +8119,176 @@
         <v>9.279999999999999</v>
       </c>
       <c r="J226" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>3</v>
+      </c>
+      <c r="D227" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E227" t="n">
+        <v>11.512</v>
+      </c>
+      <c r="F227" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G227" t="n">
+        <v>34.54</v>
+      </c>
+      <c r="H227" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="I227" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="J227" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C228" t="n">
+        <v>4</v>
+      </c>
+      <c r="D228" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E228" t="n">
+        <v>36.64</v>
+      </c>
+      <c r="F228" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G228" t="n">
+        <v>146.56</v>
+      </c>
+      <c r="H228" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="I228" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="J228" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>3</v>
+      </c>
+      <c r="D229" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E229" t="n">
+        <v>23.07</v>
+      </c>
+      <c r="F229" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G229" t="n">
+        <v>69.20999999999999</v>
+      </c>
+      <c r="H229" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="I229" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="J229" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>1</v>
+      </c>
+      <c r="D230" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E230" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="F230" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G230" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="H230" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="I230" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="J230" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="1" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>IWSC</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>9</v>
+      </c>
+      <c r="D231" t="n">
+        <v>6.239</v>
+      </c>
+      <c r="E231" t="n">
+        <v>6.779</v>
+      </c>
+      <c r="F231" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="G231" t="n">
+        <v>61.01</v>
+      </c>
+      <c r="H231" t="n">
+        <v>4.86</v>
+      </c>
+      <c r="I231" t="n">
+        <v>8.66</v>
+      </c>
+      <c r="J231" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 31/07/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J231"/>
+  <dimension ref="A1:J236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D12" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E12" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F12" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G12" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I12" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E13" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F13" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G13" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H13" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I13" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D14" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E14" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F14" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G14" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H14" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I14" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D15" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E15" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F15" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G15" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H15" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I15" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E16" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F16" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G16" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H16" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I16" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E27" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F27" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G27" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H27" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I27" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D28" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E28" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F28" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G28" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H28" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I28" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E29" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F29" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G29" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H29" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I29" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E30" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F30" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G30" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H30" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I30" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C31" t="n">
         <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E31" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F31" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G31" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H31" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I31" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D42" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E42" t="n">
-        <v>22</v>
+        <v>38.497</v>
       </c>
       <c r="F42" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G42" t="n">
-        <v>66</v>
+        <v>153.99</v>
       </c>
       <c r="H42" t="n">
-        <v>0.33</v>
+        <v>14.97</v>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>10.77</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E43" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F43" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G43" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I43" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D44" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E44" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F44" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G44" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H44" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I44" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E45" t="n">
-        <v>6.629</v>
+        <v>100.06</v>
       </c>
       <c r="F45" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G45" t="n">
-        <v>59.66</v>
+        <v>100.06</v>
       </c>
       <c r="H45" t="n">
-        <v>3.51</v>
+        <v>-0.03</v>
       </c>
       <c r="I45" t="n">
-        <v>6.25</v>
+        <v>-0.03</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C46" t="n">
         <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E46" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F46" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G46" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H46" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I46" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E57" t="n">
-        <v>10.75</v>
+        <v>22.289</v>
       </c>
       <c r="F57" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G57" t="n">
-        <v>32.25</v>
+        <v>66.87</v>
       </c>
       <c r="H57" t="n">
-        <v>1.09</v>
+        <v>1.2</v>
       </c>
       <c r="I57" t="n">
-        <v>3.5</v>
+        <v>1.83</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E58" t="n">
-        <v>39.845</v>
+        <v>102.86</v>
       </c>
       <c r="F58" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G58" t="n">
-        <v>159.38</v>
+        <v>102.86</v>
       </c>
       <c r="H58" t="n">
-        <v>20.36</v>
+        <v>2.77</v>
       </c>
       <c r="I58" t="n">
-        <v>14.65</v>
+        <v>2.77</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D59" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E59" t="n">
-        <v>102.86</v>
+        <v>6.736</v>
       </c>
       <c r="F59" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G59" t="n">
-        <v>102.86</v>
+        <v>60.62</v>
       </c>
       <c r="H59" t="n">
-        <v>2.77</v>
+        <v>4.47</v>
       </c>
       <c r="I59" t="n">
-        <v>2.77</v>
+        <v>7.96</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D60" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E60" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F60" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G60" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H60" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I60" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E61" t="n">
-        <v>22.289</v>
+        <v>10.75</v>
       </c>
       <c r="F61" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G61" t="n">
-        <v>66.87</v>
+        <v>32.25</v>
       </c>
       <c r="H61" t="n">
-        <v>1.2</v>
+        <v>1.09</v>
       </c>
       <c r="I61" t="n">
-        <v>1.83</v>
+        <v>3.5</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E72" t="n">
-        <v>41.15</v>
+        <v>104.22</v>
       </c>
       <c r="F72" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G72" t="n">
-        <v>164.6</v>
+        <v>104.22</v>
       </c>
       <c r="H72" t="n">
-        <v>25.58</v>
+        <v>4.13</v>
       </c>
       <c r="I72" t="n">
-        <v>18.4</v>
+        <v>4.13</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E73" t="n">
-        <v>6.811</v>
+        <v>23</v>
       </c>
       <c r="F73" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G73" t="n">
-        <v>61.3</v>
+        <v>69</v>
       </c>
       <c r="H73" t="n">
-        <v>5.15</v>
+        <v>3.33</v>
       </c>
       <c r="I73" t="n">
-        <v>9.17</v>
+        <v>5.07</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D75" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E75" t="n">
-        <v>23</v>
+        <v>6.811</v>
       </c>
       <c r="F75" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G75" t="n">
-        <v>69</v>
+        <v>61.3</v>
       </c>
       <c r="H75" t="n">
-        <v>3.33</v>
+        <v>5.15</v>
       </c>
       <c r="I75" t="n">
-        <v>5.07</v>
+        <v>9.17</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D76" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E76" t="n">
-        <v>104.22</v>
+        <v>41.15</v>
       </c>
       <c r="F76" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G76" t="n">
-        <v>104.22</v>
+        <v>164.6</v>
       </c>
       <c r="H76" t="n">
-        <v>4.13</v>
+        <v>25.58</v>
       </c>
       <c r="I76" t="n">
-        <v>4.13</v>
+        <v>18.4</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E87" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F87" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G87" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H87" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I87" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E88" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F88" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G88" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H88" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I88" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C90" t="n">
         <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E90" t="n">
-        <v>23.32</v>
+        <v>10.852</v>
       </c>
       <c r="F90" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G90" t="n">
-        <v>69.95999999999999</v>
+        <v>32.56</v>
       </c>
       <c r="H90" t="n">
-        <v>4.29</v>
+        <v>1.4</v>
       </c>
       <c r="I90" t="n">
-        <v>6.53</v>
+        <v>4.49</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D91" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E91" t="n">
-        <v>106.28</v>
+        <v>43.005</v>
       </c>
       <c r="F91" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G91" t="n">
-        <v>106.28</v>
+        <v>172.02</v>
       </c>
       <c r="H91" t="n">
-        <v>6.19</v>
+        <v>33</v>
       </c>
       <c r="I91" t="n">
-        <v>6.18</v>
+        <v>23.74</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E102" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F102" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G102" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H102" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I102" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E103" t="n">
-        <v>6.804</v>
+        <v>23.29</v>
       </c>
       <c r="F103" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G103" t="n">
-        <v>61.24</v>
+        <v>69.87</v>
       </c>
       <c r="H103" t="n">
-        <v>5.09</v>
+        <v>4.2</v>
       </c>
       <c r="I103" t="n">
-        <v>9.07</v>
+        <v>6.4</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D104" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E104" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F104" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G104" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H104" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I104" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D105" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E105" t="n">
-        <v>23.29</v>
+        <v>40.97</v>
       </c>
       <c r="F105" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G105" t="n">
-        <v>69.87</v>
+        <v>163.88</v>
       </c>
       <c r="H105" t="n">
-        <v>4.2</v>
+        <v>24.86</v>
       </c>
       <c r="I105" t="n">
-        <v>6.4</v>
+        <v>17.88</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D106" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E106" t="n">
-        <v>10.556</v>
+        <v>103.46</v>
       </c>
       <c r="F106" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G106" t="n">
-        <v>31.67</v>
+        <v>103.46</v>
       </c>
       <c r="H106" t="n">
-        <v>0.51</v>
+        <v>3.37</v>
       </c>
       <c r="I106" t="n">
-        <v>1.64</v>
+        <v>3.37</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D112" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E112" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F112" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G112" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H112" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I112" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D113" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E113" t="n">
-        <v>6.797</v>
+        <v>23.025</v>
       </c>
       <c r="F113" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G113" t="n">
-        <v>61.17</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H113" t="n">
-        <v>5.02</v>
+        <v>3.4</v>
       </c>
       <c r="I113" t="n">
-        <v>8.94</v>
+        <v>5.18</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D114" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E114" t="n">
-        <v>10.568</v>
+        <v>6.797</v>
       </c>
       <c r="F114" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G114" t="n">
-        <v>31.7</v>
+        <v>61.17</v>
       </c>
       <c r="H114" t="n">
-        <v>0.54</v>
+        <v>5.02</v>
       </c>
       <c r="I114" t="n">
-        <v>1.73</v>
+        <v>8.94</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D115" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E115" t="n">
-        <v>103.56</v>
+        <v>10.568</v>
       </c>
       <c r="F115" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G115" t="n">
-        <v>103.56</v>
+        <v>31.7</v>
       </c>
       <c r="H115" t="n">
-        <v>3.47</v>
+        <v>0.54</v>
       </c>
       <c r="I115" t="n">
-        <v>3.47</v>
+        <v>1.73</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E117" t="n">
-        <v>41</v>
+        <v>23.145</v>
       </c>
       <c r="F117" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G117" t="n">
-        <v>164</v>
+        <v>69.44</v>
       </c>
       <c r="H117" t="n">
-        <v>24.98</v>
+        <v>3.77</v>
       </c>
       <c r="I117" t="n">
-        <v>17.97</v>
+        <v>5.74</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D118" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E118" t="n">
-        <v>6.861</v>
+        <v>105.96</v>
       </c>
       <c r="F118" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G118" t="n">
-        <v>61.75</v>
+        <v>105.96</v>
       </c>
       <c r="H118" t="n">
-        <v>5.6</v>
+        <v>5.87</v>
       </c>
       <c r="I118" t="n">
-        <v>9.970000000000001</v>
+        <v>5.86</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D120" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E120" t="n">
-        <v>105.96</v>
+        <v>6.861</v>
       </c>
       <c r="F120" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G120" t="n">
-        <v>105.96</v>
+        <v>61.75</v>
       </c>
       <c r="H120" t="n">
-        <v>5.87</v>
+        <v>5.6</v>
       </c>
       <c r="I120" t="n">
-        <v>5.86</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D121" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E121" t="n">
-        <v>23.145</v>
+        <v>41</v>
       </c>
       <c r="F121" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G121" t="n">
-        <v>69.44</v>
+        <v>164</v>
       </c>
       <c r="H121" t="n">
-        <v>3.77</v>
+        <v>24.98</v>
       </c>
       <c r="I121" t="n">
-        <v>5.74</v>
+        <v>17.97</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C132" t="n">
         <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E132" t="n">
-        <v>23.18</v>
+        <v>11.516</v>
       </c>
       <c r="F132" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G132" t="n">
-        <v>69.54000000000001</v>
+        <v>34.55</v>
       </c>
       <c r="H132" t="n">
-        <v>3.87</v>
+        <v>3.39</v>
       </c>
       <c r="I132" t="n">
-        <v>5.89</v>
+        <v>10.88</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E133" t="n">
-        <v>6.895</v>
+        <v>40.54</v>
       </c>
       <c r="F133" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G133" t="n">
-        <v>62.05</v>
+        <v>162.16</v>
       </c>
       <c r="H133" t="n">
-        <v>5.9</v>
+        <v>23.14</v>
       </c>
       <c r="I133" t="n">
-        <v>10.51</v>
+        <v>16.65</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D135" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E135" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F135" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G135" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H135" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I135" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C136" t="n">
         <v>3</v>
       </c>
       <c r="D136" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E136" t="n">
-        <v>11.516</v>
+        <v>23.18</v>
       </c>
       <c r="F136" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G136" t="n">
-        <v>34.55</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H136" t="n">
-        <v>3.39</v>
+        <v>3.87</v>
       </c>
       <c r="I136" t="n">
-        <v>10.88</v>
+        <v>5.89</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D147" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E147" t="n">
-        <v>101.7</v>
+        <v>6.826</v>
       </c>
       <c r="F147" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G147" t="n">
-        <v>101.7</v>
+        <v>61.43</v>
       </c>
       <c r="H147" t="n">
-        <v>1.61</v>
+        <v>5.28</v>
       </c>
       <c r="I147" t="n">
-        <v>1.61</v>
+        <v>9.4</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D148" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E148" t="n">
-        <v>38.955</v>
+        <v>22.755</v>
       </c>
       <c r="F148" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G148" t="n">
-        <v>155.82</v>
+        <v>68.27</v>
       </c>
       <c r="H148" t="n">
-        <v>16.8</v>
+        <v>2.6</v>
       </c>
       <c r="I148" t="n">
-        <v>12.08</v>
+        <v>3.96</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D150" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E150" t="n">
-        <v>22.755</v>
+        <v>38.955</v>
       </c>
       <c r="F150" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G150" t="n">
-        <v>68.27</v>
+        <v>155.82</v>
       </c>
       <c r="H150" t="n">
-        <v>2.6</v>
+        <v>16.8</v>
       </c>
       <c r="I150" t="n">
-        <v>3.96</v>
+        <v>12.08</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D151" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E151" t="n">
-        <v>6.826</v>
+        <v>101.7</v>
       </c>
       <c r="F151" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G151" t="n">
-        <v>61.43</v>
+        <v>101.7</v>
       </c>
       <c r="H151" t="n">
-        <v>5.28</v>
+        <v>1.61</v>
       </c>
       <c r="I151" t="n">
-        <v>9.4</v>
+        <v>1.61</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C162" t="n">
         <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E162" t="n">
-        <v>10.748</v>
+        <v>23.01</v>
       </c>
       <c r="F162" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G162" t="n">
-        <v>32.24</v>
+        <v>69.03</v>
       </c>
       <c r="H162" t="n">
-        <v>1.08</v>
+        <v>3.36</v>
       </c>
       <c r="I162" t="n">
-        <v>3.47</v>
+        <v>5.12</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D163" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E163" t="n">
-        <v>103.84</v>
+        <v>6.927</v>
       </c>
       <c r="F163" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G163" t="n">
-        <v>103.84</v>
+        <v>62.34</v>
       </c>
       <c r="H163" t="n">
-        <v>3.75</v>
+        <v>6.19</v>
       </c>
       <c r="I163" t="n">
-        <v>3.75</v>
+        <v>11.02</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D165" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E165" t="n">
-        <v>6.927</v>
+        <v>103.84</v>
       </c>
       <c r="F165" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G165" t="n">
-        <v>62.34</v>
+        <v>103.84</v>
       </c>
       <c r="H165" t="n">
-        <v>6.19</v>
+        <v>3.75</v>
       </c>
       <c r="I165" t="n">
-        <v>11.02</v>
+        <v>3.75</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C166" t="n">
         <v>3</v>
       </c>
       <c r="D166" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E166" t="n">
-        <v>23.01</v>
+        <v>10.748</v>
       </c>
       <c r="F166" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G166" t="n">
-        <v>69.03</v>
+        <v>32.24</v>
       </c>
       <c r="H166" t="n">
-        <v>3.36</v>
+        <v>1.08</v>
       </c>
       <c r="I166" t="n">
-        <v>5.12</v>
+        <v>3.47</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D177" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E177" t="n">
-        <v>22.95</v>
+        <v>38.245</v>
       </c>
       <c r="F177" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G177" t="n">
-        <v>68.84999999999999</v>
+        <v>152.98</v>
       </c>
       <c r="H177" t="n">
-        <v>3.18</v>
+        <v>13.96</v>
       </c>
       <c r="I177" t="n">
-        <v>4.84</v>
+        <v>10.04</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D178" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E178" t="n">
-        <v>102.54</v>
+        <v>6.922</v>
       </c>
       <c r="F178" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G178" t="n">
-        <v>102.54</v>
+        <v>62.3</v>
       </c>
       <c r="H178" t="n">
-        <v>2.45</v>
+        <v>6.15</v>
       </c>
       <c r="I178" t="n">
-        <v>2.45</v>
+        <v>10.95</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D179" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E179" t="n">
-        <v>10.642</v>
+        <v>102.54</v>
       </c>
       <c r="F179" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G179" t="n">
-        <v>31.93</v>
+        <v>102.54</v>
       </c>
       <c r="H179" t="n">
-        <v>0.77</v>
+        <v>2.45</v>
       </c>
       <c r="I179" t="n">
-        <v>2.47</v>
+        <v>2.45</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D180" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E180" t="n">
-        <v>6.922</v>
+        <v>10.642</v>
       </c>
       <c r="F180" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G180" t="n">
-        <v>62.3</v>
+        <v>31.93</v>
       </c>
       <c r="H180" t="n">
-        <v>6.15</v>
+        <v>0.77</v>
       </c>
       <c r="I180" t="n">
-        <v>10.95</v>
+        <v>2.47</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,29 +6564,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D181" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E181" t="n">
-        <v>38.245</v>
+        <v>22.95</v>
       </c>
       <c r="F181" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G181" t="n">
-        <v>152.98</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H181" t="n">
-        <v>13.96</v>
+        <v>3.18</v>
       </c>
       <c r="I181" t="n">
-        <v>10.04</v>
+        <v>4.84</v>
       </c>
       <c r="J181" t="n">
         <v>7.91</v>
@@ -6938,29 +6938,29 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D192" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E192" t="n">
-        <v>22.82</v>
+        <v>38.755</v>
       </c>
       <c r="F192" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G192" t="n">
-        <v>68.45999999999999</v>
+        <v>155.02</v>
       </c>
       <c r="H192" t="n">
-        <v>2.79</v>
+        <v>16</v>
       </c>
       <c r="I192" t="n">
-        <v>4.25</v>
+        <v>11.51</v>
       </c>
       <c r="J192" t="n">
         <v>7.91</v>
@@ -6972,29 +6972,29 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D193" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E193" t="n">
-        <v>6.894</v>
+        <v>102.46</v>
       </c>
       <c r="F193" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G193" t="n">
-        <v>62.05</v>
+        <v>102.46</v>
       </c>
       <c r="H193" t="n">
-        <v>5.9</v>
+        <v>2.37</v>
       </c>
       <c r="I193" t="n">
-        <v>10.51</v>
+        <v>2.37</v>
       </c>
       <c r="J193" t="n">
         <v>7.91</v>
@@ -7040,29 +7040,29 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D195" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E195" t="n">
-        <v>102.46</v>
+        <v>6.894</v>
       </c>
       <c r="F195" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G195" t="n">
-        <v>102.46</v>
+        <v>62.05</v>
       </c>
       <c r="H195" t="n">
-        <v>2.37</v>
+        <v>5.9</v>
       </c>
       <c r="I195" t="n">
-        <v>2.37</v>
+        <v>10.51</v>
       </c>
       <c r="J195" t="n">
         <v>7.91</v>
@@ -7074,29 +7074,29 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D196" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E196" t="n">
-        <v>38.755</v>
+        <v>22.82</v>
       </c>
       <c r="F196" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G196" t="n">
-        <v>155.02</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="H196" t="n">
-        <v>16</v>
+        <v>2.79</v>
       </c>
       <c r="I196" t="n">
-        <v>11.51</v>
+        <v>4.25</v>
       </c>
       <c r="J196" t="n">
         <v>7.91</v>
@@ -7448,29 +7448,29 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D207" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E207" t="n">
-        <v>99.90000000000001</v>
+        <v>11.172</v>
       </c>
       <c r="F207" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G207" t="n">
-        <v>99.90000000000001</v>
+        <v>33.52</v>
       </c>
       <c r="H207" t="n">
-        <v>-0.19</v>
+        <v>2.36</v>
       </c>
       <c r="I207" t="n">
-        <v>-0.19</v>
+        <v>7.57</v>
       </c>
       <c r="J207" t="n">
         <v>7.91</v>
@@ -7482,29 +7482,29 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D208" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E208" t="n">
-        <v>22.725</v>
+        <v>37.82</v>
       </c>
       <c r="F208" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G208" t="n">
-        <v>68.18000000000001</v>
+        <v>151.28</v>
       </c>
       <c r="H208" t="n">
-        <v>2.51</v>
+        <v>12.26</v>
       </c>
       <c r="I208" t="n">
-        <v>3.82</v>
+        <v>8.82</v>
       </c>
       <c r="J208" t="n">
         <v>7.91</v>
@@ -7516,29 +7516,29 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D209" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E209" t="n">
-        <v>6.865</v>
+        <v>22.725</v>
       </c>
       <c r="F209" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G209" t="n">
-        <v>61.79</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H209" t="n">
-        <v>5.64</v>
+        <v>2.51</v>
       </c>
       <c r="I209" t="n">
-        <v>10.04</v>
+        <v>3.82</v>
       </c>
       <c r="J209" t="n">
         <v>7.91</v>
@@ -7550,29 +7550,29 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D210" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E210" t="n">
-        <v>37.82</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F210" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G210" t="n">
-        <v>151.28</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H210" t="n">
-        <v>12.26</v>
+        <v>-0.19</v>
       </c>
       <c r="I210" t="n">
-        <v>8.82</v>
+        <v>-0.19</v>
       </c>
       <c r="J210" t="n">
         <v>7.91</v>
@@ -7584,29 +7584,29 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D211" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E211" t="n">
-        <v>11.172</v>
+        <v>6.865</v>
       </c>
       <c r="F211" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G211" t="n">
-        <v>33.52</v>
+        <v>61.79</v>
       </c>
       <c r="H211" t="n">
-        <v>2.36</v>
+        <v>5.64</v>
       </c>
       <c r="I211" t="n">
-        <v>7.57</v>
+        <v>10.04</v>
       </c>
       <c r="J211" t="n">
         <v>7.91</v>
@@ -7788,29 +7788,29 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D217" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E217" t="n">
-        <v>98.02</v>
+        <v>6.864</v>
       </c>
       <c r="F217" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G217" t="n">
-        <v>98.02</v>
+        <v>61.78</v>
       </c>
       <c r="H217" t="n">
-        <v>-2.07</v>
+        <v>5.63</v>
       </c>
       <c r="I217" t="n">
-        <v>-2.07</v>
+        <v>10.03</v>
       </c>
       <c r="J217" t="n">
         <v>7.91</v>
@@ -7822,29 +7822,29 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C218" t="n">
         <v>3</v>
       </c>
       <c r="D218" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E218" t="n">
-        <v>23.175</v>
+        <v>11.546</v>
       </c>
       <c r="F218" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G218" t="n">
-        <v>69.53</v>
+        <v>34.64</v>
       </c>
       <c r="H218" t="n">
-        <v>3.86</v>
+        <v>3.48</v>
       </c>
       <c r="I218" t="n">
-        <v>5.88</v>
+        <v>11.17</v>
       </c>
       <c r="J218" t="n">
         <v>7.91</v>
@@ -7856,29 +7856,29 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D219" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E219" t="n">
-        <v>11.546</v>
+        <v>36.75</v>
       </c>
       <c r="F219" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G219" t="n">
-        <v>34.64</v>
+        <v>147</v>
       </c>
       <c r="H219" t="n">
-        <v>3.48</v>
+        <v>7.98</v>
       </c>
       <c r="I219" t="n">
-        <v>11.17</v>
+        <v>5.74</v>
       </c>
       <c r="J219" t="n">
         <v>7.91</v>
@@ -7890,29 +7890,29 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D220" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E220" t="n">
-        <v>6.864</v>
+        <v>98.02</v>
       </c>
       <c r="F220" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G220" t="n">
-        <v>61.78</v>
+        <v>98.02</v>
       </c>
       <c r="H220" t="n">
-        <v>5.63</v>
+        <v>-2.07</v>
       </c>
       <c r="I220" t="n">
-        <v>10.03</v>
+        <v>-2.07</v>
       </c>
       <c r="J220" t="n">
         <v>7.91</v>
@@ -7924,29 +7924,29 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D221" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E221" t="n">
-        <v>36.75</v>
+        <v>23.175</v>
       </c>
       <c r="F221" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G221" t="n">
-        <v>147</v>
+        <v>69.53</v>
       </c>
       <c r="H221" t="n">
-        <v>7.98</v>
+        <v>3.86</v>
       </c>
       <c r="I221" t="n">
-        <v>5.74</v>
+        <v>5.88</v>
       </c>
       <c r="J221" t="n">
         <v>7.91</v>
@@ -8128,29 +8128,29 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D227" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E227" t="n">
-        <v>11.512</v>
+        <v>6.779</v>
       </c>
       <c r="F227" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G227" t="n">
-        <v>34.54</v>
+        <v>61.01</v>
       </c>
       <c r="H227" t="n">
-        <v>3.38</v>
+        <v>4.86</v>
       </c>
       <c r="I227" t="n">
-        <v>10.85</v>
+        <v>8.66</v>
       </c>
       <c r="J227" t="n">
         <v>7.91</v>
@@ -8162,29 +8162,29 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D228" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E228" t="n">
-        <v>36.64</v>
+        <v>11.512</v>
       </c>
       <c r="F228" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G228" t="n">
-        <v>146.56</v>
+        <v>34.54</v>
       </c>
       <c r="H228" t="n">
-        <v>7.54</v>
+        <v>3.38</v>
       </c>
       <c r="I228" t="n">
-        <v>5.42</v>
+        <v>10.85</v>
       </c>
       <c r="J228" t="n">
         <v>7.91</v>
@@ -8196,29 +8196,29 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D229" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E229" t="n">
-        <v>23.07</v>
+        <v>36.64</v>
       </c>
       <c r="F229" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G229" t="n">
-        <v>69.20999999999999</v>
+        <v>146.56</v>
       </c>
       <c r="H229" t="n">
-        <v>3.54</v>
+        <v>7.54</v>
       </c>
       <c r="I229" t="n">
-        <v>5.39</v>
+        <v>5.42</v>
       </c>
       <c r="J229" t="n">
         <v>7.91</v>
@@ -8230,29 +8230,29 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D230" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E230" t="n">
-        <v>97.34</v>
+        <v>23.07</v>
       </c>
       <c r="F230" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G230" t="n">
-        <v>97.34</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="H230" t="n">
-        <v>-2.75</v>
+        <v>3.54</v>
       </c>
       <c r="I230" t="n">
-        <v>-2.75</v>
+        <v>5.39</v>
       </c>
       <c r="J230" t="n">
         <v>7.91</v>
@@ -8264,31 +8264,201 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>1</v>
+      </c>
+      <c r="D231" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E231" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="F231" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G231" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="H231" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="I231" t="n">
+        <v>-2.75</v>
+      </c>
+      <c r="J231" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>1</v>
+      </c>
+      <c r="D232" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E232" t="n">
+        <v>97.86</v>
+      </c>
+      <c r="F232" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G232" t="n">
+        <v>97.86</v>
+      </c>
+      <c r="H232" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="I232" t="n">
+        <v>-2.23</v>
+      </c>
+      <c r="J232" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>3</v>
+      </c>
+      <c r="D233" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E233" t="n">
+        <v>11.544</v>
+      </c>
+      <c r="F233" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G233" t="n">
+        <v>34.63</v>
+      </c>
+      <c r="H233" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="I233" t="n">
+        <v>11.14</v>
+      </c>
+      <c r="J233" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>4</v>
+      </c>
+      <c r="D234" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E234" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="F234" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G234" t="n">
+        <v>149.76</v>
+      </c>
+      <c r="H234" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="I234" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="J234" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>3</v>
+      </c>
+      <c r="D235" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E235" t="n">
+        <v>23.17</v>
+      </c>
+      <c r="F235" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G235" t="n">
+        <v>69.51000000000001</v>
+      </c>
+      <c r="H235" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="I235" t="n">
+        <v>5.85</v>
+      </c>
+      <c r="J235" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="1" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C231" t="n">
+      <c r="C236" t="n">
         <v>9</v>
       </c>
-      <c r="D231" t="n">
+      <c r="D236" t="n">
         <v>6.239</v>
       </c>
-      <c r="E231" t="n">
-        <v>6.779</v>
-      </c>
-      <c r="F231" t="n">
+      <c r="E236" t="n">
+        <v>6.812</v>
+      </c>
+      <c r="F236" t="n">
         <v>56.15</v>
       </c>
-      <c r="G231" t="n">
-        <v>61.01</v>
-      </c>
-      <c r="H231" t="n">
-        <v>4.86</v>
-      </c>
-      <c r="I231" t="n">
-        <v>8.66</v>
-      </c>
-      <c r="J231" t="n">
+      <c r="G236" t="n">
+        <v>61.31</v>
+      </c>
+      <c r="H236" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="I236" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="J236" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 03/08/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J236"/>
+  <dimension ref="A1:J241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -818,29 +818,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E12" t="n">
-        <v>41.121</v>
+        <v>10.756</v>
       </c>
       <c r="F12" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G12" t="n">
-        <v>164.48</v>
+        <v>32.27</v>
       </c>
       <c r="H12" t="n">
-        <v>25.46</v>
+        <v>1.11</v>
       </c>
       <c r="I12" t="n">
-        <v>18.31</v>
+        <v>3.56</v>
       </c>
       <c r="J12" t="n">
         <v>7.91</v>
@@ -852,29 +852,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D13" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E13" t="n">
-        <v>105.22</v>
+        <v>6.788</v>
       </c>
       <c r="F13" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G13" t="n">
-        <v>105.22</v>
+        <v>61.09</v>
       </c>
       <c r="H13" t="n">
-        <v>5.13</v>
+        <v>4.94</v>
       </c>
       <c r="I13" t="n">
-        <v>5.13</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J13" t="n">
         <v>7.91</v>
@@ -886,29 +886,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E14" t="n">
-        <v>6.788</v>
+        <v>21.907</v>
       </c>
       <c r="F14" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G14" t="n">
-        <v>61.09</v>
+        <v>65.72</v>
       </c>
       <c r="H14" t="n">
-        <v>4.94</v>
+        <v>0.05</v>
       </c>
       <c r="I14" t="n">
-        <v>8.800000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J14" t="n">
         <v>7.91</v>
@@ -920,29 +920,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E15" t="n">
-        <v>21.907</v>
+        <v>41.121</v>
       </c>
       <c r="F15" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G15" t="n">
-        <v>65.72</v>
+        <v>164.48</v>
       </c>
       <c r="H15" t="n">
-        <v>0.05</v>
+        <v>25.46</v>
       </c>
       <c r="I15" t="n">
-        <v>0.08</v>
+        <v>18.31</v>
       </c>
       <c r="J15" t="n">
         <v>7.91</v>
@@ -954,29 +954,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E16" t="n">
-        <v>10.756</v>
+        <v>105.22</v>
       </c>
       <c r="F16" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G16" t="n">
-        <v>32.27</v>
+        <v>105.22</v>
       </c>
       <c r="H16" t="n">
-        <v>1.11</v>
+        <v>5.13</v>
       </c>
       <c r="I16" t="n">
-        <v>3.56</v>
+        <v>5.13</v>
       </c>
       <c r="J16" t="n">
         <v>7.91</v>
@@ -1328,29 +1328,29 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E27" t="n">
-        <v>21.98</v>
+        <v>10.66</v>
       </c>
       <c r="F27" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G27" t="n">
-        <v>65.94</v>
+        <v>31.98</v>
       </c>
       <c r="H27" t="n">
-        <v>0.27</v>
+        <v>0.82</v>
       </c>
       <c r="I27" t="n">
-        <v>0.41</v>
+        <v>2.63</v>
       </c>
       <c r="J27" t="n">
         <v>7.91</v>
@@ -1362,29 +1362,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D28" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E28" t="n">
-        <v>6.795</v>
+        <v>40.532</v>
       </c>
       <c r="F28" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G28" t="n">
-        <v>61.16</v>
+        <v>162.13</v>
       </c>
       <c r="H28" t="n">
-        <v>5.01</v>
+        <v>23.11</v>
       </c>
       <c r="I28" t="n">
-        <v>8.92</v>
+        <v>16.62</v>
       </c>
       <c r="J28" t="n">
         <v>7.91</v>
@@ -1396,29 +1396,29 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E29" t="n">
-        <v>40.532</v>
+        <v>104.9</v>
       </c>
       <c r="F29" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G29" t="n">
-        <v>162.13</v>
+        <v>104.9</v>
       </c>
       <c r="H29" t="n">
-        <v>23.11</v>
+        <v>4.81</v>
       </c>
       <c r="I29" t="n">
-        <v>16.62</v>
+        <v>4.81</v>
       </c>
       <c r="J29" t="n">
         <v>7.91</v>
@@ -1430,29 +1430,29 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D30" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E30" t="n">
-        <v>104.9</v>
+        <v>21.98</v>
       </c>
       <c r="F30" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G30" t="n">
-        <v>104.9</v>
+        <v>65.94</v>
       </c>
       <c r="H30" t="n">
-        <v>4.81</v>
+        <v>0.27</v>
       </c>
       <c r="I30" t="n">
-        <v>4.81</v>
+        <v>0.41</v>
       </c>
       <c r="J30" t="n">
         <v>7.91</v>
@@ -1464,29 +1464,29 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E31" t="n">
-        <v>10.66</v>
+        <v>6.795</v>
       </c>
       <c r="F31" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G31" t="n">
-        <v>31.98</v>
+        <v>61.16</v>
       </c>
       <c r="H31" t="n">
-        <v>0.82</v>
+        <v>5.01</v>
       </c>
       <c r="I31" t="n">
-        <v>2.63</v>
+        <v>8.92</v>
       </c>
       <c r="J31" t="n">
         <v>7.91</v>
@@ -1838,29 +1838,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D42" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E42" t="n">
-        <v>38.497</v>
+        <v>6.629</v>
       </c>
       <c r="F42" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G42" t="n">
-        <v>153.99</v>
+        <v>59.66</v>
       </c>
       <c r="H42" t="n">
-        <v>14.97</v>
+        <v>3.51</v>
       </c>
       <c r="I42" t="n">
-        <v>10.77</v>
+        <v>6.25</v>
       </c>
       <c r="J42" t="n">
         <v>7.91</v>
@@ -1872,29 +1872,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C43" t="n">
         <v>3</v>
       </c>
       <c r="D43" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E43" t="n">
-        <v>10.61</v>
+        <v>22</v>
       </c>
       <c r="F43" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G43" t="n">
-        <v>31.83</v>
+        <v>66</v>
       </c>
       <c r="H43" t="n">
-        <v>0.67</v>
+        <v>0.33</v>
       </c>
       <c r="I43" t="n">
-        <v>2.15</v>
+        <v>0.5</v>
       </c>
       <c r="J43" t="n">
         <v>7.91</v>
@@ -1906,29 +1906,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E44" t="n">
-        <v>6.629</v>
+        <v>100.06</v>
       </c>
       <c r="F44" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G44" t="n">
-        <v>59.66</v>
+        <v>100.06</v>
       </c>
       <c r="H44" t="n">
-        <v>3.51</v>
+        <v>-0.03</v>
       </c>
       <c r="I44" t="n">
-        <v>6.25</v>
+        <v>-0.03</v>
       </c>
       <c r="J44" t="n">
         <v>7.91</v>
@@ -1940,29 +1940,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E45" t="n">
-        <v>100.06</v>
+        <v>10.61</v>
       </c>
       <c r="F45" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G45" t="n">
-        <v>100.06</v>
+        <v>31.83</v>
       </c>
       <c r="H45" t="n">
-        <v>-0.03</v>
+        <v>0.67</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03</v>
+        <v>2.15</v>
       </c>
       <c r="J45" t="n">
         <v>7.91</v>
@@ -1974,29 +1974,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D46" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E46" t="n">
-        <v>22</v>
+        <v>38.497</v>
       </c>
       <c r="F46" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G46" t="n">
-        <v>66</v>
+        <v>153.99</v>
       </c>
       <c r="H46" t="n">
-        <v>0.33</v>
+        <v>14.97</v>
       </c>
       <c r="I46" t="n">
-        <v>0.5</v>
+        <v>10.77</v>
       </c>
       <c r="J46" t="n">
         <v>7.91</v>
@@ -2348,29 +2348,29 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C57" t="n">
         <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E57" t="n">
-        <v>22.289</v>
+        <v>10.75</v>
       </c>
       <c r="F57" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G57" t="n">
-        <v>66.87</v>
+        <v>32.25</v>
       </c>
       <c r="H57" t="n">
-        <v>1.2</v>
+        <v>1.09</v>
       </c>
       <c r="I57" t="n">
-        <v>1.83</v>
+        <v>3.5</v>
       </c>
       <c r="J57" t="n">
         <v>7.91</v>
@@ -2382,29 +2382,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D58" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E58" t="n">
-        <v>102.86</v>
+        <v>6.736</v>
       </c>
       <c r="F58" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G58" t="n">
-        <v>102.86</v>
+        <v>60.62</v>
       </c>
       <c r="H58" t="n">
-        <v>2.77</v>
+        <v>4.47</v>
       </c>
       <c r="I58" t="n">
-        <v>2.77</v>
+        <v>7.96</v>
       </c>
       <c r="J58" t="n">
         <v>7.91</v>
@@ -2416,29 +2416,29 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D59" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E59" t="n">
-        <v>6.736</v>
+        <v>39.845</v>
       </c>
       <c r="F59" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G59" t="n">
-        <v>60.62</v>
+        <v>159.38</v>
       </c>
       <c r="H59" t="n">
-        <v>4.47</v>
+        <v>20.36</v>
       </c>
       <c r="I59" t="n">
-        <v>7.96</v>
+        <v>14.65</v>
       </c>
       <c r="J59" t="n">
         <v>7.91</v>
@@ -2450,29 +2450,29 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E60" t="n">
-        <v>39.845</v>
+        <v>102.86</v>
       </c>
       <c r="F60" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G60" t="n">
-        <v>159.38</v>
+        <v>102.86</v>
       </c>
       <c r="H60" t="n">
-        <v>20.36</v>
+        <v>2.77</v>
       </c>
       <c r="I60" t="n">
-        <v>14.65</v>
+        <v>2.77</v>
       </c>
       <c r="J60" t="n">
         <v>7.91</v>
@@ -2484,29 +2484,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C61" t="n">
         <v>3</v>
       </c>
       <c r="D61" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E61" t="n">
-        <v>10.75</v>
+        <v>22.289</v>
       </c>
       <c r="F61" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G61" t="n">
-        <v>32.25</v>
+        <v>66.87</v>
       </c>
       <c r="H61" t="n">
-        <v>1.09</v>
+        <v>1.2</v>
       </c>
       <c r="I61" t="n">
-        <v>3.5</v>
+        <v>1.83</v>
       </c>
       <c r="J61" t="n">
         <v>7.91</v>
@@ -2858,29 +2858,29 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E72" t="n">
-        <v>104.22</v>
+        <v>41.15</v>
       </c>
       <c r="F72" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G72" t="n">
-        <v>104.22</v>
+        <v>164.6</v>
       </c>
       <c r="H72" t="n">
-        <v>4.13</v>
+        <v>25.58</v>
       </c>
       <c r="I72" t="n">
-        <v>4.13</v>
+        <v>18.4</v>
       </c>
       <c r="J72" t="n">
         <v>7.91</v>
@@ -2892,29 +2892,29 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D73" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E73" t="n">
-        <v>23</v>
+        <v>6.811</v>
       </c>
       <c r="F73" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G73" t="n">
-        <v>69</v>
+        <v>61.3</v>
       </c>
       <c r="H73" t="n">
-        <v>3.33</v>
+        <v>5.15</v>
       </c>
       <c r="I73" t="n">
-        <v>5.07</v>
+        <v>9.17</v>
       </c>
       <c r="J73" t="n">
         <v>7.91</v>
@@ -2960,29 +2960,29 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E75" t="n">
-        <v>6.811</v>
+        <v>23</v>
       </c>
       <c r="F75" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G75" t="n">
-        <v>61.3</v>
+        <v>69</v>
       </c>
       <c r="H75" t="n">
-        <v>5.15</v>
+        <v>3.33</v>
       </c>
       <c r="I75" t="n">
-        <v>9.17</v>
+        <v>5.07</v>
       </c>
       <c r="J75" t="n">
         <v>7.91</v>
@@ -2994,29 +2994,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E76" t="n">
-        <v>41.15</v>
+        <v>104.22</v>
       </c>
       <c r="F76" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G76" t="n">
-        <v>164.6</v>
+        <v>104.22</v>
       </c>
       <c r="H76" t="n">
-        <v>25.58</v>
+        <v>4.13</v>
       </c>
       <c r="I76" t="n">
-        <v>18.4</v>
+        <v>4.13</v>
       </c>
       <c r="J76" t="n">
         <v>7.91</v>
@@ -3368,29 +3368,29 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D87" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E87" t="n">
-        <v>106.28</v>
+        <v>43.005</v>
       </c>
       <c r="F87" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G87" t="n">
-        <v>106.28</v>
+        <v>172.02</v>
       </c>
       <c r="H87" t="n">
-        <v>6.19</v>
+        <v>33</v>
       </c>
       <c r="I87" t="n">
-        <v>6.18</v>
+        <v>23.74</v>
       </c>
       <c r="J87" t="n">
         <v>7.91</v>
@@ -3402,29 +3402,29 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E88" t="n">
-        <v>23.32</v>
+        <v>10.852</v>
       </c>
       <c r="F88" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G88" t="n">
-        <v>69.95999999999999</v>
+        <v>32.56</v>
       </c>
       <c r="H88" t="n">
-        <v>4.29</v>
+        <v>1.4</v>
       </c>
       <c r="I88" t="n">
-        <v>6.53</v>
+        <v>4.49</v>
       </c>
       <c r="J88" t="n">
         <v>7.91</v>
@@ -3470,29 +3470,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C90" t="n">
         <v>3</v>
       </c>
       <c r="D90" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E90" t="n">
-        <v>10.852</v>
+        <v>23.32</v>
       </c>
       <c r="F90" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G90" t="n">
-        <v>32.56</v>
+        <v>69.95999999999999</v>
       </c>
       <c r="H90" t="n">
-        <v>1.4</v>
+        <v>4.29</v>
       </c>
       <c r="I90" t="n">
-        <v>4.49</v>
+        <v>6.53</v>
       </c>
       <c r="J90" t="n">
         <v>7.91</v>
@@ -3504,29 +3504,29 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E91" t="n">
-        <v>43.005</v>
+        <v>106.28</v>
       </c>
       <c r="F91" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G91" t="n">
-        <v>172.02</v>
+        <v>106.28</v>
       </c>
       <c r="H91" t="n">
-        <v>33</v>
+        <v>6.19</v>
       </c>
       <c r="I91" t="n">
-        <v>23.74</v>
+        <v>6.18</v>
       </c>
       <c r="J91" t="n">
         <v>7.91</v>
@@ -3878,29 +3878,29 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D102" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E102" t="n">
-        <v>10.556</v>
+        <v>103.46</v>
       </c>
       <c r="F102" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G102" t="n">
-        <v>31.67</v>
+        <v>103.46</v>
       </c>
       <c r="H102" t="n">
-        <v>0.51</v>
+        <v>3.37</v>
       </c>
       <c r="I102" t="n">
-        <v>1.64</v>
+        <v>3.37</v>
       </c>
       <c r="J102" t="n">
         <v>7.91</v>
@@ -3912,29 +3912,29 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D103" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E103" t="n">
-        <v>23.29</v>
+        <v>40.97</v>
       </c>
       <c r="F103" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G103" t="n">
-        <v>69.87</v>
+        <v>163.88</v>
       </c>
       <c r="H103" t="n">
-        <v>4.2</v>
+        <v>24.86</v>
       </c>
       <c r="I103" t="n">
-        <v>6.4</v>
+        <v>17.88</v>
       </c>
       <c r="J103" t="n">
         <v>7.91</v>
@@ -3946,29 +3946,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D104" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E104" t="n">
-        <v>6.804</v>
+        <v>23.29</v>
       </c>
       <c r="F104" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G104" t="n">
-        <v>61.24</v>
+        <v>69.87</v>
       </c>
       <c r="H104" t="n">
-        <v>5.09</v>
+        <v>4.2</v>
       </c>
       <c r="I104" t="n">
-        <v>9.07</v>
+        <v>6.4</v>
       </c>
       <c r="J104" t="n">
         <v>7.91</v>
@@ -3980,29 +3980,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E105" t="n">
-        <v>40.97</v>
+        <v>10.556</v>
       </c>
       <c r="F105" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G105" t="n">
-        <v>163.88</v>
+        <v>31.67</v>
       </c>
       <c r="H105" t="n">
-        <v>24.86</v>
+        <v>0.51</v>
       </c>
       <c r="I105" t="n">
-        <v>17.88</v>
+        <v>1.64</v>
       </c>
       <c r="J105" t="n">
         <v>7.91</v>
@@ -4014,29 +4014,29 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D106" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E106" t="n">
-        <v>103.46</v>
+        <v>6.804</v>
       </c>
       <c r="F106" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G106" t="n">
-        <v>103.46</v>
+        <v>61.24</v>
       </c>
       <c r="H106" t="n">
-        <v>3.37</v>
+        <v>5.09</v>
       </c>
       <c r="I106" t="n">
-        <v>3.37</v>
+        <v>9.07</v>
       </c>
       <c r="J106" t="n">
         <v>7.91</v>
@@ -4218,29 +4218,29 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D112" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E112" t="n">
-        <v>103.56</v>
+        <v>10.568</v>
       </c>
       <c r="F112" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G112" t="n">
-        <v>103.56</v>
+        <v>31.7</v>
       </c>
       <c r="H112" t="n">
-        <v>3.47</v>
+        <v>0.54</v>
       </c>
       <c r="I112" t="n">
-        <v>3.47</v>
+        <v>1.73</v>
       </c>
       <c r="J112" t="n">
         <v>7.91</v>
@@ -4252,29 +4252,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D113" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E113" t="n">
-        <v>23.025</v>
+        <v>103.56</v>
       </c>
       <c r="F113" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G113" t="n">
-        <v>69.06999999999999</v>
+        <v>103.56</v>
       </c>
       <c r="H113" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="I113" t="n">
-        <v>5.18</v>
+        <v>3.47</v>
       </c>
       <c r="J113" t="n">
         <v>7.91</v>
@@ -4286,29 +4286,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D114" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E114" t="n">
-        <v>6.797</v>
+        <v>23.025</v>
       </c>
       <c r="F114" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G114" t="n">
-        <v>61.17</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H114" t="n">
-        <v>5.02</v>
+        <v>3.4</v>
       </c>
       <c r="I114" t="n">
-        <v>8.94</v>
+        <v>5.18</v>
       </c>
       <c r="J114" t="n">
         <v>7.91</v>
@@ -4320,29 +4320,29 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D115" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E115" t="n">
-        <v>10.568</v>
+        <v>6.797</v>
       </c>
       <c r="F115" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G115" t="n">
-        <v>31.7</v>
+        <v>61.17</v>
       </c>
       <c r="H115" t="n">
-        <v>0.54</v>
+        <v>5.02</v>
       </c>
       <c r="I115" t="n">
-        <v>1.73</v>
+        <v>8.94</v>
       </c>
       <c r="J115" t="n">
         <v>7.91</v>
@@ -4388,29 +4388,29 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D117" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E117" t="n">
-        <v>23.145</v>
+        <v>6.861</v>
       </c>
       <c r="F117" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G117" t="n">
-        <v>69.44</v>
+        <v>61.75</v>
       </c>
       <c r="H117" t="n">
-        <v>3.77</v>
+        <v>5.6</v>
       </c>
       <c r="I117" t="n">
-        <v>5.74</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="J117" t="n">
         <v>7.91</v>
@@ -4422,29 +4422,29 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E118" t="n">
-        <v>105.96</v>
+        <v>10.756</v>
       </c>
       <c r="F118" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G118" t="n">
-        <v>105.96</v>
+        <v>32.27</v>
       </c>
       <c r="H118" t="n">
-        <v>5.87</v>
+        <v>1.11</v>
       </c>
       <c r="I118" t="n">
-        <v>5.86</v>
+        <v>3.56</v>
       </c>
       <c r="J118" t="n">
         <v>7.91</v>
@@ -4456,29 +4456,29 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D119" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E119" t="n">
-        <v>10.756</v>
+        <v>41</v>
       </c>
       <c r="F119" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G119" t="n">
-        <v>32.27</v>
+        <v>164</v>
       </c>
       <c r="H119" t="n">
-        <v>1.11</v>
+        <v>24.98</v>
       </c>
       <c r="I119" t="n">
-        <v>3.56</v>
+        <v>17.97</v>
       </c>
       <c r="J119" t="n">
         <v>7.91</v>
@@ -4490,29 +4490,29 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D120" t="n">
-        <v>6.239</v>
+        <v>21.89</v>
       </c>
       <c r="E120" t="n">
-        <v>6.861</v>
+        <v>23.145</v>
       </c>
       <c r="F120" t="n">
-        <v>56.15</v>
+        <v>65.67</v>
       </c>
       <c r="G120" t="n">
-        <v>61.75</v>
+        <v>69.44</v>
       </c>
       <c r="H120" t="n">
-        <v>5.6</v>
+        <v>3.77</v>
       </c>
       <c r="I120" t="n">
-        <v>9.970000000000001</v>
+        <v>5.74</v>
       </c>
       <c r="J120" t="n">
         <v>7.91</v>
@@ -4524,29 +4524,29 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D121" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E121" t="n">
-        <v>41</v>
+        <v>105.96</v>
       </c>
       <c r="F121" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G121" t="n">
-        <v>164</v>
+        <v>105.96</v>
       </c>
       <c r="H121" t="n">
-        <v>24.98</v>
+        <v>5.87</v>
       </c>
       <c r="I121" t="n">
-        <v>17.97</v>
+        <v>5.86</v>
       </c>
       <c r="J121" t="n">
         <v>7.91</v>
@@ -4898,29 +4898,29 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C132" t="n">
         <v>3</v>
       </c>
       <c r="D132" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E132" t="n">
-        <v>11.516</v>
+        <v>23.18</v>
       </c>
       <c r="F132" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G132" t="n">
-        <v>34.55</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="H132" t="n">
-        <v>3.39</v>
+        <v>3.87</v>
       </c>
       <c r="I132" t="n">
-        <v>10.88</v>
+        <v>5.89</v>
       </c>
       <c r="J132" t="n">
         <v>7.91</v>
@@ -4932,29 +4932,29 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D133" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E133" t="n">
-        <v>40.54</v>
+        <v>6.895</v>
       </c>
       <c r="F133" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G133" t="n">
-        <v>162.16</v>
+        <v>62.05</v>
       </c>
       <c r="H133" t="n">
-        <v>23.14</v>
+        <v>5.9</v>
       </c>
       <c r="I133" t="n">
-        <v>16.65</v>
+        <v>10.51</v>
       </c>
       <c r="J133" t="n">
         <v>7.91</v>
@@ -4966,29 +4966,29 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D134" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E134" t="n">
-        <v>104.02</v>
+        <v>11.516</v>
       </c>
       <c r="F134" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G134" t="n">
-        <v>104.02</v>
+        <v>34.55</v>
       </c>
       <c r="H134" t="n">
-        <v>3.93</v>
+        <v>3.39</v>
       </c>
       <c r="I134" t="n">
-        <v>3.93</v>
+        <v>10.88</v>
       </c>
       <c r="J134" t="n">
         <v>7.91</v>
@@ -5000,29 +5000,29 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E135" t="n">
-        <v>6.895</v>
+        <v>40.54</v>
       </c>
       <c r="F135" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G135" t="n">
-        <v>62.05</v>
+        <v>162.16</v>
       </c>
       <c r="H135" t="n">
-        <v>5.9</v>
+        <v>23.14</v>
       </c>
       <c r="I135" t="n">
-        <v>10.51</v>
+        <v>16.65</v>
       </c>
       <c r="J135" t="n">
         <v>7.91</v>
@@ -5034,29 +5034,29 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D136" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E136" t="n">
-        <v>23.18</v>
+        <v>104.02</v>
       </c>
       <c r="F136" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G136" t="n">
-        <v>69.54000000000001</v>
+        <v>104.02</v>
       </c>
       <c r="H136" t="n">
-        <v>3.87</v>
+        <v>3.93</v>
       </c>
       <c r="I136" t="n">
-        <v>5.89</v>
+        <v>3.93</v>
       </c>
       <c r="J136" t="n">
         <v>7.91</v>
@@ -5408,29 +5408,29 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D147" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E147" t="n">
-        <v>6.826</v>
+        <v>38.955</v>
       </c>
       <c r="F147" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G147" t="n">
-        <v>61.43</v>
+        <v>155.82</v>
       </c>
       <c r="H147" t="n">
-        <v>5.28</v>
+        <v>16.8</v>
       </c>
       <c r="I147" t="n">
-        <v>9.4</v>
+        <v>12.08</v>
       </c>
       <c r="J147" t="n">
         <v>7.91</v>
@@ -5442,29 +5442,29 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D148" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E148" t="n">
-        <v>22.755</v>
+        <v>101.7</v>
       </c>
       <c r="F148" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G148" t="n">
-        <v>68.27</v>
+        <v>101.7</v>
       </c>
       <c r="H148" t="n">
-        <v>2.6</v>
+        <v>1.61</v>
       </c>
       <c r="I148" t="n">
-        <v>3.96</v>
+        <v>1.61</v>
       </c>
       <c r="J148" t="n">
         <v>7.91</v>
@@ -5510,29 +5510,29 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D150" t="n">
-        <v>34.755</v>
+        <v>6.239</v>
       </c>
       <c r="E150" t="n">
-        <v>38.955</v>
+        <v>6.826</v>
       </c>
       <c r="F150" t="n">
-        <v>139.02</v>
+        <v>56.15</v>
       </c>
       <c r="G150" t="n">
-        <v>155.82</v>
+        <v>61.43</v>
       </c>
       <c r="H150" t="n">
-        <v>16.8</v>
+        <v>5.28</v>
       </c>
       <c r="I150" t="n">
-        <v>12.08</v>
+        <v>9.4</v>
       </c>
       <c r="J150" t="n">
         <v>7.91</v>
@@ -5544,29 +5544,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E151" t="n">
-        <v>101.7</v>
+        <v>22.755</v>
       </c>
       <c r="F151" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G151" t="n">
-        <v>101.7</v>
+        <v>68.27</v>
       </c>
       <c r="H151" t="n">
-        <v>1.61</v>
+        <v>2.6</v>
       </c>
       <c r="I151" t="n">
-        <v>1.61</v>
+        <v>3.96</v>
       </c>
       <c r="J151" t="n">
         <v>7.91</v>
@@ -5918,29 +5918,29 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C162" t="n">
         <v>3</v>
       </c>
       <c r="D162" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E162" t="n">
-        <v>23.01</v>
+        <v>10.748</v>
       </c>
       <c r="F162" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G162" t="n">
-        <v>69.03</v>
+        <v>32.24</v>
       </c>
       <c r="H162" t="n">
-        <v>3.36</v>
+        <v>1.08</v>
       </c>
       <c r="I162" t="n">
-        <v>5.12</v>
+        <v>3.47</v>
       </c>
       <c r="J162" t="n">
         <v>7.91</v>
@@ -5952,29 +5952,29 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D163" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E163" t="n">
-        <v>6.927</v>
+        <v>103.84</v>
       </c>
       <c r="F163" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G163" t="n">
-        <v>62.34</v>
+        <v>103.84</v>
       </c>
       <c r="H163" t="n">
-        <v>6.19</v>
+        <v>3.75</v>
       </c>
       <c r="I163" t="n">
-        <v>11.02</v>
+        <v>3.75</v>
       </c>
       <c r="J163" t="n">
         <v>7.91</v>
@@ -6020,29 +6020,29 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D165" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E165" t="n">
-        <v>103.84</v>
+        <v>23.01</v>
       </c>
       <c r="F165" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G165" t="n">
-        <v>103.84</v>
+        <v>69.03</v>
       </c>
       <c r="H165" t="n">
-        <v>3.75</v>
+        <v>3.36</v>
       </c>
       <c r="I165" t="n">
-        <v>3.75</v>
+        <v>5.12</v>
       </c>
       <c r="J165" t="n">
         <v>7.91</v>
@@ -6054,29 +6054,29 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D166" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E166" t="n">
-        <v>10.748</v>
+        <v>6.927</v>
       </c>
       <c r="F166" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G166" t="n">
-        <v>32.24</v>
+        <v>62.34</v>
       </c>
       <c r="H166" t="n">
-        <v>1.08</v>
+        <v>6.19</v>
       </c>
       <c r="I166" t="n">
-        <v>3.47</v>
+        <v>11.02</v>
       </c>
       <c r="J166" t="n">
         <v>7.91</v>
@@ -6428,29 +6428,29 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D177" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E177" t="n">
-        <v>38.245</v>
+        <v>22.95</v>
       </c>
       <c r="F177" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G177" t="n">
-        <v>152.98</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="H177" t="n">
-        <v>13.96</v>
+        <v>3.18</v>
       </c>
       <c r="I177" t="n">
-        <v>10.04</v>
+        <v>4.84</v>
       </c>
       <c r="J177" t="n">
         <v>7.91</v>
@@ -6462,29 +6462,29 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D178" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E178" t="n">
-        <v>6.922</v>
+        <v>102.54</v>
       </c>
       <c r="F178" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G178" t="n">
-        <v>62.3</v>
+        <v>102.54</v>
       </c>
       <c r="H178" t="n">
-        <v>6.15</v>
+        <v>2.45</v>
       </c>
       <c r="I178" t="n">
-        <v>10.95</v>
+        <v>2.45</v>
       </c>
       <c r="J178" t="n">
         <v>7.91</v>
@@ -6496,29 +6496,29 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D179" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E179" t="n">
-        <v>102.54</v>
+        <v>10.642</v>
       </c>
       <c r="F179" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G179" t="n">
-        <v>102.54</v>
+        <v>31.93</v>
       </c>
       <c r="H179" t="n">
-        <v>2.45</v>
+        <v>0.77</v>
       </c>
       <c r="I179" t="n">
-        <v>2.45</v>
+        <v>2.47</v>
       </c>
       <c r="J179" t="n">
         <v>7.91</v>
@@ -6530,29 +6530,29 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D180" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E180" t="n">
-        <v>10.642</v>
+        <v>38.245</v>
       </c>
       <c r="F180" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G180" t="n">
-        <v>31.93</v>
+        <v>152.98</v>
       </c>
       <c r="H180" t="n">
-        <v>0.77</v>
+        <v>13.96</v>
       </c>
       <c r="I180" t="n">
-        <v>2.47</v>
+        <v>10.04</v>
       </c>
       <c r="J180" t="n">
         <v>7.91</v>
@@ -6564,29 +6564,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D181" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E181" t="n">
-        <v>22.95</v>
+        <v>6.922</v>
       </c>
       <c r="F181" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G181" t="n">
-        <v>68.84999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="H181" t="n">
-        <v>3.18</v>
+        <v>6.15</v>
       </c>
       <c r="I181" t="n">
-        <v>4.84</v>
+        <v>10.95</v>
       </c>
       <c r="J181" t="n">
         <v>7.91</v>
@@ -6938,29 +6938,29 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D192" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E192" t="n">
-        <v>38.755</v>
+        <v>22.82</v>
       </c>
       <c r="F192" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G192" t="n">
-        <v>155.02</v>
+        <v>68.45999999999999</v>
       </c>
       <c r="H192" t="n">
-        <v>16</v>
+        <v>2.79</v>
       </c>
       <c r="I192" t="n">
-        <v>11.51</v>
+        <v>4.25</v>
       </c>
       <c r="J192" t="n">
         <v>7.91</v>
@@ -6972,29 +6972,29 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D193" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E193" t="n">
-        <v>102.46</v>
+        <v>6.894</v>
       </c>
       <c r="F193" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G193" t="n">
-        <v>102.46</v>
+        <v>62.05</v>
       </c>
       <c r="H193" t="n">
-        <v>2.37</v>
+        <v>5.9</v>
       </c>
       <c r="I193" t="n">
-        <v>2.37</v>
+        <v>10.51</v>
       </c>
       <c r="J193" t="n">
         <v>7.91</v>
@@ -7040,29 +7040,29 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D195" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E195" t="n">
-        <v>6.894</v>
+        <v>38.755</v>
       </c>
       <c r="F195" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G195" t="n">
-        <v>62.05</v>
+        <v>155.02</v>
       </c>
       <c r="H195" t="n">
-        <v>5.9</v>
+        <v>16</v>
       </c>
       <c r="I195" t="n">
-        <v>10.51</v>
+        <v>11.51</v>
       </c>
       <c r="J195" t="n">
         <v>7.91</v>
@@ -7074,29 +7074,29 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D196" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E196" t="n">
-        <v>22.82</v>
+        <v>102.46</v>
       </c>
       <c r="F196" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G196" t="n">
-        <v>68.45999999999999</v>
+        <v>102.46</v>
       </c>
       <c r="H196" t="n">
-        <v>2.79</v>
+        <v>2.37</v>
       </c>
       <c r="I196" t="n">
-        <v>4.25</v>
+        <v>2.37</v>
       </c>
       <c r="J196" t="n">
         <v>7.91</v>
@@ -7448,29 +7448,29 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D207" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E207" t="n">
-        <v>11.172</v>
+        <v>6.865</v>
       </c>
       <c r="F207" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G207" t="n">
-        <v>33.52</v>
+        <v>61.79</v>
       </c>
       <c r="H207" t="n">
-        <v>2.36</v>
+        <v>5.64</v>
       </c>
       <c r="I207" t="n">
-        <v>7.57</v>
+        <v>10.04</v>
       </c>
       <c r="J207" t="n">
         <v>7.91</v>
@@ -7482,29 +7482,29 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D208" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E208" t="n">
-        <v>37.82</v>
+        <v>22.725</v>
       </c>
       <c r="F208" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G208" t="n">
-        <v>151.28</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="H208" t="n">
-        <v>12.26</v>
+        <v>2.51</v>
       </c>
       <c r="I208" t="n">
-        <v>8.82</v>
+        <v>3.82</v>
       </c>
       <c r="J208" t="n">
         <v>7.91</v>
@@ -7516,29 +7516,29 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D209" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E209" t="n">
-        <v>22.725</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F209" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G209" t="n">
-        <v>68.18000000000001</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="H209" t="n">
-        <v>2.51</v>
+        <v>-0.19</v>
       </c>
       <c r="I209" t="n">
-        <v>3.82</v>
+        <v>-0.19</v>
       </c>
       <c r="J209" t="n">
         <v>7.91</v>
@@ -7550,29 +7550,29 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D210" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E210" t="n">
-        <v>99.90000000000001</v>
+        <v>11.172</v>
       </c>
       <c r="F210" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G210" t="n">
-        <v>99.90000000000001</v>
+        <v>33.52</v>
       </c>
       <c r="H210" t="n">
-        <v>-0.19</v>
+        <v>2.36</v>
       </c>
       <c r="I210" t="n">
-        <v>-0.19</v>
+        <v>7.57</v>
       </c>
       <c r="J210" t="n">
         <v>7.91</v>
@@ -7584,29 +7584,29 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D211" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E211" t="n">
-        <v>6.865</v>
+        <v>37.82</v>
       </c>
       <c r="F211" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G211" t="n">
-        <v>61.79</v>
+        <v>151.28</v>
       </c>
       <c r="H211" t="n">
-        <v>5.64</v>
+        <v>12.26</v>
       </c>
       <c r="I211" t="n">
-        <v>10.04</v>
+        <v>8.82</v>
       </c>
       <c r="J211" t="n">
         <v>7.91</v>
@@ -7958,29 +7958,29 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D222" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E222" t="n">
-        <v>96.67</v>
+        <v>6.818</v>
       </c>
       <c r="F222" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G222" t="n">
-        <v>96.67</v>
+        <v>61.36</v>
       </c>
       <c r="H222" t="n">
-        <v>-3.42</v>
+        <v>5.21</v>
       </c>
       <c r="I222" t="n">
-        <v>-3.42</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="J222" t="n">
         <v>7.91</v>
@@ -7992,29 +7992,29 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D223" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E223" t="n">
-        <v>11.5</v>
+        <v>35.89</v>
       </c>
       <c r="F223" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G223" t="n">
-        <v>34.5</v>
+        <v>143.56</v>
       </c>
       <c r="H223" t="n">
-        <v>3.34</v>
+        <v>4.54</v>
       </c>
       <c r="I223" t="n">
-        <v>10.72</v>
+        <v>3.27</v>
       </c>
       <c r="J223" t="n">
         <v>7.91</v>
@@ -8026,29 +8026,29 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D224" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E224" t="n">
-        <v>35.89</v>
+        <v>23.12</v>
       </c>
       <c r="F224" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G224" t="n">
-        <v>143.56</v>
+        <v>69.36</v>
       </c>
       <c r="H224" t="n">
-        <v>4.54</v>
+        <v>3.69</v>
       </c>
       <c r="I224" t="n">
-        <v>3.27</v>
+        <v>5.62</v>
       </c>
       <c r="J224" t="n">
         <v>7.91</v>
@@ -8060,29 +8060,29 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D225" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E225" t="n">
-        <v>23.12</v>
+        <v>96.67</v>
       </c>
       <c r="F225" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G225" t="n">
-        <v>69.36</v>
+        <v>96.67</v>
       </c>
       <c r="H225" t="n">
-        <v>3.69</v>
+        <v>-3.42</v>
       </c>
       <c r="I225" t="n">
-        <v>5.62</v>
+        <v>-3.42</v>
       </c>
       <c r="J225" t="n">
         <v>7.91</v>
@@ -8094,29 +8094,29 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D226" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E226" t="n">
-        <v>6.818</v>
+        <v>11.5</v>
       </c>
       <c r="F226" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G226" t="n">
-        <v>61.36</v>
+        <v>34.5</v>
       </c>
       <c r="H226" t="n">
-        <v>5.21</v>
+        <v>3.34</v>
       </c>
       <c r="I226" t="n">
-        <v>9.279999999999999</v>
+        <v>10.72</v>
       </c>
       <c r="J226" t="n">
         <v>7.91</v>
@@ -8298,29 +8298,29 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D232" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E232" t="n">
-        <v>97.86</v>
+        <v>6.812</v>
       </c>
       <c r="F232" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G232" t="n">
-        <v>97.86</v>
+        <v>61.31</v>
       </c>
       <c r="H232" t="n">
-        <v>-2.23</v>
+        <v>5.16</v>
       </c>
       <c r="I232" t="n">
-        <v>-2.23</v>
+        <v>9.19</v>
       </c>
       <c r="J232" t="n">
         <v>7.91</v>
@@ -8332,29 +8332,29 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C233" t="n">
         <v>3</v>
       </c>
       <c r="D233" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E233" t="n">
-        <v>11.544</v>
+        <v>23.17</v>
       </c>
       <c r="F233" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G233" t="n">
-        <v>34.63</v>
+        <v>69.51000000000001</v>
       </c>
       <c r="H233" t="n">
-        <v>3.47</v>
+        <v>3.84</v>
       </c>
       <c r="I233" t="n">
-        <v>11.14</v>
+        <v>5.85</v>
       </c>
       <c r="J233" t="n">
         <v>7.91</v>
@@ -8366,29 +8366,29 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D234" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E234" t="n">
-        <v>37.44</v>
+        <v>11.544</v>
       </c>
       <c r="F234" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G234" t="n">
-        <v>149.76</v>
+        <v>34.63</v>
       </c>
       <c r="H234" t="n">
-        <v>10.74</v>
+        <v>3.47</v>
       </c>
       <c r="I234" t="n">
-        <v>7.73</v>
+        <v>11.14</v>
       </c>
       <c r="J234" t="n">
         <v>7.91</v>
@@ -8400,29 +8400,29 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E235" t="n">
-        <v>23.17</v>
+        <v>97.86</v>
       </c>
       <c r="F235" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G235" t="n">
-        <v>69.51000000000001</v>
+        <v>97.86</v>
       </c>
       <c r="H235" t="n">
-        <v>3.84</v>
+        <v>-2.23</v>
       </c>
       <c r="I235" t="n">
-        <v>5.85</v>
+        <v>-2.23</v>
       </c>
       <c r="J235" t="n">
         <v>7.91</v>
@@ -8434,31 +8434,201 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>4</v>
+      </c>
+      <c r="D236" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E236" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="F236" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G236" t="n">
+        <v>149.76</v>
+      </c>
+      <c r="H236" t="n">
+        <v>10.74</v>
+      </c>
+      <c r="I236" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="J236" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>EFENSE</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>3</v>
+      </c>
+      <c r="D237" t="n">
+        <v>10.387</v>
+      </c>
+      <c r="E237" t="n">
+        <v>11.842</v>
+      </c>
+      <c r="F237" t="n">
+        <v>31.16</v>
+      </c>
+      <c r="G237" t="n">
+        <v>35.53</v>
+      </c>
+      <c r="H237" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="I237" t="n">
+        <v>14.02</v>
+      </c>
+      <c r="J237" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>PAASI</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>4</v>
+      </c>
+      <c r="D238" t="n">
+        <v>34.755</v>
+      </c>
+      <c r="E238" t="n">
+        <v>37.315</v>
+      </c>
+      <c r="F238" t="n">
+        <v>139.02</v>
+      </c>
+      <c r="G238" t="n">
+        <v>149.26</v>
+      </c>
+      <c r="H238" t="n">
+        <v>10.24</v>
+      </c>
+      <c r="I238" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="J238" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>PINDIA</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>3</v>
+      </c>
+      <c r="D239" t="n">
+        <v>21.89</v>
+      </c>
+      <c r="E239" t="n">
+        <v>23.245</v>
+      </c>
+      <c r="F239" t="n">
+        <v>65.67</v>
+      </c>
+      <c r="G239" t="n">
+        <v>69.73</v>
+      </c>
+      <c r="H239" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="I239" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="J239" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>PUST</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>1</v>
+      </c>
+      <c r="D240" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="E240" t="n">
+        <v>99.84999999999999</v>
+      </c>
+      <c r="F240" t="n">
+        <v>100.09</v>
+      </c>
+      <c r="G240" t="n">
+        <v>99.84999999999999</v>
+      </c>
+      <c r="H240" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="I240" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="J240" t="n">
+        <v>7.91</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
           <t>IWSC</t>
         </is>
       </c>
-      <c r="C236" t="n">
+      <c r="C241" t="n">
         <v>9</v>
       </c>
-      <c r="D236" t="n">
+      <c r="D241" t="n">
         <v>6.239</v>
       </c>
-      <c r="E236" t="n">
-        <v>6.812</v>
-      </c>
-      <c r="F236" t="n">
+      <c r="E241" t="n">
+        <v>6.914</v>
+      </c>
+      <c r="F241" t="n">
         <v>56.15</v>
       </c>
-      <c r="G236" t="n">
-        <v>61.31</v>
-      </c>
-      <c r="H236" t="n">
-        <v>5.16</v>
-      </c>
-      <c r="I236" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="J236" t="n">
+      <c r="G241" t="n">
+        <v>62.23</v>
+      </c>
+      <c r="H241" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="I241" t="n">
+        <v>10.83</v>
+      </c>
+      <c r="J241" t="n">
         <v>7.91</v>
       </c>
     </row>

</xml_diff>

<commit_message>
📈 Pointage automatique du 04/08/2026
</commit_message>
<xml_diff>
--- a/suivi_pea_detail.xlsx
+++ b/suivi_pea_detail.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J241"/>
+  <dimension ref="A1:J246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,29 +648,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E7" t="n">
-        <v>40.247</v>
+        <v>11.262</v>
       </c>
       <c r="F7" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G7" t="n">
-        <v>160.99</v>
+        <v>33.79</v>
       </c>
       <c r="H7" t="n">
-        <v>21.97</v>
+        <v>2.63</v>
       </c>
       <c r="I7" t="n">
-        <v>15.8</v>
+        <v>8.44</v>
       </c>
       <c r="J7" t="n">
         <v>7.91</v>
@@ -682,29 +682,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E8" t="n">
-        <v>22.34</v>
+        <v>104.22</v>
       </c>
       <c r="F8" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G8" t="n">
-        <v>67.02</v>
+        <v>104.22</v>
       </c>
       <c r="H8" t="n">
-        <v>1.35</v>
+        <v>4.13</v>
       </c>
       <c r="I8" t="n">
-        <v>2.06</v>
+        <v>4.13</v>
       </c>
       <c r="J8" t="n">
         <v>7.91</v>
@@ -716,29 +716,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E9" t="n">
-        <v>104.22</v>
+        <v>6.781</v>
       </c>
       <c r="F9" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G9" t="n">
-        <v>104.22</v>
+        <v>61.03</v>
       </c>
       <c r="H9" t="n">
-        <v>4.13</v>
+        <v>4.88</v>
       </c>
       <c r="I9" t="n">
-        <v>4.13</v>
+        <v>8.69</v>
       </c>
       <c r="J9" t="n">
         <v>7.91</v>
@@ -750,29 +750,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D10" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E10" t="n">
-        <v>6.781</v>
+        <v>40.247</v>
       </c>
       <c r="F10" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G10" t="n">
-        <v>61.03</v>
+        <v>160.99</v>
       </c>
       <c r="H10" t="n">
-        <v>4.88</v>
+        <v>21.97</v>
       </c>
       <c r="I10" t="n">
-        <v>8.69</v>
+        <v>15.8</v>
       </c>
       <c r="J10" t="n">
         <v>7.91</v>
@@ -784,29 +784,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C11" t="n">
         <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E11" t="n">
-        <v>11.262</v>
+        <v>22.34</v>
       </c>
       <c r="F11" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G11" t="n">
-        <v>33.79</v>
+        <v>67.02</v>
       </c>
       <c r="H11" t="n">
-        <v>2.63</v>
+        <v>1.35</v>
       </c>
       <c r="I11" t="n">
-        <v>8.44</v>
+        <v>2.06</v>
       </c>
       <c r="J11" t="n">
         <v>7.91</v>
@@ -988,29 +988,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E17" t="n">
-        <v>41.789</v>
+        <v>105.6</v>
       </c>
       <c r="F17" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G17" t="n">
-        <v>167.16</v>
+        <v>105.6</v>
       </c>
       <c r="H17" t="n">
-        <v>28.14</v>
+        <v>5.51</v>
       </c>
       <c r="I17" t="n">
-        <v>20.24</v>
+        <v>5.51</v>
       </c>
       <c r="J17" t="n">
         <v>7.91</v>
@@ -1022,29 +1022,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C18" t="n">
         <v>3</v>
       </c>
       <c r="D18" t="n">
-        <v>10.387</v>
+        <v>21.89</v>
       </c>
       <c r="E18" t="n">
-        <v>10.662</v>
+        <v>21.915</v>
       </c>
       <c r="F18" t="n">
-        <v>31.16</v>
+        <v>65.67</v>
       </c>
       <c r="G18" t="n">
-        <v>31.99</v>
+        <v>65.75</v>
       </c>
       <c r="H18" t="n">
-        <v>0.83</v>
+        <v>0.08</v>
       </c>
       <c r="I18" t="n">
-        <v>2.66</v>
+        <v>0.12</v>
       </c>
       <c r="J18" t="n">
         <v>7.91</v>
@@ -1056,29 +1056,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>6.239</v>
+        <v>34.755</v>
       </c>
       <c r="E19" t="n">
-        <v>6.82</v>
+        <v>41.789</v>
       </c>
       <c r="F19" t="n">
-        <v>56.15</v>
+        <v>139.02</v>
       </c>
       <c r="G19" t="n">
-        <v>61.38</v>
+        <v>167.16</v>
       </c>
       <c r="H19" t="n">
-        <v>5.23</v>
+        <v>28.14</v>
       </c>
       <c r="I19" t="n">
-        <v>9.31</v>
+        <v>20.24</v>
       </c>
       <c r="J19" t="n">
         <v>7.91</v>
@@ -1090,29 +1090,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C20" t="n">
         <v>3</v>
       </c>
       <c r="D20" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E20" t="n">
-        <v>21.915</v>
+        <v>10.662</v>
       </c>
       <c r="F20" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G20" t="n">
-        <v>65.75</v>
+        <v>31.99</v>
       </c>
       <c r="H20" t="n">
-        <v>0.08</v>
+        <v>0.83</v>
       </c>
       <c r="I20" t="n">
-        <v>0.12</v>
+        <v>2.66</v>
       </c>
       <c r="J20" t="n">
         <v>7.91</v>
@@ -1124,29 +1124,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D21" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E21" t="n">
-        <v>105.6</v>
+        <v>6.82</v>
       </c>
       <c r="F21" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G21" t="n">
-        <v>105.6</v>
+        <v>61.38</v>
       </c>
       <c r="H21" t="n">
-        <v>5.51</v>
+        <v>5.23</v>
       </c>
       <c r="I21" t="n">
-        <v>5.51</v>
+        <v>9.31</v>
       </c>
       <c r="J21" t="n">
         <v>7.91</v>
@@ -1498,29 +1498,29 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C32" t="n">
         <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E32" t="n">
-        <v>22.053</v>
+        <v>10.714</v>
       </c>
       <c r="F32" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G32" t="n">
-        <v>66.16</v>
+        <v>32.14</v>
       </c>
       <c r="H32" t="n">
-        <v>0.49</v>
+        <v>0.98</v>
       </c>
       <c r="I32" t="n">
-        <v>0.75</v>
+        <v>3.15</v>
       </c>
       <c r="J32" t="n">
         <v>7.91</v>
@@ -1532,29 +1532,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D33" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E33" t="n">
-        <v>6.762</v>
+        <v>103.08</v>
       </c>
       <c r="F33" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G33" t="n">
-        <v>60.86</v>
+        <v>103.08</v>
       </c>
       <c r="H33" t="n">
-        <v>4.71</v>
+        <v>2.99</v>
       </c>
       <c r="I33" t="n">
-        <v>8.390000000000001</v>
+        <v>2.99</v>
       </c>
       <c r="J33" t="n">
         <v>7.91</v>
@@ -1566,29 +1566,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D34" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E34" t="n">
-        <v>38.849</v>
+        <v>22.053</v>
       </c>
       <c r="F34" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G34" t="n">
-        <v>155.4</v>
+        <v>66.16</v>
       </c>
       <c r="H34" t="n">
-        <v>16.38</v>
+        <v>0.49</v>
       </c>
       <c r="I34" t="n">
-        <v>11.78</v>
+        <v>0.75</v>
       </c>
       <c r="J34" t="n">
         <v>7.91</v>
@@ -1600,29 +1600,29 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D35" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E35" t="n">
-        <v>103.08</v>
+        <v>6.762</v>
       </c>
       <c r="F35" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G35" t="n">
-        <v>103.08</v>
+        <v>60.86</v>
       </c>
       <c r="H35" t="n">
-        <v>2.99</v>
+        <v>4.71</v>
       </c>
       <c r="I35" t="n">
-        <v>2.99</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="J35" t="n">
         <v>7.91</v>
@@ -1634,29 +1634,29 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D36" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E36" t="n">
-        <v>10.714</v>
+        <v>38.849</v>
       </c>
       <c r="F36" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G36" t="n">
-        <v>32.14</v>
+        <v>155.4</v>
       </c>
       <c r="H36" t="n">
-        <v>0.98</v>
+        <v>16.38</v>
       </c>
       <c r="I36" t="n">
-        <v>3.15</v>
+        <v>11.78</v>
       </c>
       <c r="J36" t="n">
         <v>7.91</v>
@@ -2008,29 +2008,29 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D47" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E47" t="n">
-        <v>99.83</v>
+        <v>21.778</v>
       </c>
       <c r="F47" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G47" t="n">
-        <v>99.83</v>
+        <v>65.33</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.26</v>
+        <v>-0.34</v>
       </c>
       <c r="I47" t="n">
-        <v>-0.26</v>
+        <v>-0.52</v>
       </c>
       <c r="J47" t="n">
         <v>7.91</v>
@@ -2042,29 +2042,29 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D48" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E48" t="n">
-        <v>10.562</v>
+        <v>6.622</v>
       </c>
       <c r="F48" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G48" t="n">
-        <v>31.69</v>
+        <v>59.6</v>
       </c>
       <c r="H48" t="n">
-        <v>0.53</v>
+        <v>3.45</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>6.14</v>
       </c>
       <c r="J48" t="n">
         <v>7.91</v>
@@ -2110,29 +2110,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E50" t="n">
-        <v>6.622</v>
+        <v>99.83</v>
       </c>
       <c r="F50" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G50" t="n">
-        <v>59.6</v>
+        <v>99.83</v>
       </c>
       <c r="H50" t="n">
-        <v>3.45</v>
+        <v>-0.26</v>
       </c>
       <c r="I50" t="n">
-        <v>6.14</v>
+        <v>-0.26</v>
       </c>
       <c r="J50" t="n">
         <v>7.91</v>
@@ -2144,29 +2144,29 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C51" t="n">
         <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>21.89</v>
+        <v>10.387</v>
       </c>
       <c r="E51" t="n">
-        <v>21.778</v>
+        <v>10.562</v>
       </c>
       <c r="F51" t="n">
-        <v>65.67</v>
+        <v>31.16</v>
       </c>
       <c r="G51" t="n">
-        <v>65.33</v>
+        <v>31.69</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.34</v>
+        <v>0.53</v>
       </c>
       <c r="I51" t="n">
-        <v>-0.52</v>
+        <v>1.7</v>
       </c>
       <c r="J51" t="n">
         <v>7.91</v>
@@ -2518,29 +2518,29 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E62" t="n">
-        <v>105.5</v>
+        <v>41.064</v>
       </c>
       <c r="F62" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G62" t="n">
-        <v>105.5</v>
+        <v>164.26</v>
       </c>
       <c r="H62" t="n">
-        <v>5.41</v>
+        <v>25.24</v>
       </c>
       <c r="I62" t="n">
-        <v>5.41</v>
+        <v>18.16</v>
       </c>
       <c r="J62" t="n">
         <v>7.91</v>
@@ -2552,29 +2552,29 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D63" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E63" t="n">
-        <v>10.712</v>
+        <v>6.817</v>
       </c>
       <c r="F63" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G63" t="n">
-        <v>32.14</v>
+        <v>61.35</v>
       </c>
       <c r="H63" t="n">
-        <v>0.98</v>
+        <v>5.2</v>
       </c>
       <c r="I63" t="n">
-        <v>3.15</v>
+        <v>9.26</v>
       </c>
       <c r="J63" t="n">
         <v>7.91</v>
@@ -2586,29 +2586,29 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E64" t="n">
-        <v>22.7</v>
+        <v>105.5</v>
       </c>
       <c r="F64" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G64" t="n">
-        <v>68.09999999999999</v>
+        <v>105.5</v>
       </c>
       <c r="H64" t="n">
-        <v>2.43</v>
+        <v>5.41</v>
       </c>
       <c r="I64" t="n">
-        <v>3.7</v>
+        <v>5.41</v>
       </c>
       <c r="J64" t="n">
         <v>7.91</v>
@@ -2620,29 +2620,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D65" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E65" t="n">
-        <v>6.817</v>
+        <v>10.712</v>
       </c>
       <c r="F65" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G65" t="n">
-        <v>61.35</v>
+        <v>32.14</v>
       </c>
       <c r="H65" t="n">
-        <v>5.2</v>
+        <v>0.98</v>
       </c>
       <c r="I65" t="n">
-        <v>9.26</v>
+        <v>3.15</v>
       </c>
       <c r="J65" t="n">
         <v>7.91</v>
@@ -2654,29 +2654,29 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E66" t="n">
-        <v>41.064</v>
+        <v>22.7</v>
       </c>
       <c r="F66" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G66" t="n">
-        <v>164.26</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="H66" t="n">
-        <v>25.24</v>
+        <v>2.43</v>
       </c>
       <c r="I66" t="n">
-        <v>18.16</v>
+        <v>3.7</v>
       </c>
       <c r="J66" t="n">
         <v>7.91</v>
@@ -3028,29 +3028,29 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D77" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E77" t="n">
-        <v>23.4</v>
+        <v>42.25</v>
       </c>
       <c r="F77" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G77" t="n">
-        <v>70.2</v>
+        <v>169</v>
       </c>
       <c r="H77" t="n">
-        <v>4.53</v>
+        <v>29.98</v>
       </c>
       <c r="I77" t="n">
-        <v>6.9</v>
+        <v>21.57</v>
       </c>
       <c r="J77" t="n">
         <v>7.91</v>
@@ -3062,29 +3062,29 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D78" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E78" t="n">
-        <v>10.958</v>
+        <v>6.836</v>
       </c>
       <c r="F78" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G78" t="n">
-        <v>32.87</v>
+        <v>61.52</v>
       </c>
       <c r="H78" t="n">
-        <v>1.71</v>
+        <v>5.37</v>
       </c>
       <c r="I78" t="n">
-        <v>5.49</v>
+        <v>9.56</v>
       </c>
       <c r="J78" t="n">
         <v>7.91</v>
@@ -3096,29 +3096,29 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D79" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E79" t="n">
-        <v>105.8</v>
+        <v>23.4</v>
       </c>
       <c r="F79" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G79" t="n">
-        <v>105.8</v>
+        <v>70.2</v>
       </c>
       <c r="H79" t="n">
-        <v>5.71</v>
+        <v>4.53</v>
       </c>
       <c r="I79" t="n">
-        <v>5.7</v>
+        <v>6.9</v>
       </c>
       <c r="J79" t="n">
         <v>7.91</v>
@@ -3130,29 +3130,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E80" t="n">
-        <v>6.836</v>
+        <v>10.958</v>
       </c>
       <c r="F80" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G80" t="n">
-        <v>61.52</v>
+        <v>32.87</v>
       </c>
       <c r="H80" t="n">
-        <v>5.37</v>
+        <v>1.71</v>
       </c>
       <c r="I80" t="n">
-        <v>9.56</v>
+        <v>5.49</v>
       </c>
       <c r="J80" t="n">
         <v>7.91</v>
@@ -3164,29 +3164,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D81" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E81" t="n">
-        <v>42.25</v>
+        <v>105.8</v>
       </c>
       <c r="F81" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G81" t="n">
-        <v>169</v>
+        <v>105.8</v>
       </c>
       <c r="H81" t="n">
-        <v>29.98</v>
+        <v>5.71</v>
       </c>
       <c r="I81" t="n">
-        <v>21.57</v>
+        <v>5.7</v>
       </c>
       <c r="J81" t="n">
         <v>7.91</v>
@@ -3538,29 +3538,29 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D92" t="n">
-        <v>100.09</v>
+        <v>34.755</v>
       </c>
       <c r="E92" t="n">
-        <v>103.88</v>
+        <v>40.575</v>
       </c>
       <c r="F92" t="n">
-        <v>100.09</v>
+        <v>139.02</v>
       </c>
       <c r="G92" t="n">
-        <v>103.88</v>
+        <v>162.3</v>
       </c>
       <c r="H92" t="n">
-        <v>3.79</v>
+        <v>23.28</v>
       </c>
       <c r="I92" t="n">
-        <v>3.79</v>
+        <v>16.75</v>
       </c>
       <c r="J92" t="n">
         <v>7.91</v>
@@ -3572,29 +3572,29 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E93" t="n">
-        <v>6.797</v>
+        <v>10.876</v>
       </c>
       <c r="F93" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G93" t="n">
-        <v>61.17</v>
+        <v>32.63</v>
       </c>
       <c r="H93" t="n">
-        <v>5.02</v>
+        <v>1.47</v>
       </c>
       <c r="I93" t="n">
-        <v>8.94</v>
+        <v>4.72</v>
       </c>
       <c r="J93" t="n">
         <v>7.91</v>
@@ -3640,29 +3640,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D95" t="n">
-        <v>34.755</v>
+        <v>100.09</v>
       </c>
       <c r="E95" t="n">
-        <v>40.575</v>
+        <v>103.88</v>
       </c>
       <c r="F95" t="n">
-        <v>139.02</v>
+        <v>100.09</v>
       </c>
       <c r="G95" t="n">
-        <v>162.3</v>
+        <v>103.88</v>
       </c>
       <c r="H95" t="n">
-        <v>23.28</v>
+        <v>3.79</v>
       </c>
       <c r="I95" t="n">
-        <v>16.75</v>
+        <v>3.79</v>
       </c>
       <c r="J95" t="n">
         <v>7.91</v>
@@ -3674,29 +3674,29 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D96" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E96" t="n">
-        <v>10.876</v>
+        <v>6.797</v>
       </c>
       <c r="F96" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G96" t="n">
-        <v>32.63</v>
+        <v>61.17</v>
       </c>
       <c r="H96" t="n">
-        <v>1.47</v>
+        <v>5.02</v>
       </c>
       <c r="I96" t="n">
-        <v>4.72</v>
+        <v>8.94</v>
       </c>
       <c r="J96" t="n">
         <v>7.91</v>
@@ -4048,29 +4048,29 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D107" t="n">
-        <v>21.89</v>
+        <v>6.239</v>
       </c>
       <c r="E107" t="n">
-        <v>23.33</v>
+        <v>6.785</v>
       </c>
       <c r="F107" t="n">
-        <v>65.67</v>
+        <v>56.15</v>
       </c>
       <c r="G107" t="n">
-        <v>69.98999999999999</v>
+        <v>61.06</v>
       </c>
       <c r="H107" t="n">
-        <v>4.32</v>
+        <v>4.91</v>
       </c>
       <c r="I107" t="n">
-        <v>6.58</v>
+        <v>8.74</v>
       </c>
       <c r="J107" t="n">
         <v>7.91</v>
@@ -4082,29 +4082,29 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D108" t="n">
-        <v>10.387</v>
+        <v>100.09</v>
       </c>
       <c r="E108" t="n">
-        <v>10.456</v>
+        <v>103.14</v>
       </c>
       <c r="F108" t="n">
-        <v>31.16</v>
+        <v>100.09</v>
       </c>
       <c r="G108" t="n">
-        <v>31.37</v>
+        <v>103.14</v>
       </c>
       <c r="H108" t="n">
-        <v>0.21</v>
+        <v>3.05</v>
       </c>
       <c r="I108" t="n">
-        <v>0.67</v>
+        <v>3.05</v>
       </c>
       <c r="J108" t="n">
         <v>7.91</v>
@@ -4150,29 +4150,29 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D110" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E110" t="n">
-        <v>103.14</v>
+        <v>23.33</v>
       </c>
       <c r="F110" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G110" t="n">
-        <v>103.14</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="H110" t="n">
-        <v>3.05</v>
+        <v>4.32</v>
       </c>
       <c r="I110" t="n">
-        <v>3.05</v>
+        <v>6.58</v>
       </c>
       <c r="J110" t="n">
         <v>7.91</v>
@@ -4184,29 +4184,29 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D111" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E111" t="n">
-        <v>6.785</v>
+        <v>10.456</v>
       </c>
       <c r="F111" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G111" t="n">
-        <v>61.06</v>
+        <v>31.37</v>
       </c>
       <c r="H111" t="n">
-        <v>4.91</v>
+        <v>0.21</v>
       </c>
       <c r="I111" t="n">
-        <v>8.74</v>
+        <v>0.67</v>
       </c>
       <c r="J111" t="n">
         <v>7.91</v>
@@ -4558,29 +4558,29 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="D122" t="n">
-        <v>100.09</v>
+        <v>6.239</v>
       </c>
       <c r="E122" t="n">
-        <v>106</v>
+        <v>6.901</v>
       </c>
       <c r="F122" t="n">
-        <v>100.09</v>
+        <v>56.15</v>
       </c>
       <c r="G122" t="n">
-        <v>106</v>
+        <v>62.11</v>
       </c>
       <c r="H122" t="n">
-        <v>5.91</v>
+        <v>5.96</v>
       </c>
       <c r="I122" t="n">
-        <v>5.9</v>
+        <v>10.61</v>
       </c>
       <c r="J122" t="n">
         <v>7.91</v>
@@ -4592,29 +4592,29 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D123" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E123" t="n">
-        <v>11.038</v>
+        <v>40.395</v>
       </c>
       <c r="F123" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G123" t="n">
-        <v>33.11</v>
+        <v>161.58</v>
       </c>
       <c r="H123" t="n">
-        <v>1.95</v>
+        <v>22.56</v>
       </c>
       <c r="I123" t="n">
-        <v>6.26</v>
+        <v>16.23</v>
       </c>
       <c r="J123" t="n">
         <v>7.91</v>
@@ -4660,29 +4660,29 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D125" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E125" t="n">
-        <v>40.395</v>
+        <v>11.038</v>
       </c>
       <c r="F125" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G125" t="n">
-        <v>161.58</v>
+        <v>33.11</v>
       </c>
       <c r="H125" t="n">
-        <v>22.56</v>
+        <v>1.95</v>
       </c>
       <c r="I125" t="n">
-        <v>16.23</v>
+        <v>6.26</v>
       </c>
       <c r="J125" t="n">
         <v>7.91</v>
@@ -4694,29 +4694,29 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D126" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E126" t="n">
-        <v>6.901</v>
+        <v>106</v>
       </c>
       <c r="F126" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G126" t="n">
-        <v>62.11</v>
+        <v>106</v>
       </c>
       <c r="H126" t="n">
-        <v>5.96</v>
+        <v>5.91</v>
       </c>
       <c r="I126" t="n">
-        <v>10.61</v>
+        <v>5.9</v>
       </c>
       <c r="J126" t="n">
         <v>7.91</v>
@@ -5068,29 +5068,29 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D137" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E137" t="n">
-        <v>11.728</v>
+        <v>40.61</v>
       </c>
       <c r="F137" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G137" t="n">
-        <v>35.18</v>
+        <v>162.44</v>
       </c>
       <c r="H137" t="n">
-        <v>4.02</v>
+        <v>23.42</v>
       </c>
       <c r="I137" t="n">
-        <v>12.9</v>
+        <v>16.85</v>
       </c>
       <c r="J137" t="n">
         <v>7.91</v>
@@ -5102,29 +5102,29 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D138" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E138" t="n">
-        <v>23.3</v>
+        <v>104.76</v>
       </c>
       <c r="F138" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G138" t="n">
-        <v>69.90000000000001</v>
+        <v>104.76</v>
       </c>
       <c r="H138" t="n">
-        <v>4.23</v>
+        <v>4.67</v>
       </c>
       <c r="I138" t="n">
-        <v>6.44</v>
+        <v>4.67</v>
       </c>
       <c r="J138" t="n">
         <v>7.91</v>
@@ -5170,29 +5170,29 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D140" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E140" t="n">
-        <v>104.76</v>
+        <v>23.3</v>
       </c>
       <c r="F140" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G140" t="n">
-        <v>104.76</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="H140" t="n">
-        <v>4.67</v>
+        <v>4.23</v>
       </c>
       <c r="I140" t="n">
-        <v>4.67</v>
+        <v>6.44</v>
       </c>
       <c r="J140" t="n">
         <v>7.91</v>
@@ -5204,29 +5204,29 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D141" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E141" t="n">
-        <v>40.61</v>
+        <v>11.728</v>
       </c>
       <c r="F141" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G141" t="n">
-        <v>162.44</v>
+        <v>35.18</v>
       </c>
       <c r="H141" t="n">
-        <v>23.42</v>
+        <v>4.02</v>
       </c>
       <c r="I141" t="n">
-        <v>16.85</v>
+        <v>12.9</v>
       </c>
       <c r="J141" t="n">
         <v>7.91</v>
@@ -5578,29 +5578,29 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D152" t="n">
-        <v>10.387</v>
+        <v>34.755</v>
       </c>
       <c r="E152" t="n">
-        <v>11.034</v>
+        <v>39.915</v>
       </c>
       <c r="F152" t="n">
-        <v>31.16</v>
+        <v>139.02</v>
       </c>
       <c r="G152" t="n">
-        <v>33.1</v>
+        <v>159.66</v>
       </c>
       <c r="H152" t="n">
-        <v>1.94</v>
+        <v>20.64</v>
       </c>
       <c r="I152" t="n">
-        <v>6.23</v>
+        <v>14.85</v>
       </c>
       <c r="J152" t="n">
         <v>7.91</v>
@@ -5612,29 +5612,29 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D153" t="n">
-        <v>100.09</v>
+        <v>21.89</v>
       </c>
       <c r="E153" t="n">
-        <v>104.12</v>
+        <v>23.045</v>
       </c>
       <c r="F153" t="n">
-        <v>100.09</v>
+        <v>65.67</v>
       </c>
       <c r="G153" t="n">
-        <v>104.12</v>
+        <v>69.14</v>
       </c>
       <c r="H153" t="n">
-        <v>4.03</v>
+        <v>3.47</v>
       </c>
       <c r="I153" t="n">
-        <v>4.03</v>
+        <v>5.28</v>
       </c>
       <c r="J153" t="n">
         <v>7.91</v>
@@ -5680,29 +5680,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D155" t="n">
-        <v>21.89</v>
+        <v>100.09</v>
       </c>
       <c r="E155" t="n">
-        <v>23.045</v>
+        <v>104.12</v>
       </c>
       <c r="F155" t="n">
-        <v>65.67</v>
+        <v>100.09</v>
       </c>
       <c r="G155" t="n">
-        <v>69.14</v>
+        <v>104.12</v>
       </c>
       <c r="H155" t="n">
-        <v>3.47</v>
+        <v>4.03</v>
       </c>
       <c r="I155" t="n">
-        <v>5.28</v>
+        <v>4.03</v>
       </c>
       <c r="J155" t="n">
         <v>7.91</v>
@@ -5714,29 +5714,29 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D156" t="n">
-        <v>34.755</v>
+        <v>10.387</v>
       </c>
       <c r="E156" t="n">
-        <v>39.915</v>
+        <v>11.034</v>
       </c>
       <c r="F156" t="n">
-        <v>139.02</v>
+        <v>31.16</v>
       </c>
       <c r="G156" t="n">
-        <v>159.66</v>
+        <v>33.1</v>
       </c>
       <c r="H156" t="n">
-        <v>20.64</v>
+        <v>1.94</v>
       </c>
       <c r="I156" t="n">
-        <v>14.85</v>
+        <v>6.23</v>
       </c>
       <c r="J156" t="n">
         <v>7.91</v>
@@ -6088,29 +6088,29 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E167" t="n">
-        <v>22.92</v>
+        <v>38.98</v>
       </c>
       <c r="F167" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G167" t="n">
-        <v>68.76000000000001</v>
+        <v>155.92</v>
       </c>
       <c r="H167" t="n">
-        <v>3.09</v>
+        <v>16.9</v>
       </c>
       <c r="I167" t="n">
-        <v>4.71</v>
+        <v>12.16</v>
       </c>
       <c r="J167" t="n">
         <v>7.91</v>
@@ -6122,29 +6122,29 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>EFENSE</t>
+          <t>IWSC</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D168" t="n">
-        <v>10.387</v>
+        <v>6.239</v>
       </c>
       <c r="E168" t="n">
-        <v>10.726</v>
+        <v>6.911</v>
       </c>
       <c r="F168" t="n">
-        <v>31.16</v>
+        <v>56.15</v>
       </c>
       <c r="G168" t="n">
-        <v>32.18</v>
+        <v>62.2</v>
       </c>
       <c r="H168" t="n">
-        <v>1.02</v>
+        <v>6.05</v>
       </c>
       <c r="I168" t="n">
-        <v>3.27</v>
+        <v>10.77</v>
       </c>
       <c r="J168" t="n">
         <v>7.91</v>
@@ -6190,29 +6190,29 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="D170" t="n">
-        <v>6.239</v>
+        <v>10.387</v>
       </c>
       <c r="E170" t="n">
-        <v>6.911</v>
+        <v>10.726</v>
       </c>
       <c r="F170" t="n">
-        <v>56.15</v>
+        <v>31.16</v>
       </c>
       <c r="G170" t="n">
-        <v>62.2</v>
+        <v>32.18</v>
       </c>
       <c r="H170" t="n">
-        <v>6.05</v>
+        <v>1.02</v>
       </c>
       <c r="I170" t="n">
-        <v>10.77</v>
+        <v>3.27</v>
       </c>
       <c r="J170" t="n">
         <v>7.91</v>
@@ -6224,29 +6224,29 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>PAASI</t>
+          <t>PINDIA</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D171" t="n">
-        <v>34.755</v>
+        <v>21.89</v>
       </c>
       <c r="E171" t="n">
-        <v>38.98</v>
+        <v>22.92</v>
       </c>
       <c r="F171" t="n">
-        <v>139.02</v>
+        <v>65.67</v>
       </c>
       <c r="G171" t="n">
-        <v>155.92</v>
+        <v>68.76000000000001</v>
       </c>
       <c r="H171" t="n">
-        <v>16.9</v>
+        <v>3.09</v>
       </c>
       <c r="I171" t="n">
-        <v>12.16</v>
+        <v>4.71</v>
       </c>
       <c r="J171" t="n">
         <v>7.91</v>
@@ -6598,29 +6598,29 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>PINDIA</t>
+          <t>PAASI</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D182" t="n">
-        <v>21.89</v>
+        <v>34.755</v>
       </c>
       <c r="E182" t="n">
-        <v>22.835</v>
+        <v>37.235</v>
       </c>
       <c r="F182" t="n">
-        <v>65.67</v>
+        <v>139.02</v>
       </c>
       <c r="G182" t="n">
-        <v>68.5</v>
+        <v>148.94</v>
       </c>
       <c r="H182" t="n">
-        <v>2.83</v>
+        <v>9.92</v>
       </c>
       <c r="I182" t="n">
-        <v>4.31</v>
+        <v>7.14</v>
       </c>
       <c r="J182" t="n">
         <v>7.91</v>
@@ -6632,29 +6632,29 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>IWSC</t>
+          <t>PUST</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="D183" t="n">
-        <v>6.239</v>
+        <v>100.09</v>
       </c>
       <c r="E183" t="n">
-        <v>6.848</v>
+        <v>100.14</v>
       </c>
       <c r="F183" t="n">
-        <v>56.15</v>
+        <v>100.09</v>
       </c>
       <c r="G183" t="n">
-        <v>61.63</v>
+        <v>100.14</v>
       </c>
       <c r="H183" t="n">
-        <v>5.48</v>
+        <v>0.05</v>
       </c>
       <c r="I183" t="n">
-        <v>9.76</v>
+        <v>0.05</v>
       </c>
       <c r="J183" t="n">
         <v>7.91</v>
@@ -6666,29 +6666,29 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>PUST</t>
+          <t>EFENSE</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D184" t="n">
-        <v>100.09</v>
+        <v>10.387</v>
       </c>
       <c r="E184" t="n">
-        <v>100.14</v>
+        <v>10.776</v>
       </c>
       <c r="F184" t="n">
-        <v>100.09</v>
+        <v>31.16</v>
       </c>
       <c r="G184" t="n">
-        <v>100.14</v>
+        <v>32.33</v>
       </c>
       <c r="H184" t="n">
-        <v>0.05</v>
+       